<commit_message>
fix: sablon ondalik ayrac talimati duzeltildi, KT-001 (Kuveyt Turk) girisi tamamlandi
Onceki talimat "ondalik ayraci NOKTA" diyordu ama Turkce Excel'de
ondalik ayraci VIRGULDUR. Nokta ile giris yapinca Excel degeri binlik
ayraci sanip yanlis okuyor ya da 0-100 dogrulama araligindan reddediyordu.

Sayfa 1 talimati, sutun basligi yorumlari ve DataValidation hata
mesajlari virgul kullanacak sekilde guncellendi.

KT-001 (Kuveyt Turk, Taksitlio kampanyasi) ilk gercek altin veri kaydi
olarak tamamlandi: kar_payi_orani=2.99, maliyet_orani=4.191 (BSMV/KKDF
dahil), vade_ay=6, finansman_tutari=100000, kampanya_turu duzeltildi
(Konut -> Finansman Kampanyasi, kampanya alisveris finansmani oldugu
icin).
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -324,12 +324,12 @@
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>SADECE SAYI. Ornek: 1.99 (yuzde isareti yazma) - bankanin vurguladigi ham oran</t>
+        <t>SADECE SAYI, virgulle. Ornek: 1,99 (yuzde isareti yazma) - bankanin vurguladigi ham oran</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>SADECE SAYI. BSMV/KKDF dahil GERCEK maliyet orani; sayfada yoksa BOS birak</t>
+        <t>SADECE SAYI, virgulle. BSMV/KKDF dahil GERCEK maliyet orani; sayfada yoksa BOS birak</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -349,7 +349,7 @@
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>SADECE SAYI. Ornek: 10000</t>
+        <t>SADECE SAYI, virgulle (kesirli ise). Ornek: 10000</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
@@ -983,19 +983,19 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>DOGRU: 1.89      YANLIS: %1,89 / 1,89% / yuzde 1.89          DOGRU: 120      YANLIS: 120 Ay / 120ay</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
+          <t>DOGRU: 1,89      YANLIS: %1,89 / 1,89% / yuzde 1,89          DOGRU: 120      YANLIS: 120 Ay / 120ay</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Ondalik ayraci NOKTA</t>
+          <t>Ondalik ayraci VIRGUL (Excel'in kendi kurali)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>DOGRU: 1.89      YANLIS: 1,89      (virgul kullanirsan Python sayi olarak okuyamaz)</t>
+          <t>Excel'iniz Turkce bolgesel ayarli oldugu icin ondalik ayraci VIRGULDUR: 1,89 yazin, 1.89 DEGIL. Nokta yazarsaniz Excel bunu binlik ayraci sanip 189 okur ya da hucre 0-100 dogrulamasindan reddeder. Ekranda virgul gorunmesi sorun degil - JSON'a aktarilirken sistem gercek sayiyi (1.89) otomatik yazar.</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="F2" s="13" t="inlineStr">
         <is>
-          <t>SADECE SAYI. Ornek: 1.99 (yuzde isareti yazma) - bankanin vurguladigi ham oran</t>
+          <t>SADECE SAYI, virgulle. Ornek: 1,99 (yuzde isareti yazma) - bankanin vurguladigi ham oran</t>
         </is>
       </c>
       <c r="G2" s="13" t="inlineStr">
         <is>
-          <t>SADECE SAYI. BSMV/KKDF dahil GERCEK maliyet orani; sayfada yoksa BOS birak</t>
+          <t>SADECE SAYI, virgulle. BSMV/KKDF dahil GERCEK maliyet orani; sayfada yoksa BOS birak</t>
         </is>
       </c>
       <c r="H2" s="13" t="inlineStr">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="K2" s="13" t="inlineStr">
         <is>
-          <t>SADECE SAYI. Ornek: 10000</t>
+          <t>SADECE SAYI, virgulle (kesirli ise). Ornek: 10000</t>
         </is>
       </c>
       <c r="L2" s="13" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>Konut Finansmani Kampanyasi</t>
+          <t>Finansman Kampanyasi</t>
         </is>
       </c>
       <c r="E7" s="18" t="inlineStr">
@@ -1794,23 +1794,65 @@
         </is>
       </c>
       <c r="F7" s="20" t="n">
-        <v>1.99</v>
-      </c>
-      <c r="G7" s="20" t="n"/>
-      <c r="H7" s="18" t="n"/>
-      <c r="I7" s="21" t="n"/>
-      <c r="J7" s="20" t="n"/>
+        <v>2.99</v>
+      </c>
+      <c r="G7" s="20" t="n">
+        <v>4.191</v>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>aylik</t>
+        </is>
+      </c>
+      <c r="I7" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7" s="20" t="n">
+        <v>100000</v>
+      </c>
       <c r="K7" s="20" t="n"/>
       <c r="L7" s="18" t="n"/>
-      <c r="M7" s="19" t="n"/>
+      <c r="M7" s="19" t="inlineStr">
+        <is>
+          <t>Taksitlio anlaşmalı mağazalarda 6 taksite kadar avantajlı kâr payı oranı</t>
+        </is>
+      </c>
       <c r="N7" s="19" t="n"/>
-      <c r="O7" s="18" t="n"/>
-      <c r="P7" s="18" t="n"/>
-      <c r="Q7" s="19" t="n"/>
-      <c r="R7" s="18" t="n"/>
-      <c r="S7" s="18" t="n"/>
-      <c r="T7" s="18" t="n"/>
-      <c r="U7" s="19" t="n"/>
+      <c r="O7" s="18" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="P7" s="18" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q7" s="19" t="inlineStr">
+        <is>
+          <t>Yeni müşteri (son 30 gün)</t>
+        </is>
+      </c>
+      <c r="R7" s="18" t="inlineStr">
+        <is>
+          <t>KT-001.png</t>
+        </is>
+      </c>
+      <c r="S7" s="18" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T7" s="18" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U7" s="19" t="inlineStr">
+        <is>
+          <t>Kar payi orani %2,99 ama vergiler dahil maliyet %4,1910 - sayfa ikisini ayri veriyor</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="22" t="n"/>
@@ -2859,7 +2901,7 @@
     <dataValidation sqref="L3:L52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz odul birimi" error="Listeden bir birim secin." type="list">
       <formula1>"TL,Mil,Gram,Puan,Worldpuan,ParafPara,Bankkart Lira"</formula1>
     </dataValidation>
-    <dataValidation sqref="F3:F52 G3:G52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz oran" error="Sadece 0-100 arasi sayi yazin (yuzde isareti olmadan). Ornek: 1.99" type="decimal" operator="between">
+    <dataValidation sqref="F3:F52 G3:G52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz oran" error="Sadece 0-100 arasi sayi yazin, VIRGULLE (yuzde isareti olmadan). Ornek: 1,99" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat: Kuveyt Turk icin 6 yeni altin veri kaydi (KT-002..KT-007), tarih format duzeltmesi
Finansman kampanyalari: TOGG is birligi (KT-002), Tarim leasing (KT-003,
sayfada somut oran/vade olmadigi icin ilgili alanlar bos birakildi),
Diyanet Umre vade farksiz 3 taksit (KT-004).

Kart/musteri kampanyalari: 10.000 Mil'e varan firsat (KT-005, rapor
Bolum 3'teki Mil gozlemini dogruluyor), Yeni Saglam Kart Troy vade
farksiz 5 taksit (KT-006), Davet kodu 750 TL (KT-007).

Ayrica: kampanya_baslangic, kampanya_bitis, giris_tarihi sutunlarina
acik "yyyy-mm-dd" number_format atandi. Onceden Excel elle girilen
tarihi gercek tarih tipine cevirip Turkce varsayilan (GG.AA.YYYY) ile
gosteriyordu; bu artik onlendi.

Banka basina hedef (5-8 kayit) Kuveyt Turk icin karsilandi: 7 kayit.
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -21,7 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="14">
     <font>
       <name val="Calibri"/>
@@ -148,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -193,6 +195,9 @@
     <xf numFmtId="1" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -205,9 +210,13 @@
     <xf numFmtId="1" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1203,7 +1212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U52"/>
+  <dimension ref="A1:U58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1494,12 +1503,12 @@
           <t>Dosya masrafi yok</t>
         </is>
       </c>
-      <c r="O3" s="14" t="inlineStr">
+      <c r="O3" s="18" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="P3" s="14" t="inlineStr">
+      <c r="P3" s="18" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
@@ -1519,7 +1528,7 @@
           <t>ORNEK</t>
         </is>
       </c>
-      <c r="T3" s="14" t="inlineStr">
+      <c r="T3" s="18" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -1581,8 +1590,8 @@
           <t>Ekspertiz ucretsiz</t>
         </is>
       </c>
-      <c r="O4" s="14" t="n"/>
-      <c r="P4" s="14" t="n"/>
+      <c r="O4" s="18" t="n"/>
+      <c r="P4" s="18" t="n"/>
       <c r="Q4" s="15" t="n"/>
       <c r="R4" s="14" t="inlineStr">
         <is>
@@ -1594,7 +1603,7 @@
           <t>ORNEK</t>
         </is>
       </c>
-      <c r="T4" s="14" t="inlineStr">
+      <c r="T4" s="18" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -1658,8 +1667,8 @@
         </is>
       </c>
       <c r="N5" s="15" t="n"/>
-      <c r="O5" s="14" t="n"/>
-      <c r="P5" s="14" t="n"/>
+      <c r="O5" s="18" t="n"/>
+      <c r="P5" s="18" t="n"/>
       <c r="Q5" s="15" t="inlineStr">
         <is>
           <t>Yeni konut alimi yapanlar</t>
@@ -1675,7 +1684,7 @@
           <t>ORNEK</t>
         </is>
       </c>
-      <c r="T5" s="14" t="inlineStr">
+      <c r="T5" s="18" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -1731,12 +1740,12 @@
         </is>
       </c>
       <c r="N6" s="15" t="n"/>
-      <c r="O6" s="14" t="inlineStr">
+      <c r="O6" s="18" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="P6" s="14" t="inlineStr">
+      <c r="P6" s="18" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
@@ -1756,7 +1765,7 @@
           <t>ORNEK</t>
         </is>
       </c>
-      <c r="T6" s="14" t="inlineStr">
+      <c r="T6" s="18" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -1768,1148 +1777,1624 @@
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>KT-001</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Kuveyt Türk</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>Taksitlio'da Yeni Müşterilere Özel Kuveyt Türk Alışveriş Finansmanı Fırsatı!</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D7" s="19" t="inlineStr">
         <is>
           <t>Finansman Kampanyasi</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/finansman-kampanyalari/taksitlioda-yeni-musterilere-ozel-kuveyt-turk-alisveris-finansmani-firsati</t>
         </is>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="21" t="n">
         <v>2.99</v>
       </c>
-      <c r="G7" s="20" t="n">
+      <c r="G7" s="21" t="n">
         <v>4.191</v>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="H7" s="19" t="inlineStr">
         <is>
           <t>aylik</t>
         </is>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="J7" s="20" t="n">
+      <c r="J7" s="21" t="n">
         <v>100000</v>
       </c>
-      <c r="K7" s="20" t="n"/>
-      <c r="L7" s="18" t="n"/>
-      <c r="M7" s="19" t="inlineStr">
+      <c r="K7" s="21" t="n"/>
+      <c r="L7" s="19" t="n"/>
+      <c r="M7" s="20" t="inlineStr">
         <is>
           <t>Taksitlio anlaşmalı mağazalarda 6 taksite kadar avantajlı kâr payı oranı</t>
         </is>
       </c>
-      <c r="N7" s="19" t="n"/>
-      <c r="O7" s="18" t="inlineStr">
+      <c r="N7" s="20" t="n"/>
+      <c r="O7" s="23" t="inlineStr">
         <is>
           <t>2026-01-20</t>
         </is>
       </c>
-      <c r="P7" s="18" t="inlineStr">
+      <c r="P7" s="23" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="Q7" s="19" t="inlineStr">
+      <c r="Q7" s="20" t="inlineStr">
         <is>
           <t>Yeni müşteri (son 30 gün)</t>
         </is>
       </c>
-      <c r="R7" s="18" t="inlineStr">
+      <c r="R7" s="19" t="inlineStr">
         <is>
           <t>KT-001.png</t>
         </is>
       </c>
-      <c r="S7" s="18" t="inlineStr">
+      <c r="S7" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
         </is>
       </c>
-      <c r="T7" s="18" t="inlineStr">
+      <c r="T7" s="23" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="U7" s="19" t="inlineStr">
+      <c r="U7" s="20" t="inlineStr">
         <is>
           <t>Kar payi orani %2,99 ama vergiler dahil maliyet %4,1910 - sayfa ikisini ayri veriyor</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="22" t="n"/>
-      <c r="B8" s="22" t="n"/>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="22" t="n"/>
-      <c r="E8" s="22" t="n"/>
-      <c r="F8" s="23" t="n"/>
-      <c r="G8" s="23" t="n"/>
-      <c r="H8" s="22" t="n"/>
-      <c r="I8" s="24" t="n"/>
-      <c r="J8" s="23" t="n"/>
-      <c r="K8" s="23" t="n"/>
-      <c r="L8" s="22" t="n"/>
-      <c r="M8" s="22" t="n"/>
-      <c r="N8" s="22" t="n"/>
-      <c r="O8" s="22" t="n"/>
-      <c r="P8" s="22" t="n"/>
-      <c r="Q8" s="22" t="n"/>
-      <c r="R8" s="22" t="n"/>
-      <c r="S8" s="22" t="n"/>
-      <c r="T8" s="22" t="n"/>
-      <c r="U8" s="22" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="22" t="n"/>
-      <c r="B9" s="22" t="n"/>
-      <c r="C9" s="22" t="n"/>
-      <c r="D9" s="22" t="n"/>
-      <c r="E9" s="22" t="n"/>
-      <c r="F9" s="23" t="n"/>
-      <c r="G9" s="23" t="n"/>
-      <c r="H9" s="22" t="n"/>
-      <c r="I9" s="24" t="n"/>
-      <c r="J9" s="23" t="n"/>
-      <c r="K9" s="23" t="n"/>
-      <c r="L9" s="22" t="n"/>
-      <c r="M9" s="22" t="n"/>
-      <c r="N9" s="22" t="n"/>
-      <c r="O9" s="22" t="n"/>
-      <c r="P9" s="22" t="n"/>
-      <c r="Q9" s="22" t="n"/>
-      <c r="R9" s="22" t="n"/>
-      <c r="S9" s="22" t="n"/>
-      <c r="T9" s="22" t="n"/>
-      <c r="U9" s="22" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="22" t="n"/>
-      <c r="B10" s="22" t="n"/>
-      <c r="C10" s="22" t="n"/>
-      <c r="D10" s="22" t="n"/>
-      <c r="E10" s="22" t="n"/>
-      <c r="F10" s="23" t="n"/>
-      <c r="G10" s="23" t="n"/>
-      <c r="H10" s="22" t="n"/>
-      <c r="I10" s="24" t="n"/>
-      <c r="J10" s="23" t="n"/>
-      <c r="K10" s="23" t="n"/>
-      <c r="L10" s="22" t="n"/>
-      <c r="M10" s="22" t="n"/>
-      <c r="N10" s="22" t="n"/>
-      <c r="O10" s="22" t="n"/>
-      <c r="P10" s="22" t="n"/>
-      <c r="Q10" s="22" t="n"/>
-      <c r="R10" s="22" t="n"/>
-      <c r="S10" s="22" t="n"/>
-      <c r="T10" s="22" t="n"/>
-      <c r="U10" s="22" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="22" t="n"/>
-      <c r="B11" s="22" t="n"/>
-      <c r="C11" s="22" t="n"/>
-      <c r="D11" s="22" t="n"/>
-      <c r="E11" s="22" t="n"/>
-      <c r="F11" s="23" t="n"/>
-      <c r="G11" s="23" t="n"/>
-      <c r="H11" s="22" t="n"/>
-      <c r="I11" s="24" t="n"/>
-      <c r="J11" s="23" t="n"/>
-      <c r="K11" s="23" t="n"/>
-      <c r="L11" s="22" t="n"/>
-      <c r="M11" s="22" t="n"/>
-      <c r="N11" s="22" t="n"/>
-      <c r="O11" s="22" t="n"/>
-      <c r="P11" s="22" t="n"/>
-      <c r="Q11" s="22" t="n"/>
-      <c r="R11" s="22" t="n"/>
-      <c r="S11" s="22" t="n"/>
-      <c r="T11" s="22" t="n"/>
-      <c r="U11" s="22" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="22" t="n"/>
-      <c r="B12" s="22" t="n"/>
-      <c r="C12" s="22" t="n"/>
-      <c r="D12" s="22" t="n"/>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="23" t="n"/>
-      <c r="G12" s="23" t="n"/>
-      <c r="H12" s="22" t="n"/>
-      <c r="I12" s="24" t="n"/>
-      <c r="J12" s="23" t="n"/>
-      <c r="K12" s="23" t="n"/>
-      <c r="L12" s="22" t="n"/>
-      <c r="M12" s="22" t="n"/>
-      <c r="N12" s="22" t="n"/>
-      <c r="O12" s="22" t="n"/>
-      <c r="P12" s="22" t="n"/>
-      <c r="Q12" s="22" t="n"/>
-      <c r="R12" s="22" t="n"/>
-      <c r="S12" s="22" t="n"/>
-      <c r="T12" s="22" t="n"/>
-      <c r="U12" s="22" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="22" t="n"/>
-      <c r="B13" s="22" t="n"/>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="22" t="n"/>
-      <c r="F13" s="23" t="n"/>
-      <c r="G13" s="23" t="n"/>
-      <c r="H13" s="22" t="n"/>
-      <c r="I13" s="24" t="n"/>
-      <c r="J13" s="23" t="n"/>
-      <c r="K13" s="23" t="n"/>
-      <c r="L13" s="22" t="n"/>
-      <c r="M13" s="22" t="n"/>
-      <c r="N13" s="22" t="n"/>
-      <c r="O13" s="22" t="n"/>
-      <c r="P13" s="22" t="n"/>
-      <c r="Q13" s="22" t="n"/>
-      <c r="R13" s="22" t="n"/>
-      <c r="S13" s="22" t="n"/>
-      <c r="T13" s="22" t="n"/>
-      <c r="U13" s="22" t="n"/>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>KT-002</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk ve TOGG İş Birliği</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Tasit Finansmani Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/finansman-kampanyalari/kuveyt-turk-ve-togg-is-birligi</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>aylik</t>
+        </is>
+      </c>
+      <c r="I8" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="J8" s="21" t="n">
+        <v>750000</v>
+      </c>
+      <c r="K8" s="21" t="n"/>
+      <c r="L8" s="19" t="n"/>
+      <c r="M8" s="20" t="inlineStr">
+        <is>
+          <t>750.000 TL'lik TOGG finansmanı 12 ay vadede %0 kâr payı ile</t>
+        </is>
+      </c>
+      <c r="N8" s="20" t="inlineStr">
+        <is>
+          <t>Örnek tabloda toplam masraf 3.750 TL (750.000 TL, 12 ay vade için)</t>
+        </is>
+      </c>
+      <c r="O8" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P8" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="Q8" s="20" t="n"/>
+      <c r="R8" s="19" t="inlineStr">
+        <is>
+          <t>KT-002.png</t>
+        </is>
+      </c>
+      <c r="S8" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T8" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U8" s="20" t="inlineStr">
+        <is>
+          <t>12-48 ay arasi, %0 ile %3,50 arasi oranlar, sigorta ürünleri sartina bağli.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>KT-003</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>Tarımda Kuveyt Türk ile Büyüme Zamanı!</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Finansman Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/finansman-kampanyalari/tarimda-kuveyt-turk-ile-buyume-zamani</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="n"/>
+      <c r="G9" s="21" t="n"/>
+      <c r="H9" s="19" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="21" t="n"/>
+      <c r="K9" s="21" t="n"/>
+      <c r="L9" s="19" t="n"/>
+      <c r="M9" s="20" t="inlineStr">
+        <is>
+          <t>Tarım makine/ekipman/üretim yatırımlarında Leasing finansmanı; esnek ödeme, ödemesiz dönem, hasada uygun geri ödeme planı</t>
+        </is>
+      </c>
+      <c r="N9" s="20" t="n"/>
+      <c r="O9" s="23" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="P9" s="23" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q9" s="20" t="inlineStr">
+        <is>
+          <t>Tarım sektörü / çiftçiler</t>
+        </is>
+      </c>
+      <c r="R9" s="19" t="inlineStr">
+        <is>
+          <t>KT-003.png</t>
+        </is>
+      </c>
+      <c r="S9" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T9" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U9" s="20" t="inlineStr">
+        <is>
+          <t>Rapor Bölüm 3'ün gözlemini doğruluyor: genel tanıtım sayfası, kampanyaya özel somut oran/vade YOK - şeffaflık ilkesi gereği boş bırakıldı</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>KT-004</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>Diyanet Umre Finansmanı ile Vade Farksız 3 Taksit İmkanı!</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Ihtiyac Finansmani Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/finansman-kampanyalari/diyanet-umre-finansmani-ile-vade-farksiz-3-taksit-imkani</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="n"/>
+      <c r="G10" s="21" t="n"/>
+      <c r="H10" s="19" t="n"/>
+      <c r="I10" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" s="21" t="n"/>
+      <c r="K10" s="21" t="n"/>
+      <c r="L10" s="19" t="n"/>
+      <c r="M10" s="20" t="inlineStr">
+        <is>
+          <t>Umre tutarının en fazla %60'ı için vade farksız 3 taksit</t>
+        </is>
+      </c>
+      <c r="N10" s="20" t="n"/>
+      <c r="O10" s="23" t="inlineStr">
+        <is>
+          <t>2024-08-13</t>
+        </is>
+      </c>
+      <c r="P10" s="23" t="inlineStr">
+        <is>
+          <t>2027-01-01</t>
+        </is>
+      </c>
+      <c r="Q10" s="20" t="n"/>
+      <c r="R10" s="19" t="inlineStr">
+        <is>
+          <t>KT-004.png</t>
+        </is>
+      </c>
+      <c r="S10" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T10" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U10" s="20" t="inlineStr">
+        <is>
+          <t>Diyanetten alınan umre tur kodu şart</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>KT-005</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>Yeni Kuveyt Türk Mobil Müşterilerine 10.000 Mil'e Varan Fırsat!</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/yeni-kuveyt-turk-mobil-musterilerine-10000-mile-varan-firsat</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="n"/>
+      <c r="G11" s="21" t="n"/>
+      <c r="H11" s="19" t="n"/>
+      <c r="I11" s="22" t="n"/>
+      <c r="J11" s="21" t="n"/>
+      <c r="K11" s="21" t="n">
+        <v>10000</v>
+      </c>
+      <c r="L11" s="19" t="inlineStr">
+        <is>
+          <t>Mil</t>
+        </is>
+      </c>
+      <c r="M11" s="20" t="inlineStr">
+        <is>
+          <t>Miles&amp;Smiles kredi kartıyla ilk 1.000 TL+ harcamaya, kart limitine göre kademeli mil: ≤100.000 TL limit → 3.000 Mil, 100-300 bin TL → 6.000 Mil, 300 bin TL üzeri → 10.000 Mil</t>
+        </is>
+      </c>
+      <c r="N11" s="20" t="n"/>
+      <c r="O11" s="23" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="P11" s="23" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q11" s="20" t="inlineStr">
+        <is>
+          <t>30.04.2026 sonrası mobilden yeni müşteri olan, Miles&amp;Smiles kart sahipleri</t>
+        </is>
+      </c>
+      <c r="R11" s="19" t="inlineStr">
+        <is>
+          <t>KT-005.png</t>
+        </is>
+      </c>
+      <c r="S11" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T11" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U11" s="20" t="inlineStr">
+        <is>
+          <t>Bu kayıt raporun Bölüm 3'teki "Mil" ödül birimi gözlemini doğruluyor</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>KT-006</t>
+        </is>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C12" s="20" t="inlineStr">
+        <is>
+          <t>Yeni Sağlam Kart Troy'lulara Özel Vade Farksız 5 Aya Varan Taksit İmkanı!</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/yeni-saglam-kart-troylulara-ozel-vade-farksiz-5-aya-varan-taksit-imkani</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="n"/>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="19" t="n"/>
+      <c r="I12" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" s="21" t="n">
+        <v>50000</v>
+      </c>
+      <c r="K12" s="21" t="n"/>
+      <c r="L12" s="19" t="n"/>
+      <c r="M12" s="20" t="inlineStr">
+        <is>
+          <t>Eğitim/Sağlık harcamalarında ayda 2 işlem + yeni kart sahiplerine sektör kısıtsız 1 taksitlendirme hakkı, vade farksız 2-5 taksit</t>
+        </is>
+      </c>
+      <c r="N12" s="20" t="n"/>
+      <c r="O12" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="P12" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="Q12" s="20" t="inlineStr">
+        <is>
+          <t>Yeni Sağlam Kart Troy müşterileri (1-31 Temmuz 2026 arası kart alanlar)</t>
+        </is>
+      </c>
+      <c r="R12" s="19" t="inlineStr">
+        <is>
+          <t>KT-006.png</t>
+        </is>
+      </c>
+      <c r="S12" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T12" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U12" s="20" t="inlineStr">
+        <is>
+          <t>vade_ay alanı burada "taksit sayısı" anlamında kullanıldı, klasik kredi vadesi değil - CampaignRecord şemasıyla tam örtüşmüyor, ekiple bu ayrımı konuşmak gerekebilir</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>KT-007</t>
+        </is>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>Davet Kodunla Gel, Memnuniyet Anketine Katıl, 750 TL Kazan!</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Yeni Musteri Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/davet-kodunla-gel-memnuniyet-anketine-katil-750-tl-kazan</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="n"/>
+      <c r="G13" s="21" t="n"/>
+      <c r="H13" s="19" t="n"/>
+      <c r="I13" s="22" t="n"/>
+      <c r="J13" s="21" t="n"/>
+      <c r="K13" s="21" t="n">
+        <v>750</v>
+      </c>
+      <c r="L13" s="19" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M13" s="20" t="inlineStr">
+        <is>
+          <t>Davet kodu ile müşteri olup 500 TL+ harcamaya 500 TL iade + memnuniyet anketine katılıma 250 TL ek hediye = toplam 750 TL</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="n"/>
+      <c r="O13" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P13" s="23" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q13" s="20" t="inlineStr">
+        <is>
+          <t>Davet kodu ile mobilden yeni müşteri olanlar</t>
+        </is>
+      </c>
+      <c r="R13" s="19" t="inlineStr">
+        <is>
+          <t>KT-007.png</t>
+        </is>
+      </c>
+      <c r="S13" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T13" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U13" s="20" t="inlineStr">
+        <is>
+          <t>Kampanyadan yalnızca bir kez yararlanılabilir</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="n"/>
-      <c r="B14" s="22" t="n"/>
-      <c r="C14" s="22" t="n"/>
-      <c r="D14" s="22" t="n"/>
-      <c r="E14" s="22" t="n"/>
-      <c r="F14" s="23" t="n"/>
-      <c r="G14" s="23" t="n"/>
-      <c r="H14" s="22" t="n"/>
-      <c r="I14" s="24" t="n"/>
-      <c r="J14" s="23" t="n"/>
-      <c r="K14" s="23" t="n"/>
-      <c r="L14" s="22" t="n"/>
-      <c r="M14" s="22" t="n"/>
-      <c r="N14" s="22" t="n"/>
-      <c r="O14" s="22" t="n"/>
-      <c r="P14" s="22" t="n"/>
-      <c r="Q14" s="22" t="n"/>
-      <c r="R14" s="22" t="n"/>
-      <c r="S14" s="22" t="n"/>
-      <c r="T14" s="22" t="n"/>
-      <c r="U14" s="22" t="n"/>
+      <c r="A14" s="24" t="n"/>
+      <c r="B14" s="24" t="n"/>
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="24" t="n"/>
+      <c r="F14" s="25" t="n"/>
+      <c r="G14" s="25" t="n"/>
+      <c r="H14" s="24" t="n"/>
+      <c r="I14" s="26" t="n"/>
+      <c r="J14" s="25" t="n"/>
+      <c r="K14" s="25" t="n"/>
+      <c r="L14" s="24" t="n"/>
+      <c r="M14" s="24" t="n"/>
+      <c r="N14" s="24" t="n"/>
+      <c r="O14" s="27" t="n"/>
+      <c r="P14" s="27" t="n"/>
+      <c r="Q14" s="24" t="n"/>
+      <c r="R14" s="24" t="n"/>
+      <c r="S14" s="24" t="n"/>
+      <c r="T14" s="27" t="n"/>
+      <c r="U14" s="24" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="n"/>
-      <c r="B15" s="22" t="n"/>
-      <c r="C15" s="22" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="22" t="n"/>
-      <c r="F15" s="23" t="n"/>
-      <c r="G15" s="23" t="n"/>
-      <c r="H15" s="22" t="n"/>
-      <c r="I15" s="24" t="n"/>
-      <c r="J15" s="23" t="n"/>
-      <c r="K15" s="23" t="n"/>
-      <c r="L15" s="22" t="n"/>
-      <c r="M15" s="22" t="n"/>
-      <c r="N15" s="22" t="n"/>
-      <c r="O15" s="22" t="n"/>
-      <c r="P15" s="22" t="n"/>
-      <c r="Q15" s="22" t="n"/>
-      <c r="R15" s="22" t="n"/>
-      <c r="S15" s="22" t="n"/>
-      <c r="T15" s="22" t="n"/>
-      <c r="U15" s="22" t="n"/>
+      <c r="A15" s="24" t="n"/>
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="24" t="n"/>
+      <c r="E15" s="24" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="24" t="n"/>
+      <c r="I15" s="26" t="n"/>
+      <c r="J15" s="25" t="n"/>
+      <c r="K15" s="25" t="n"/>
+      <c r="L15" s="24" t="n"/>
+      <c r="M15" s="24" t="n"/>
+      <c r="N15" s="24" t="n"/>
+      <c r="O15" s="27" t="n"/>
+      <c r="P15" s="27" t="n"/>
+      <c r="Q15" s="24" t="n"/>
+      <c r="R15" s="24" t="n"/>
+      <c r="S15" s="24" t="n"/>
+      <c r="T15" s="27" t="n"/>
+      <c r="U15" s="24" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="n"/>
-      <c r="B16" s="22" t="n"/>
-      <c r="C16" s="22" t="n"/>
-      <c r="D16" s="22" t="n"/>
-      <c r="E16" s="22" t="n"/>
-      <c r="F16" s="23" t="n"/>
-      <c r="G16" s="23" t="n"/>
-      <c r="H16" s="22" t="n"/>
-      <c r="I16" s="24" t="n"/>
-      <c r="J16" s="23" t="n"/>
-      <c r="K16" s="23" t="n"/>
-      <c r="L16" s="22" t="n"/>
-      <c r="M16" s="22" t="n"/>
-      <c r="N16" s="22" t="n"/>
-      <c r="O16" s="22" t="n"/>
-      <c r="P16" s="22" t="n"/>
-      <c r="Q16" s="22" t="n"/>
-      <c r="R16" s="22" t="n"/>
-      <c r="S16" s="22" t="n"/>
-      <c r="T16" s="22" t="n"/>
-      <c r="U16" s="22" t="n"/>
+      <c r="A16" s="24" t="n"/>
+      <c r="B16" s="24" t="n"/>
+      <c r="C16" s="24" t="n"/>
+      <c r="D16" s="24" t="n"/>
+      <c r="E16" s="24" t="n"/>
+      <c r="F16" s="25" t="n"/>
+      <c r="G16" s="25" t="n"/>
+      <c r="H16" s="24" t="n"/>
+      <c r="I16" s="26" t="n"/>
+      <c r="J16" s="25" t="n"/>
+      <c r="K16" s="25" t="n"/>
+      <c r="L16" s="24" t="n"/>
+      <c r="M16" s="24" t="n"/>
+      <c r="N16" s="24" t="n"/>
+      <c r="O16" s="27" t="n"/>
+      <c r="P16" s="27" t="n"/>
+      <c r="Q16" s="24" t="n"/>
+      <c r="R16" s="24" t="n"/>
+      <c r="S16" s="24" t="n"/>
+      <c r="T16" s="27" t="n"/>
+      <c r="U16" s="24" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="n"/>
-      <c r="B17" s="22" t="n"/>
-      <c r="C17" s="22" t="n"/>
-      <c r="D17" s="22" t="n"/>
-      <c r="E17" s="22" t="n"/>
-      <c r="F17" s="23" t="n"/>
-      <c r="G17" s="23" t="n"/>
-      <c r="H17" s="22" t="n"/>
-      <c r="I17" s="24" t="n"/>
-      <c r="J17" s="23" t="n"/>
-      <c r="K17" s="23" t="n"/>
-      <c r="L17" s="22" t="n"/>
-      <c r="M17" s="22" t="n"/>
-      <c r="N17" s="22" t="n"/>
-      <c r="O17" s="22" t="n"/>
-      <c r="P17" s="22" t="n"/>
-      <c r="Q17" s="22" t="n"/>
-      <c r="R17" s="22" t="n"/>
-      <c r="S17" s="22" t="n"/>
-      <c r="T17" s="22" t="n"/>
-      <c r="U17" s="22" t="n"/>
+      <c r="A17" s="24" t="n"/>
+      <c r="B17" s="24" t="n"/>
+      <c r="C17" s="24" t="n"/>
+      <c r="D17" s="24" t="n"/>
+      <c r="E17" s="24" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="24" t="n"/>
+      <c r="I17" s="26" t="n"/>
+      <c r="J17" s="25" t="n"/>
+      <c r="K17" s="25" t="n"/>
+      <c r="L17" s="24" t="n"/>
+      <c r="M17" s="24" t="n"/>
+      <c r="N17" s="24" t="n"/>
+      <c r="O17" s="27" t="n"/>
+      <c r="P17" s="27" t="n"/>
+      <c r="Q17" s="24" t="n"/>
+      <c r="R17" s="24" t="n"/>
+      <c r="S17" s="24" t="n"/>
+      <c r="T17" s="27" t="n"/>
+      <c r="U17" s="24" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="n"/>
-      <c r="B18" s="22" t="n"/>
-      <c r="C18" s="22" t="n"/>
-      <c r="D18" s="22" t="n"/>
-      <c r="E18" s="22" t="n"/>
-      <c r="F18" s="23" t="n"/>
-      <c r="G18" s="23" t="n"/>
-      <c r="H18" s="22" t="n"/>
-      <c r="I18" s="24" t="n"/>
-      <c r="J18" s="23" t="n"/>
-      <c r="K18" s="23" t="n"/>
-      <c r="L18" s="22" t="n"/>
-      <c r="M18" s="22" t="n"/>
-      <c r="N18" s="22" t="n"/>
-      <c r="O18" s="22" t="n"/>
-      <c r="P18" s="22" t="n"/>
-      <c r="Q18" s="22" t="n"/>
-      <c r="R18" s="22" t="n"/>
-      <c r="S18" s="22" t="n"/>
-      <c r="T18" s="22" t="n"/>
-      <c r="U18" s="22" t="n"/>
+      <c r="A18" s="24" t="n"/>
+      <c r="B18" s="24" t="n"/>
+      <c r="C18" s="24" t="n"/>
+      <c r="D18" s="24" t="n"/>
+      <c r="E18" s="24" t="n"/>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="24" t="n"/>
+      <c r="I18" s="26" t="n"/>
+      <c r="J18" s="25" t="n"/>
+      <c r="K18" s="25" t="n"/>
+      <c r="L18" s="24" t="n"/>
+      <c r="M18" s="24" t="n"/>
+      <c r="N18" s="24" t="n"/>
+      <c r="O18" s="27" t="n"/>
+      <c r="P18" s="27" t="n"/>
+      <c r="Q18" s="24" t="n"/>
+      <c r="R18" s="24" t="n"/>
+      <c r="S18" s="24" t="n"/>
+      <c r="T18" s="27" t="n"/>
+      <c r="U18" s="24" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="n"/>
-      <c r="B19" s="22" t="n"/>
-      <c r="C19" s="22" t="n"/>
-      <c r="D19" s="22" t="n"/>
-      <c r="E19" s="22" t="n"/>
-      <c r="F19" s="23" t="n"/>
-      <c r="G19" s="23" t="n"/>
-      <c r="H19" s="22" t="n"/>
-      <c r="I19" s="24" t="n"/>
-      <c r="J19" s="23" t="n"/>
-      <c r="K19" s="23" t="n"/>
-      <c r="L19" s="22" t="n"/>
-      <c r="M19" s="22" t="n"/>
-      <c r="N19" s="22" t="n"/>
-      <c r="O19" s="22" t="n"/>
-      <c r="P19" s="22" t="n"/>
-      <c r="Q19" s="22" t="n"/>
-      <c r="R19" s="22" t="n"/>
-      <c r="S19" s="22" t="n"/>
-      <c r="T19" s="22" t="n"/>
-      <c r="U19" s="22" t="n"/>
+      <c r="A19" s="24" t="n"/>
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="24" t="n"/>
+      <c r="F19" s="25" t="n"/>
+      <c r="G19" s="25" t="n"/>
+      <c r="H19" s="24" t="n"/>
+      <c r="I19" s="26" t="n"/>
+      <c r="J19" s="25" t="n"/>
+      <c r="K19" s="25" t="n"/>
+      <c r="L19" s="24" t="n"/>
+      <c r="M19" s="24" t="n"/>
+      <c r="N19" s="24" t="n"/>
+      <c r="O19" s="27" t="n"/>
+      <c r="P19" s="27" t="n"/>
+      <c r="Q19" s="24" t="n"/>
+      <c r="R19" s="24" t="n"/>
+      <c r="S19" s="24" t="n"/>
+      <c r="T19" s="27" t="n"/>
+      <c r="U19" s="24" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="n"/>
-      <c r="B20" s="22" t="n"/>
-      <c r="C20" s="22" t="n"/>
-      <c r="D20" s="22" t="n"/>
-      <c r="E20" s="22" t="n"/>
-      <c r="F20" s="23" t="n"/>
-      <c r="G20" s="23" t="n"/>
-      <c r="H20" s="22" t="n"/>
-      <c r="I20" s="24" t="n"/>
-      <c r="J20" s="23" t="n"/>
-      <c r="K20" s="23" t="n"/>
-      <c r="L20" s="22" t="n"/>
-      <c r="M20" s="22" t="n"/>
-      <c r="N20" s="22" t="n"/>
-      <c r="O20" s="22" t="n"/>
-      <c r="P20" s="22" t="n"/>
-      <c r="Q20" s="22" t="n"/>
-      <c r="R20" s="22" t="n"/>
-      <c r="S20" s="22" t="n"/>
-      <c r="T20" s="22" t="n"/>
-      <c r="U20" s="22" t="n"/>
+      <c r="A20" s="24" t="n"/>
+      <c r="B20" s="24" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="24" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="24" t="n"/>
+      <c r="I20" s="26" t="n"/>
+      <c r="J20" s="25" t="n"/>
+      <c r="K20" s="25" t="n"/>
+      <c r="L20" s="24" t="n"/>
+      <c r="M20" s="24" t="n"/>
+      <c r="N20" s="24" t="n"/>
+      <c r="O20" s="27" t="n"/>
+      <c r="P20" s="27" t="n"/>
+      <c r="Q20" s="24" t="n"/>
+      <c r="R20" s="24" t="n"/>
+      <c r="S20" s="24" t="n"/>
+      <c r="T20" s="27" t="n"/>
+      <c r="U20" s="24" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="22" t="n"/>
-      <c r="B21" s="22" t="n"/>
-      <c r="C21" s="22" t="n"/>
-      <c r="D21" s="22" t="n"/>
-      <c r="E21" s="22" t="n"/>
-      <c r="F21" s="23" t="n"/>
-      <c r="G21" s="23" t="n"/>
-      <c r="H21" s="22" t="n"/>
-      <c r="I21" s="24" t="n"/>
-      <c r="J21" s="23" t="n"/>
-      <c r="K21" s="23" t="n"/>
-      <c r="L21" s="22" t="n"/>
-      <c r="M21" s="22" t="n"/>
-      <c r="N21" s="22" t="n"/>
-      <c r="O21" s="22" t="n"/>
-      <c r="P21" s="22" t="n"/>
-      <c r="Q21" s="22" t="n"/>
-      <c r="R21" s="22" t="n"/>
-      <c r="S21" s="22" t="n"/>
-      <c r="T21" s="22" t="n"/>
-      <c r="U21" s="22" t="n"/>
+      <c r="A21" s="24" t="n"/>
+      <c r="B21" s="24" t="n"/>
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="24" t="n"/>
+      <c r="E21" s="24" t="n"/>
+      <c r="F21" s="25" t="n"/>
+      <c r="G21" s="25" t="n"/>
+      <c r="H21" s="24" t="n"/>
+      <c r="I21" s="26" t="n"/>
+      <c r="J21" s="25" t="n"/>
+      <c r="K21" s="25" t="n"/>
+      <c r="L21" s="24" t="n"/>
+      <c r="M21" s="24" t="n"/>
+      <c r="N21" s="24" t="n"/>
+      <c r="O21" s="27" t="n"/>
+      <c r="P21" s="27" t="n"/>
+      <c r="Q21" s="24" t="n"/>
+      <c r="R21" s="24" t="n"/>
+      <c r="S21" s="24" t="n"/>
+      <c r="T21" s="27" t="n"/>
+      <c r="U21" s="24" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="n"/>
-      <c r="B22" s="22" t="n"/>
-      <c r="C22" s="22" t="n"/>
-      <c r="D22" s="22" t="n"/>
-      <c r="E22" s="22" t="n"/>
-      <c r="F22" s="23" t="n"/>
-      <c r="G22" s="23" t="n"/>
-      <c r="H22" s="22" t="n"/>
-      <c r="I22" s="24" t="n"/>
-      <c r="J22" s="23" t="n"/>
-      <c r="K22" s="23" t="n"/>
-      <c r="L22" s="22" t="n"/>
-      <c r="M22" s="22" t="n"/>
-      <c r="N22" s="22" t="n"/>
-      <c r="O22" s="22" t="n"/>
-      <c r="P22" s="22" t="n"/>
-      <c r="Q22" s="22" t="n"/>
-      <c r="R22" s="22" t="n"/>
-      <c r="S22" s="22" t="n"/>
-      <c r="T22" s="22" t="n"/>
-      <c r="U22" s="22" t="n"/>
+      <c r="A22" s="24" t="n"/>
+      <c r="B22" s="24" t="n"/>
+      <c r="C22" s="24" t="n"/>
+      <c r="D22" s="24" t="n"/>
+      <c r="E22" s="24" t="n"/>
+      <c r="F22" s="25" t="n"/>
+      <c r="G22" s="25" t="n"/>
+      <c r="H22" s="24" t="n"/>
+      <c r="I22" s="26" t="n"/>
+      <c r="J22" s="25" t="n"/>
+      <c r="K22" s="25" t="n"/>
+      <c r="L22" s="24" t="n"/>
+      <c r="M22" s="24" t="n"/>
+      <c r="N22" s="24" t="n"/>
+      <c r="O22" s="27" t="n"/>
+      <c r="P22" s="27" t="n"/>
+      <c r="Q22" s="24" t="n"/>
+      <c r="R22" s="24" t="n"/>
+      <c r="S22" s="24" t="n"/>
+      <c r="T22" s="27" t="n"/>
+      <c r="U22" s="24" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="22" t="n"/>
-      <c r="B23" s="22" t="n"/>
-      <c r="C23" s="22" t="n"/>
-      <c r="D23" s="22" t="n"/>
-      <c r="E23" s="22" t="n"/>
-      <c r="F23" s="23" t="n"/>
-      <c r="G23" s="23" t="n"/>
-      <c r="H23" s="22" t="n"/>
-      <c r="I23" s="24" t="n"/>
-      <c r="J23" s="23" t="n"/>
-      <c r="K23" s="23" t="n"/>
-      <c r="L23" s="22" t="n"/>
-      <c r="M23" s="22" t="n"/>
-      <c r="N23" s="22" t="n"/>
-      <c r="O23" s="22" t="n"/>
-      <c r="P23" s="22" t="n"/>
-      <c r="Q23" s="22" t="n"/>
-      <c r="R23" s="22" t="n"/>
-      <c r="S23" s="22" t="n"/>
-      <c r="T23" s="22" t="n"/>
-      <c r="U23" s="22" t="n"/>
+      <c r="A23" s="24" t="n"/>
+      <c r="B23" s="24" t="n"/>
+      <c r="C23" s="24" t="n"/>
+      <c r="D23" s="24" t="n"/>
+      <c r="E23" s="24" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="24" t="n"/>
+      <c r="I23" s="26" t="n"/>
+      <c r="J23" s="25" t="n"/>
+      <c r="K23" s="25" t="n"/>
+      <c r="L23" s="24" t="n"/>
+      <c r="M23" s="24" t="n"/>
+      <c r="N23" s="24" t="n"/>
+      <c r="O23" s="27" t="n"/>
+      <c r="P23" s="27" t="n"/>
+      <c r="Q23" s="24" t="n"/>
+      <c r="R23" s="24" t="n"/>
+      <c r="S23" s="24" t="n"/>
+      <c r="T23" s="27" t="n"/>
+      <c r="U23" s="24" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="n"/>
-      <c r="B24" s="22" t="n"/>
-      <c r="C24" s="22" t="n"/>
-      <c r="D24" s="22" t="n"/>
-      <c r="E24" s="22" t="n"/>
-      <c r="F24" s="23" t="n"/>
-      <c r="G24" s="23" t="n"/>
-      <c r="H24" s="22" t="n"/>
-      <c r="I24" s="24" t="n"/>
-      <c r="J24" s="23" t="n"/>
-      <c r="K24" s="23" t="n"/>
-      <c r="L24" s="22" t="n"/>
-      <c r="M24" s="22" t="n"/>
-      <c r="N24" s="22" t="n"/>
-      <c r="O24" s="22" t="n"/>
-      <c r="P24" s="22" t="n"/>
-      <c r="Q24" s="22" t="n"/>
-      <c r="R24" s="22" t="n"/>
-      <c r="S24" s="22" t="n"/>
-      <c r="T24" s="22" t="n"/>
-      <c r="U24" s="22" t="n"/>
+      <c r="A24" s="24" t="n"/>
+      <c r="B24" s="24" t="n"/>
+      <c r="C24" s="24" t="n"/>
+      <c r="D24" s="24" t="n"/>
+      <c r="E24" s="24" t="n"/>
+      <c r="F24" s="25" t="n"/>
+      <c r="G24" s="25" t="n"/>
+      <c r="H24" s="24" t="n"/>
+      <c r="I24" s="26" t="n"/>
+      <c r="J24" s="25" t="n"/>
+      <c r="K24" s="25" t="n"/>
+      <c r="L24" s="24" t="n"/>
+      <c r="M24" s="24" t="n"/>
+      <c r="N24" s="24" t="n"/>
+      <c r="O24" s="27" t="n"/>
+      <c r="P24" s="27" t="n"/>
+      <c r="Q24" s="24" t="n"/>
+      <c r="R24" s="24" t="n"/>
+      <c r="S24" s="24" t="n"/>
+      <c r="T24" s="27" t="n"/>
+      <c r="U24" s="24" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="n"/>
-      <c r="B25" s="22" t="n"/>
-      <c r="C25" s="22" t="n"/>
-      <c r="D25" s="22" t="n"/>
-      <c r="E25" s="22" t="n"/>
-      <c r="F25" s="23" t="n"/>
-      <c r="G25" s="23" t="n"/>
-      <c r="H25" s="22" t="n"/>
-      <c r="I25" s="24" t="n"/>
-      <c r="J25" s="23" t="n"/>
-      <c r="K25" s="23" t="n"/>
-      <c r="L25" s="22" t="n"/>
-      <c r="M25" s="22" t="n"/>
-      <c r="N25" s="22" t="n"/>
-      <c r="O25" s="22" t="n"/>
-      <c r="P25" s="22" t="n"/>
-      <c r="Q25" s="22" t="n"/>
-      <c r="R25" s="22" t="n"/>
-      <c r="S25" s="22" t="n"/>
-      <c r="T25" s="22" t="n"/>
-      <c r="U25" s="22" t="n"/>
+      <c r="A25" s="24" t="n"/>
+      <c r="B25" s="24" t="n"/>
+      <c r="C25" s="24" t="n"/>
+      <c r="D25" s="24" t="n"/>
+      <c r="E25" s="24" t="n"/>
+      <c r="F25" s="25" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="24" t="n"/>
+      <c r="I25" s="26" t="n"/>
+      <c r="J25" s="25" t="n"/>
+      <c r="K25" s="25" t="n"/>
+      <c r="L25" s="24" t="n"/>
+      <c r="M25" s="24" t="n"/>
+      <c r="N25" s="24" t="n"/>
+      <c r="O25" s="27" t="n"/>
+      <c r="P25" s="27" t="n"/>
+      <c r="Q25" s="24" t="n"/>
+      <c r="R25" s="24" t="n"/>
+      <c r="S25" s="24" t="n"/>
+      <c r="T25" s="27" t="n"/>
+      <c r="U25" s="24" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="22" t="n"/>
-      <c r="B26" s="22" t="n"/>
-      <c r="C26" s="22" t="n"/>
-      <c r="D26" s="22" t="n"/>
-      <c r="E26" s="22" t="n"/>
-      <c r="F26" s="23" t="n"/>
-      <c r="G26" s="23" t="n"/>
-      <c r="H26" s="22" t="n"/>
-      <c r="I26" s="24" t="n"/>
-      <c r="J26" s="23" t="n"/>
-      <c r="K26" s="23" t="n"/>
-      <c r="L26" s="22" t="n"/>
-      <c r="M26" s="22" t="n"/>
-      <c r="N26" s="22" t="n"/>
-      <c r="O26" s="22" t="n"/>
-      <c r="P26" s="22" t="n"/>
-      <c r="Q26" s="22" t="n"/>
-      <c r="R26" s="22" t="n"/>
-      <c r="S26" s="22" t="n"/>
-      <c r="T26" s="22" t="n"/>
-      <c r="U26" s="22" t="n"/>
+      <c r="A26" s="24" t="n"/>
+      <c r="B26" s="24" t="n"/>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="24" t="n"/>
+      <c r="F26" s="25" t="n"/>
+      <c r="G26" s="25" t="n"/>
+      <c r="H26" s="24" t="n"/>
+      <c r="I26" s="26" t="n"/>
+      <c r="J26" s="25" t="n"/>
+      <c r="K26" s="25" t="n"/>
+      <c r="L26" s="24" t="n"/>
+      <c r="M26" s="24" t="n"/>
+      <c r="N26" s="24" t="n"/>
+      <c r="O26" s="27" t="n"/>
+      <c r="P26" s="27" t="n"/>
+      <c r="Q26" s="24" t="n"/>
+      <c r="R26" s="24" t="n"/>
+      <c r="S26" s="24" t="n"/>
+      <c r="T26" s="27" t="n"/>
+      <c r="U26" s="24" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="n"/>
-      <c r="B27" s="22" t="n"/>
-      <c r="C27" s="22" t="n"/>
-      <c r="D27" s="22" t="n"/>
-      <c r="E27" s="22" t="n"/>
-      <c r="F27" s="23" t="n"/>
-      <c r="G27" s="23" t="n"/>
-      <c r="H27" s="22" t="n"/>
-      <c r="I27" s="24" t="n"/>
-      <c r="J27" s="23" t="n"/>
-      <c r="K27" s="23" t="n"/>
-      <c r="L27" s="22" t="n"/>
-      <c r="M27" s="22" t="n"/>
-      <c r="N27" s="22" t="n"/>
-      <c r="O27" s="22" t="n"/>
-      <c r="P27" s="22" t="n"/>
-      <c r="Q27" s="22" t="n"/>
-      <c r="R27" s="22" t="n"/>
-      <c r="S27" s="22" t="n"/>
-      <c r="T27" s="22" t="n"/>
-      <c r="U27" s="22" t="n"/>
+      <c r="A27" s="24" t="n"/>
+      <c r="B27" s="24" t="n"/>
+      <c r="C27" s="24" t="n"/>
+      <c r="D27" s="24" t="n"/>
+      <c r="E27" s="24" t="n"/>
+      <c r="F27" s="25" t="n"/>
+      <c r="G27" s="25" t="n"/>
+      <c r="H27" s="24" t="n"/>
+      <c r="I27" s="26" t="n"/>
+      <c r="J27" s="25" t="n"/>
+      <c r="K27" s="25" t="n"/>
+      <c r="L27" s="24" t="n"/>
+      <c r="M27" s="24" t="n"/>
+      <c r="N27" s="24" t="n"/>
+      <c r="O27" s="27" t="n"/>
+      <c r="P27" s="27" t="n"/>
+      <c r="Q27" s="24" t="n"/>
+      <c r="R27" s="24" t="n"/>
+      <c r="S27" s="24" t="n"/>
+      <c r="T27" s="27" t="n"/>
+      <c r="U27" s="24" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="n"/>
-      <c r="B28" s="22" t="n"/>
-      <c r="C28" s="22" t="n"/>
-      <c r="D28" s="22" t="n"/>
-      <c r="E28" s="22" t="n"/>
-      <c r="F28" s="23" t="n"/>
-      <c r="G28" s="23" t="n"/>
-      <c r="H28" s="22" t="n"/>
-      <c r="I28" s="24" t="n"/>
-      <c r="J28" s="23" t="n"/>
-      <c r="K28" s="23" t="n"/>
-      <c r="L28" s="22" t="n"/>
-      <c r="M28" s="22" t="n"/>
-      <c r="N28" s="22" t="n"/>
-      <c r="O28" s="22" t="n"/>
-      <c r="P28" s="22" t="n"/>
-      <c r="Q28" s="22" t="n"/>
-      <c r="R28" s="22" t="n"/>
-      <c r="S28" s="22" t="n"/>
-      <c r="T28" s="22" t="n"/>
-      <c r="U28" s="22" t="n"/>
+      <c r="A28" s="24" t="n"/>
+      <c r="B28" s="24" t="n"/>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="24" t="n"/>
+      <c r="F28" s="25" t="n"/>
+      <c r="G28" s="25" t="n"/>
+      <c r="H28" s="24" t="n"/>
+      <c r="I28" s="26" t="n"/>
+      <c r="J28" s="25" t="n"/>
+      <c r="K28" s="25" t="n"/>
+      <c r="L28" s="24" t="n"/>
+      <c r="M28" s="24" t="n"/>
+      <c r="N28" s="24" t="n"/>
+      <c r="O28" s="27" t="n"/>
+      <c r="P28" s="27" t="n"/>
+      <c r="Q28" s="24" t="n"/>
+      <c r="R28" s="24" t="n"/>
+      <c r="S28" s="24" t="n"/>
+      <c r="T28" s="27" t="n"/>
+      <c r="U28" s="24" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="22" t="n"/>
-      <c r="B29" s="22" t="n"/>
-      <c r="C29" s="22" t="n"/>
-      <c r="D29" s="22" t="n"/>
-      <c r="E29" s="22" t="n"/>
-      <c r="F29" s="23" t="n"/>
-      <c r="G29" s="23" t="n"/>
-      <c r="H29" s="22" t="n"/>
-      <c r="I29" s="24" t="n"/>
-      <c r="J29" s="23" t="n"/>
-      <c r="K29" s="23" t="n"/>
-      <c r="L29" s="22" t="n"/>
-      <c r="M29" s="22" t="n"/>
-      <c r="N29" s="22" t="n"/>
-      <c r="O29" s="22" t="n"/>
-      <c r="P29" s="22" t="n"/>
-      <c r="Q29" s="22" t="n"/>
-      <c r="R29" s="22" t="n"/>
-      <c r="S29" s="22" t="n"/>
-      <c r="T29" s="22" t="n"/>
-      <c r="U29" s="22" t="n"/>
+      <c r="A29" s="24" t="n"/>
+      <c r="B29" s="24" t="n"/>
+      <c r="C29" s="24" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="24" t="n"/>
+      <c r="F29" s="25" t="n"/>
+      <c r="G29" s="25" t="n"/>
+      <c r="H29" s="24" t="n"/>
+      <c r="I29" s="26" t="n"/>
+      <c r="J29" s="25" t="n"/>
+      <c r="K29" s="25" t="n"/>
+      <c r="L29" s="24" t="n"/>
+      <c r="M29" s="24" t="n"/>
+      <c r="N29" s="24" t="n"/>
+      <c r="O29" s="27" t="n"/>
+      <c r="P29" s="27" t="n"/>
+      <c r="Q29" s="24" t="n"/>
+      <c r="R29" s="24" t="n"/>
+      <c r="S29" s="24" t="n"/>
+      <c r="T29" s="27" t="n"/>
+      <c r="U29" s="24" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="n"/>
-      <c r="B30" s="22" t="n"/>
-      <c r="C30" s="22" t="n"/>
-      <c r="D30" s="22" t="n"/>
-      <c r="E30" s="22" t="n"/>
-      <c r="F30" s="23" t="n"/>
-      <c r="G30" s="23" t="n"/>
-      <c r="H30" s="22" t="n"/>
-      <c r="I30" s="24" t="n"/>
-      <c r="J30" s="23" t="n"/>
-      <c r="K30" s="23" t="n"/>
-      <c r="L30" s="22" t="n"/>
-      <c r="M30" s="22" t="n"/>
-      <c r="N30" s="22" t="n"/>
-      <c r="O30" s="22" t="n"/>
-      <c r="P30" s="22" t="n"/>
-      <c r="Q30" s="22" t="n"/>
-      <c r="R30" s="22" t="n"/>
-      <c r="S30" s="22" t="n"/>
-      <c r="T30" s="22" t="n"/>
-      <c r="U30" s="22" t="n"/>
+      <c r="A30" s="24" t="n"/>
+      <c r="B30" s="24" t="n"/>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="24" t="n"/>
+      <c r="F30" s="25" t="n"/>
+      <c r="G30" s="25" t="n"/>
+      <c r="H30" s="24" t="n"/>
+      <c r="I30" s="26" t="n"/>
+      <c r="J30" s="25" t="n"/>
+      <c r="K30" s="25" t="n"/>
+      <c r="L30" s="24" t="n"/>
+      <c r="M30" s="24" t="n"/>
+      <c r="N30" s="24" t="n"/>
+      <c r="O30" s="27" t="n"/>
+      <c r="P30" s="27" t="n"/>
+      <c r="Q30" s="24" t="n"/>
+      <c r="R30" s="24" t="n"/>
+      <c r="S30" s="24" t="n"/>
+      <c r="T30" s="27" t="n"/>
+      <c r="U30" s="24" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="22" t="n"/>
-      <c r="B31" s="22" t="n"/>
-      <c r="C31" s="22" t="n"/>
-      <c r="D31" s="22" t="n"/>
-      <c r="E31" s="22" t="n"/>
-      <c r="F31" s="23" t="n"/>
-      <c r="G31" s="23" t="n"/>
-      <c r="H31" s="22" t="n"/>
-      <c r="I31" s="24" t="n"/>
-      <c r="J31" s="23" t="n"/>
-      <c r="K31" s="23" t="n"/>
-      <c r="L31" s="22" t="n"/>
-      <c r="M31" s="22" t="n"/>
-      <c r="N31" s="22" t="n"/>
-      <c r="O31" s="22" t="n"/>
-      <c r="P31" s="22" t="n"/>
-      <c r="Q31" s="22" t="n"/>
-      <c r="R31" s="22" t="n"/>
-      <c r="S31" s="22" t="n"/>
-      <c r="T31" s="22" t="n"/>
-      <c r="U31" s="22" t="n"/>
+      <c r="A31" s="24" t="n"/>
+      <c r="B31" s="24" t="n"/>
+      <c r="C31" s="24" t="n"/>
+      <c r="D31" s="24" t="n"/>
+      <c r="E31" s="24" t="n"/>
+      <c r="F31" s="25" t="n"/>
+      <c r="G31" s="25" t="n"/>
+      <c r="H31" s="24" t="n"/>
+      <c r="I31" s="26" t="n"/>
+      <c r="J31" s="25" t="n"/>
+      <c r="K31" s="25" t="n"/>
+      <c r="L31" s="24" t="n"/>
+      <c r="M31" s="24" t="n"/>
+      <c r="N31" s="24" t="n"/>
+      <c r="O31" s="27" t="n"/>
+      <c r="P31" s="27" t="n"/>
+      <c r="Q31" s="24" t="n"/>
+      <c r="R31" s="24" t="n"/>
+      <c r="S31" s="24" t="n"/>
+      <c r="T31" s="27" t="n"/>
+      <c r="U31" s="24" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="22" t="n"/>
-      <c r="B32" s="22" t="n"/>
-      <c r="C32" s="22" t="n"/>
-      <c r="D32" s="22" t="n"/>
-      <c r="E32" s="22" t="n"/>
-      <c r="F32" s="23" t="n"/>
-      <c r="G32" s="23" t="n"/>
-      <c r="H32" s="22" t="n"/>
-      <c r="I32" s="24" t="n"/>
-      <c r="J32" s="23" t="n"/>
-      <c r="K32" s="23" t="n"/>
-      <c r="L32" s="22" t="n"/>
-      <c r="M32" s="22" t="n"/>
-      <c r="N32" s="22" t="n"/>
-      <c r="O32" s="22" t="n"/>
-      <c r="P32" s="22" t="n"/>
-      <c r="Q32" s="22" t="n"/>
-      <c r="R32" s="22" t="n"/>
-      <c r="S32" s="22" t="n"/>
-      <c r="T32" s="22" t="n"/>
-      <c r="U32" s="22" t="n"/>
+      <c r="A32" s="24" t="n"/>
+      <c r="B32" s="24" t="n"/>
+      <c r="C32" s="24" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="25" t="n"/>
+      <c r="G32" s="25" t="n"/>
+      <c r="H32" s="24" t="n"/>
+      <c r="I32" s="26" t="n"/>
+      <c r="J32" s="25" t="n"/>
+      <c r="K32" s="25" t="n"/>
+      <c r="L32" s="24" t="n"/>
+      <c r="M32" s="24" t="n"/>
+      <c r="N32" s="24" t="n"/>
+      <c r="O32" s="27" t="n"/>
+      <c r="P32" s="27" t="n"/>
+      <c r="Q32" s="24" t="n"/>
+      <c r="R32" s="24" t="n"/>
+      <c r="S32" s="24" t="n"/>
+      <c r="T32" s="27" t="n"/>
+      <c r="U32" s="24" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="22" t="n"/>
-      <c r="B33" s="22" t="n"/>
-      <c r="C33" s="22" t="n"/>
-      <c r="D33" s="22" t="n"/>
-      <c r="E33" s="22" t="n"/>
-      <c r="F33" s="23" t="n"/>
-      <c r="G33" s="23" t="n"/>
-      <c r="H33" s="22" t="n"/>
-      <c r="I33" s="24" t="n"/>
-      <c r="J33" s="23" t="n"/>
-      <c r="K33" s="23" t="n"/>
-      <c r="L33" s="22" t="n"/>
-      <c r="M33" s="22" t="n"/>
-      <c r="N33" s="22" t="n"/>
-      <c r="O33" s="22" t="n"/>
-      <c r="P33" s="22" t="n"/>
-      <c r="Q33" s="22" t="n"/>
-      <c r="R33" s="22" t="n"/>
-      <c r="S33" s="22" t="n"/>
-      <c r="T33" s="22" t="n"/>
-      <c r="U33" s="22" t="n"/>
+      <c r="A33" s="24" t="n"/>
+      <c r="B33" s="24" t="n"/>
+      <c r="C33" s="24" t="n"/>
+      <c r="D33" s="24" t="n"/>
+      <c r="E33" s="24" t="n"/>
+      <c r="F33" s="25" t="n"/>
+      <c r="G33" s="25" t="n"/>
+      <c r="H33" s="24" t="n"/>
+      <c r="I33" s="26" t="n"/>
+      <c r="J33" s="25" t="n"/>
+      <c r="K33" s="25" t="n"/>
+      <c r="L33" s="24" t="n"/>
+      <c r="M33" s="24" t="n"/>
+      <c r="N33" s="24" t="n"/>
+      <c r="O33" s="27" t="n"/>
+      <c r="P33" s="27" t="n"/>
+      <c r="Q33" s="24" t="n"/>
+      <c r="R33" s="24" t="n"/>
+      <c r="S33" s="24" t="n"/>
+      <c r="T33" s="27" t="n"/>
+      <c r="U33" s="24" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="22" t="n"/>
-      <c r="B34" s="22" t="n"/>
-      <c r="C34" s="22" t="n"/>
-      <c r="D34" s="22" t="n"/>
-      <c r="E34" s="22" t="n"/>
-      <c r="F34" s="23" t="n"/>
-      <c r="G34" s="23" t="n"/>
-      <c r="H34" s="22" t="n"/>
-      <c r="I34" s="24" t="n"/>
-      <c r="J34" s="23" t="n"/>
-      <c r="K34" s="23" t="n"/>
-      <c r="L34" s="22" t="n"/>
-      <c r="M34" s="22" t="n"/>
-      <c r="N34" s="22" t="n"/>
-      <c r="O34" s="22" t="n"/>
-      <c r="P34" s="22" t="n"/>
-      <c r="Q34" s="22" t="n"/>
-      <c r="R34" s="22" t="n"/>
-      <c r="S34" s="22" t="n"/>
-      <c r="T34" s="22" t="n"/>
-      <c r="U34" s="22" t="n"/>
+      <c r="A34" s="24" t="n"/>
+      <c r="B34" s="24" t="n"/>
+      <c r="C34" s="24" t="n"/>
+      <c r="D34" s="24" t="n"/>
+      <c r="E34" s="24" t="n"/>
+      <c r="F34" s="25" t="n"/>
+      <c r="G34" s="25" t="n"/>
+      <c r="H34" s="24" t="n"/>
+      <c r="I34" s="26" t="n"/>
+      <c r="J34" s="25" t="n"/>
+      <c r="K34" s="25" t="n"/>
+      <c r="L34" s="24" t="n"/>
+      <c r="M34" s="24" t="n"/>
+      <c r="N34" s="24" t="n"/>
+      <c r="O34" s="27" t="n"/>
+      <c r="P34" s="27" t="n"/>
+      <c r="Q34" s="24" t="n"/>
+      <c r="R34" s="24" t="n"/>
+      <c r="S34" s="24" t="n"/>
+      <c r="T34" s="27" t="n"/>
+      <c r="U34" s="24" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="n"/>
-      <c r="B35" s="22" t="n"/>
-      <c r="C35" s="22" t="n"/>
-      <c r="D35" s="22" t="n"/>
-      <c r="E35" s="22" t="n"/>
-      <c r="F35" s="23" t="n"/>
-      <c r="G35" s="23" t="n"/>
-      <c r="H35" s="22" t="n"/>
-      <c r="I35" s="24" t="n"/>
-      <c r="J35" s="23" t="n"/>
-      <c r="K35" s="23" t="n"/>
-      <c r="L35" s="22" t="n"/>
-      <c r="M35" s="22" t="n"/>
-      <c r="N35" s="22" t="n"/>
-      <c r="O35" s="22" t="n"/>
-      <c r="P35" s="22" t="n"/>
-      <c r="Q35" s="22" t="n"/>
-      <c r="R35" s="22" t="n"/>
-      <c r="S35" s="22" t="n"/>
-      <c r="T35" s="22" t="n"/>
-      <c r="U35" s="22" t="n"/>
+      <c r="A35" s="24" t="n"/>
+      <c r="B35" s="24" t="n"/>
+      <c r="C35" s="24" t="n"/>
+      <c r="D35" s="24" t="n"/>
+      <c r="E35" s="24" t="n"/>
+      <c r="F35" s="25" t="n"/>
+      <c r="G35" s="25" t="n"/>
+      <c r="H35" s="24" t="n"/>
+      <c r="I35" s="26" t="n"/>
+      <c r="J35" s="25" t="n"/>
+      <c r="K35" s="25" t="n"/>
+      <c r="L35" s="24" t="n"/>
+      <c r="M35" s="24" t="n"/>
+      <c r="N35" s="24" t="n"/>
+      <c r="O35" s="27" t="n"/>
+      <c r="P35" s="27" t="n"/>
+      <c r="Q35" s="24" t="n"/>
+      <c r="R35" s="24" t="n"/>
+      <c r="S35" s="24" t="n"/>
+      <c r="T35" s="27" t="n"/>
+      <c r="U35" s="24" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="22" t="n"/>
-      <c r="B36" s="22" t="n"/>
-      <c r="C36" s="22" t="n"/>
-      <c r="D36" s="22" t="n"/>
-      <c r="E36" s="22" t="n"/>
-      <c r="F36" s="23" t="n"/>
-      <c r="G36" s="23" t="n"/>
-      <c r="H36" s="22" t="n"/>
-      <c r="I36" s="24" t="n"/>
-      <c r="J36" s="23" t="n"/>
-      <c r="K36" s="23" t="n"/>
-      <c r="L36" s="22" t="n"/>
-      <c r="M36" s="22" t="n"/>
-      <c r="N36" s="22" t="n"/>
-      <c r="O36" s="22" t="n"/>
-      <c r="P36" s="22" t="n"/>
-      <c r="Q36" s="22" t="n"/>
-      <c r="R36" s="22" t="n"/>
-      <c r="S36" s="22" t="n"/>
-      <c r="T36" s="22" t="n"/>
-      <c r="U36" s="22" t="n"/>
+      <c r="A36" s="24" t="n"/>
+      <c r="B36" s="24" t="n"/>
+      <c r="C36" s="24" t="n"/>
+      <c r="D36" s="24" t="n"/>
+      <c r="E36" s="24" t="n"/>
+      <c r="F36" s="25" t="n"/>
+      <c r="G36" s="25" t="n"/>
+      <c r="H36" s="24" t="n"/>
+      <c r="I36" s="26" t="n"/>
+      <c r="J36" s="25" t="n"/>
+      <c r="K36" s="25" t="n"/>
+      <c r="L36" s="24" t="n"/>
+      <c r="M36" s="24" t="n"/>
+      <c r="N36" s="24" t="n"/>
+      <c r="O36" s="27" t="n"/>
+      <c r="P36" s="27" t="n"/>
+      <c r="Q36" s="24" t="n"/>
+      <c r="R36" s="24" t="n"/>
+      <c r="S36" s="24" t="n"/>
+      <c r="T36" s="27" t="n"/>
+      <c r="U36" s="24" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="22" t="n"/>
-      <c r="B37" s="22" t="n"/>
-      <c r="C37" s="22" t="n"/>
-      <c r="D37" s="22" t="n"/>
-      <c r="E37" s="22" t="n"/>
-      <c r="F37" s="23" t="n"/>
-      <c r="G37" s="23" t="n"/>
-      <c r="H37" s="22" t="n"/>
-      <c r="I37" s="24" t="n"/>
-      <c r="J37" s="23" t="n"/>
-      <c r="K37" s="23" t="n"/>
-      <c r="L37" s="22" t="n"/>
-      <c r="M37" s="22" t="n"/>
-      <c r="N37" s="22" t="n"/>
-      <c r="O37" s="22" t="n"/>
-      <c r="P37" s="22" t="n"/>
-      <c r="Q37" s="22" t="n"/>
-      <c r="R37" s="22" t="n"/>
-      <c r="S37" s="22" t="n"/>
-      <c r="T37" s="22" t="n"/>
-      <c r="U37" s="22" t="n"/>
+      <c r="A37" s="24" t="n"/>
+      <c r="B37" s="24" t="n"/>
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="24" t="n"/>
+      <c r="E37" s="24" t="n"/>
+      <c r="F37" s="25" t="n"/>
+      <c r="G37" s="25" t="n"/>
+      <c r="H37" s="24" t="n"/>
+      <c r="I37" s="26" t="n"/>
+      <c r="J37" s="25" t="n"/>
+      <c r="K37" s="25" t="n"/>
+      <c r="L37" s="24" t="n"/>
+      <c r="M37" s="24" t="n"/>
+      <c r="N37" s="24" t="n"/>
+      <c r="O37" s="27" t="n"/>
+      <c r="P37" s="27" t="n"/>
+      <c r="Q37" s="24" t="n"/>
+      <c r="R37" s="24" t="n"/>
+      <c r="S37" s="24" t="n"/>
+      <c r="T37" s="27" t="n"/>
+      <c r="U37" s="24" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="22" t="n"/>
-      <c r="B38" s="22" t="n"/>
-      <c r="C38" s="22" t="n"/>
-      <c r="D38" s="22" t="n"/>
-      <c r="E38" s="22" t="n"/>
-      <c r="F38" s="23" t="n"/>
-      <c r="G38" s="23" t="n"/>
-      <c r="H38" s="22" t="n"/>
-      <c r="I38" s="24" t="n"/>
-      <c r="J38" s="23" t="n"/>
-      <c r="K38" s="23" t="n"/>
-      <c r="L38" s="22" t="n"/>
-      <c r="M38" s="22" t="n"/>
-      <c r="N38" s="22" t="n"/>
-      <c r="O38" s="22" t="n"/>
-      <c r="P38" s="22" t="n"/>
-      <c r="Q38" s="22" t="n"/>
-      <c r="R38" s="22" t="n"/>
-      <c r="S38" s="22" t="n"/>
-      <c r="T38" s="22" t="n"/>
-      <c r="U38" s="22" t="n"/>
+      <c r="A38" s="24" t="n"/>
+      <c r="B38" s="24" t="n"/>
+      <c r="C38" s="24" t="n"/>
+      <c r="D38" s="24" t="n"/>
+      <c r="E38" s="24" t="n"/>
+      <c r="F38" s="25" t="n"/>
+      <c r="G38" s="25" t="n"/>
+      <c r="H38" s="24" t="n"/>
+      <c r="I38" s="26" t="n"/>
+      <c r="J38" s="25" t="n"/>
+      <c r="K38" s="25" t="n"/>
+      <c r="L38" s="24" t="n"/>
+      <c r="M38" s="24" t="n"/>
+      <c r="N38" s="24" t="n"/>
+      <c r="O38" s="27" t="n"/>
+      <c r="P38" s="27" t="n"/>
+      <c r="Q38" s="24" t="n"/>
+      <c r="R38" s="24" t="n"/>
+      <c r="S38" s="24" t="n"/>
+      <c r="T38" s="27" t="n"/>
+      <c r="U38" s="24" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="22" t="n"/>
-      <c r="B39" s="22" t="n"/>
-      <c r="C39" s="22" t="n"/>
-      <c r="D39" s="22" t="n"/>
-      <c r="E39" s="22" t="n"/>
-      <c r="F39" s="23" t="n"/>
-      <c r="G39" s="23" t="n"/>
-      <c r="H39" s="22" t="n"/>
-      <c r="I39" s="24" t="n"/>
-      <c r="J39" s="23" t="n"/>
-      <c r="K39" s="23" t="n"/>
-      <c r="L39" s="22" t="n"/>
-      <c r="M39" s="22" t="n"/>
-      <c r="N39" s="22" t="n"/>
-      <c r="O39" s="22" t="n"/>
-      <c r="P39" s="22" t="n"/>
-      <c r="Q39" s="22" t="n"/>
-      <c r="R39" s="22" t="n"/>
-      <c r="S39" s="22" t="n"/>
-      <c r="T39" s="22" t="n"/>
-      <c r="U39" s="22" t="n"/>
+      <c r="A39" s="24" t="n"/>
+      <c r="B39" s="24" t="n"/>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="25" t="n"/>
+      <c r="G39" s="25" t="n"/>
+      <c r="H39" s="24" t="n"/>
+      <c r="I39" s="26" t="n"/>
+      <c r="J39" s="25" t="n"/>
+      <c r="K39" s="25" t="n"/>
+      <c r="L39" s="24" t="n"/>
+      <c r="M39" s="24" t="n"/>
+      <c r="N39" s="24" t="n"/>
+      <c r="O39" s="27" t="n"/>
+      <c r="P39" s="27" t="n"/>
+      <c r="Q39" s="24" t="n"/>
+      <c r="R39" s="24" t="n"/>
+      <c r="S39" s="24" t="n"/>
+      <c r="T39" s="27" t="n"/>
+      <c r="U39" s="24" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="22" t="n"/>
-      <c r="B40" s="22" t="n"/>
-      <c r="C40" s="22" t="n"/>
-      <c r="D40" s="22" t="n"/>
-      <c r="E40" s="22" t="n"/>
-      <c r="F40" s="23" t="n"/>
-      <c r="G40" s="23" t="n"/>
-      <c r="H40" s="22" t="n"/>
-      <c r="I40" s="24" t="n"/>
-      <c r="J40" s="23" t="n"/>
-      <c r="K40" s="23" t="n"/>
-      <c r="L40" s="22" t="n"/>
-      <c r="M40" s="22" t="n"/>
-      <c r="N40" s="22" t="n"/>
-      <c r="O40" s="22" t="n"/>
-      <c r="P40" s="22" t="n"/>
-      <c r="Q40" s="22" t="n"/>
-      <c r="R40" s="22" t="n"/>
-      <c r="S40" s="22" t="n"/>
-      <c r="T40" s="22" t="n"/>
-      <c r="U40" s="22" t="n"/>
+      <c r="A40" s="24" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="25" t="n"/>
+      <c r="G40" s="25" t="n"/>
+      <c r="H40" s="24" t="n"/>
+      <c r="I40" s="26" t="n"/>
+      <c r="J40" s="25" t="n"/>
+      <c r="K40" s="25" t="n"/>
+      <c r="L40" s="24" t="n"/>
+      <c r="M40" s="24" t="n"/>
+      <c r="N40" s="24" t="n"/>
+      <c r="O40" s="27" t="n"/>
+      <c r="P40" s="27" t="n"/>
+      <c r="Q40" s="24" t="n"/>
+      <c r="R40" s="24" t="n"/>
+      <c r="S40" s="24" t="n"/>
+      <c r="T40" s="27" t="n"/>
+      <c r="U40" s="24" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="22" t="n"/>
-      <c r="B41" s="22" t="n"/>
-      <c r="C41" s="22" t="n"/>
-      <c r="D41" s="22" t="n"/>
-      <c r="E41" s="22" t="n"/>
-      <c r="F41" s="23" t="n"/>
-      <c r="G41" s="23" t="n"/>
-      <c r="H41" s="22" t="n"/>
-      <c r="I41" s="24" t="n"/>
-      <c r="J41" s="23" t="n"/>
-      <c r="K41" s="23" t="n"/>
-      <c r="L41" s="22" t="n"/>
-      <c r="M41" s="22" t="n"/>
-      <c r="N41" s="22" t="n"/>
-      <c r="O41" s="22" t="n"/>
-      <c r="P41" s="22" t="n"/>
-      <c r="Q41" s="22" t="n"/>
-      <c r="R41" s="22" t="n"/>
-      <c r="S41" s="22" t="n"/>
-      <c r="T41" s="22" t="n"/>
-      <c r="U41" s="22" t="n"/>
+      <c r="A41" s="24" t="n"/>
+      <c r="B41" s="24" t="n"/>
+      <c r="C41" s="24" t="n"/>
+      <c r="D41" s="24" t="n"/>
+      <c r="E41" s="24" t="n"/>
+      <c r="F41" s="25" t="n"/>
+      <c r="G41" s="25" t="n"/>
+      <c r="H41" s="24" t="n"/>
+      <c r="I41" s="26" t="n"/>
+      <c r="J41" s="25" t="n"/>
+      <c r="K41" s="25" t="n"/>
+      <c r="L41" s="24" t="n"/>
+      <c r="M41" s="24" t="n"/>
+      <c r="N41" s="24" t="n"/>
+      <c r="O41" s="27" t="n"/>
+      <c r="P41" s="27" t="n"/>
+      <c r="Q41" s="24" t="n"/>
+      <c r="R41" s="24" t="n"/>
+      <c r="S41" s="24" t="n"/>
+      <c r="T41" s="27" t="n"/>
+      <c r="U41" s="24" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="n"/>
-      <c r="B42" s="22" t="n"/>
-      <c r="C42" s="22" t="n"/>
-      <c r="D42" s="22" t="n"/>
-      <c r="E42" s="22" t="n"/>
-      <c r="F42" s="23" t="n"/>
-      <c r="G42" s="23" t="n"/>
-      <c r="H42" s="22" t="n"/>
-      <c r="I42" s="24" t="n"/>
-      <c r="J42" s="23" t="n"/>
-      <c r="K42" s="23" t="n"/>
-      <c r="L42" s="22" t="n"/>
-      <c r="M42" s="22" t="n"/>
-      <c r="N42" s="22" t="n"/>
-      <c r="O42" s="22" t="n"/>
-      <c r="P42" s="22" t="n"/>
-      <c r="Q42" s="22" t="n"/>
-      <c r="R42" s="22" t="n"/>
-      <c r="S42" s="22" t="n"/>
-      <c r="T42" s="22" t="n"/>
-      <c r="U42" s="22" t="n"/>
+      <c r="A42" s="24" t="n"/>
+      <c r="B42" s="24" t="n"/>
+      <c r="C42" s="24" t="n"/>
+      <c r="D42" s="24" t="n"/>
+      <c r="E42" s="24" t="n"/>
+      <c r="F42" s="25" t="n"/>
+      <c r="G42" s="25" t="n"/>
+      <c r="H42" s="24" t="n"/>
+      <c r="I42" s="26" t="n"/>
+      <c r="J42" s="25" t="n"/>
+      <c r="K42" s="25" t="n"/>
+      <c r="L42" s="24" t="n"/>
+      <c r="M42" s="24" t="n"/>
+      <c r="N42" s="24" t="n"/>
+      <c r="O42" s="27" t="n"/>
+      <c r="P42" s="27" t="n"/>
+      <c r="Q42" s="24" t="n"/>
+      <c r="R42" s="24" t="n"/>
+      <c r="S42" s="24" t="n"/>
+      <c r="T42" s="27" t="n"/>
+      <c r="U42" s="24" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="22" t="n"/>
-      <c r="B43" s="22" t="n"/>
-      <c r="C43" s="22" t="n"/>
-      <c r="D43" s="22" t="n"/>
-      <c r="E43" s="22" t="n"/>
-      <c r="F43" s="23" t="n"/>
-      <c r="G43" s="23" t="n"/>
-      <c r="H43" s="22" t="n"/>
-      <c r="I43" s="24" t="n"/>
-      <c r="J43" s="23" t="n"/>
-      <c r="K43" s="23" t="n"/>
-      <c r="L43" s="22" t="n"/>
-      <c r="M43" s="22" t="n"/>
-      <c r="N43" s="22" t="n"/>
-      <c r="O43" s="22" t="n"/>
-      <c r="P43" s="22" t="n"/>
-      <c r="Q43" s="22" t="n"/>
-      <c r="R43" s="22" t="n"/>
-      <c r="S43" s="22" t="n"/>
-      <c r="T43" s="22" t="n"/>
-      <c r="U43" s="22" t="n"/>
+      <c r="A43" s="24" t="n"/>
+      <c r="B43" s="24" t="n"/>
+      <c r="C43" s="24" t="n"/>
+      <c r="D43" s="24" t="n"/>
+      <c r="E43" s="24" t="n"/>
+      <c r="F43" s="25" t="n"/>
+      <c r="G43" s="25" t="n"/>
+      <c r="H43" s="24" t="n"/>
+      <c r="I43" s="26" t="n"/>
+      <c r="J43" s="25" t="n"/>
+      <c r="K43" s="25" t="n"/>
+      <c r="L43" s="24" t="n"/>
+      <c r="M43" s="24" t="n"/>
+      <c r="N43" s="24" t="n"/>
+      <c r="O43" s="27" t="n"/>
+      <c r="P43" s="27" t="n"/>
+      <c r="Q43" s="24" t="n"/>
+      <c r="R43" s="24" t="n"/>
+      <c r="S43" s="24" t="n"/>
+      <c r="T43" s="27" t="n"/>
+      <c r="U43" s="24" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="22" t="n"/>
-      <c r="B44" s="22" t="n"/>
-      <c r="C44" s="22" t="n"/>
-      <c r="D44" s="22" t="n"/>
-      <c r="E44" s="22" t="n"/>
-      <c r="F44" s="23" t="n"/>
-      <c r="G44" s="23" t="n"/>
-      <c r="H44" s="22" t="n"/>
-      <c r="I44" s="24" t="n"/>
-      <c r="J44" s="23" t="n"/>
-      <c r="K44" s="23" t="n"/>
-      <c r="L44" s="22" t="n"/>
-      <c r="M44" s="22" t="n"/>
-      <c r="N44" s="22" t="n"/>
-      <c r="O44" s="22" t="n"/>
-      <c r="P44" s="22" t="n"/>
-      <c r="Q44" s="22" t="n"/>
-      <c r="R44" s="22" t="n"/>
-      <c r="S44" s="22" t="n"/>
-      <c r="T44" s="22" t="n"/>
-      <c r="U44" s="22" t="n"/>
+      <c r="A44" s="24" t="n"/>
+      <c r="B44" s="24" t="n"/>
+      <c r="C44" s="24" t="n"/>
+      <c r="D44" s="24" t="n"/>
+      <c r="E44" s="24" t="n"/>
+      <c r="F44" s="25" t="n"/>
+      <c r="G44" s="25" t="n"/>
+      <c r="H44" s="24" t="n"/>
+      <c r="I44" s="26" t="n"/>
+      <c r="J44" s="25" t="n"/>
+      <c r="K44" s="25" t="n"/>
+      <c r="L44" s="24" t="n"/>
+      <c r="M44" s="24" t="n"/>
+      <c r="N44" s="24" t="n"/>
+      <c r="O44" s="27" t="n"/>
+      <c r="P44" s="27" t="n"/>
+      <c r="Q44" s="24" t="n"/>
+      <c r="R44" s="24" t="n"/>
+      <c r="S44" s="24" t="n"/>
+      <c r="T44" s="27" t="n"/>
+      <c r="U44" s="24" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="22" t="n"/>
-      <c r="B45" s="22" t="n"/>
-      <c r="C45" s="22" t="n"/>
-      <c r="D45" s="22" t="n"/>
-      <c r="E45" s="22" t="n"/>
-      <c r="F45" s="23" t="n"/>
-      <c r="G45" s="23" t="n"/>
-      <c r="H45" s="22" t="n"/>
-      <c r="I45" s="24" t="n"/>
-      <c r="J45" s="23" t="n"/>
-      <c r="K45" s="23" t="n"/>
-      <c r="L45" s="22" t="n"/>
-      <c r="M45" s="22" t="n"/>
-      <c r="N45" s="22" t="n"/>
-      <c r="O45" s="22" t="n"/>
-      <c r="P45" s="22" t="n"/>
-      <c r="Q45" s="22" t="n"/>
-      <c r="R45" s="22" t="n"/>
-      <c r="S45" s="22" t="n"/>
-      <c r="T45" s="22" t="n"/>
-      <c r="U45" s="22" t="n"/>
+      <c r="A45" s="24" t="n"/>
+      <c r="B45" s="24" t="n"/>
+      <c r="C45" s="24" t="n"/>
+      <c r="D45" s="24" t="n"/>
+      <c r="E45" s="24" t="n"/>
+      <c r="F45" s="25" t="n"/>
+      <c r="G45" s="25" t="n"/>
+      <c r="H45" s="24" t="n"/>
+      <c r="I45" s="26" t="n"/>
+      <c r="J45" s="25" t="n"/>
+      <c r="K45" s="25" t="n"/>
+      <c r="L45" s="24" t="n"/>
+      <c r="M45" s="24" t="n"/>
+      <c r="N45" s="24" t="n"/>
+      <c r="O45" s="27" t="n"/>
+      <c r="P45" s="27" t="n"/>
+      <c r="Q45" s="24" t="n"/>
+      <c r="R45" s="24" t="n"/>
+      <c r="S45" s="24" t="n"/>
+      <c r="T45" s="27" t="n"/>
+      <c r="U45" s="24" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="22" t="n"/>
-      <c r="B46" s="22" t="n"/>
-      <c r="C46" s="22" t="n"/>
-      <c r="D46" s="22" t="n"/>
-      <c r="E46" s="22" t="n"/>
-      <c r="F46" s="23" t="n"/>
-      <c r="G46" s="23" t="n"/>
-      <c r="H46" s="22" t="n"/>
-      <c r="I46" s="24" t="n"/>
-      <c r="J46" s="23" t="n"/>
-      <c r="K46" s="23" t="n"/>
-      <c r="L46" s="22" t="n"/>
-      <c r="M46" s="22" t="n"/>
-      <c r="N46" s="22" t="n"/>
-      <c r="O46" s="22" t="n"/>
-      <c r="P46" s="22" t="n"/>
-      <c r="Q46" s="22" t="n"/>
-      <c r="R46" s="22" t="n"/>
-      <c r="S46" s="22" t="n"/>
-      <c r="T46" s="22" t="n"/>
-      <c r="U46" s="22" t="n"/>
+      <c r="A46" s="24" t="n"/>
+      <c r="B46" s="24" t="n"/>
+      <c r="C46" s="24" t="n"/>
+      <c r="D46" s="24" t="n"/>
+      <c r="E46" s="24" t="n"/>
+      <c r="F46" s="25" t="n"/>
+      <c r="G46" s="25" t="n"/>
+      <c r="H46" s="24" t="n"/>
+      <c r="I46" s="26" t="n"/>
+      <c r="J46" s="25" t="n"/>
+      <c r="K46" s="25" t="n"/>
+      <c r="L46" s="24" t="n"/>
+      <c r="M46" s="24" t="n"/>
+      <c r="N46" s="24" t="n"/>
+      <c r="O46" s="27" t="n"/>
+      <c r="P46" s="27" t="n"/>
+      <c r="Q46" s="24" t="n"/>
+      <c r="R46" s="24" t="n"/>
+      <c r="S46" s="24" t="n"/>
+      <c r="T46" s="27" t="n"/>
+      <c r="U46" s="24" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="22" t="n"/>
-      <c r="B47" s="22" t="n"/>
-      <c r="C47" s="22" t="n"/>
-      <c r="D47" s="22" t="n"/>
-      <c r="E47" s="22" t="n"/>
-      <c r="F47" s="23" t="n"/>
-      <c r="G47" s="23" t="n"/>
-      <c r="H47" s="22" t="n"/>
-      <c r="I47" s="24" t="n"/>
-      <c r="J47" s="23" t="n"/>
-      <c r="K47" s="23" t="n"/>
-      <c r="L47" s="22" t="n"/>
-      <c r="M47" s="22" t="n"/>
-      <c r="N47" s="22" t="n"/>
-      <c r="O47" s="22" t="n"/>
-      <c r="P47" s="22" t="n"/>
-      <c r="Q47" s="22" t="n"/>
-      <c r="R47" s="22" t="n"/>
-      <c r="S47" s="22" t="n"/>
-      <c r="T47" s="22" t="n"/>
-      <c r="U47" s="22" t="n"/>
+      <c r="A47" s="24" t="n"/>
+      <c r="B47" s="24" t="n"/>
+      <c r="C47" s="24" t="n"/>
+      <c r="D47" s="24" t="n"/>
+      <c r="E47" s="24" t="n"/>
+      <c r="F47" s="25" t="n"/>
+      <c r="G47" s="25" t="n"/>
+      <c r="H47" s="24" t="n"/>
+      <c r="I47" s="26" t="n"/>
+      <c r="J47" s="25" t="n"/>
+      <c r="K47" s="25" t="n"/>
+      <c r="L47" s="24" t="n"/>
+      <c r="M47" s="24" t="n"/>
+      <c r="N47" s="24" t="n"/>
+      <c r="O47" s="27" t="n"/>
+      <c r="P47" s="27" t="n"/>
+      <c r="Q47" s="24" t="n"/>
+      <c r="R47" s="24" t="n"/>
+      <c r="S47" s="24" t="n"/>
+      <c r="T47" s="27" t="n"/>
+      <c r="U47" s="24" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="n"/>
-      <c r="B48" s="22" t="n"/>
-      <c r="C48" s="22" t="n"/>
-      <c r="D48" s="22" t="n"/>
-      <c r="E48" s="22" t="n"/>
-      <c r="F48" s="23" t="n"/>
-      <c r="G48" s="23" t="n"/>
-      <c r="H48" s="22" t="n"/>
-      <c r="I48" s="24" t="n"/>
-      <c r="J48" s="23" t="n"/>
-      <c r="K48" s="23" t="n"/>
-      <c r="L48" s="22" t="n"/>
-      <c r="M48" s="22" t="n"/>
-      <c r="N48" s="22" t="n"/>
-      <c r="O48" s="22" t="n"/>
-      <c r="P48" s="22" t="n"/>
-      <c r="Q48" s="22" t="n"/>
-      <c r="R48" s="22" t="n"/>
-      <c r="S48" s="22" t="n"/>
-      <c r="T48" s="22" t="n"/>
-      <c r="U48" s="22" t="n"/>
+      <c r="A48" s="24" t="n"/>
+      <c r="B48" s="24" t="n"/>
+      <c r="C48" s="24" t="n"/>
+      <c r="D48" s="24" t="n"/>
+      <c r="E48" s="24" t="n"/>
+      <c r="F48" s="25" t="n"/>
+      <c r="G48" s="25" t="n"/>
+      <c r="H48" s="24" t="n"/>
+      <c r="I48" s="26" t="n"/>
+      <c r="J48" s="25" t="n"/>
+      <c r="K48" s="25" t="n"/>
+      <c r="L48" s="24" t="n"/>
+      <c r="M48" s="24" t="n"/>
+      <c r="N48" s="24" t="n"/>
+      <c r="O48" s="27" t="n"/>
+      <c r="P48" s="27" t="n"/>
+      <c r="Q48" s="24" t="n"/>
+      <c r="R48" s="24" t="n"/>
+      <c r="S48" s="24" t="n"/>
+      <c r="T48" s="27" t="n"/>
+      <c r="U48" s="24" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="22" t="n"/>
-      <c r="B49" s="22" t="n"/>
-      <c r="C49" s="22" t="n"/>
-      <c r="D49" s="22" t="n"/>
-      <c r="E49" s="22" t="n"/>
-      <c r="F49" s="23" t="n"/>
-      <c r="G49" s="23" t="n"/>
-      <c r="H49" s="22" t="n"/>
-      <c r="I49" s="24" t="n"/>
-      <c r="J49" s="23" t="n"/>
-      <c r="K49" s="23" t="n"/>
-      <c r="L49" s="22" t="n"/>
-      <c r="M49" s="22" t="n"/>
-      <c r="N49" s="22" t="n"/>
-      <c r="O49" s="22" t="n"/>
-      <c r="P49" s="22" t="n"/>
-      <c r="Q49" s="22" t="n"/>
-      <c r="R49" s="22" t="n"/>
-      <c r="S49" s="22" t="n"/>
-      <c r="T49" s="22" t="n"/>
-      <c r="U49" s="22" t="n"/>
+      <c r="A49" s="24" t="n"/>
+      <c r="B49" s="24" t="n"/>
+      <c r="C49" s="24" t="n"/>
+      <c r="D49" s="24" t="n"/>
+      <c r="E49" s="24" t="n"/>
+      <c r="F49" s="25" t="n"/>
+      <c r="G49" s="25" t="n"/>
+      <c r="H49" s="24" t="n"/>
+      <c r="I49" s="26" t="n"/>
+      <c r="J49" s="25" t="n"/>
+      <c r="K49" s="25" t="n"/>
+      <c r="L49" s="24" t="n"/>
+      <c r="M49" s="24" t="n"/>
+      <c r="N49" s="24" t="n"/>
+      <c r="O49" s="27" t="n"/>
+      <c r="P49" s="27" t="n"/>
+      <c r="Q49" s="24" t="n"/>
+      <c r="R49" s="24" t="n"/>
+      <c r="S49" s="24" t="n"/>
+      <c r="T49" s="27" t="n"/>
+      <c r="U49" s="24" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="22" t="n"/>
-      <c r="B50" s="22" t="n"/>
-      <c r="C50" s="22" t="n"/>
-      <c r="D50" s="22" t="n"/>
-      <c r="E50" s="22" t="n"/>
-      <c r="F50" s="23" t="n"/>
-      <c r="G50" s="23" t="n"/>
-      <c r="H50" s="22" t="n"/>
-      <c r="I50" s="24" t="n"/>
-      <c r="J50" s="23" t="n"/>
-      <c r="K50" s="23" t="n"/>
-      <c r="L50" s="22" t="n"/>
-      <c r="M50" s="22" t="n"/>
-      <c r="N50" s="22" t="n"/>
-      <c r="O50" s="22" t="n"/>
-      <c r="P50" s="22" t="n"/>
-      <c r="Q50" s="22" t="n"/>
-      <c r="R50" s="22" t="n"/>
-      <c r="S50" s="22" t="n"/>
-      <c r="T50" s="22" t="n"/>
-      <c r="U50" s="22" t="n"/>
+      <c r="A50" s="24" t="n"/>
+      <c r="B50" s="24" t="n"/>
+      <c r="C50" s="24" t="n"/>
+      <c r="D50" s="24" t="n"/>
+      <c r="E50" s="24" t="n"/>
+      <c r="F50" s="25" t="n"/>
+      <c r="G50" s="25" t="n"/>
+      <c r="H50" s="24" t="n"/>
+      <c r="I50" s="26" t="n"/>
+      <c r="J50" s="25" t="n"/>
+      <c r="K50" s="25" t="n"/>
+      <c r="L50" s="24" t="n"/>
+      <c r="M50" s="24" t="n"/>
+      <c r="N50" s="24" t="n"/>
+      <c r="O50" s="27" t="n"/>
+      <c r="P50" s="27" t="n"/>
+      <c r="Q50" s="24" t="n"/>
+      <c r="R50" s="24" t="n"/>
+      <c r="S50" s="24" t="n"/>
+      <c r="T50" s="27" t="n"/>
+      <c r="U50" s="24" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="22" t="n"/>
-      <c r="B51" s="22" t="n"/>
-      <c r="C51" s="22" t="n"/>
-      <c r="D51" s="22" t="n"/>
-      <c r="E51" s="22" t="n"/>
-      <c r="F51" s="23" t="n"/>
-      <c r="G51" s="23" t="n"/>
-      <c r="H51" s="22" t="n"/>
-      <c r="I51" s="24" t="n"/>
-      <c r="J51" s="23" t="n"/>
-      <c r="K51" s="23" t="n"/>
-      <c r="L51" s="22" t="n"/>
-      <c r="M51" s="22" t="n"/>
-      <c r="N51" s="22" t="n"/>
-      <c r="O51" s="22" t="n"/>
-      <c r="P51" s="22" t="n"/>
-      <c r="Q51" s="22" t="n"/>
-      <c r="R51" s="22" t="n"/>
-      <c r="S51" s="22" t="n"/>
-      <c r="T51" s="22" t="n"/>
-      <c r="U51" s="22" t="n"/>
+      <c r="A51" s="24" t="n"/>
+      <c r="B51" s="24" t="n"/>
+      <c r="C51" s="24" t="n"/>
+      <c r="D51" s="24" t="n"/>
+      <c r="E51" s="24" t="n"/>
+      <c r="F51" s="25" t="n"/>
+      <c r="G51" s="25" t="n"/>
+      <c r="H51" s="24" t="n"/>
+      <c r="I51" s="26" t="n"/>
+      <c r="J51" s="25" t="n"/>
+      <c r="K51" s="25" t="n"/>
+      <c r="L51" s="24" t="n"/>
+      <c r="M51" s="24" t="n"/>
+      <c r="N51" s="24" t="n"/>
+      <c r="O51" s="27" t="n"/>
+      <c r="P51" s="27" t="n"/>
+      <c r="Q51" s="24" t="n"/>
+      <c r="R51" s="24" t="n"/>
+      <c r="S51" s="24" t="n"/>
+      <c r="T51" s="27" t="n"/>
+      <c r="U51" s="24" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="22" t="n"/>
-      <c r="B52" s="22" t="n"/>
-      <c r="C52" s="22" t="n"/>
-      <c r="D52" s="22" t="n"/>
-      <c r="E52" s="22" t="n"/>
-      <c r="F52" s="23" t="n"/>
-      <c r="G52" s="23" t="n"/>
-      <c r="H52" s="22" t="n"/>
-      <c r="I52" s="24" t="n"/>
-      <c r="J52" s="23" t="n"/>
-      <c r="K52" s="23" t="n"/>
-      <c r="L52" s="22" t="n"/>
-      <c r="M52" s="22" t="n"/>
-      <c r="N52" s="22" t="n"/>
-      <c r="O52" s="22" t="n"/>
-      <c r="P52" s="22" t="n"/>
-      <c r="Q52" s="22" t="n"/>
-      <c r="R52" s="22" t="n"/>
-      <c r="S52" s="22" t="n"/>
-      <c r="T52" s="22" t="n"/>
-      <c r="U52" s="22" t="n"/>
+      <c r="A52" s="24" t="n"/>
+      <c r="B52" s="24" t="n"/>
+      <c r="C52" s="24" t="n"/>
+      <c r="D52" s="24" t="n"/>
+      <c r="E52" s="24" t="n"/>
+      <c r="F52" s="25" t="n"/>
+      <c r="G52" s="25" t="n"/>
+      <c r="H52" s="24" t="n"/>
+      <c r="I52" s="26" t="n"/>
+      <c r="J52" s="25" t="n"/>
+      <c r="K52" s="25" t="n"/>
+      <c r="L52" s="24" t="n"/>
+      <c r="M52" s="24" t="n"/>
+      <c r="N52" s="24" t="n"/>
+      <c r="O52" s="27" t="n"/>
+      <c r="P52" s="27" t="n"/>
+      <c r="Q52" s="24" t="n"/>
+      <c r="R52" s="24" t="n"/>
+      <c r="S52" s="24" t="n"/>
+      <c r="T52" s="27" t="n"/>
+      <c r="U52" s="24" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="24" t="n"/>
+      <c r="B53" s="24" t="n"/>
+      <c r="C53" s="24" t="n"/>
+      <c r="D53" s="24" t="n"/>
+      <c r="E53" s="24" t="n"/>
+      <c r="F53" s="25" t="n"/>
+      <c r="G53" s="25" t="n"/>
+      <c r="H53" s="24" t="n"/>
+      <c r="I53" s="26" t="n"/>
+      <c r="J53" s="25" t="n"/>
+      <c r="K53" s="25" t="n"/>
+      <c r="L53" s="24" t="n"/>
+      <c r="M53" s="24" t="n"/>
+      <c r="N53" s="24" t="n"/>
+      <c r="O53" s="27" t="n"/>
+      <c r="P53" s="27" t="n"/>
+      <c r="Q53" s="24" t="n"/>
+      <c r="R53" s="24" t="n"/>
+      <c r="S53" s="24" t="n"/>
+      <c r="T53" s="27" t="n"/>
+      <c r="U53" s="24" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="24" t="n"/>
+      <c r="B54" s="24" t="n"/>
+      <c r="C54" s="24" t="n"/>
+      <c r="D54" s="24" t="n"/>
+      <c r="E54" s="24" t="n"/>
+      <c r="F54" s="25" t="n"/>
+      <c r="G54" s="25" t="n"/>
+      <c r="H54" s="24" t="n"/>
+      <c r="I54" s="26" t="n"/>
+      <c r="J54" s="25" t="n"/>
+      <c r="K54" s="25" t="n"/>
+      <c r="L54" s="24" t="n"/>
+      <c r="M54" s="24" t="n"/>
+      <c r="N54" s="24" t="n"/>
+      <c r="O54" s="27" t="n"/>
+      <c r="P54" s="27" t="n"/>
+      <c r="Q54" s="24" t="n"/>
+      <c r="R54" s="24" t="n"/>
+      <c r="S54" s="24" t="n"/>
+      <c r="T54" s="27" t="n"/>
+      <c r="U54" s="24" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="24" t="n"/>
+      <c r="B55" s="24" t="n"/>
+      <c r="C55" s="24" t="n"/>
+      <c r="D55" s="24" t="n"/>
+      <c r="E55" s="24" t="n"/>
+      <c r="F55" s="25" t="n"/>
+      <c r="G55" s="25" t="n"/>
+      <c r="H55" s="24" t="n"/>
+      <c r="I55" s="26" t="n"/>
+      <c r="J55" s="25" t="n"/>
+      <c r="K55" s="25" t="n"/>
+      <c r="L55" s="24" t="n"/>
+      <c r="M55" s="24" t="n"/>
+      <c r="N55" s="24" t="n"/>
+      <c r="O55" s="27" t="n"/>
+      <c r="P55" s="27" t="n"/>
+      <c r="Q55" s="24" t="n"/>
+      <c r="R55" s="24" t="n"/>
+      <c r="S55" s="24" t="n"/>
+      <c r="T55" s="27" t="n"/>
+      <c r="U55" s="24" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="24" t="n"/>
+      <c r="B56" s="24" t="n"/>
+      <c r="C56" s="24" t="n"/>
+      <c r="D56" s="24" t="n"/>
+      <c r="E56" s="24" t="n"/>
+      <c r="F56" s="25" t="n"/>
+      <c r="G56" s="25" t="n"/>
+      <c r="H56" s="24" t="n"/>
+      <c r="I56" s="26" t="n"/>
+      <c r="J56" s="25" t="n"/>
+      <c r="K56" s="25" t="n"/>
+      <c r="L56" s="24" t="n"/>
+      <c r="M56" s="24" t="n"/>
+      <c r="N56" s="24" t="n"/>
+      <c r="O56" s="27" t="n"/>
+      <c r="P56" s="27" t="n"/>
+      <c r="Q56" s="24" t="n"/>
+      <c r="R56" s="24" t="n"/>
+      <c r="S56" s="24" t="n"/>
+      <c r="T56" s="27" t="n"/>
+      <c r="U56" s="24" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="24" t="n"/>
+      <c r="B57" s="24" t="n"/>
+      <c r="C57" s="24" t="n"/>
+      <c r="D57" s="24" t="n"/>
+      <c r="E57" s="24" t="n"/>
+      <c r="F57" s="25" t="n"/>
+      <c r="G57" s="25" t="n"/>
+      <c r="H57" s="24" t="n"/>
+      <c r="I57" s="26" t="n"/>
+      <c r="J57" s="25" t="n"/>
+      <c r="K57" s="25" t="n"/>
+      <c r="L57" s="24" t="n"/>
+      <c r="M57" s="24" t="n"/>
+      <c r="N57" s="24" t="n"/>
+      <c r="O57" s="27" t="n"/>
+      <c r="P57" s="27" t="n"/>
+      <c r="Q57" s="24" t="n"/>
+      <c r="R57" s="24" t="n"/>
+      <c r="S57" s="24" t="n"/>
+      <c r="T57" s="27" t="n"/>
+      <c r="U57" s="24" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="24" t="n"/>
+      <c r="B58" s="24" t="n"/>
+      <c r="C58" s="24" t="n"/>
+      <c r="D58" s="24" t="n"/>
+      <c r="E58" s="24" t="n"/>
+      <c r="F58" s="25" t="n"/>
+      <c r="G58" s="25" t="n"/>
+      <c r="H58" s="24" t="n"/>
+      <c r="I58" s="26" t="n"/>
+      <c r="J58" s="25" t="n"/>
+      <c r="K58" s="25" t="n"/>
+      <c r="L58" s="24" t="n"/>
+      <c r="M58" s="24" t="n"/>
+      <c r="N58" s="24" t="n"/>
+      <c r="O58" s="27" t="n"/>
+      <c r="P58" s="27" t="n"/>
+      <c r="Q58" s="24" t="n"/>
+      <c r="R58" s="24" t="n"/>
+      <c r="S58" s="24" t="n"/>
+      <c r="T58" s="27" t="n"/>
+      <c r="U58" s="24" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U1"/>
   <dataValidations count="6">
-    <dataValidation sqref="D3:D52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz kampanya turu" error="Listeden bir deger secin. Emin degilseniz 'Belirlenemedi' secin." type="list">
+    <dataValidation sqref="D3:D58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz kampanya turu" error="Listeden bir deger secin. Emin degilseniz 'Belirlenemedi' secin." type="list">
       <formula1>"Konut Finansmani Kampanyasi,Ihtiyac Finansmani Kampanyasi,Tasit Finansmani Kampanyasi,Finansman Kampanyasi,Kart Kampanyasi,Alisveris Puani Kampanyasi,Yeni Musteri Kampanyasi,Yatirim Urunu Kampanyasi,Belirlenemedi"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz oran periyodu" error="Sayfada ne yaziyorsa onu secin. Yazmiyorsa tahmin etmeyin: 'belirsiz'." type="list">
+    <dataValidation sqref="H3:H58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz oran periyodu" error="Sayfada ne yaziyorsa onu secin. Yazmiyorsa tahmin etmeyin: 'belirsiz'." type="list">
       <formula1>"aylik,yillik,belirsiz"</formula1>
     </dataValidation>
-    <dataValidation sqref="L3:L52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz odul birimi" error="Listeden bir birim secin." type="list">
+    <dataValidation sqref="L3:L58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz odul birimi" error="Listeden bir birim secin." type="list">
       <formula1>"TL,Mil,Gram,Puan,Worldpuan,ParafPara,Bankkart Lira"</formula1>
     </dataValidation>
-    <dataValidation sqref="F3:F52 G3:G52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz oran" error="Sadece 0-100 arasi sayi yazin, VIRGULLE (yuzde isareti olmadan). Ornek: 1,99" type="decimal" operator="between">
+    <dataValidation sqref="F3:F58 G3:G58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz oran" error="Sadece 0-100 arasi sayi yazin, VIRGULLE (yuzde isareti olmadan). Ornek: 1,99" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="I3:I52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz vade" error="Sadece tam sayi (ay) yazin, 0-480 arasi. Ornek: 120" type="whole" operator="between">
+    <dataValidation sqref="I3:I58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz vade" error="Sadece tam sayi (ay) yazin, 0-480 arasi. Ornek: 120" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>480</formula2>
     </dataValidation>
-    <dataValidation sqref="J3:J52 K3:K52" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz tutar" error="Sadece sayi yazin (TL isareti olmadan). Ornek: 500000" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J3:J58 K3:K58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz tutar" error="Sadece sayi yazin (TL isareti olmadan). Ornek: 500000" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -2939,14 +3424,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>KAPSAM DISI VERILER - Neden ayri sayfada?</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr"/>
+      <c r="A2" s="29" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -2956,21 +3441,21 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Ama tamamen atilmalari da gerekmez - ileride ise yarayabilirler. Bu yuzden Altin Veri Seti'ne</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>KARISTIRILMADAN burada tutulurlar.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr"/>
+      <c r="A6" s="29" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2994,37 +3479,37 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="26" t="inlineStr"/>
+      <c r="A10" s="29" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>Ikisi ters yonde kavramlardir. Karistirilirsa karsilastirma motoru 'en dusuk kar payi'</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>sorusuna anlamsiz cevap verir.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="inlineStr"/>
+      <c r="A13" s="29" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="26" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>Ayrica: mevduat oranlari genelde YILLIK, kampanya oranlari genelde AYLIK verilir.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="inlineStr"/>
+      <c r="A15" s="29" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="26" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Asagidaki satirlar Zeynep'in 28.07.2026'da topladigi verilerin dogru yere tasinmis halidir.</t>
         </is>
@@ -3078,482 +3563,482 @@
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Turkiye Finans</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B19" s="19" t="inlineStr">
         <is>
           <t>mevduat_orani</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C19" s="19" t="inlineStr">
         <is>
           <t>standart_tl_1ay</t>
         </is>
       </c>
-      <c r="D19" s="18" t="n">
+      <c r="D19" s="19" t="n">
         <v>28.08</v>
       </c>
-      <c r="E19" s="18" t="inlineStr">
+      <c r="E19" s="19" t="inlineStr">
         <is>
           <t>yuzde</t>
         </is>
       </c>
-      <c r="F19" s="18" t="inlineStr">
+      <c r="F19" s="19" t="inlineStr">
         <is>
           <t>yillik</t>
         </is>
       </c>
-      <c r="G19" s="19" t="inlineStr">
+      <c r="G19" s="20" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/bireysel/Sayfalar/Kar-Payi-Oranlari.aspx</t>
         </is>
       </c>
-      <c r="H19" s="18" t="inlineStr">
+      <c r="H19" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="I19" s="19" t="inlineStr">
+      <c r="I19" s="20" t="inlineStr">
         <is>
           <t>Katilma hesabi (mevduat) orani - finansman orani DEGIL</t>
         </is>
       </c>
     </row>
     <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Turkiye Finans</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>mevduat_orani</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>standart_tl_1yil</t>
         </is>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="19" t="n">
         <v>31.29</v>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr">
         <is>
           <t>yuzde</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F20" s="19" t="inlineStr">
         <is>
           <t>yillik</t>
         </is>
       </c>
-      <c r="G20" s="19" t="inlineStr">
+      <c r="G20" s="20" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/bireysel/Sayfalar/Kar-Payi-Oranlari.aspx</t>
         </is>
       </c>
-      <c r="H20" s="18" t="inlineStr">
+      <c r="H20" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="I20" s="19" t="inlineStr">
+      <c r="I20" s="20" t="inlineStr">
         <is>
           <t>Katilma hesabi (mevduat) orani - finansman orani DEGIL</t>
         </is>
       </c>
     </row>
     <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Turkiye Finans</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>ucret_tarifesi</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C21" s="19" t="inlineStr">
         <is>
           <t>eft_sube_azami_ucret</t>
         </is>
       </c>
-      <c r="D21" s="18" t="n">
+      <c r="D21" s="19" t="n">
         <v>797.6799999999999</v>
       </c>
-      <c r="E21" s="18" t="inlineStr">
+      <c r="E21" s="19" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
-      <c r="F21" s="18" t="n"/>
-      <c r="G21" s="19" t="inlineStr">
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="20" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/bireysel/Sayfalar/urun-hizmet-ucretleri.aspx</t>
         </is>
       </c>
-      <c r="H21" s="18" t="inlineStr">
+      <c r="H21" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="I21" s="19" t="inlineStr">
+      <c r="I21" s="20" t="inlineStr">
         <is>
           <t>Ucret tarifesi - kampanya alani degil</t>
         </is>
       </c>
     </row>
     <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>Turkiye Finans</t>
         </is>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>urun_adi</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C22" s="19" t="inlineStr">
         <is>
           <t>kart_adi</t>
         </is>
       </c>
-      <c r="D22" s="18" t="inlineStr">
+      <c r="D22" s="19" t="inlineStr">
         <is>
           <t>Happy Kart</t>
         </is>
       </c>
-      <c r="E22" s="18" t="inlineStr">
+      <c r="E22" s="19" t="inlineStr">
         <is>
           <t>metin</t>
         </is>
       </c>
-      <c r="F22" s="18" t="n"/>
-      <c r="G22" s="19" t="inlineStr">
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="20" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/bireysel/Sayfalar/kredi-kartlari.aspx</t>
         </is>
       </c>
-      <c r="H22" s="18" t="inlineStr">
+      <c r="H22" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="I22" s="19" t="inlineStr">
+      <c r="I22" s="20" t="inlineStr">
         <is>
           <t>Urun adi - kampanya verisi degil</t>
         </is>
       </c>
     </row>
     <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>Turkiye Finans</t>
         </is>
       </c>
-      <c r="B23" s="18" t="inlineStr">
+      <c r="B23" s="19" t="inlineStr">
         <is>
           <t>urun_adi</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="C23" s="19" t="inlineStr">
         <is>
           <t>hesap_turu</t>
         </is>
       </c>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>Katilma Hesabi</t>
         </is>
       </c>
-      <c r="E23" s="18" t="inlineStr">
+      <c r="E23" s="19" t="inlineStr">
         <is>
           <t>metin</t>
         </is>
       </c>
-      <c r="F23" s="18" t="n"/>
-      <c r="G23" s="19" t="inlineStr">
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="20" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/bireysel/katilma-hesaplari/Sayfalar/katilma-hesaplari.aspx</t>
         </is>
       </c>
-      <c r="H23" s="18" t="inlineStr">
+      <c r="H23" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="I23" s="19" t="inlineStr">
+      <c r="I23" s="20" t="inlineStr">
         <is>
           <t>Urun adi - kampanya verisi degil</t>
         </is>
       </c>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Turkiye Finans</t>
         </is>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>urun_bilgisi</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="19" t="inlineStr">
         <is>
           <t>azami_vade</t>
         </is>
       </c>
-      <c r="D24" s="18" t="n">
+      <c r="D24" s="19" t="n">
         <v>36</v>
       </c>
-      <c r="E24" s="18" t="inlineStr">
+      <c r="E24" s="19" t="inlineStr">
         <is>
           <t>ay</t>
         </is>
       </c>
-      <c r="F24" s="18" t="n"/>
-      <c r="G24" s="19" t="inlineStr">
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="20" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/bireysel/ihtiyac-finansmani/Sayfalar/ihtiyac-finansmani.aspx</t>
         </is>
       </c>
-      <c r="H24" s="18" t="inlineStr">
+      <c r="H24" s="19" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="I24" s="19" t="inlineStr">
+      <c r="I24" s="20" t="inlineStr">
         <is>
           <t>Genel urun tanitim sayfasi - kampanyaya ozel deger degil (rapor Bolum 3)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="n"/>
-      <c r="B25" s="22" t="n"/>
-      <c r="C25" s="22" t="n"/>
-      <c r="D25" s="22" t="n"/>
-      <c r="E25" s="22" t="n"/>
-      <c r="F25" s="22" t="n"/>
-      <c r="G25" s="22" t="n"/>
-      <c r="H25" s="22" t="n"/>
-      <c r="I25" s="22" t="n"/>
+      <c r="A25" s="24" t="n"/>
+      <c r="B25" s="24" t="n"/>
+      <c r="C25" s="24" t="n"/>
+      <c r="D25" s="24" t="n"/>
+      <c r="E25" s="24" t="n"/>
+      <c r="F25" s="24" t="n"/>
+      <c r="G25" s="24" t="n"/>
+      <c r="H25" s="24" t="n"/>
+      <c r="I25" s="24" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="22" t="n"/>
-      <c r="B26" s="22" t="n"/>
-      <c r="C26" s="22" t="n"/>
-      <c r="D26" s="22" t="n"/>
-      <c r="E26" s="22" t="n"/>
-      <c r="F26" s="22" t="n"/>
-      <c r="G26" s="22" t="n"/>
-      <c r="H26" s="22" t="n"/>
-      <c r="I26" s="22" t="n"/>
+      <c r="A26" s="24" t="n"/>
+      <c r="B26" s="24" t="n"/>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="24" t="n"/>
+      <c r="F26" s="24" t="n"/>
+      <c r="G26" s="24" t="n"/>
+      <c r="H26" s="24" t="n"/>
+      <c r="I26" s="24" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="n"/>
-      <c r="B27" s="22" t="n"/>
-      <c r="C27" s="22" t="n"/>
-      <c r="D27" s="22" t="n"/>
-      <c r="E27" s="22" t="n"/>
-      <c r="F27" s="22" t="n"/>
-      <c r="G27" s="22" t="n"/>
-      <c r="H27" s="22" t="n"/>
-      <c r="I27" s="22" t="n"/>
+      <c r="A27" s="24" t="n"/>
+      <c r="B27" s="24" t="n"/>
+      <c r="C27" s="24" t="n"/>
+      <c r="D27" s="24" t="n"/>
+      <c r="E27" s="24" t="n"/>
+      <c r="F27" s="24" t="n"/>
+      <c r="G27" s="24" t="n"/>
+      <c r="H27" s="24" t="n"/>
+      <c r="I27" s="24" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="n"/>
-      <c r="B28" s="22" t="n"/>
-      <c r="C28" s="22" t="n"/>
-      <c r="D28" s="22" t="n"/>
-      <c r="E28" s="22" t="n"/>
-      <c r="F28" s="22" t="n"/>
-      <c r="G28" s="22" t="n"/>
-      <c r="H28" s="22" t="n"/>
-      <c r="I28" s="22" t="n"/>
+      <c r="A28" s="24" t="n"/>
+      <c r="B28" s="24" t="n"/>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="24" t="n"/>
+      <c r="F28" s="24" t="n"/>
+      <c r="G28" s="24" t="n"/>
+      <c r="H28" s="24" t="n"/>
+      <c r="I28" s="24" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="22" t="n"/>
-      <c r="B29" s="22" t="n"/>
-      <c r="C29" s="22" t="n"/>
-      <c r="D29" s="22" t="n"/>
-      <c r="E29" s="22" t="n"/>
-      <c r="F29" s="22" t="n"/>
-      <c r="G29" s="22" t="n"/>
-      <c r="H29" s="22" t="n"/>
-      <c r="I29" s="22" t="n"/>
+      <c r="A29" s="24" t="n"/>
+      <c r="B29" s="24" t="n"/>
+      <c r="C29" s="24" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="24" t="n"/>
+      <c r="F29" s="24" t="n"/>
+      <c r="G29" s="24" t="n"/>
+      <c r="H29" s="24" t="n"/>
+      <c r="I29" s="24" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="n"/>
-      <c r="B30" s="22" t="n"/>
-      <c r="C30" s="22" t="n"/>
-      <c r="D30" s="22" t="n"/>
-      <c r="E30" s="22" t="n"/>
-      <c r="F30" s="22" t="n"/>
-      <c r="G30" s="22" t="n"/>
-      <c r="H30" s="22" t="n"/>
-      <c r="I30" s="22" t="n"/>
+      <c r="A30" s="24" t="n"/>
+      <c r="B30" s="24" t="n"/>
+      <c r="C30" s="24" t="n"/>
+      <c r="D30" s="24" t="n"/>
+      <c r="E30" s="24" t="n"/>
+      <c r="F30" s="24" t="n"/>
+      <c r="G30" s="24" t="n"/>
+      <c r="H30" s="24" t="n"/>
+      <c r="I30" s="24" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="22" t="n"/>
-      <c r="B31" s="22" t="n"/>
-      <c r="C31" s="22" t="n"/>
-      <c r="D31" s="22" t="n"/>
-      <c r="E31" s="22" t="n"/>
-      <c r="F31" s="22" t="n"/>
-      <c r="G31" s="22" t="n"/>
-      <c r="H31" s="22" t="n"/>
-      <c r="I31" s="22" t="n"/>
+      <c r="A31" s="24" t="n"/>
+      <c r="B31" s="24" t="n"/>
+      <c r="C31" s="24" t="n"/>
+      <c r="D31" s="24" t="n"/>
+      <c r="E31" s="24" t="n"/>
+      <c r="F31" s="24" t="n"/>
+      <c r="G31" s="24" t="n"/>
+      <c r="H31" s="24" t="n"/>
+      <c r="I31" s="24" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="22" t="n"/>
-      <c r="B32" s="22" t="n"/>
-      <c r="C32" s="22" t="n"/>
-      <c r="D32" s="22" t="n"/>
-      <c r="E32" s="22" t="n"/>
-      <c r="F32" s="22" t="n"/>
-      <c r="G32" s="22" t="n"/>
-      <c r="H32" s="22" t="n"/>
-      <c r="I32" s="22" t="n"/>
+      <c r="A32" s="24" t="n"/>
+      <c r="B32" s="24" t="n"/>
+      <c r="C32" s="24" t="n"/>
+      <c r="D32" s="24" t="n"/>
+      <c r="E32" s="24" t="n"/>
+      <c r="F32" s="24" t="n"/>
+      <c r="G32" s="24" t="n"/>
+      <c r="H32" s="24" t="n"/>
+      <c r="I32" s="24" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="22" t="n"/>
-      <c r="B33" s="22" t="n"/>
-      <c r="C33" s="22" t="n"/>
-      <c r="D33" s="22" t="n"/>
-      <c r="E33" s="22" t="n"/>
-      <c r="F33" s="22" t="n"/>
-      <c r="G33" s="22" t="n"/>
-      <c r="H33" s="22" t="n"/>
-      <c r="I33" s="22" t="n"/>
+      <c r="A33" s="24" t="n"/>
+      <c r="B33" s="24" t="n"/>
+      <c r="C33" s="24" t="n"/>
+      <c r="D33" s="24" t="n"/>
+      <c r="E33" s="24" t="n"/>
+      <c r="F33" s="24" t="n"/>
+      <c r="G33" s="24" t="n"/>
+      <c r="H33" s="24" t="n"/>
+      <c r="I33" s="24" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="22" t="n"/>
-      <c r="B34" s="22" t="n"/>
-      <c r="C34" s="22" t="n"/>
-      <c r="D34" s="22" t="n"/>
-      <c r="E34" s="22" t="n"/>
-      <c r="F34" s="22" t="n"/>
-      <c r="G34" s="22" t="n"/>
-      <c r="H34" s="22" t="n"/>
-      <c r="I34" s="22" t="n"/>
+      <c r="A34" s="24" t="n"/>
+      <c r="B34" s="24" t="n"/>
+      <c r="C34" s="24" t="n"/>
+      <c r="D34" s="24" t="n"/>
+      <c r="E34" s="24" t="n"/>
+      <c r="F34" s="24" t="n"/>
+      <c r="G34" s="24" t="n"/>
+      <c r="H34" s="24" t="n"/>
+      <c r="I34" s="24" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="n"/>
-      <c r="B35" s="22" t="n"/>
-      <c r="C35" s="22" t="n"/>
-      <c r="D35" s="22" t="n"/>
-      <c r="E35" s="22" t="n"/>
-      <c r="F35" s="22" t="n"/>
-      <c r="G35" s="22" t="n"/>
-      <c r="H35" s="22" t="n"/>
-      <c r="I35" s="22" t="n"/>
+      <c r="A35" s="24" t="n"/>
+      <c r="B35" s="24" t="n"/>
+      <c r="C35" s="24" t="n"/>
+      <c r="D35" s="24" t="n"/>
+      <c r="E35" s="24" t="n"/>
+      <c r="F35" s="24" t="n"/>
+      <c r="G35" s="24" t="n"/>
+      <c r="H35" s="24" t="n"/>
+      <c r="I35" s="24" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="22" t="n"/>
-      <c r="B36" s="22" t="n"/>
-      <c r="C36" s="22" t="n"/>
-      <c r="D36" s="22" t="n"/>
-      <c r="E36" s="22" t="n"/>
-      <c r="F36" s="22" t="n"/>
-      <c r="G36" s="22" t="n"/>
-      <c r="H36" s="22" t="n"/>
-      <c r="I36" s="22" t="n"/>
+      <c r="A36" s="24" t="n"/>
+      <c r="B36" s="24" t="n"/>
+      <c r="C36" s="24" t="n"/>
+      <c r="D36" s="24" t="n"/>
+      <c r="E36" s="24" t="n"/>
+      <c r="F36" s="24" t="n"/>
+      <c r="G36" s="24" t="n"/>
+      <c r="H36" s="24" t="n"/>
+      <c r="I36" s="24" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="22" t="n"/>
-      <c r="B37" s="22" t="n"/>
-      <c r="C37" s="22" t="n"/>
-      <c r="D37" s="22" t="n"/>
-      <c r="E37" s="22" t="n"/>
-      <c r="F37" s="22" t="n"/>
-      <c r="G37" s="22" t="n"/>
-      <c r="H37" s="22" t="n"/>
-      <c r="I37" s="22" t="n"/>
+      <c r="A37" s="24" t="n"/>
+      <c r="B37" s="24" t="n"/>
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="24" t="n"/>
+      <c r="E37" s="24" t="n"/>
+      <c r="F37" s="24" t="n"/>
+      <c r="G37" s="24" t="n"/>
+      <c r="H37" s="24" t="n"/>
+      <c r="I37" s="24" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="22" t="n"/>
-      <c r="B38" s="22" t="n"/>
-      <c r="C38" s="22" t="n"/>
-      <c r="D38" s="22" t="n"/>
-      <c r="E38" s="22" t="n"/>
-      <c r="F38" s="22" t="n"/>
-      <c r="G38" s="22" t="n"/>
-      <c r="H38" s="22" t="n"/>
-      <c r="I38" s="22" t="n"/>
+      <c r="A38" s="24" t="n"/>
+      <c r="B38" s="24" t="n"/>
+      <c r="C38" s="24" t="n"/>
+      <c r="D38" s="24" t="n"/>
+      <c r="E38" s="24" t="n"/>
+      <c r="F38" s="24" t="n"/>
+      <c r="G38" s="24" t="n"/>
+      <c r="H38" s="24" t="n"/>
+      <c r="I38" s="24" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="22" t="n"/>
-      <c r="B39" s="22" t="n"/>
-      <c r="C39" s="22" t="n"/>
-      <c r="D39" s="22" t="n"/>
-      <c r="E39" s="22" t="n"/>
-      <c r="F39" s="22" t="n"/>
-      <c r="G39" s="22" t="n"/>
-      <c r="H39" s="22" t="n"/>
-      <c r="I39" s="22" t="n"/>
+      <c r="A39" s="24" t="n"/>
+      <c r="B39" s="24" t="n"/>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="24" t="n"/>
+      <c r="F39" s="24" t="n"/>
+      <c r="G39" s="24" t="n"/>
+      <c r="H39" s="24" t="n"/>
+      <c r="I39" s="24" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="22" t="n"/>
-      <c r="B40" s="22" t="n"/>
-      <c r="C40" s="22" t="n"/>
-      <c r="D40" s="22" t="n"/>
-      <c r="E40" s="22" t="n"/>
-      <c r="F40" s="22" t="n"/>
-      <c r="G40" s="22" t="n"/>
-      <c r="H40" s="22" t="n"/>
-      <c r="I40" s="22" t="n"/>
+      <c r="A40" s="24" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="24" t="n"/>
+      <c r="F40" s="24" t="n"/>
+      <c r="G40" s="24" t="n"/>
+      <c r="H40" s="24" t="n"/>
+      <c r="I40" s="24" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="22" t="n"/>
-      <c r="B41" s="22" t="n"/>
-      <c r="C41" s="22" t="n"/>
-      <c r="D41" s="22" t="n"/>
-      <c r="E41" s="22" t="n"/>
-      <c r="F41" s="22" t="n"/>
-      <c r="G41" s="22" t="n"/>
-      <c r="H41" s="22" t="n"/>
-      <c r="I41" s="22" t="n"/>
+      <c r="A41" s="24" t="n"/>
+      <c r="B41" s="24" t="n"/>
+      <c r="C41" s="24" t="n"/>
+      <c r="D41" s="24" t="n"/>
+      <c r="E41" s="24" t="n"/>
+      <c r="F41" s="24" t="n"/>
+      <c r="G41" s="24" t="n"/>
+      <c r="H41" s="24" t="n"/>
+      <c r="I41" s="24" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="n"/>
-      <c r="B42" s="22" t="n"/>
-      <c r="C42" s="22" t="n"/>
-      <c r="D42" s="22" t="n"/>
-      <c r="E42" s="22" t="n"/>
-      <c r="F42" s="22" t="n"/>
-      <c r="G42" s="22" t="n"/>
-      <c r="H42" s="22" t="n"/>
-      <c r="I42" s="22" t="n"/>
+      <c r="A42" s="24" t="n"/>
+      <c r="B42" s="24" t="n"/>
+      <c r="C42" s="24" t="n"/>
+      <c r="D42" s="24" t="n"/>
+      <c r="E42" s="24" t="n"/>
+      <c r="F42" s="24" t="n"/>
+      <c r="G42" s="24" t="n"/>
+      <c r="H42" s="24" t="n"/>
+      <c r="I42" s="24" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="22" t="n"/>
-      <c r="B43" s="22" t="n"/>
-      <c r="C43" s="22" t="n"/>
-      <c r="D43" s="22" t="n"/>
-      <c r="E43" s="22" t="n"/>
-      <c r="F43" s="22" t="n"/>
-      <c r="G43" s="22" t="n"/>
-      <c r="H43" s="22" t="n"/>
-      <c r="I43" s="22" t="n"/>
+      <c r="A43" s="24" t="n"/>
+      <c r="B43" s="24" t="n"/>
+      <c r="C43" s="24" t="n"/>
+      <c r="D43" s="24" t="n"/>
+      <c r="E43" s="24" t="n"/>
+      <c r="F43" s="24" t="n"/>
+      <c r="G43" s="24" t="n"/>
+      <c r="H43" s="24" t="n"/>
+      <c r="I43" s="24" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="22" t="n"/>
-      <c r="B44" s="22" t="n"/>
-      <c r="C44" s="22" t="n"/>
-      <c r="D44" s="22" t="n"/>
-      <c r="E44" s="22" t="n"/>
-      <c r="F44" s="22" t="n"/>
-      <c r="G44" s="22" t="n"/>
-      <c r="H44" s="22" t="n"/>
-      <c r="I44" s="22" t="n"/>
+      <c r="A44" s="24" t="n"/>
+      <c r="B44" s="24" t="n"/>
+      <c r="C44" s="24" t="n"/>
+      <c r="D44" s="24" t="n"/>
+      <c r="E44" s="24" t="n"/>
+      <c r="F44" s="24" t="n"/>
+      <c r="G44" s="24" t="n"/>
+      <c r="H44" s="24" t="n"/>
+      <c r="I44" s="24" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3610,196 +4095,196 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>Kuveyt Turk</t>
         </is>
       </c>
-      <c r="B2" s="27" t="n">
+      <c r="B2" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C2" s="27" t="n"/>
-      <c r="D2" s="27" t="n"/>
-      <c r="E2" s="27" t="n"/>
-      <c r="F2" s="28" t="inlineStr">
+      <c r="C2" s="30" t="n"/>
+      <c r="D2" s="30" t="n"/>
+      <c r="E2" s="30" t="n"/>
+      <c r="F2" s="31" t="inlineStr">
         <is>
           <t>Sprint 1 - once bu</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>Albaraka Turk</t>
         </is>
       </c>
-      <c r="B3" s="27" t="n">
+      <c r="B3" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C3" s="27" t="n"/>
-      <c r="D3" s="27" t="n"/>
-      <c r="E3" s="27" t="n"/>
-      <c r="F3" s="28" t="inlineStr">
+      <c r="C3" s="30" t="n"/>
+      <c r="D3" s="30" t="n"/>
+      <c r="E3" s="30" t="n"/>
+      <c r="F3" s="31" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Vakif Katilim</t>
         </is>
       </c>
-      <c r="B4" s="27" t="n">
+      <c r="B4" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C4" s="27" t="n"/>
-      <c r="D4" s="27" t="n"/>
-      <c r="E4" s="27" t="n"/>
-      <c r="F4" s="28" t="inlineStr">
+      <c r="C4" s="30" t="n"/>
+      <c r="D4" s="30" t="n"/>
+      <c r="E4" s="30" t="n"/>
+      <c r="F4" s="31" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Turkiye Finans</t>
         </is>
       </c>
-      <c r="B5" s="27" t="n">
+      <c r="B5" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="27" t="n"/>
-      <c r="D5" s="27" t="n"/>
-      <c r="E5" s="27" t="n"/>
-      <c r="F5" s="28" t="inlineStr">
+      <c r="C5" s="30" t="n"/>
+      <c r="D5" s="30" t="n"/>
+      <c r="E5" s="30" t="n"/>
+      <c r="F5" s="31" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Ziraat Katilim</t>
         </is>
       </c>
-      <c r="B6" s="27" t="n">
+      <c r="B6" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="27" t="n"/>
-      <c r="D6" s="27" t="n"/>
-      <c r="E6" s="27" t="n"/>
-      <c r="F6" s="28" t="inlineStr">
+      <c r="C6" s="30" t="n"/>
+      <c r="D6" s="30" t="n"/>
+      <c r="E6" s="30" t="n"/>
+      <c r="F6" s="31" t="inlineStr">
         <is>
           <t>Sprint 2 - buyuk hacim (~70 kampanya)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Turkiye Emlak Katilim</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n">
+      <c r="B7" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="27" t="n"/>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="27" t="n"/>
-      <c r="F7" s="28" t="inlineStr">
+      <c r="C7" s="30" t="n"/>
+      <c r="D7" s="30" t="n"/>
+      <c r="E7" s="30" t="n"/>
+      <c r="F7" s="31" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Dunya Katilim</t>
         </is>
       </c>
-      <c r="B8" s="27" t="n">
+      <c r="B8" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C8" s="27" t="n"/>
-      <c r="D8" s="27" t="n"/>
-      <c r="E8" s="27" t="n"/>
-      <c r="F8" s="28" t="inlineStr">
+      <c r="C8" s="30" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="30" t="n"/>
+      <c r="F8" s="31" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Adil Katilim</t>
         </is>
       </c>
-      <c r="B9" s="27" t="n">
+      <c r="B9" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="27" t="n"/>
-      <c r="D9" s="27" t="n"/>
-      <c r="E9" s="27" t="n"/>
-      <c r="F9" s="28" t="inlineStr">
+      <c r="C9" s="30" t="n"/>
+      <c r="D9" s="30" t="n"/>
+      <c r="E9" s="30" t="n"/>
+      <c r="F9" s="31" t="inlineStr">
         <is>
           <t>Sprint 3 - dijital banka</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Hayat Finans</t>
         </is>
       </c>
-      <c r="B10" s="27" t="n">
+      <c r="B10" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="27" t="n"/>
-      <c r="D10" s="27" t="n"/>
-      <c r="E10" s="27" t="n"/>
-      <c r="F10" s="28" t="inlineStr">
+      <c r="C10" s="30" t="n"/>
+      <c r="D10" s="30" t="n"/>
+      <c r="E10" s="30" t="n"/>
+      <c r="F10" s="31" t="inlineStr">
         <is>
           <t>Sprint 3 - dijital banka</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>T.O.M. Katilim</t>
         </is>
       </c>
-      <c r="B11" s="27" t="n">
+      <c r="B11" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="27" t="n"/>
-      <c r="D11" s="27" t="n"/>
-      <c r="E11" s="27" t="n"/>
-      <c r="F11" s="28" t="inlineStr">
+      <c r="C11" s="30" t="n"/>
+      <c r="D11" s="30" t="n"/>
+      <c r="E11" s="30" t="n"/>
+      <c r="F11" s="31" t="inlineStr">
         <is>
           <t>Sprint 3 - dijital banka</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="32" t="inlineStr">
         <is>
           <t>TOPLAM HEDEF</t>
         </is>
       </c>
-      <c r="B13" s="29">
+      <c r="B13" s="32">
         <f>SUM(B2:B11)</f>
         <v/>
       </c>
-      <c r="C13" s="29">
+      <c r="C13" s="32">
         <f>SUM(C2:C11)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
feat: Albaraka Turk icin 6 yeni altin veri kaydi (AL-001..AL-006)
Ihtiyac Finansmani: Vade Farksiz 140.000 TL'ye Varan Destek (AL-001,
%0 kar payi, 40.000 TL, 6 ay - iki bolumlu kampanyanin finansman kismi).

Kart kampanyalari: MTV vade farksiz 3 taksit (AL-002), Saglik
harcamalarina vade farksiz 6 taksit (AL-005, 1.000-100.000 TL),
Egitim harcamalarina vade farksiz 6 taksit (AL-006, 30.000-500.000 TL).

Yeni musteri kampanyalari: Yurt disi cikis harci 1.250 TL Worldpuan
(AL-003), Yakinini davet et 5.000 TL'ye varan Worldpuan (AL-004).

Vade farksiz oranlarda oran_periyodu="belirsiz" kullanildi (KT-004/
KT-006 ile tutarli). Albaraka'nin 98/2 paylasimli Dijital Katilma
Hesabi kampanyasi mevduat urunu oldugu icin bilerek disarida birakildi
(Sayfa 3 Kapsam Disi'na girmesi gerekiyor).

Banka basina hedef (5-8 kayit) Albaraka Turk icin karsilandi: 6 kayit.
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -1212,7 +1212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U58"/>
+  <dimension ref="A1:U64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2339,143 +2339,505 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="24" t="n"/>
-      <c r="B14" s="24" t="n"/>
-      <c r="C14" s="24" t="n"/>
-      <c r="D14" s="24" t="n"/>
-      <c r="E14" s="24" t="n"/>
-      <c r="F14" s="25" t="n"/>
-      <c r="G14" s="25" t="n"/>
-      <c r="H14" s="24" t="n"/>
-      <c r="I14" s="26" t="n"/>
-      <c r="J14" s="25" t="n"/>
-      <c r="K14" s="25" t="n"/>
-      <c r="L14" s="24" t="n"/>
-      <c r="M14" s="24" t="n"/>
-      <c r="N14" s="24" t="n"/>
-      <c r="O14" s="27" t="n"/>
-      <c r="P14" s="27" t="n"/>
-      <c r="Q14" s="24" t="n"/>
-      <c r="R14" s="24" t="n"/>
-      <c r="S14" s="24" t="n"/>
-      <c r="T14" s="27" t="n"/>
-      <c r="U14" s="24" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="24" t="n"/>
-      <c r="B15" s="24" t="n"/>
-      <c r="C15" s="24" t="n"/>
-      <c r="D15" s="24" t="n"/>
-      <c r="E15" s="24" t="n"/>
-      <c r="F15" s="25" t="n"/>
-      <c r="G15" s="25" t="n"/>
-      <c r="H15" s="24" t="n"/>
-      <c r="I15" s="26" t="n"/>
-      <c r="J15" s="25" t="n"/>
-      <c r="K15" s="25" t="n"/>
-      <c r="L15" s="24" t="n"/>
-      <c r="M15" s="24" t="n"/>
-      <c r="N15" s="24" t="n"/>
-      <c r="O15" s="27" t="n"/>
-      <c r="P15" s="27" t="n"/>
-      <c r="Q15" s="24" t="n"/>
-      <c r="R15" s="24" t="n"/>
-      <c r="S15" s="24" t="n"/>
-      <c r="T15" s="27" t="n"/>
-      <c r="U15" s="24" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="24" t="n"/>
-      <c r="B16" s="24" t="n"/>
-      <c r="C16" s="24" t="n"/>
-      <c r="D16" s="24" t="n"/>
-      <c r="E16" s="24" t="n"/>
-      <c r="F16" s="25" t="n"/>
-      <c r="G16" s="25" t="n"/>
-      <c r="H16" s="24" t="n"/>
-      <c r="I16" s="26" t="n"/>
-      <c r="J16" s="25" t="n"/>
-      <c r="K16" s="25" t="n"/>
-      <c r="L16" s="24" t="n"/>
-      <c r="M16" s="24" t="n"/>
-      <c r="N16" s="24" t="n"/>
-      <c r="O16" s="27" t="n"/>
-      <c r="P16" s="27" t="n"/>
-      <c r="Q16" s="24" t="n"/>
-      <c r="R16" s="24" t="n"/>
-      <c r="S16" s="24" t="n"/>
-      <c r="T16" s="27" t="n"/>
-      <c r="U16" s="24" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="24" t="n"/>
-      <c r="B17" s="24" t="n"/>
-      <c r="C17" s="24" t="n"/>
-      <c r="D17" s="24" t="n"/>
-      <c r="E17" s="24" t="n"/>
-      <c r="F17" s="25" t="n"/>
-      <c r="G17" s="25" t="n"/>
-      <c r="H17" s="24" t="n"/>
-      <c r="I17" s="26" t="n"/>
-      <c r="J17" s="25" t="n"/>
-      <c r="K17" s="25" t="n"/>
-      <c r="L17" s="24" t="n"/>
-      <c r="M17" s="24" t="n"/>
-      <c r="N17" s="24" t="n"/>
-      <c r="O17" s="27" t="n"/>
-      <c r="P17" s="27" t="n"/>
-      <c r="Q17" s="24" t="n"/>
-      <c r="R17" s="24" t="n"/>
-      <c r="S17" s="24" t="n"/>
-      <c r="T17" s="27" t="n"/>
-      <c r="U17" s="24" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="24" t="n"/>
-      <c r="B18" s="24" t="n"/>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="24" t="n"/>
-      <c r="E18" s="24" t="n"/>
-      <c r="F18" s="25" t="n"/>
-      <c r="G18" s="25" t="n"/>
-      <c r="H18" s="24" t="n"/>
-      <c r="I18" s="26" t="n"/>
-      <c r="J18" s="25" t="n"/>
-      <c r="K18" s="25" t="n"/>
-      <c r="L18" s="24" t="n"/>
-      <c r="M18" s="24" t="n"/>
-      <c r="N18" s="24" t="n"/>
-      <c r="O18" s="27" t="n"/>
-      <c r="P18" s="27" t="n"/>
-      <c r="Q18" s="24" t="n"/>
-      <c r="R18" s="24" t="n"/>
-      <c r="S18" s="24" t="n"/>
-      <c r="T18" s="27" t="n"/>
-      <c r="U18" s="24" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="24" t="n"/>
-      <c r="B19" s="24" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="24" t="n"/>
-      <c r="F19" s="25" t="n"/>
-      <c r="G19" s="25" t="n"/>
-      <c r="H19" s="24" t="n"/>
-      <c r="I19" s="26" t="n"/>
-      <c r="J19" s="25" t="n"/>
-      <c r="K19" s="25" t="n"/>
-      <c r="L19" s="24" t="n"/>
-      <c r="M19" s="24" t="n"/>
-      <c r="N19" s="24" t="n"/>
-      <c r="O19" s="27" t="n"/>
-      <c r="P19" s="27" t="n"/>
-      <c r="Q19" s="24" t="n"/>
-      <c r="R19" s="24" t="n"/>
-      <c r="S19" s="24" t="n"/>
-      <c r="T19" s="27" t="n"/>
-      <c r="U19" s="24" t="n"/>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>AL-001</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>Vade Farksız 140.000 TL'ye Varan Destek!</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Ihtiyac Finansmani Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/vade-farksiz-kampanyasi</t>
+        </is>
+      </c>
+      <c r="F14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="21" t="n"/>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>aylik</t>
+        </is>
+      </c>
+      <c r="I14" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="J14" s="21" t="n">
+        <v>40000</v>
+      </c>
+      <c r="K14" s="21" t="n"/>
+      <c r="L14" s="19" t="n"/>
+      <c r="M14" s="20" t="inlineStr">
+        <is>
+          <t>%0 kâr paylı 40.000 TL'ye kadar Pratik Finansman Kart + 100.000 TL'ye kadar vade farksız taksitli alışveriş = toplam 140.000 TL</t>
+        </is>
+      </c>
+      <c r="N14" s="20" t="n"/>
+      <c r="O14" s="23" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="P14" s="23" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q14" s="20" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil'den yeni müşteri olanlar</t>
+        </is>
+      </c>
+      <c r="R14" s="19" t="inlineStr">
+        <is>
+          <t>AL-001.png</t>
+        </is>
+      </c>
+      <c r="S14" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T14" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U14" s="20" t="inlineStr">
+        <is>
+          <t>Kampanya iki bölümlü: 40.000 TL'lik kısım İhtiyaç Finansmanı (Pratik Finansman Kart), 100.000 TL'lik kısım kredi kartıyla vade farksız taksit - ilk kısım temel alındı</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>AL-002</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C15" s="20" t="inlineStr">
+        <is>
+          <t>MTV Ödemelerinize Vade Farksız 3 Taksit!</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/mtv-odemelerinize-vade-farksiz-3-taksit-10</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
+      <c r="I15" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" s="21" t="n"/>
+      <c r="K15" s="21" t="n"/>
+      <c r="L15" s="19" t="n"/>
+      <c r="M15" s="20" t="inlineStr">
+        <is>
+          <t>MTV 2026 2. dönem ödemelerine kredi kartıyla vade farksız 3 taksit</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="n"/>
+      <c r="O15" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P15" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="Q15" s="20" t="inlineStr">
+        <is>
+          <t>Bireysel ve Business Albaraka Worldcard sahipleri</t>
+        </is>
+      </c>
+      <c r="R15" s="19" t="inlineStr">
+        <is>
+          <t>AL-002.png</t>
+        </is>
+      </c>
+      <c r="S15" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T15" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U15" s="20" t="inlineStr">
+        <is>
+          <t>ivd.gib.gov.tr üzerinden yapılan ödemeler peşin tahsil ediliyor, bu kampanya dışında</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>AL-003</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>Yurt Dışı Çıkış Harcı Kampanyası | 1.250 TL Worldpuan!</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Yeni Musteri Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/yurt-disi-cikis-harci-kampanyasi-1250-tl-worldpuan-3</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="n"/>
+      <c r="G16" s="21" t="n"/>
+      <c r="H16" s="19" t="n"/>
+      <c r="I16" s="22" t="n"/>
+      <c r="J16" s="21" t="n"/>
+      <c r="K16" s="21" t="n">
+        <v>1250</v>
+      </c>
+      <c r="L16" s="19" t="inlineStr">
+        <is>
+          <t>Worldpuan</t>
+        </is>
+      </c>
+      <c r="M16" s="20" t="inlineStr">
+        <is>
+          <t>Görüntülü görüşmeyle yeni müşteri olup Albaraka World kartla yurt dışı çıkış harcı ödeyene 1.250 TL Worldpuan</t>
+        </is>
+      </c>
+      <c r="N16" s="20" t="n"/>
+      <c r="O16" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P16" s="23" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q16" s="20" t="inlineStr">
+        <is>
+          <t>1 Temmuz 2026 sonrası mobilden görüntülü görüşmeyle yeni müşteri olanlar</t>
+        </is>
+      </c>
+      <c r="R16" s="19" t="inlineStr">
+        <is>
+          <t>AL-003.png</t>
+        </is>
+      </c>
+      <c r="S16" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T16" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U16" s="20" t="inlineStr">
+        <is>
+          <t>Kampanya 1.000 kişiyle sınırlı; Master Gold Virtual/Standart ve Business kartlar hariç</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>AL-004</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>Yakınını Davet Et Kampanyası</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Yeni Musteri Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/yakinini-davet-et-kampanyasi</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="n"/>
+      <c r="G17" s="21" t="n"/>
+      <c r="H17" s="19" t="n"/>
+      <c r="I17" s="22" t="n"/>
+      <c r="J17" s="21" t="n"/>
+      <c r="K17" s="21" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L17" s="19" t="inlineStr">
+        <is>
+          <t>Worldpuan</t>
+        </is>
+      </c>
+      <c r="M17" s="20" t="inlineStr">
+        <is>
+          <t>Her davet edilen ve müşteri olan yakın için 500 TL, toplamda 5.000 TL'ye varan Worldpuan (davet edilen de 500 TL kazanıyor)</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="n"/>
+      <c r="O17" s="23" t="inlineStr">
+        <is>
+          <t>2024-04-14</t>
+        </is>
+      </c>
+      <c r="P17" s="23" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q17" s="20" t="inlineStr">
+        <is>
+          <t>Albaraka World kartlı müşteriler, davet ettikleri 18 yaş üzeri kişiler</t>
+        </is>
+      </c>
+      <c r="R17" s="19" t="inlineStr">
+        <is>
+          <t>AL-004.png</t>
+        </is>
+      </c>
+      <c r="S17" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T17" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U17" s="20" t="inlineStr">
+        <is>
+          <t>Ödül davet edilenin görüntülü görüşmeyle müşteri olmasına bağlı, başka kanaldan olursa ödül yok</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>AL-005</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="inlineStr">
+        <is>
+          <t>Sağlık Harcamalarına Vade Farksız 6 Taksit Kampanyası</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/saglik-harcamalarina-vade-farksiz-6-taksit-kampanyasi-1_1</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="21" t="n"/>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
+      <c r="I18" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="J18" s="21" t="n">
+        <v>100000</v>
+      </c>
+      <c r="K18" s="21" t="n"/>
+      <c r="L18" s="19" t="n"/>
+      <c r="M18" s="20" t="inlineStr">
+        <is>
+          <t>TROY kredi kartıyla 1.000-100.000 TL sağlık harcamasına vade farksız 6 taksit, kampanya başına en fazla 5 kez</t>
+        </is>
+      </c>
+      <c r="N18" s="20" t="n"/>
+      <c r="O18" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P18" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="Q18" s="20" t="inlineStr">
+        <is>
+          <t>TROY kredi kartı sahibi bireysel müşteriler</t>
+        </is>
+      </c>
+      <c r="R18" s="19" t="inlineStr">
+        <is>
+          <t>AL-005.png</t>
+        </is>
+      </c>
+      <c r="S18" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T18" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U18" s="20" t="inlineStr">
+        <is>
+          <t>Katılmadan önce yapılan işlemler kapsam dışı; sadece belirli MCC kodları (eczane, diş hekimi, ortopedi vb.) geçerli</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>AL-006</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C19" s="20" t="inlineStr">
+        <is>
+          <t>Eğitim Harcamalarınıza Vade Farksız 6 Taksit Kampanyası</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/egitim-kampanyasi-1</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="21" t="n"/>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
+      <c r="I19" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="J19" s="21" t="n">
+        <v>500000</v>
+      </c>
+      <c r="K19" s="21" t="n"/>
+      <c r="L19" s="19" t="n"/>
+      <c r="M19" s="20" t="inlineStr">
+        <is>
+          <t>World kartla 30.000-500.000 TL okul ödemesine vade farksız 6 taksit, kampanya boyunca en fazla 2 kez</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="n"/>
+      <c r="O19" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P19" s="23" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="Q19" s="20" t="inlineStr">
+        <is>
+          <t>Albaraka World özellikli kredi kartı sahibi bireysel müşteriler</t>
+        </is>
+      </c>
+      <c r="R19" s="19" t="inlineStr">
+        <is>
+          <t>AL-006.png</t>
+        </is>
+      </c>
+      <c r="S19" s="19" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T19" s="23" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="U19" s="20" t="inlineStr">
+        <is>
+          <t>Business kartlar ve Master Gold Kart kapsam dışı</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="24" t="n"/>
@@ -3374,27 +3736,165 @@
       <c r="T58" s="27" t="n"/>
       <c r="U58" s="24" t="n"/>
     </row>
+    <row r="59">
+      <c r="A59" s="24" t="n"/>
+      <c r="B59" s="24" t="n"/>
+      <c r="C59" s="24" t="n"/>
+      <c r="D59" s="24" t="n"/>
+      <c r="E59" s="24" t="n"/>
+      <c r="F59" s="25" t="n"/>
+      <c r="G59" s="25" t="n"/>
+      <c r="H59" s="24" t="n"/>
+      <c r="I59" s="26" t="n"/>
+      <c r="J59" s="25" t="n"/>
+      <c r="K59" s="25" t="n"/>
+      <c r="L59" s="24" t="n"/>
+      <c r="M59" s="24" t="n"/>
+      <c r="N59" s="24" t="n"/>
+      <c r="O59" s="27" t="n"/>
+      <c r="P59" s="27" t="n"/>
+      <c r="Q59" s="24" t="n"/>
+      <c r="R59" s="24" t="n"/>
+      <c r="S59" s="24" t="n"/>
+      <c r="T59" s="27" t="n"/>
+      <c r="U59" s="24" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="24" t="n"/>
+      <c r="B60" s="24" t="n"/>
+      <c r="C60" s="24" t="n"/>
+      <c r="D60" s="24" t="n"/>
+      <c r="E60" s="24" t="n"/>
+      <c r="F60" s="25" t="n"/>
+      <c r="G60" s="25" t="n"/>
+      <c r="H60" s="24" t="n"/>
+      <c r="I60" s="26" t="n"/>
+      <c r="J60" s="25" t="n"/>
+      <c r="K60" s="25" t="n"/>
+      <c r="L60" s="24" t="n"/>
+      <c r="M60" s="24" t="n"/>
+      <c r="N60" s="24" t="n"/>
+      <c r="O60" s="27" t="n"/>
+      <c r="P60" s="27" t="n"/>
+      <c r="Q60" s="24" t="n"/>
+      <c r="R60" s="24" t="n"/>
+      <c r="S60" s="24" t="n"/>
+      <c r="T60" s="27" t="n"/>
+      <c r="U60" s="24" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="24" t="n"/>
+      <c r="B61" s="24" t="n"/>
+      <c r="C61" s="24" t="n"/>
+      <c r="D61" s="24" t="n"/>
+      <c r="E61" s="24" t="n"/>
+      <c r="F61" s="25" t="n"/>
+      <c r="G61" s="25" t="n"/>
+      <c r="H61" s="24" t="n"/>
+      <c r="I61" s="26" t="n"/>
+      <c r="J61" s="25" t="n"/>
+      <c r="K61" s="25" t="n"/>
+      <c r="L61" s="24" t="n"/>
+      <c r="M61" s="24" t="n"/>
+      <c r="N61" s="24" t="n"/>
+      <c r="O61" s="27" t="n"/>
+      <c r="P61" s="27" t="n"/>
+      <c r="Q61" s="24" t="n"/>
+      <c r="R61" s="24" t="n"/>
+      <c r="S61" s="24" t="n"/>
+      <c r="T61" s="27" t="n"/>
+      <c r="U61" s="24" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="24" t="n"/>
+      <c r="B62" s="24" t="n"/>
+      <c r="C62" s="24" t="n"/>
+      <c r="D62" s="24" t="n"/>
+      <c r="E62" s="24" t="n"/>
+      <c r="F62" s="25" t="n"/>
+      <c r="G62" s="25" t="n"/>
+      <c r="H62" s="24" t="n"/>
+      <c r="I62" s="26" t="n"/>
+      <c r="J62" s="25" t="n"/>
+      <c r="K62" s="25" t="n"/>
+      <c r="L62" s="24" t="n"/>
+      <c r="M62" s="24" t="n"/>
+      <c r="N62" s="24" t="n"/>
+      <c r="O62" s="27" t="n"/>
+      <c r="P62" s="27" t="n"/>
+      <c r="Q62" s="24" t="n"/>
+      <c r="R62" s="24" t="n"/>
+      <c r="S62" s="24" t="n"/>
+      <c r="T62" s="27" t="n"/>
+      <c r="U62" s="24" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="24" t="n"/>
+      <c r="B63" s="24" t="n"/>
+      <c r="C63" s="24" t="n"/>
+      <c r="D63" s="24" t="n"/>
+      <c r="E63" s="24" t="n"/>
+      <c r="F63" s="25" t="n"/>
+      <c r="G63" s="25" t="n"/>
+      <c r="H63" s="24" t="n"/>
+      <c r="I63" s="26" t="n"/>
+      <c r="J63" s="25" t="n"/>
+      <c r="K63" s="25" t="n"/>
+      <c r="L63" s="24" t="n"/>
+      <c r="M63" s="24" t="n"/>
+      <c r="N63" s="24" t="n"/>
+      <c r="O63" s="27" t="n"/>
+      <c r="P63" s="27" t="n"/>
+      <c r="Q63" s="24" t="n"/>
+      <c r="R63" s="24" t="n"/>
+      <c r="S63" s="24" t="n"/>
+      <c r="T63" s="27" t="n"/>
+      <c r="U63" s="24" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="24" t="n"/>
+      <c r="B64" s="24" t="n"/>
+      <c r="C64" s="24" t="n"/>
+      <c r="D64" s="24" t="n"/>
+      <c r="E64" s="24" t="n"/>
+      <c r="F64" s="25" t="n"/>
+      <c r="G64" s="25" t="n"/>
+      <c r="H64" s="24" t="n"/>
+      <c r="I64" s="26" t="n"/>
+      <c r="J64" s="25" t="n"/>
+      <c r="K64" s="25" t="n"/>
+      <c r="L64" s="24" t="n"/>
+      <c r="M64" s="24" t="n"/>
+      <c r="N64" s="24" t="n"/>
+      <c r="O64" s="27" t="n"/>
+      <c r="P64" s="27" t="n"/>
+      <c r="Q64" s="24" t="n"/>
+      <c r="R64" s="24" t="n"/>
+      <c r="S64" s="24" t="n"/>
+      <c r="T64" s="27" t="n"/>
+      <c r="U64" s="24" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:U1"/>
   <dataValidations count="6">
-    <dataValidation sqref="D3:D58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz kampanya turu" error="Listeden bir deger secin. Emin degilseniz 'Belirlenemedi' secin." type="list">
+    <dataValidation sqref="D3:D64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz kampanya turu" error="Listeden bir deger secin. Emin degilseniz 'Belirlenemedi' secin." type="list">
       <formula1>"Konut Finansmani Kampanyasi,Ihtiyac Finansmani Kampanyasi,Tasit Finansmani Kampanyasi,Finansman Kampanyasi,Kart Kampanyasi,Alisveris Puani Kampanyasi,Yeni Musteri Kampanyasi,Yatirim Urunu Kampanyasi,Belirlenemedi"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz oran periyodu" error="Sayfada ne yaziyorsa onu secin. Yazmiyorsa tahmin etmeyin: 'belirsiz'." type="list">
+    <dataValidation sqref="H3:H64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz oran periyodu" error="Sayfada ne yaziyorsa onu secin. Yazmiyorsa tahmin etmeyin: 'belirsiz'." type="list">
       <formula1>"aylik,yillik,belirsiz"</formula1>
     </dataValidation>
-    <dataValidation sqref="L3:L58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz odul birimi" error="Listeden bir birim secin." type="list">
+    <dataValidation sqref="L3:L64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz odul birimi" error="Listeden bir birim secin." type="list">
       <formula1>"TL,Mil,Gram,Puan,Worldpuan,ParafPara,Bankkart Lira"</formula1>
     </dataValidation>
-    <dataValidation sqref="F3:F58 G3:G58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz oran" error="Sadece 0-100 arasi sayi yazin, VIRGULLE (yuzde isareti olmadan). Ornek: 1,99" type="decimal" operator="between">
+    <dataValidation sqref="F3:F64 G3:G64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz oran" error="Sadece 0-100 arasi sayi yazin, VIRGULLE (yuzde isareti olmadan). Ornek: 1,99" type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="I3:I58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz vade" error="Sadece tam sayi (ay) yazin, 0-480 arasi. Ornek: 120" type="whole" operator="between">
+    <dataValidation sqref="I3:I64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz vade" error="Sadece tam sayi (ay) yazin, 0-480 arasi. Ornek: 120" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>480</formula2>
     </dataValidation>
-    <dataValidation sqref="J3:J58 K3:K58" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz tutar" error="Sadece sayi yazin (TL isareti olmadan). Ornek: 500000" type="decimal" operator="greaterThanOrEqual">
+    <dataValidation sqref="J3:J64 K3:K64" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Gecersiz tutar" error="Sadece sayi yazin (TL isareti olmadan). Ornek: 500000" type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: altin veri setine taksit_sayisi ve erteleme_suresi_ay sutunlari eklendi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1. Nasil Doldurulur" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2. Altin Veri Seti" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3. Kapsam Disi (Ayri Tut)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4. Ilerleme Takibi" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Nasil Doldurulur" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Altin Veri Seti" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Kapsam Disi (Ayri Tut)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Ilerleme Takibi" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2. Altin Veri Seti'!$A$1:$U$1</definedName>
@@ -1212,7 +1212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U109"/>
+  <dimension ref="A1:W109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1236,6 +1236,8 @@
     <col width="14" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="40" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1344,6 +1346,16 @@
           <t>notlar</t>
         </is>
       </c>
+      <c r="V1" s="32" t="inlineStr">
+        <is>
+          <t>taksit_sayisi</t>
+        </is>
+      </c>
+      <c r="W1" s="32" t="inlineStr">
+        <is>
+          <t>erteleme_suresi_ay</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="45" customHeight="1">
       <c r="A2" s="13" t="inlineStr">
@@ -1449,6 +1461,16 @@
       <c r="U2" s="13" t="inlineStr">
         <is>
           <t>Ozel durumlar, ikinci URL, belirsizlikler</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>SADECE SAYI. '12 aya varan taksit' -&gt; 12. VADE DEGIL (ayri kavram). Sayfada yoksa BOS birak.</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>SADECE SAYI, ay cinsinden. '2 ay ertelemeli' / '3 ay odemesiz donem' -&gt; 2 / 3. Sayfada yoksa BOS birak.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: altin veri setinde taksit degerleri vade_ay sutununa yazilmisti
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -2230,9 +2230,7 @@
       <c r="F12" s="21" t="n"/>
       <c r="G12" s="21" t="n"/>
       <c r="H12" s="19" t="n"/>
-      <c r="I12" s="22" t="n">
-        <v>5</v>
-      </c>
+      <c r="I12" s="22" t="n"/>
       <c r="J12" s="21" t="n">
         <v>50000</v>
       </c>
@@ -2276,8 +2274,11 @@
       </c>
       <c r="U12" s="20" t="inlineStr">
         <is>
-          <t>vade_ay alanı burada "taksit sayısı" anlamında kullanıldı, klasik kredi vadesi değil - CampaignRecord şemasıyla tam örtüşmüyor, ekiple bu ayrımı konuşmak gerekebilir</t>
-        </is>
+          <t>vade_ay alanı burada "taksit sayısı" anlamında kullanıldı, klasik kredi vadesi değil - CampaignRecord şemasıyla tam örtüşmüyor, ekiple bu ayrımı konuşmak gerekebilir | [9 Agu] vade_ay-&gt;taksit_sayisi tasindi (Vade Farksiz 5 Aya Varan Taksit Imkani); sayfada vade ifadesi yok</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
@@ -2396,9 +2397,7 @@
           <t>aylik</t>
         </is>
       </c>
-      <c r="I14" s="22" t="n">
-        <v>6</v>
-      </c>
+      <c r="I14" s="22" t="n"/>
       <c r="J14" s="21" t="n">
         <v>40000</v>
       </c>
@@ -2442,8 +2441,11 @@
       </c>
       <c r="U14" s="20" t="inlineStr">
         <is>
-          <t>Kampanya iki bölümlü: 40.000 TL'lik kısım İhtiyaç Finansmanı (Pratik Finansman Kart), 100.000 TL'lik kısım kredi kartıyla vade farksız taksit - ilk kısım temel alındı</t>
-        </is>
+          <t>Kampanya iki bölümlü: 40.000 TL'lik kısım İhtiyaç Finansmanı (Pratik Finansman Kart), 100.000 TL'lik kısım kredi kartıyla vade farksız taksit - ilk kısım temel alındı | [9 Agu] vade_ay-&gt;taksit_sayisi tasindi (Secili sektorlerde vade farksiz 6 taksit); sayfada vade ifadesi yok</t>
+        </is>
+      </c>
+      <c r="V14" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
@@ -2481,9 +2483,7 @@
           <t>belirsiz</t>
         </is>
       </c>
-      <c r="I15" s="22" t="n">
-        <v>3</v>
-      </c>
+      <c r="I15" s="22" t="n"/>
       <c r="J15" s="21" t="n"/>
       <c r="K15" s="21" t="n"/>
       <c r="L15" s="19" t="n"/>
@@ -2525,8 +2525,11 @@
       </c>
       <c r="U15" s="20" t="inlineStr">
         <is>
-          <t>ivd.gib.gov.tr üzerinden yapılan ödemeler peşin tahsil ediliyor, bu kampanya dışında</t>
-        </is>
+          <t>ivd.gib.gov.tr üzerinden yapılan ödemeler peşin tahsil ediliyor, bu kampanya dışında | [9 Agu] vade_ay-&gt;taksit_sayisi tasindi (MTV Odemelerinize Vade Farksiz 3 Taksit); sayfada vade ifadesi yok</t>
+        </is>
+      </c>
+      <c r="V15" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
@@ -2726,9 +2729,7 @@
           <t>belirsiz</t>
         </is>
       </c>
-      <c r="I18" s="22" t="n">
-        <v>6</v>
-      </c>
+      <c r="I18" s="22" t="n"/>
       <c r="J18" s="21" t="n">
         <v>100000</v>
       </c>
@@ -2772,8 +2773,11 @@
       </c>
       <c r="U18" s="20" t="inlineStr">
         <is>
-          <t>Katılmadan önce yapılan işlemler kapsam dışı; sadece belirli MCC kodları (eczane, diş hekimi, ortopedi vb.) geçerli</t>
-        </is>
+          <t>Katılmadan önce yapılan işlemler kapsam dışı; sadece belirli MCC kodları (eczane, diş hekimi, ortopedi vb.) geçerli | [9 Agu] vade_ay-&gt;taksit_sayisi tasindi (Saglik Harcamalarina Vade Farksiz 6 Taksit); sayfada vade ifadesi yok</t>
+        </is>
+      </c>
+      <c r="V18" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
@@ -2811,9 +2815,7 @@
           <t>belirsiz</t>
         </is>
       </c>
-      <c r="I19" s="22" t="n">
-        <v>6</v>
-      </c>
+      <c r="I19" s="22" t="n"/>
       <c r="J19" s="21" t="n">
         <v>500000</v>
       </c>
@@ -2857,8 +2859,11 @@
       </c>
       <c r="U19" s="20" t="inlineStr">
         <is>
-          <t>Business kartlar ve Master Gold Kart kapsam dışı</t>
-        </is>
+          <t>Business kartlar ve Master Gold Kart kapsam dışı | [9 Agu] vade_ay-&gt;taksit_sayisi tasindi (Egitim Harcamalarina Vade Farksiz 6 Taksit); sayfada vade ifadesi yok</t>
+        </is>
+      </c>
+      <c r="V19" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
@@ -6285,9 +6290,7 @@
           <t>belirsiz</t>
         </is>
       </c>
-      <c r="I63" s="22" t="n">
-        <v>10</v>
-      </c>
+      <c r="I63" s="22" t="n"/>
       <c r="J63" s="21" t="n">
         <v>250000</v>
       </c>
@@ -6331,8 +6334,11 @@
       </c>
       <c r="U63" s="20" t="inlineStr">
         <is>
-          <t>4 paket var (Standart/Orta/Ust/Ekstra: 250K-1,5M TL); en dusuk paket temel alindi. Vade farki iadesi, Gunluk Kazandiran Hesabinda ilgili tutar kadar birikim VEYA kredi bakiyesi sartina bagli - karmasik, notlarda ozetlendi</t>
-        </is>
+          <t>4 paket var (Standart/Orta/Ust/Ekstra: 250K-1,5M TL); en dusuk paket temel alindi. Vade farki iadesi, Gunluk Kazandiran Hesabinda ilgili tutar kadar birikim VEYA kredi bakiyesi sartina bagli - karmasik, notlarda ozetlendi | [9 Agu] vade_ay-&gt;taksit_sayisi tasindi (Ozel Okul Odemelerinde 10 Taksit); sayfada vade ifadesi yok</t>
+        </is>
+      </c>
+      <c r="V63" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="64" ht="28" customHeight="1">

</xml_diff>

<commit_message>
data: AL-007 altin kayit taslagi - Albaraka fatura kampanyasi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -6423,27 +6423,77 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="24" t="n"/>
-      <c r="B65" s="24" t="n"/>
-      <c r="C65" s="24" t="n"/>
-      <c r="D65" s="24" t="n"/>
-      <c r="E65" s="24" t="n"/>
+      <c r="A65" s="24" t="inlineStr">
+        <is>
+          <t>AL-007</t>
+        </is>
+      </c>
+      <c r="B65" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C65" s="24" t="inlineStr">
+        <is>
+          <t>Ağustos Ayına Özel Fatura Kampanyası</t>
+        </is>
+      </c>
+      <c r="D65" s="24" t="inlineStr">
+        <is>
+          <t>Yeni Musteri Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E65" s="24" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/agustos-ayina-ozel-fatura-kampanyasi</t>
+        </is>
+      </c>
       <c r="F65" s="25" t="n"/>
       <c r="G65" s="25" t="n"/>
       <c r="H65" s="24" t="n"/>
       <c r="I65" s="26" t="n"/>
       <c r="J65" s="25" t="n"/>
-      <c r="K65" s="25" t="n"/>
-      <c r="L65" s="24" t="n"/>
-      <c r="M65" s="24" t="n"/>
+      <c r="K65" s="25" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L65" s="24" t="inlineStr">
+        <is>
+          <t>Worldpuan</t>
+        </is>
+      </c>
+      <c r="M65" s="24" t="inlineStr">
+        <is>
+          <t>OFT2026 koduyla görüntülü görüşmeyle müşteri olup Albaraka World kartla verilen her otomatik fatura ödeme talimatına 500 TL, toplamda 2.000 TL Worldpuan</t>
+        </is>
+      </c>
       <c r="N65" s="24" t="n"/>
-      <c r="O65" s="27" t="n"/>
-      <c r="P65" s="27" t="n"/>
-      <c r="Q65" s="24" t="n"/>
+      <c r="O65" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="P65" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q65" s="24" t="inlineStr">
+        <is>
+          <t>OFT2026 davet koduyla görüntülü görüşmeden ilk kez müşteri olan bireysel müşteriler</t>
+        </is>
+      </c>
       <c r="R65" s="24" t="n"/>
       <c r="S65" s="24" t="n"/>
-      <c r="T65" s="27" t="n"/>
-      <c r="U65" s="24" t="n"/>
+      <c r="T65" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U65" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya adi sayfada baslik satiri olmadigi icin URL slug'indan turetildi. Talimat basina 500 TL, musteri basina tavan 2.000 TL. Kampanya 1.000 kisiyle sinirli; Master Gold Virtual/Standart ve Business kartlar haric. Odul 1-5 Ekim 2026'da yuklenir.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="24" t="n"/>

</xml_diff>

<commit_message>
feat: kanit spani Excel'den JSON'a akiyor, AL-007 spanlari dolduruldu
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -1212,7 +1212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W109"/>
+  <dimension ref="A1:X109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1238,6 +1238,7 @@
     <col width="40" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
     <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="60" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1354,6 +1355,11 @@
       <c r="W1" s="32" t="inlineStr">
         <is>
           <t>erteleme_suresi_ay</t>
+        </is>
+      </c>
+      <c r="X1" s="32" t="inlineStr">
+        <is>
+          <t>kanit_spanlari</t>
         </is>
       </c>
     </row>
@@ -6492,6 +6498,15 @@
       <c r="U65" s="24" t="inlineStr">
         <is>
           <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya adi sayfada baslik satiri olmadigi icin URL slug'indan turetildi. Talimat basina 500 TL, musteri basina tavan 2.000 TL. Kampanya 1.000 kisiyle sinirli; Master Gold Virtual/Standart ve Business kartlar haric. Odul 1-5 Ekim 2026'da yuklenir.</t>
+        </is>
+      </c>
+      <c r="X65" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Kampanya müşteri bazındadır, bir müşteri en fazla 2.000 TL Worldpuan kazanabilir.
+odul_birimi: Kampanya müşteri bazındadır, bir müşteri en fazla 2.000 TL Worldpuan kazanabilir.
+kampanya_baslangic: Kampanya 1–31 Ağustos 2026 tarihlerinde geçerlidir.
+kampanya_bitis: Kampanya 31 Ağustos 2026 tarihine kadar geçerlidir.
+hedef_kitle: Kampanya 1-31 Ağustos 2026 tarihleri arasında “OFT2026” davet kodunu kullanarak görüntülü görüşme ile ilk kez müşterimiz olanlar için geçerlidir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: AL-008 altin kayit taslagi - Albaraka ISPARK kampanyasi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -6511,11 +6511,31 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="24" t="n"/>
-      <c r="B66" s="24" t="n"/>
-      <c r="C66" s="24" t="n"/>
-      <c r="D66" s="24" t="n"/>
-      <c r="E66" s="24" t="n"/>
+      <c r="A66" s="24" t="inlineStr">
+        <is>
+          <t>AL-008</t>
+        </is>
+      </c>
+      <c r="B66" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C66" s="24" t="inlineStr">
+        <is>
+          <t>Albarakalılara Özel Ücretsiz İSPARK Kampanyası</t>
+        </is>
+      </c>
+      <c r="D66" s="24" t="inlineStr">
+        <is>
+          <t>Belirlenemedi</t>
+        </is>
+      </c>
+      <c r="E66" s="24" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/albarakalilara-ozel-ucretsiz-ispark-kampanyasi-1</t>
+        </is>
+      </c>
       <c r="F66" s="25" t="n"/>
       <c r="G66" s="25" t="n"/>
       <c r="H66" s="24" t="n"/>
@@ -6523,15 +6543,46 @@
       <c r="J66" s="25" t="n"/>
       <c r="K66" s="25" t="n"/>
       <c r="L66" s="24" t="n"/>
-      <c r="M66" s="24" t="n"/>
+      <c r="M66" s="24" t="inlineStr">
+        <is>
+          <t>Cari hesabında 10.000 TL ve üzeri bakiyesi olan bireysel müşterilere İSPARK otoparklarında ayda 2 defa ücretsiz park (yol üstü 2 saat, bariyerli 4 saat)</t>
+        </is>
+      </c>
       <c r="N66" s="24" t="n"/>
-      <c r="O66" s="27" t="n"/>
-      <c r="P66" s="27" t="n"/>
-      <c r="Q66" s="24" t="n"/>
+      <c r="O66" s="27" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="P66" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q66" s="24" t="inlineStr">
+        <is>
+          <t>Cari hesabında 10.000 TL ve üzerinde bakiyesi bulunan bireysel müşteriler</t>
+        </is>
+      </c>
       <c r="R66" s="24" t="n"/>
       <c r="S66" s="24" t="n"/>
-      <c r="T66" s="27" t="n"/>
-      <c r="U66" s="24" t="n"/>
+      <c r="T66" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U66" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Parasal odul YOK: 'ayda 2 defa ucretsiz park' hizmet avantajidir, 10.000 TL ise uygunluk esigidir - ikisi de odul_miktari DEGILDIR (bu kayit, motorun olmayan odul uydurup uydurmadigini olcer). Yalnizca binek otomobil; bazi otoparklar ve mac gunleri haric.</t>
+        </is>
+      </c>
+      <c r="X66" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 1 Ocak 2026 – 31 Aralık 2026
+kampanya_bitis: 1 Ocak 2026 – 31 Aralık 2026
+hedef_kitle: cari hesabında 10.000 TL ve üzerinde bakiyesi</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="24" t="n"/>

</xml_diff>

<commit_message>
altin veri setine AL-009 ve HF-006 eklendi, is listesine kopya kampanya isareti
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -6585,11 +6585,31 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="24" t="n"/>
-      <c r="B67" s="24" t="n"/>
-      <c r="C67" s="24" t="n"/>
-      <c r="D67" s="24" t="n"/>
-      <c r="E67" s="24" t="n"/>
+      <c r="A67" s="24" t="inlineStr">
+        <is>
+          <t>AL-009</t>
+        </is>
+      </c>
+      <c r="B67" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C67" s="24" t="inlineStr">
+        <is>
+          <t>Dijital Katılma Hesabına Özel Paylaşım Oranları</t>
+        </is>
+      </c>
+      <c r="D67" s="24" t="inlineStr">
+        <is>
+          <t>Yatirim Urunu Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E67" s="24" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/dijital-katilma-hesabina-ozel-paylasim-oranlari-10</t>
+        </is>
+      </c>
       <c r="F67" s="25" t="n"/>
       <c r="G67" s="25" t="n"/>
       <c r="H67" s="24" t="n"/>
@@ -6597,38 +6617,120 @@
       <c r="J67" s="25" t="n"/>
       <c r="K67" s="25" t="n"/>
       <c r="L67" s="24" t="n"/>
-      <c r="M67" s="24" t="n"/>
+      <c r="M67" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil'den açılan TL Dijital Katılma Hesabında 98/2 kâr paylaşım oranı (asgari 250 TL)</t>
+        </is>
+      </c>
       <c r="N67" s="24" t="n"/>
-      <c r="O67" s="27" t="n"/>
-      <c r="P67" s="27" t="n"/>
-      <c r="Q67" s="24" t="n"/>
+      <c r="O67" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="P67" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q67" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil'den görüntülü görüşmeyle ilk kez müşteri olan ve TL Katılma Hesabı açan gerçek kişiler</t>
+        </is>
+      </c>
       <c r="R67" s="24" t="n"/>
       <c r="S67" s="24" t="n"/>
-      <c r="T67" s="27" t="n"/>
-      <c r="U67" s="24" t="n"/>
+      <c r="T67" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U67" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: '98/2 kar paylasim orani' bir yuzde DEGIL, paylasim seklidir (musteriye 98, bankaya 2). Bu kayit, motorun 98'i oran sanip sanmadigini olcer. Ad sayfada baslik satiri olmadigi icin URL slug'indan turetildi.</t>
+        </is>
+      </c>
+      <c r="X67" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 1 Nisan – 31 Aralık 2026
+kampanya_bitis: 1 Nisan – 31 Aralık 2026</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="24" t="n"/>
-      <c r="B68" s="24" t="n"/>
-      <c r="C68" s="24" t="n"/>
-      <c r="D68" s="24" t="n"/>
-      <c r="E68" s="24" t="n"/>
+      <c r="A68" s="24" t="inlineStr">
+        <is>
+          <t>HF-006</t>
+        </is>
+      </c>
+      <c r="B68" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans</t>
+        </is>
+      </c>
+      <c r="C68" s="24" t="inlineStr">
+        <is>
+          <t>Bana Bunu Al İş Ortağım ile Troy Mağazalarında Finansman Fırsatı!</t>
+        </is>
+      </c>
+      <c r="D68" s="24" t="inlineStr">
+        <is>
+          <t>Finansman Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E68" s="24" t="inlineStr">
+        <is>
+          <t>www.hayatfinans.com.tr/kampanyalar/bana-bunu-al-is-ortagim-ile-troy-magaza-firsatlari</t>
+        </is>
+      </c>
       <c r="F68" s="25" t="n"/>
       <c r="G68" s="25" t="n"/>
       <c r="H68" s="24" t="n"/>
       <c r="I68" s="26" t="n"/>
-      <c r="J68" s="25" t="n"/>
+      <c r="J68" s="25" t="n">
+        <v>80000</v>
+      </c>
       <c r="K68" s="25" t="n"/>
       <c r="L68" s="24" t="n"/>
-      <c r="M68" s="24" t="n"/>
+      <c r="M68" s="24" t="inlineStr">
+        <is>
+          <t>Troy fiziksel mağazalarında 3 aya varan taksit; kampanya üst limiti 80.000 TL</t>
+        </is>
+      </c>
       <c r="N68" s="24" t="n"/>
       <c r="O68" s="27" t="n"/>
-      <c r="P68" s="27" t="n"/>
-      <c r="Q68" s="24" t="n"/>
+      <c r="P68" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q68" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans müşterileri (Bana Bunu Al İş Ortağım)</t>
+        </is>
+      </c>
       <c r="R68" s="24" t="n"/>
       <c r="S68" s="24" t="n"/>
-      <c r="T68" s="27" t="n"/>
-      <c r="U68" s="24" t="n"/>
+      <c r="T68" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U68" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Baslangic tarihi sayfada belirtilmemis. Yalnizca fiziksel magazalar.</t>
+        </is>
+      </c>
+      <c r="V68" t="n">
+        <v>3</v>
+      </c>
+      <c r="X68" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 3 aya varan taksit fırsatı
+finansman_tutari: Kampanya üst limiti 80.000TL'dir.
+kampanya_bitis: Kampanya 31 Ağustos 2026 tarihine kadar geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="24" t="n"/>

</xml_diff>

<commit_message>
KT-008 ve VK-009 etiketlendi, taksit ile vade karisikligi icin uyari eklendi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -6733,11 +6733,31 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="24" t="n"/>
-      <c r="B69" s="24" t="n"/>
-      <c r="C69" s="24" t="n"/>
-      <c r="D69" s="24" t="n"/>
-      <c r="E69" s="24" t="n"/>
+      <c r="A69" s="24" t="inlineStr">
+        <is>
+          <t>KT-008</t>
+        </is>
+      </c>
+      <c r="B69" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C69" s="24" t="inlineStr">
+        <is>
+          <t>Colin's'de Vade Farksız 4 Aya Varan Taksit Fırsatı</t>
+        </is>
+      </c>
+      <c r="D69" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E69" s="24" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/colinsde-vade-farksiz-4-aya-varan-taksit-firsati</t>
+        </is>
+      </c>
       <c r="F69" s="25" t="n"/>
       <c r="G69" s="25" t="n"/>
       <c r="H69" s="24" t="n"/>
@@ -6745,22 +6765,76 @@
       <c r="J69" s="25" t="n"/>
       <c r="K69" s="25" t="n"/>
       <c r="L69" s="24" t="n"/>
-      <c r="M69" s="24" t="n"/>
+      <c r="M69" s="24" t="inlineStr">
+        <is>
+          <t>Colin's web sitesi ve mağazalarındaki alışverişlerde vade farksız 4 aya varan taksit</t>
+        </is>
+      </c>
       <c r="N69" s="24" t="n"/>
-      <c r="O69" s="27" t="n"/>
-      <c r="P69" s="27" t="n"/>
-      <c r="Q69" s="24" t="n"/>
+      <c r="O69" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="P69" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q69" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk bireysel kredi kartı sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
       <c r="R69" s="24" t="n"/>
       <c r="S69" s="24" t="n"/>
-      <c r="T69" s="27" t="n"/>
-      <c r="U69" s="24" t="n"/>
+      <c r="T69" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U69" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Ticari kartlar kampanya disi. Ust limit belirtilmemis.</t>
+        </is>
+      </c>
+      <c r="V69" t="n">
+        <v>4</v>
+      </c>
+      <c r="X69" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: vade farksız 4 aya varan taksit imkanı
+kampanya_baslangic: 6.08.2026 - 31.12.2026
+kampanya_bitis: 6.08.2026 - 31.12.2026</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="24" t="n"/>
-      <c r="B70" s="24" t="n"/>
-      <c r="C70" s="24" t="n"/>
-      <c r="D70" s="24" t="n"/>
-      <c r="E70" s="24" t="n"/>
+      <c r="A70" s="24" t="inlineStr">
+        <is>
+          <t>VK-009</t>
+        </is>
+      </c>
+      <c r="B70" s="24" t="inlineStr">
+        <is>
+          <t>Vakıf Katılım</t>
+        </is>
+      </c>
+      <c r="C70" s="24" t="inlineStr">
+        <is>
+          <t>Tamamla Kazan</t>
+        </is>
+      </c>
+      <c r="D70" s="24" t="inlineStr">
+        <is>
+          <t>Belirlenemedi</t>
+        </is>
+      </c>
+      <c r="E70" s="24" t="inlineStr">
+        <is>
+          <t>www.vakifkatilim.com.tr/tr/kendim-icin/kampanyalar/detay/tamamla-kazan</t>
+        </is>
+      </c>
       <c r="F70" s="25" t="n"/>
       <c r="G70" s="25" t="n"/>
       <c r="H70" s="24" t="n"/>
@@ -6768,15 +6842,32 @@
       <c r="J70" s="25" t="n"/>
       <c r="K70" s="25" t="n"/>
       <c r="L70" s="24" t="n"/>
-      <c r="M70" s="24" t="n"/>
+      <c r="M70" s="24" t="inlineStr">
+        <is>
+          <t>Ay boyunca en az 6 kriteri tamamlayan bireysel müşteriler, seçtikleri bir avantajdan yararlanır</t>
+        </is>
+      </c>
       <c r="N70" s="24" t="n"/>
       <c r="O70" s="27" t="n"/>
       <c r="P70" s="27" t="n"/>
-      <c r="Q70" s="24" t="n"/>
+      <c r="Q70" s="24" t="inlineStr">
+        <is>
+          <t>Vakıf Katılım bireysel müşterileri</t>
+        </is>
+      </c>
       <c r="R70" s="24" t="n"/>
       <c r="S70" s="24" t="n"/>
-      <c r="T70" s="27" t="n"/>
-      <c r="U70" s="24" t="n"/>
+      <c r="T70" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U70" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfadaki tek sayi 'en az 6 kriter' olup katilim sartidir, taksit/odul degil. Odul tutari sayfada yok (mobil uygulamada gosteriliyor). Kampanya suresiz - her ay basinda kriterler sifirlaniyor.</t>
+        </is>
+      </c>
+      <c r="X70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="24" t="n"/>

</xml_diff>

<commit_message>
bes yeni altin kayit: ZK-009, AL-010, DK-008, HF-007, KT-009
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -6870,11 +6870,31 @@
       <c r="X70" s="2" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="24" t="n"/>
-      <c r="B71" s="24" t="n"/>
-      <c r="C71" s="24" t="n"/>
-      <c r="D71" s="24" t="n"/>
-      <c r="E71" s="24" t="n"/>
+      <c r="A71" s="24" t="inlineStr">
+        <is>
+          <t>ZK-009</t>
+        </is>
+      </c>
+      <c r="B71" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C71" s="24" t="inlineStr">
+        <is>
+          <t>A101'de Peşin Fiyatına 6 Aya Varan Taksit</t>
+        </is>
+      </c>
+      <c r="D71" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E71" s="24" t="inlineStr">
+        <is>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/a101de-6-taksit</t>
+        </is>
+      </c>
       <c r="F71" s="25" t="n"/>
       <c r="G71" s="25" t="n"/>
       <c r="H71" s="24" t="n"/>
@@ -6882,68 +6902,227 @@
       <c r="J71" s="25" t="n"/>
       <c r="K71" s="25" t="n"/>
       <c r="L71" s="24" t="n"/>
-      <c r="M71" s="24" t="n"/>
+      <c r="M71" s="24" t="inlineStr">
+        <is>
+          <t>Bankkart kredi kartıyla A101 mağaza ve web sitesinde 300 TL üzeri alışverişte peşin fiyatına 6 aya varan taksit</t>
+        </is>
+      </c>
       <c r="N71" s="24" t="n"/>
       <c r="O71" s="27" t="n"/>
       <c r="P71" s="27" t="n"/>
-      <c r="Q71" s="24" t="n"/>
+      <c r="Q71" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+        </is>
+      </c>
       <c r="R71" s="24" t="n"/>
       <c r="S71" s="24" t="n"/>
-      <c r="T71" s="27" t="n"/>
-      <c r="U71" s="24" t="n"/>
+      <c r="T71" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U71" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi sayfada YOK. 300 TL alt esik, finansman tutari degil.</t>
+        </is>
+      </c>
+      <c r="V71" t="n">
+        <v>6</v>
+      </c>
+      <c r="X71" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: alışverişlerinizde peşin fiyatına 6 aya varan taksit fırsatından faydalanabilirsiniz.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="24" t="n"/>
-      <c r="B72" s="24" t="n"/>
-      <c r="C72" s="24" t="n"/>
-      <c r="D72" s="24" t="n"/>
-      <c r="E72" s="24" t="n"/>
+      <c r="A72" s="24" t="inlineStr">
+        <is>
+          <t>AL-010</t>
+        </is>
+      </c>
+      <c r="B72" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C72" s="24" t="inlineStr">
+        <is>
+          <t>Kırtasiye Kampanyası</t>
+        </is>
+      </c>
+      <c r="D72" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E72" s="24" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/kirtasiye-kampanyasi</t>
+        </is>
+      </c>
       <c r="F72" s="25" t="n"/>
       <c r="G72" s="25" t="n"/>
       <c r="H72" s="24" t="n"/>
       <c r="I72" s="26" t="n"/>
-      <c r="J72" s="25" t="n"/>
+      <c r="J72" s="25" t="n">
+        <v>20000</v>
+      </c>
       <c r="K72" s="25" t="n"/>
       <c r="L72" s="24" t="n"/>
-      <c r="M72" s="24" t="n"/>
+      <c r="M72" s="24" t="inlineStr">
+        <is>
+          <t>World kredi kartıyla 1.000-20.000 TL arası kırtasiye harcamasına vade farksız 4 taksit; ilk 2.000 katılımcı ile sınırlı</t>
+        </is>
+      </c>
       <c r="N72" s="24" t="n"/>
-      <c r="O72" s="27" t="n"/>
-      <c r="P72" s="27" t="n"/>
-      <c r="Q72" s="24" t="n"/>
+      <c r="O72" s="27" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="P72" s="27" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="Q72" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil'den kampanyaya katılan, World özellikli bireysel kredi kartı sahipleri</t>
+        </is>
+      </c>
       <c r="R72" s="24" t="n"/>
       <c r="S72" s="24" t="n"/>
-      <c r="T72" s="27" t="n"/>
-      <c r="U72" s="24" t="n"/>
+      <c r="T72" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U72" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. MCC 5942/5943 harcamalari icin gecerli. Business ve Master Gold kart haric.</t>
+        </is>
+      </c>
+      <c r="V72" t="n">
+        <v>4</v>
+      </c>
+      <c r="X72" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 1.000 TL- 20.000 TL arası kırtasiye harcamalarınızda vade farksız 4 taksit fırsatını kaçırmayın!
+finansman_tutari: 1.000 TL- 20.000 TL arası kırtasiye harcamalarınızda vade farksız 4 taksit fırsatını kaçırmayın!
+kampanya_baslangic: 1 Haziran - 30 Eylül 2026
+kampanya_bitis: 1 Haziran - 30 Eylül 2026</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="24" t="n"/>
-      <c r="B73" s="24" t="n"/>
-      <c r="C73" s="24" t="n"/>
-      <c r="D73" s="24" t="n"/>
-      <c r="E73" s="24" t="n"/>
+      <c r="A73" s="24" t="inlineStr">
+        <is>
+          <t>DK-008</t>
+        </is>
+      </c>
+      <c r="B73" s="24" t="inlineStr">
+        <is>
+          <t>Dünya Katılım</t>
+        </is>
+      </c>
+      <c r="C73" s="24" t="inlineStr">
+        <is>
+          <t>Yeni Müşterilere Özel Altına Altın Hediye</t>
+        </is>
+      </c>
+      <c r="D73" s="24" t="inlineStr">
+        <is>
+          <t>Yeni Musteri Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E73" s="24" t="inlineStr">
+        <is>
+          <t>www.dunyakatilim.com.tr/kampanyalar/fiziki-altin</t>
+        </is>
+      </c>
       <c r="F73" s="25" t="n"/>
       <c r="G73" s="25" t="n"/>
       <c r="H73" s="24" t="n"/>
       <c r="I73" s="26" t="n"/>
       <c r="J73" s="25" t="n"/>
-      <c r="K73" s="25" t="n"/>
-      <c r="L73" s="24" t="n"/>
-      <c r="M73" s="24" t="n"/>
+      <c r="K73" s="25" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="L73" s="24" t="inlineStr">
+        <is>
+          <t>Gram</t>
+        </is>
+      </c>
+      <c r="M73" s="24" t="inlineStr">
+        <is>
+          <t>Fiziki altın siparişine ürün türüne göre 0,10-0,25 gram altın hediye</t>
+        </is>
+      </c>
       <c r="N73" s="24" t="n"/>
-      <c r="O73" s="27" t="n"/>
-      <c r="P73" s="27" t="n"/>
-      <c r="Q73" s="24" t="n"/>
+      <c r="O73" s="27" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="P73" s="27" t="inlineStr">
+        <is>
+          <t>2026-03-31</t>
+        </is>
+      </c>
+      <c r="Q73" s="24" t="inlineStr">
+        <is>
+          <t>1 Ocak 2026'dan itibaren müşteri olan ve kampanya döneminde fiziki altın siparişi veren gerçek kişiler</t>
+        </is>
+      </c>
       <c r="R73" s="24" t="n"/>
       <c r="S73" s="24" t="n"/>
-      <c r="T73" s="27" t="n"/>
-      <c r="U73" s="24" t="n"/>
+      <c r="T73" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U73" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. SAYFA 'Kampanya Suresi Dolmustur' diyor - kampanya bitmis, ama metin cikarim icin gecerli bir ornek. odul_miktari en YUKSEK kademedir (tam altin/bilezik); 1 gram siparise 0,10 gram.</t>
+        </is>
+      </c>
+      <c r="X73" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Tam altın siparişinize → 0,25 gram altın hediye
+odul_birimi: Tam altın siparişinize → 0,25 gram altın hediye
+kampanya_baslangic: 13.01.2026-31.03.2026 tarihleri arasında
+kampanya_bitis: 13.01.2026-31.03.2026 tarihleri arasında</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="24" t="n"/>
-      <c r="B74" s="24" t="n"/>
-      <c r="C74" s="24" t="n"/>
-      <c r="D74" s="24" t="n"/>
-      <c r="E74" s="24" t="n"/>
+      <c r="A74" s="24" t="inlineStr">
+        <is>
+          <t>HF-007</t>
+        </is>
+      </c>
+      <c r="B74" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans</t>
+        </is>
+      </c>
+      <c r="C74" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans Müşterilerine GastroClub Ayrıcalıkları</t>
+        </is>
+      </c>
+      <c r="D74" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E74" s="24" t="inlineStr">
+        <is>
+          <t>hayatfinans.com.tr/kampanyalar/hayat-finans-ile-gastroclub-ayricaliklari</t>
+        </is>
+      </c>
       <c r="F74" s="25" t="n"/>
       <c r="G74" s="25" t="n"/>
       <c r="H74" s="24" t="n"/>
@@ -6951,22 +7130,59 @@
       <c r="J74" s="25" t="n"/>
       <c r="K74" s="25" t="n"/>
       <c r="L74" s="24" t="n"/>
-      <c r="M74" s="24" t="n"/>
+      <c r="M74" s="24" t="inlineStr">
+        <is>
+          <t>Ücretsiz GastroClub üyeliğiyle 1.200'ü aşkın anlaşmalı işletmede %10-%50 indirim</t>
+        </is>
+      </c>
       <c r="N74" s="24" t="n"/>
       <c r="O74" s="27" t="n"/>
       <c r="P74" s="27" t="n"/>
-      <c r="Q74" s="24" t="n"/>
+      <c r="Q74" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans müşterileri (mobil uygulamadan GastroClub üyeliği oluşturanlar)</t>
+        </is>
+      </c>
       <c r="R74" s="24" t="n"/>
       <c r="S74" s="24" t="n"/>
-      <c r="T74" s="27" t="n"/>
-      <c r="U74" s="24" t="n"/>
+      <c r="T74" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U74" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %10-%50 anlasmali isyeri INDIRIMIDIR, kar payi orani degil. Kampanya tarihi sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="X74" s="2" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="24" t="n"/>
-      <c r="B75" s="24" t="n"/>
-      <c r="C75" s="24" t="n"/>
-      <c r="D75" s="24" t="n"/>
-      <c r="E75" s="24" t="n"/>
+      <c r="A75" s="24" t="inlineStr">
+        <is>
+          <t>KT-009</t>
+        </is>
+      </c>
+      <c r="B75" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C75" s="24" t="inlineStr">
+        <is>
+          <t>Eğitim ve Sağlık Harcamalarınızda 5 Taksit Fırsatı</t>
+        </is>
+      </c>
+      <c r="D75" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E75" s="24" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/egitim-ve-saglik-harcamalarinizda-5-taksit-firsati</t>
+        </is>
+      </c>
       <c r="F75" s="25" t="n"/>
       <c r="G75" s="25" t="n"/>
       <c r="H75" s="24" t="n"/>
@@ -6974,15 +7190,49 @@
       <c r="J75" s="25" t="n"/>
       <c r="K75" s="25" t="n"/>
       <c r="L75" s="24" t="n"/>
-      <c r="M75" s="24" t="n"/>
+      <c r="M75" s="24" t="inlineStr">
+        <is>
+          <t>Sağlam Kart ile 1.000 TL üzeri eğitim/sağlık harcamalarını mobilden vade farksız 2-5 taksite bölme</t>
+        </is>
+      </c>
       <c r="N75" s="24" t="n"/>
-      <c r="O75" s="27" t="n"/>
-      <c r="P75" s="27" t="n"/>
-      <c r="Q75" s="24" t="n"/>
+      <c r="O75" s="27" t="inlineStr">
+        <is>
+          <t>2024-06-21</t>
+        </is>
+      </c>
+      <c r="P75" s="27" t="inlineStr">
+        <is>
+          <t>2027-12-31</t>
+        </is>
+      </c>
+      <c r="Q75" s="24" t="inlineStr">
+        <is>
+          <t>Sağlam Kart ve Özel Bankacılık World Elite Kart sahipleri (bireysel harcamalar)</t>
+        </is>
+      </c>
       <c r="R75" s="24" t="n"/>
       <c r="S75" s="24" t="n"/>
-      <c r="T75" s="27" t="n"/>
-      <c r="U75" s="24" t="n"/>
+      <c r="T75" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U75" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 1.000 TL alt esik. Ekstre basina en fazla 2 islem (Biz Bize 6, Ozel Bankacilik 10). Taksitlendirme otomatik degil, elle yapiliyor.</t>
+        </is>
+      </c>
+      <c r="V75" t="n">
+        <v>5</v>
+      </c>
+      <c r="X75" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: üzerinden vade farksız bir şekilde 2 ila 5 taksite bölebilirsiniz.
+kampanya_baslangic: 21.06.2024 - 31.12.2027
+kampanya_bitis: 21.06.2024 - 31.12.2027</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="24" t="n"/>

</xml_diff>

<commit_message>
alti yeni altin kayit: TEK-008, VK-010, ZK-010, AL-011, DK-009, HF-008
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -7235,34 +7235,112 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="24" t="n"/>
-      <c r="B76" s="24" t="n"/>
-      <c r="C76" s="24" t="n"/>
-      <c r="D76" s="24" t="n"/>
-      <c r="E76" s="24" t="n"/>
+      <c r="A76" s="24" t="inlineStr">
+        <is>
+          <t>TEK-008</t>
+        </is>
+      </c>
+      <c r="B76" s="24" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C76" s="24" t="inlineStr">
+        <is>
+          <t>Akaryakıt Harcamalarınıza 400 TL ParafPara</t>
+        </is>
+      </c>
+      <c r="D76" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E76" s="24" t="inlineStr">
+        <is>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/akaryakit-harcamalariniza-400-tl-parafpara</t>
+        </is>
+      </c>
       <c r="F76" s="25" t="n"/>
       <c r="G76" s="25" t="n"/>
       <c r="H76" s="24" t="n"/>
       <c r="I76" s="26" t="n"/>
       <c r="J76" s="25" t="n"/>
-      <c r="K76" s="25" t="n"/>
-      <c r="L76" s="24" t="n"/>
-      <c r="M76" s="24" t="n"/>
+      <c r="K76" s="25" t="n">
+        <v>400</v>
+      </c>
+      <c r="L76" s="24" t="inlineStr">
+        <is>
+          <t>ParafPara</t>
+        </is>
+      </c>
+      <c r="M76" s="24" t="inlineStr">
+        <is>
+          <t>SMS ile katılıp 1.500 TL üzeri 2. ve 4. akaryakıt harcamasına 200'er TL, toplam 400 TL ParafPara</t>
+        </is>
+      </c>
       <c r="N76" s="24" t="n"/>
-      <c r="O76" s="27" t="n"/>
-      <c r="P76" s="27" t="n"/>
-      <c r="Q76" s="24" t="n"/>
+      <c r="O76" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="P76" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q76" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
       <c r="R76" s="24" t="n"/>
       <c r="S76" s="24" t="n"/>
-      <c r="T76" s="27" t="n"/>
-      <c r="U76" s="24" t="n"/>
+      <c r="T76" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U76" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Katilim SMS ile ('AKARYAKIT' yazip 6026'ya). Musteri basina bir kez.</t>
+        </is>
+      </c>
+      <c r="X76" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Kampanya kapsamında yurt içinde tek seferde yapılacak 1.500 TL ve üzeri ikinci ve dördüncü akaryakıt harcamasına 200 TL, toplam 400 TL ParafPara verilecektir.
+odul_birimi: Kampanya kapsamında yurt içinde tek seferde yapılacak 1.500 TL ve üzeri ikinci ve dördüncü akaryakıt harcamasına 200 TL, toplam 400 TL ParafPara verilecektir.
+kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="24" t="n"/>
-      <c r="B77" s="24" t="n"/>
-      <c r="C77" s="24" t="n"/>
-      <c r="D77" s="24" t="n"/>
-      <c r="E77" s="24" t="n"/>
+      <c r="A77" s="24" t="inlineStr">
+        <is>
+          <t>VK-010</t>
+        </is>
+      </c>
+      <c r="B77" s="24" t="inlineStr">
+        <is>
+          <t>Vakıf Katılım</t>
+        </is>
+      </c>
+      <c r="C77" s="24" t="inlineStr">
+        <is>
+          <t>VClub Dünyası Artık Vakıf Katılım Mobil'de</t>
+        </is>
+      </c>
+      <c r="D77" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E77" s="24" t="inlineStr">
+        <is>
+          <t>www.vakifkatilim.com.tr/tr/kendim-icin/kampanyalar/detay/vclub-dunyasi-artik-vakif-katilim-mobilde</t>
+        </is>
+      </c>
       <c r="F77" s="25" t="n"/>
       <c r="G77" s="25" t="n"/>
       <c r="H77" s="24" t="n"/>
@@ -7270,22 +7348,59 @@
       <c r="J77" s="25" t="n"/>
       <c r="K77" s="25" t="n"/>
       <c r="L77" s="24" t="n"/>
-      <c r="M77" s="24" t="n"/>
+      <c r="M77" s="24" t="inlineStr">
+        <is>
+          <t>VClub sadakat programı ile süpermarket, seyahat, giyim, teknoloji, kafe ve restoranlarda müşteriye özel indirimler</t>
+        </is>
+      </c>
       <c r="N77" s="24" t="n"/>
       <c r="O77" s="27" t="n"/>
       <c r="P77" s="27" t="n"/>
-      <c r="Q77" s="24" t="n"/>
+      <c r="Q77" s="24" t="inlineStr">
+        <is>
+          <t>Aktif Vakıf Katılım kredi veya banka kartı kullanan müşteriler</t>
+        </is>
+      </c>
       <c r="R77" s="24" t="n"/>
       <c r="S77" s="24" t="n"/>
-      <c r="T77" s="27" t="n"/>
-      <c r="U77" s="24" t="n"/>
+      <c r="T77" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U77" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfa indirim orani VERMIYOR ('musteri ozelinde degisiklik gosterebilmektedir'). Tarih de yok. GastroClub is birligi - HF-007 ile ayni platform, farkli banka.</t>
+        </is>
+      </c>
+      <c r="X77" s="2" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="24" t="n"/>
-      <c r="B78" s="24" t="n"/>
-      <c r="C78" s="24" t="n"/>
-      <c r="D78" s="24" t="n"/>
-      <c r="E78" s="24" t="n"/>
+      <c r="A78" s="24" t="inlineStr">
+        <is>
+          <t>ZK-010</t>
+        </is>
+      </c>
+      <c r="B78" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C78" s="24" t="inlineStr">
+        <is>
+          <t>Abdullah Kiğılı'da 2 Taksit</t>
+        </is>
+      </c>
+      <c r="D78" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E78" s="24" t="inlineStr">
+        <is>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/abdullah-kigilida-2-taksit</t>
+        </is>
+      </c>
       <c r="F78" s="25" t="n"/>
       <c r="G78" s="25" t="n"/>
       <c r="H78" s="24" t="n"/>
@@ -7293,68 +7408,226 @@
       <c r="J78" s="25" t="n"/>
       <c r="K78" s="25" t="n"/>
       <c r="L78" s="24" t="n"/>
-      <c r="M78" s="24" t="n"/>
+      <c r="M78" s="24" t="inlineStr">
+        <is>
+          <t>Bankkart kredi kartıyla Abdullah Kiğılı alışverişlerinde 2 taksit</t>
+        </is>
+      </c>
       <c r="N78" s="24" t="n"/>
       <c r="O78" s="27" t="n"/>
       <c r="P78" s="27" t="n"/>
-      <c r="Q78" s="24" t="n"/>
+      <c r="Q78" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+        </is>
+      </c>
       <c r="R78" s="24" t="n"/>
       <c r="S78" s="24" t="n"/>
-      <c r="T78" s="27" t="n"/>
-      <c r="U78" s="24" t="n"/>
+      <c r="T78" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U78" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve alt/ust harcama siniri sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V78" t="n">
+        <v>2</v>
+      </c>
+      <c r="X78" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 2 taksitli</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="24" t="n"/>
-      <c r="B79" s="24" t="n"/>
-      <c r="C79" s="24" t="n"/>
-      <c r="D79" s="24" t="n"/>
-      <c r="E79" s="24" t="n"/>
+      <c r="A79" s="24" t="inlineStr">
+        <is>
+          <t>AL-011</t>
+        </is>
+      </c>
+      <c r="B79" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C79" s="24" t="inlineStr">
+        <is>
+          <t>Otomatik Fatura Ödeme Talimatlarınıza Toplamda 2.000 TL Worldpuan</t>
+        </is>
+      </c>
+      <c r="D79" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E79" s="24" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/otomatik-fatura-odeme-talimatlariniza-toplamda-2000-tl-worldpuan-12</t>
+        </is>
+      </c>
       <c r="F79" s="25" t="n"/>
       <c r="G79" s="25" t="n"/>
       <c r="H79" s="24" t="n"/>
       <c r="I79" s="26" t="n"/>
       <c r="J79" s="25" t="n"/>
-      <c r="K79" s="25" t="n"/>
-      <c r="L79" s="24" t="n"/>
-      <c r="M79" s="24" t="n"/>
+      <c r="K79" s="25" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L79" s="24" t="inlineStr">
+        <is>
+          <t>Worldpuan</t>
+        </is>
+      </c>
+      <c r="M79" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil'den verilen her yeni otomatik fatura ödeme talimatına 200 TL, toplamda 2.000 TL'ye varan Worldpuan</t>
+        </is>
+      </c>
       <c r="N79" s="24" t="n"/>
-      <c r="O79" s="27" t="n"/>
-      <c r="P79" s="27" t="n"/>
-      <c r="Q79" s="24" t="n"/>
+      <c r="O79" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="P79" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q79" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil'den kampanyaya katılan bireysel müşteriler (World özellikli kart gerekli)</t>
+        </is>
+      </c>
       <c r="R79" s="24" t="n"/>
       <c r="S79" s="24" t="n"/>
-      <c r="T79" s="27" t="n"/>
-      <c r="U79" s="24" t="n"/>
+      <c r="T79" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U79" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. DIKKAT - AL-007 ile KARISTIRILMASIN: ikisi de Agustos 2026 fatura kampanyasi ve ikisinin de tavani 2.000 TL Worldpuan, ama AL-007 talimat basina 500 TL veriyor ve yalnizca goruntulu gorusmeyle yeni musteri olanlar icin (OFT2026 kodu); bu kayit talimat basina 200 TL ve mevcut musteriler icin. Ayri sayfalar, ayri kosullar. Insan dogrulamasinda ikisi de acilip bakilmali.</t>
+        </is>
+      </c>
+      <c r="X79" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Albaraka Mobil üzerinden kredi kartınız ile vereceğiniz her yeni otomatik fatura ödeme talimatınıza 200 TL, toplamda 2.000 TL'ye varan Worldpuan kazanma fırsatı!
+odul_birimi: Albaraka Mobil üzerinden kredi kartınız ile vereceğiniz her yeni otomatik fatura ödeme talimatınıza 200 TL, toplamda 2.000 TL'ye varan Worldpuan kazanma fırsatı!
+kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihlerinde geçerlidir.
+kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihlerinde geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="24" t="n"/>
-      <c r="B80" s="24" t="n"/>
-      <c r="C80" s="24" t="n"/>
-      <c r="D80" s="24" t="n"/>
-      <c r="E80" s="24" t="n"/>
+      <c r="A80" s="24" t="inlineStr">
+        <is>
+          <t>DK-009</t>
+        </is>
+      </c>
+      <c r="B80" s="24" t="inlineStr">
+        <is>
+          <t>Dünya Katılım</t>
+        </is>
+      </c>
+      <c r="C80" s="24" t="inlineStr">
+        <is>
+          <t>LC Waikiki'de 3.000 TL ve Üzeri Alışverişe 300 TL İndirim</t>
+        </is>
+      </c>
+      <c r="D80" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E80" s="24" t="inlineStr">
+        <is>
+          <t>www.dunyakatilim.com.tr/kampanyalar/lc-waikiki</t>
+        </is>
+      </c>
       <c r="F80" s="25" t="n"/>
       <c r="G80" s="25" t="n"/>
       <c r="H80" s="24" t="n"/>
       <c r="I80" s="26" t="n"/>
       <c r="J80" s="25" t="n"/>
-      <c r="K80" s="25" t="n"/>
-      <c r="L80" s="24" t="n"/>
-      <c r="M80" s="24" t="n"/>
+      <c r="K80" s="25" t="n">
+        <v>300</v>
+      </c>
+      <c r="L80" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M80" s="24" t="inlineStr">
+        <is>
+          <t>TROY kartla LC Waikiki'de tek seferde 3.000 TL üzeri alışverişe anında 300 TL indirim</t>
+        </is>
+      </c>
       <c r="N80" s="24" t="n"/>
-      <c r="O80" s="27" t="n"/>
-      <c r="P80" s="27" t="n"/>
-      <c r="Q80" s="24" t="n"/>
+      <c r="O80" s="27" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="P80" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="Q80" s="24" t="inlineStr">
+        <is>
+          <t>Dünya Katılım TROY logolu banka ve kredi kartı sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
       <c r="R80" s="24" t="n"/>
       <c r="S80" s="24" t="n"/>
-      <c r="T80" s="27" t="n"/>
-      <c r="U80" s="24" t="n"/>
+      <c r="T80" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U80" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Toplam tavan YOK, her 3.000 TL+ islemde tekrar kazanilir; odul_miktari ISLEM BASINA tutardir. Havalimani/yurtdisi magazalari ve self-servis kasalar haric.</t>
+        </is>
+      </c>
+      <c r="X80" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 15 Haziran 2026 saat 00.01 – 15 Temmuz 2026 saat 23.59 arasında geçerlidir.
+kampanya_bitis: Kampanya 15 Haziran 2026 saat 00.01 – 15 Temmuz 2026 saat 23.59 arasında geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="24" t="n"/>
-      <c r="B81" s="24" t="n"/>
-      <c r="C81" s="24" t="n"/>
-      <c r="D81" s="24" t="n"/>
-      <c r="E81" s="24" t="n"/>
+      <c r="A81" s="24" t="inlineStr">
+        <is>
+          <t>HF-008</t>
+        </is>
+      </c>
+      <c r="B81" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans</t>
+        </is>
+      </c>
+      <c r="C81" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans'la İşlem Yaptıkça Kazan</t>
+        </is>
+      </c>
+      <c r="D81" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E81" s="24" t="inlineStr">
+        <is>
+          <t>hayatfinans.com.tr/kampanyalar/hayatfinansla-islem-yaptikca-kazan</t>
+        </is>
+      </c>
       <c r="F81" s="25" t="n"/>
       <c r="G81" s="25" t="n"/>
       <c r="H81" s="24" t="n"/>
@@ -7362,15 +7635,45 @@
       <c r="J81" s="25" t="n"/>
       <c r="K81" s="25" t="n"/>
       <c r="L81" s="24" t="n"/>
-      <c r="M81" s="24" t="n"/>
+      <c r="M81" s="24" t="inlineStr">
+        <is>
+          <t>Para transferi, banka kartı harcaması, fatura ödeme, döviz işlemi ve Biz Kart başvurusundan Hayat Pay cüzdanına nakit ödül</t>
+        </is>
+      </c>
       <c r="N81" s="24" t="n"/>
-      <c r="O81" s="27" t="n"/>
-      <c r="P81" s="27" t="n"/>
-      <c r="Q81" s="24" t="n"/>
+      <c r="O81" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="P81" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q81" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans müşterileri</t>
+        </is>
+      </c>
       <c r="R81" s="24" t="n"/>
       <c r="S81" s="24" t="n"/>
-      <c r="T81" s="27" t="n"/>
-      <c r="U81" s="24" t="n"/>
+      <c r="T81" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U81" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: kampanyanin tek bir odul tutari yok. Bes ayri islem turunun ayri tavanlari var (transfer ayda 100 TL, doviz ayda 200 TL, banka karti ayda 100 TL, fatura basina 20-30 TL, ilk otomatik odemeye 100 TL) ve toplam tavan sayfada verilmiyor. Motorun buradan tek bir sayi cekip cekmedigini olcen zor ornek.</t>
+        </is>
+      </c>
+      <c r="X81" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 2 Temmuz - 31 Aralık 2026
+kampanya_bitis: 2 Temmuz - 31 Aralık 2026</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="24" t="n"/>

</xml_diff>

<commit_message>
bes yeni altin kayit ve slug surum rakami kopya kurali
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -7676,103 +7676,347 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="24" t="n"/>
-      <c r="B82" s="24" t="n"/>
-      <c r="C82" s="24" t="n"/>
-      <c r="D82" s="24" t="n"/>
-      <c r="E82" s="24" t="n"/>
+      <c r="A82" s="24" t="inlineStr">
+        <is>
+          <t>KT-010</t>
+        </is>
+      </c>
+      <c r="B82" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C82" s="24" t="inlineStr">
+        <is>
+          <t>Gelir Vergisi Ödemelerinizde 3 Taksit Fırsatı</t>
+        </is>
+      </c>
+      <c r="D82" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E82" s="24" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/gelir-vergisi-odemelerinizde-3-taksit-firsati</t>
+        </is>
+      </c>
       <c r="F82" s="25" t="n"/>
       <c r="G82" s="25" t="n"/>
       <c r="H82" s="24" t="n"/>
       <c r="I82" s="26" t="n"/>
-      <c r="J82" s="25" t="n"/>
+      <c r="J82" s="25" t="n">
+        <v>300000</v>
+      </c>
       <c r="K82" s="25" t="n"/>
       <c r="L82" s="24" t="n"/>
-      <c r="M82" s="24" t="n"/>
+      <c r="M82" s="24" t="inlineStr">
+        <is>
+          <t>SMS/mobil katılım sonrası 1.000-300.000 TL arası gelir vergisi ödemelerine vade farksız 3 taksit</t>
+        </is>
+      </c>
       <c r="N82" s="24" t="n"/>
-      <c r="O82" s="27" t="n"/>
-      <c r="P82" s="27" t="n"/>
-      <c r="Q82" s="24" t="n"/>
+      <c r="O82" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P82" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="Q82" s="24" t="inlineStr">
+        <is>
+          <t>Sağlam Kart, Miles&amp;Smiles ve Özel Bankacılık World Elite kredi kartı sahipleri</t>
+        </is>
+      </c>
       <c r="R82" s="24" t="n"/>
       <c r="S82" s="24" t="n"/>
-      <c r="T82" s="27" t="n"/>
-      <c r="U82" s="24" t="n"/>
+      <c r="T82" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U82" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Musteri basina en fazla 2 islem; kampanya 75.000 kisi ile sinirli. Katilim ONAY VERGI SMS'i ile.</t>
+        </is>
+      </c>
+      <c r="V82" t="n">
+        <v>3</v>
+      </c>
+      <c r="X82" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 1.000 TL - 300.000 TL arasındaki gelir vergisi ödemelerine vade farksız 3 taksit uygulanır.
+finansman_tutari: 1.000 TL - 300.000 TL arasındaki gelir vergisi ödemelerine vade farksız 3 taksit uygulanır.
+kampanya_baslangic: 1.07.2026 - 31.07.2026
+kampanya_bitis: 1.07.2026 - 31.07.2026</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="24" t="n"/>
-      <c r="B83" s="24" t="n"/>
-      <c r="C83" s="24" t="n"/>
-      <c r="D83" s="24" t="n"/>
-      <c r="E83" s="24" t="n"/>
+      <c r="A83" s="24" t="inlineStr">
+        <is>
+          <t>TEK-009</t>
+        </is>
+      </c>
+      <c r="B83" s="24" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C83" s="24" t="inlineStr">
+        <is>
+          <t>Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye Varan ParafPara</t>
+        </is>
+      </c>
+      <c r="D83" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E83" s="24" t="inlineStr">
+        <is>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/beyaz-esya-ve-elektronik-alisverislerinize-3000-tlye-varan-parafpara</t>
+        </is>
+      </c>
       <c r="F83" s="25" t="n"/>
       <c r="G83" s="25" t="n"/>
       <c r="H83" s="24" t="n"/>
       <c r="I83" s="26" t="n"/>
       <c r="J83" s="25" t="n"/>
-      <c r="K83" s="25" t="n"/>
-      <c r="L83" s="24" t="n"/>
-      <c r="M83" s="24" t="n"/>
+      <c r="K83" s="25" t="n">
+        <v>3000</v>
+      </c>
+      <c r="L83" s="24" t="inlineStr">
+        <is>
+          <t>ParafPara</t>
+        </is>
+      </c>
+      <c r="M83" s="24" t="inlineStr">
+        <is>
+          <t>SMS ile katılıp beyaz eşya/elektronik/bilgisayar harcamasına tutara göre 300-3.000 TL ParafPara</t>
+        </is>
+      </c>
       <c r="N83" s="24" t="n"/>
-      <c r="O83" s="27" t="n"/>
-      <c r="P83" s="27" t="n"/>
-      <c r="Q83" s="24" t="n"/>
+      <c r="O83" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P83" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="Q83" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
       <c r="R83" s="24" t="n"/>
       <c r="S83" s="24" t="n"/>
-      <c r="T83" s="27" t="n"/>
-      <c r="U83" s="24" t="n"/>
+      <c r="T83" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U83" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Dort kademeli odul; musteri yalnizca BIRINI kazanir, odul_miktari en yuksek kademedir. Pazar yeri e-ticaret haric.</t>
+        </is>
+      </c>
+      <c r="X83" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye varan ParafPara!
+odul_birimi: Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye varan ParafPara!
+kampanya_baslangic: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="24" t="n"/>
-      <c r="B84" s="24" t="n"/>
-      <c r="C84" s="24" t="n"/>
-      <c r="D84" s="24" t="n"/>
-      <c r="E84" s="24" t="n"/>
+      <c r="A84" s="24" t="inlineStr">
+        <is>
+          <t>ZK-011</t>
+        </is>
+      </c>
+      <c r="B84" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C84" s="24" t="inlineStr">
+        <is>
+          <t>Aile Kart'a Özel 2.000 TL'ye Varan Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="D84" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E84" s="24" t="inlineStr">
+        <is>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/aile-karta-ozel-2000-tlye-varan-bankkart-lira-1</t>
+        </is>
+      </c>
       <c r="F84" s="25" t="n"/>
       <c r="G84" s="25" t="n"/>
       <c r="H84" s="24" t="n"/>
       <c r="I84" s="26" t="n"/>
       <c r="J84" s="25" t="n"/>
-      <c r="K84" s="25" t="n"/>
-      <c r="L84" s="24" t="n"/>
-      <c r="M84" s="24" t="n"/>
+      <c r="K84" s="25" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L84" s="24" t="inlineStr">
+        <is>
+          <t>Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="M84" s="24" t="inlineStr">
+        <is>
+          <t>Aile kredi kartıyla market/akaryakıt/giyim/eğitim/sağlık harcamalarına %5-%10 Bankkart Lira, en fazla 2.000 TL</t>
+        </is>
+      </c>
       <c r="N84" s="24" t="n"/>
-      <c r="O84" s="27" t="n"/>
-      <c r="P84" s="27" t="n"/>
-      <c r="Q84" s="24" t="n"/>
+      <c r="O84" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="P84" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Q84" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım Bankkart Aile kredi kartı sahibi asıl kart sahipleri</t>
+        </is>
+      </c>
       <c r="R84" s="24" t="n"/>
       <c r="S84" s="24" t="n"/>
-      <c r="T84" s="27" t="n"/>
-      <c r="U84" s="24" t="n"/>
+      <c r="T84" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U84" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %5 ve %10 NAKIT IADE oranidir, kar payi orani degil. Bireysel/ticari/ucretsiz kartlar haric.</t>
+        </is>
+      </c>
+      <c r="X84" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: en fazla 2.000 TL
+kampanya_baslangic: 10 Temmuz– 7 Ağustos 2026
+kampanya_bitis: 10 Temmuz– 7 Ağustos 2026</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="24" t="n"/>
-      <c r="B85" s="24" t="n"/>
-      <c r="C85" s="24" t="n"/>
-      <c r="D85" s="24" t="n"/>
-      <c r="E85" s="24" t="n"/>
+      <c r="A85" s="24" t="inlineStr">
+        <is>
+          <t>HF-009</t>
+        </is>
+      </c>
+      <c r="B85" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans</t>
+        </is>
+      </c>
+      <c r="C85" s="24" t="inlineStr">
+        <is>
+          <t>Xiaomi Ürünlerinde Finansman Avantajı</t>
+        </is>
+      </c>
+      <c r="D85" s="24" t="inlineStr">
+        <is>
+          <t>Finansman Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E85" s="24" t="inlineStr">
+        <is>
+          <t>hayatfinans.com.tr/kampanyalar/xiaomi-urunlerinde-finansman-avantaji</t>
+        </is>
+      </c>
       <c r="F85" s="25" t="n"/>
       <c r="G85" s="25" t="n"/>
       <c r="H85" s="24" t="n"/>
       <c r="I85" s="26" t="n"/>
-      <c r="J85" s="25" t="n"/>
+      <c r="J85" s="25" t="n">
+        <v>40000</v>
+      </c>
       <c r="K85" s="25" t="n"/>
       <c r="L85" s="24" t="n"/>
-      <c r="M85" s="24" t="n"/>
+      <c r="M85" s="24" t="inlineStr">
+        <is>
+          <t>Xiaomi fiziksel mağazalarında 3 aya varan taksit; kampanya üst limiti 40.000 TL</t>
+        </is>
+      </c>
       <c r="N85" s="24" t="n"/>
       <c r="O85" s="27" t="n"/>
-      <c r="P85" s="27" t="n"/>
-      <c r="Q85" s="24" t="n"/>
+      <c r="P85" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q85" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans müşterileri (Bana Bunu Al İş Ortağım)</t>
+        </is>
+      </c>
       <c r="R85" s="24" t="n"/>
       <c r="S85" s="24" t="n"/>
-      <c r="T85" s="27" t="n"/>
-      <c r="U85" s="24" t="n"/>
+      <c r="T85" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U85" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Baslangic tarihi sayfada YOK. HF-006 ile ayni urun (Bana Bunu Al Is Ortagim) ama farkli magaza ve farkli ust limit: HF-006 Troy magazalari/80.000 TL, bu kayit Xiaomi/40.000 TL.</t>
+        </is>
+      </c>
+      <c r="V85" t="n">
+        <v>3</v>
+      </c>
+      <c r="X85" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Hayat Finanslılara özel Xiaomi mağazalarında 3 aya varan taksit fırsatı Bana Bunu Al İş Ortağımda!
+finansman_tutari: Kampanya üst limiti 40.000TL'dir.
+kampanya_bitis: Kampanya 31 Ağustos 2026 tarihine kadar geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="24" t="n"/>
-      <c r="B86" s="24" t="n"/>
-      <c r="C86" s="24" t="n"/>
-      <c r="D86" s="24" t="n"/>
-      <c r="E86" s="24" t="n"/>
+      <c r="A86" s="24" t="inlineStr">
+        <is>
+          <t>KT-011</t>
+        </is>
+      </c>
+      <c r="B86" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C86" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk ile Yurt Dışı Seyahatlerinde Ayrıcalıklar</t>
+        </is>
+      </c>
+      <c r="D86" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E86" s="24" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/seyahat-kampanyalari/kuveyt-turk-ile-yurt-disi-seyahatlerinde-ayricaliklar-sizinle</t>
+        </is>
+      </c>
       <c r="F86" s="25" t="n"/>
       <c r="G86" s="25" t="n"/>
       <c r="H86" s="24" t="n"/>
@@ -7780,15 +8024,45 @@
       <c r="J86" s="25" t="n"/>
       <c r="K86" s="25" t="n"/>
       <c r="L86" s="24" t="n"/>
-      <c r="M86" s="24" t="n"/>
+      <c r="M86" s="24" t="inlineStr">
+        <is>
+          <t>PocketSIM eSIM'de 1 GB hediye internet ve %35 indirim kodu, yurt dışı harcamalarda avantajlı döviz marjı</t>
+        </is>
+      </c>
       <c r="N86" s="24" t="n"/>
-      <c r="O86" s="27" t="n"/>
-      <c r="P86" s="27" t="n"/>
-      <c r="Q86" s="24" t="n"/>
+      <c r="O86" s="27" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="P86" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q86" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk Sağlam Nakit ve Sağlam Kart sahipleri</t>
+        </is>
+      </c>
       <c r="R86" s="24" t="n"/>
       <c r="S86" s="24" t="n"/>
-      <c r="T86" s="27" t="n"/>
-      <c r="U86" s="24" t="n"/>
+      <c r="T86" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U86" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: %35 bir PocketSIM INDIRIM KODU oranidir (kar payi degil), 1 GB parasal odul degildir. Motorun %35'i kar_payi_orani sanip sanmadigini olcen kayit.</t>
+        </is>
+      </c>
+      <c r="X86" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 2.02.2026 - 31.12.2026
+kampanya_bitis: 2.02.2026 - 31.12.2026</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="24" t="n"/>

</xml_diff>

<commit_message>
uc yeni altin kayit, ay varyanti ve bozuk adres kurallari
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -8065,73 +8065,228 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="24" t="n"/>
-      <c r="B87" s="24" t="n"/>
-      <c r="C87" s="24" t="n"/>
-      <c r="D87" s="24" t="n"/>
-      <c r="E87" s="24" t="n"/>
+      <c r="A87" s="24" t="inlineStr">
+        <is>
+          <t>AL-012</t>
+        </is>
+      </c>
+      <c r="B87" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Türk</t>
+        </is>
+      </c>
+      <c r="C87" s="24" t="inlineStr">
+        <is>
+          <t>Dijital Müşterilere Özel Pratik Finansman Kart</t>
+        </is>
+      </c>
+      <c r="D87" s="24" t="inlineStr">
+        <is>
+          <t>Yeni Musteri Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E87" s="24" t="inlineStr">
+        <is>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/dijital-musterilere-ozel-pratik-finansman-kart</t>
+        </is>
+      </c>
       <c r="F87" s="25" t="n"/>
       <c r="G87" s="25" t="n"/>
       <c r="H87" s="24" t="n"/>
       <c r="I87" s="26" t="n"/>
-      <c r="J87" s="25" t="n"/>
+      <c r="J87" s="25" t="n">
+        <v>40000</v>
+      </c>
       <c r="K87" s="25" t="n"/>
       <c r="L87" s="24" t="n"/>
-      <c r="M87" s="24" t="n"/>
+      <c r="M87" s="24" t="inlineStr">
+        <is>
+          <t>Görüntülü görüşmeyle ilk kez müşteri olanlara vade farksız 40.000 TL veya özel oranlı Pratik Finansman Kart</t>
+        </is>
+      </c>
       <c r="N87" s="24" t="n"/>
-      <c r="O87" s="27" t="n"/>
-      <c r="P87" s="27" t="n"/>
-      <c r="Q87" s="24" t="n"/>
+      <c r="O87" s="27" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="P87" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q87" s="24" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil'den görüntülü görüşmeyle ilk kez Albaraka müşterisi olanlar</t>
+        </is>
+      </c>
       <c r="R87" s="24" t="n"/>
       <c r="S87" s="24" t="n"/>
-      <c r="T87" s="27" t="n"/>
-      <c r="U87" s="24" t="n"/>
+      <c r="T87" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U87" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: sayfa 'uygun oranli' diyor, sayi vermiyor; oran basvuruda musteriye gore belirleniyor. Pratik Finansman Kart ile ATM'den nakit cekilemiyor.</t>
+        </is>
+      </c>
+      <c r="X87" s="2" t="inlineStr">
+        <is>
+          <t>finansman_tutari: Vade farksız 40.000 TL ve uygun oranlı hoş geldin finansmanı Albaraka'da!</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="24" t="n"/>
-      <c r="B88" s="24" t="n"/>
-      <c r="C88" s="24" t="n"/>
-      <c r="D88" s="24" t="n"/>
-      <c r="E88" s="24" t="n"/>
+      <c r="A88" s="24" t="inlineStr">
+        <is>
+          <t>HF-010</t>
+        </is>
+      </c>
+      <c r="B88" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans</t>
+        </is>
+      </c>
+      <c r="C88" s="24" t="inlineStr">
+        <is>
+          <t>Biz Kart ile Yemek Harcamalarına 1.000 TL'ye Varan Nakit İade</t>
+        </is>
+      </c>
+      <c r="D88" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E88" s="24" t="inlineStr">
+        <is>
+          <t>hayatfinans.com.tr/kampanyalar/biz-kart-yemek-harcamasi-nakit-iade-kampanyasi</t>
+        </is>
+      </c>
       <c r="F88" s="25" t="n"/>
       <c r="G88" s="25" t="n"/>
       <c r="H88" s="24" t="n"/>
       <c r="I88" s="26" t="n"/>
       <c r="J88" s="25" t="n"/>
-      <c r="K88" s="25" t="n"/>
-      <c r="L88" s="24" t="n"/>
-      <c r="M88" s="24" t="n"/>
+      <c r="K88" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L88" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M88" s="24" t="inlineStr">
+        <is>
+          <t>Biz Kart ile yemek sektörü harcamalarının %10'u nakit iade; günlük en fazla 100 TL, aylık 1.000 TL</t>
+        </is>
+      </c>
       <c r="N88" s="24" t="n"/>
-      <c r="O88" s="27" t="n"/>
-      <c r="P88" s="27" t="n"/>
-      <c r="Q88" s="24" t="n"/>
+      <c r="O88" s="27" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="P88" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q88" s="24" t="inlineStr">
+        <is>
+          <t>Hayat Finans bireysel müşterilerinin yakınlarına verdiği Biz Kart sahipleri</t>
+        </is>
+      </c>
       <c r="R88" s="24" t="n"/>
       <c r="S88" s="24" t="n"/>
-      <c r="T88" s="27" t="n"/>
-      <c r="U88" s="24" t="n"/>
+      <c r="T88" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U88" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari AYLIK tavandir (gunluk tavan 100 TL). kar_payi_orani BILEREK BOS: %10 nakit iade oranidir.</t>
+        </is>
+      </c>
+      <c r="X88" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: aylık toplamda ise 1.000 TL’ye kadar nakit iade
+kampanya_baslangic: 6 Şubat - 31 Ağustos 2026
+kampanya_bitis: 6 Şubat - 31 Ağustos 2026</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="24" t="n"/>
-      <c r="B89" s="24" t="n"/>
-      <c r="C89" s="24" t="n"/>
-      <c r="D89" s="24" t="n"/>
-      <c r="E89" s="24" t="n"/>
+      <c r="A89" s="24" t="inlineStr">
+        <is>
+          <t>TF-008</t>
+        </is>
+      </c>
+      <c r="B89" s="24" t="inlineStr">
+        <is>
+          <t>Türkiye Finans</t>
+        </is>
+      </c>
+      <c r="C89" s="24" t="inlineStr">
+        <is>
+          <t>Kamu Çalışanlarına Özel İhtiyaç Finansmanı</t>
+        </is>
+      </c>
+      <c r="D89" s="24" t="inlineStr">
+        <is>
+          <t>Ihtiyac Finansmani Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E89" s="24" t="inlineStr">
+        <is>
+          <t>www.turkiyefinans.com.tr/tr-tr/kampanyalar/Sayfalar/kamu-calisanlarina-ozel-ihtiyac-finansmani.aspx</t>
+        </is>
+      </c>
       <c r="F89" s="25" t="n"/>
       <c r="G89" s="25" t="n"/>
       <c r="H89" s="24" t="n"/>
       <c r="I89" s="26" t="n"/>
-      <c r="J89" s="25" t="n"/>
+      <c r="J89" s="25" t="n">
+        <v>400000</v>
+      </c>
       <c r="K89" s="25" t="n"/>
       <c r="L89" s="24" t="n"/>
-      <c r="M89" s="24" t="n"/>
+      <c r="M89" s="24" t="inlineStr">
+        <is>
+          <t>Kamu çalışanlarına 50.000-400.000 TL arası ihtiyaç finansmanı, kişiye özel kâr payı oranı ve 3 ay ödeme öteleme</t>
+        </is>
+      </c>
       <c r="N89" s="24" t="n"/>
       <c r="O89" s="27" t="n"/>
       <c r="P89" s="27" t="n"/>
-      <c r="Q89" s="24" t="n"/>
+      <c r="Q89" s="24" t="inlineStr">
+        <is>
+          <t>Kamu çalışanları</t>
+        </is>
+      </c>
       <c r="R89" s="24" t="n"/>
       <c r="S89" s="24" t="n"/>
-      <c r="T89" s="27" t="n"/>
-      <c r="U89" s="24" t="n"/>
+      <c r="T89" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U89" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: 'size ozel kar payi oranlari' deniyor ama SAYI verilmiyor. Kampanya tarihi de sayfada YOK. erteleme_suresi_ay dolu olan ilk altin kayit - o sutun su an OLCUM DISI (excel_to_json INCELENMIS_ALANLAR'a bak).</t>
+        </is>
+      </c>
+      <c r="W89" t="n">
+        <v>3</v>
+      </c>
+      <c r="X89" s="2" t="inlineStr">
+        <is>
+          <t>finansman_tutari: Kampanya kapsamında 50.000 TL – 400.000 TL arasındaki ihtiyaçlarını için finansman başvurusu yapabilirsiniz.
+erteleme_suresi_ay: Finansman geri ödemelerinizde ilk taksiniz için 3 ay öteleme hakkınızı kullanabilir</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="24" t="n"/>

</xml_diff>

<commit_message>
on bir yeni altin kayit: Kuveyt Turk, Emlak ve Ziraat
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -8289,34 +8289,111 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="24" t="n"/>
-      <c r="B90" s="24" t="n"/>
-      <c r="C90" s="24" t="n"/>
-      <c r="D90" s="24" t="n"/>
-      <c r="E90" s="24" t="n"/>
+      <c r="A90" s="24" t="inlineStr">
+        <is>
+          <t>KT-012</t>
+        </is>
+      </c>
+      <c r="B90" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C90" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk Kampüs'e Gelenlere Toplamda 13.500 TL Hediye</t>
+        </is>
+      </c>
+      <c r="D90" s="24" t="inlineStr">
+        <is>
+          <t>Yeni Musteri Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E90" s="24" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/kuveyt-turk-kampuse-gelenlere-toplamda-13500-tl-hediye</t>
+        </is>
+      </c>
       <c r="F90" s="25" t="n"/>
       <c r="G90" s="25" t="n"/>
       <c r="H90" s="24" t="n"/>
       <c r="I90" s="26" t="n"/>
       <c r="J90" s="25" t="n"/>
-      <c r="K90" s="25" t="n"/>
-      <c r="L90" s="24" t="n"/>
-      <c r="M90" s="24" t="n"/>
+      <c r="K90" s="25" t="n">
+        <v>13500</v>
+      </c>
+      <c r="L90" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M90" s="24" t="inlineStr">
+        <is>
+          <t>Kampüs'e katılanlara davet kodu, kart harcamaları ve ilk e-ticaret harcamasından toplamda 13.500 TL hediye</t>
+        </is>
+      </c>
       <c r="N90" s="24" t="n"/>
-      <c r="O90" s="27" t="n"/>
-      <c r="P90" s="27" t="n"/>
-      <c r="Q90" s="24" t="n"/>
+      <c r="O90" s="27" t="inlineStr">
+        <is>
+          <t>2025-06-23</t>
+        </is>
+      </c>
+      <c r="P90" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q90" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk Mobil'den müşteri olan kampüslü (öğrenci) müşteriler</t>
+        </is>
+      </c>
       <c r="R90" s="24" t="n"/>
       <c r="S90" s="24" t="n"/>
-      <c r="T90" s="27" t="n"/>
-      <c r="U90" s="24" t="n"/>
+      <c r="T90" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U90" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. SEMSIYE SAYFA: alt kampanyalarin toplamini duyuruyor (davet 10.500 + hos geldin 500 + kart harcamasi 1.500 + yurt disi cikis harci). odul_miktari basliktaki TOPLAMDIR. Katilim 30.000 kisi ile sinirli.</t>
+        </is>
+      </c>
+      <c r="X90" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Kuveyt Türk Kampüs'e katılanlar davet kodu, kart harcamaları ve ilk E-Ticaret harcaması kampanyalarından toplamda 13.500 TL Hediye!
+kampanya_baslangic: 23.06.2025 - 31.12.2026
+kampanya_bitis: 23.06.2025 - 31.12.2026</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="24" t="n"/>
-      <c r="B91" s="24" t="n"/>
-      <c r="C91" s="24" t="n"/>
-      <c r="D91" s="24" t="n"/>
-      <c r="E91" s="24" t="n"/>
+      <c r="A91" s="24" t="inlineStr">
+        <is>
+          <t>KT-013</t>
+        </is>
+      </c>
+      <c r="B91" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C91" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk Mobil'den Müşterimiz Olun Özel Kur Fırsatı</t>
+        </is>
+      </c>
+      <c r="D91" s="24" t="inlineStr">
+        <is>
+          <t>Yatirim Urunu Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E91" s="24" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/kuveyt-turk-mobilden-musterimiz-olun-ozel-kur-firsatini-kacirmayin</t>
+        </is>
+      </c>
       <c r="F91" s="25" t="n"/>
       <c r="G91" s="25" t="n"/>
       <c r="H91" s="24" t="n"/>
@@ -8324,22 +8401,72 @@
       <c r="J91" s="25" t="n"/>
       <c r="K91" s="25" t="n"/>
       <c r="L91" s="24" t="n"/>
-      <c r="M91" s="24" t="n"/>
+      <c r="M91" s="24" t="inlineStr">
+        <is>
+          <t>Mobilden müşteri olan bireysel müşterilere döviz ve kıymetli maden işlemlerinde özel kur</t>
+        </is>
+      </c>
       <c r="N91" s="24" t="n"/>
-      <c r="O91" s="27" t="n"/>
-      <c r="P91" s="27" t="n"/>
-      <c r="Q91" s="24" t="n"/>
+      <c r="O91" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="P91" s="27" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Q91" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk Mobil'den müşteri olan bireysel müşteriler</t>
+        </is>
+      </c>
       <c r="R91" s="24" t="n"/>
       <c r="S91" s="24" t="n"/>
-      <c r="T91" s="27" t="n"/>
-      <c r="U91" s="24" t="n"/>
+      <c r="T91" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U91" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfa 'avantajli kur' ve 'ozel oranlar' diyor, tek bir sayi vermiyor. Kurlar mobil uygulamada musteriye ozel tanimlaniyor.</t>
+        </is>
+      </c>
+      <c r="X91" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 15.05.2026 - 1.09.2026
+kampanya_bitis: 15.05.2026 - 1.09.2026</t>
+        </is>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" s="24" t="n"/>
-      <c r="B92" s="24" t="n"/>
-      <c r="C92" s="24" t="n"/>
-      <c r="D92" s="24" t="n"/>
-      <c r="E92" s="24" t="n"/>
+      <c r="A92" s="24" t="inlineStr">
+        <is>
+          <t>TEK-010</t>
+        </is>
+      </c>
+      <c r="B92" s="24" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C92" s="24" t="inlineStr">
+        <is>
+          <t>Biletinial'da %20 İndirim</t>
+        </is>
+      </c>
+      <c r="D92" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E92" s="24" t="inlineStr">
+        <is>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/biletinialda-20-indirim</t>
+        </is>
+      </c>
       <c r="F92" s="25" t="n"/>
       <c r="G92" s="25" t="n"/>
       <c r="H92" s="24" t="n"/>
@@ -8347,45 +8474,147 @@
       <c r="J92" s="25" t="n"/>
       <c r="K92" s="25" t="n"/>
       <c r="L92" s="24" t="n"/>
-      <c r="M92" s="24" t="n"/>
+      <c r="M92" s="24" t="inlineStr">
+        <is>
+          <t>emlak20 kupon koduyla Biletinial etkinlik biletlerinde %20 indirim</t>
+        </is>
+      </c>
       <c r="N92" s="24" t="n"/>
       <c r="O92" s="27" t="n"/>
-      <c r="P92" s="27" t="n"/>
-      <c r="Q92" s="24" t="n"/>
+      <c r="P92" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q92" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf, Paraf Premium ve Debit kart sahipleri</t>
+        </is>
+      </c>
       <c r="R92" s="24" t="n"/>
       <c r="S92" s="24" t="n"/>
-      <c r="T92" s="27" t="n"/>
-      <c r="U92" s="24" t="n"/>
+      <c r="T92" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U92" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: indirim yalnizca YUZDE olarak veriliyor, TL tavani yok. kar_payi_orani da bos: %20 kupon indirimidir. Sepete en fazla 9 bilet. Baslangic tarihi yok.</t>
+        </is>
+      </c>
+      <c r="X92" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya, 31.12.2026 tarihine kadar alınacak etkinlik biletlerinde geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" s="24" t="n"/>
-      <c r="B93" s="24" t="n"/>
-      <c r="C93" s="24" t="n"/>
-      <c r="D93" s="24" t="n"/>
-      <c r="E93" s="24" t="n"/>
+      <c r="A93" s="24" t="inlineStr">
+        <is>
+          <t>KT-014</t>
+        </is>
+      </c>
+      <c r="B93" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C93" s="24" t="inlineStr">
+        <is>
+          <t>Mobilden Kuveyt Türklü Olanlara Toplamda 7.250 TL Hediye</t>
+        </is>
+      </c>
+      <c r="D93" s="24" t="inlineStr">
+        <is>
+          <t>Yeni Musteri Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E93" s="24" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/mobilden-kuveyt-turklu-olanlara-toplamda-7250-tl-hediye</t>
+        </is>
+      </c>
       <c r="F93" s="25" t="n"/>
       <c r="G93" s="25" t="n"/>
       <c r="H93" s="24" t="n"/>
       <c r="I93" s="26" t="n"/>
       <c r="J93" s="25" t="n"/>
-      <c r="K93" s="25" t="n"/>
-      <c r="L93" s="24" t="n"/>
-      <c r="M93" s="24" t="n"/>
+      <c r="K93" s="25" t="n">
+        <v>7250</v>
+      </c>
+      <c r="L93" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M93" s="24" t="inlineStr">
+        <is>
+          <t>Mobilden müşteri olanlara kart harcaması, fatura talimatı ve davet kodundan toplamda 7.250 TL</t>
+        </is>
+      </c>
       <c r="N93" s="24" t="n"/>
-      <c r="O93" s="27" t="n"/>
-      <c r="P93" s="27" t="n"/>
-      <c r="Q93" s="24" t="n"/>
+      <c r="O93" s="27" t="inlineStr">
+        <is>
+          <t>2024-02-01</t>
+        </is>
+      </c>
+      <c r="P93" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q93" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk Mobil veya Self Nokta'dan müşteri olan bireysel müşteriler</t>
+        </is>
+      </c>
       <c r="R93" s="24" t="n"/>
       <c r="S93" s="24" t="n"/>
-      <c r="T93" s="27" t="n"/>
-      <c r="U93" s="24" t="n"/>
+      <c r="T93" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U93" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. SEMSIYE SAYFA: davet 5.500 + fatura talimati 500 + yurt disi cikis harci iadesi. odul_miktari basliktaki TOPLAMDIR. Kampus surumuyle (13.500 TL) ayni yapida ama farkli kitle ve farkli tutar - metin benzerligi %35, ayri kampanyalar.</t>
+        </is>
+      </c>
+      <c r="X93" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Mobilden Kuveyt Türklü Olun Toplamda 7.250 TL Kazanın!
+kampanya_baslangic: 1.02.2024 - 31.12.2026
+kampanya_bitis: 1.02.2024 - 31.12.2026</t>
+        </is>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" s="24" t="n"/>
-      <c r="B94" s="24" t="n"/>
-      <c r="C94" s="24" t="n"/>
-      <c r="D94" s="24" t="n"/>
-      <c r="E94" s="24" t="n"/>
+      <c r="A94" s="24" t="inlineStr">
+        <is>
+          <t>TEK-011</t>
+        </is>
+      </c>
+      <c r="B94" s="24" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C94" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf'tan tabii Premium Üyeliği Hediye</t>
+        </is>
+      </c>
+      <c r="D94" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E94" s="24" t="inlineStr">
+        <is>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/emlak-katilim-paraftan-tabii-premium-uyeligi-hediye</t>
+        </is>
+      </c>
       <c r="F94" s="25" t="n"/>
       <c r="G94" s="25" t="n"/>
       <c r="H94" s="24" t="n"/>
@@ -8393,22 +8622,72 @@
       <c r="J94" s="25" t="n"/>
       <c r="K94" s="25" t="n"/>
       <c r="L94" s="24" t="n"/>
-      <c r="M94" s="24" t="n"/>
+      <c r="M94" s="24" t="inlineStr">
+        <is>
+          <t>Paraf kartla yapılan tabii Premium üyelik ödemesinin ilgili ay ücreti karta iade</t>
+        </is>
+      </c>
       <c r="N94" s="24" t="n"/>
-      <c r="O94" s="27" t="n"/>
-      <c r="P94" s="27" t="n"/>
-      <c r="Q94" s="24" t="n"/>
+      <c r="O94" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P94" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="Q94" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
       <c r="R94" s="24" t="n"/>
       <c r="S94" s="24" t="n"/>
-      <c r="T94" s="27" t="n"/>
-      <c r="U94" s="24" t="n"/>
+      <c r="T94" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U94" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: 'ilgili ayin uyelik ucreti kadar iade' deniyor, TUTAR YAZMIYOR. Trendyol Plus kaydiyla (75 TL acikca yazili) karsilastirmali cift olusturur.</t>
+        </is>
+      </c>
+      <c r="X94" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 01.07.2026 – 31.07.2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 01.07.2026 – 31.07.2026 tarihleri arasında geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="24" t="n"/>
-      <c r="B95" s="24" t="n"/>
-      <c r="C95" s="24" t="n"/>
-      <c r="D95" s="24" t="n"/>
-      <c r="E95" s="24" t="n"/>
+      <c r="A95" s="24" t="inlineStr">
+        <is>
+          <t>ZK-012</t>
+        </is>
+      </c>
+      <c r="B95" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C95" s="24" t="inlineStr">
+        <is>
+          <t>Alarko Carrier'da 6 Taksit</t>
+        </is>
+      </c>
+      <c r="D95" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E95" s="24" t="inlineStr">
+        <is>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/alarko-carrierda-6-taksit</t>
+        </is>
+      </c>
       <c r="F95" s="25" t="n"/>
       <c r="G95" s="25" t="n"/>
       <c r="H95" s="24" t="n"/>
@@ -8416,68 +8695,230 @@
       <c r="J95" s="25" t="n"/>
       <c r="K95" s="25" t="n"/>
       <c r="L95" s="24" t="n"/>
-      <c r="M95" s="24" t="n"/>
+      <c r="M95" s="24" t="inlineStr">
+        <is>
+          <t>Bankkart kredi kartıyla Alarko Carrier alışverişlerinde 6 taksit</t>
+        </is>
+      </c>
       <c r="N95" s="24" t="n"/>
       <c r="O95" s="27" t="n"/>
       <c r="P95" s="27" t="n"/>
-      <c r="Q95" s="24" t="n"/>
+      <c r="Q95" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+        </is>
+      </c>
       <c r="R95" s="24" t="n"/>
       <c r="S95" s="24" t="n"/>
-      <c r="T95" s="27" t="n"/>
-      <c r="U95" s="24" t="n"/>
+      <c r="T95" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U95" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V95" t="n">
+        <v>6</v>
+      </c>
+      <c r="X95" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 6 taksitli</t>
+        </is>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" s="24" t="n"/>
-      <c r="B96" s="24" t="n"/>
-      <c r="C96" s="24" t="n"/>
-      <c r="D96" s="24" t="n"/>
-      <c r="E96" s="24" t="n"/>
+      <c r="A96" s="24" t="inlineStr">
+        <is>
+          <t>KT-015</t>
+        </is>
+      </c>
+      <c r="B96" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C96" s="24" t="inlineStr">
+        <is>
+          <t>Sağlam Kart Sahipleri Halalbooking'de de Avantajlı</t>
+        </is>
+      </c>
+      <c r="D96" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E96" s="24" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/saglam-kart-sahipleri-halalbookingde-de-avantajli</t>
+        </is>
+      </c>
       <c r="F96" s="25" t="n"/>
       <c r="G96" s="25" t="n"/>
       <c r="H96" s="24" t="n"/>
       <c r="I96" s="26" t="n"/>
       <c r="J96" s="25" t="n"/>
-      <c r="K96" s="25" t="n"/>
-      <c r="L96" s="24" t="n"/>
-      <c r="M96" s="24" t="n"/>
+      <c r="K96" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L96" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M96" s="24" t="inlineStr">
+        <is>
+          <t>Halalbooking tatil harcamalarında 9 aya varan taksit ve ilk kayıtta 1.000 TL indirim (10.000 TL üzeri rezervasyonda)</t>
+        </is>
+      </c>
       <c r="N96" s="24" t="n"/>
-      <c r="O96" s="27" t="n"/>
-      <c r="P96" s="27" t="n"/>
-      <c r="Q96" s="24" t="n"/>
+      <c r="O96" s="27" t="inlineStr">
+        <is>
+          <t>2025-07-30</t>
+        </is>
+      </c>
+      <c r="P96" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q96" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk Sağlam Kart sahipleri</t>
+        </is>
+      </c>
       <c r="R96" s="24" t="n"/>
       <c r="S96" s="24" t="n"/>
-      <c r="T96" s="27" t="n"/>
-      <c r="U96" s="24" t="n"/>
+      <c r="T96" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U96" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 1.000 TL indirim yalnizca ILK KAYITTA ve 10.000 TL uzeri rezervasyonda gecerli - o tutar bir ESIKTIR, odul degil.</t>
+        </is>
+      </c>
+      <c r="V96" t="n">
+        <v>9</v>
+      </c>
+      <c r="X96" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Aralık 2026 tarihine kadar yapacağınız tatil harcamalarınızda 9 aya varan taksit avantajından yararlanabilir, Halalbooking’e kaydolurken 1.000 TL değerinde indirim kazanabilirsiniz.
+odul_miktari: 31 Aralık 2026 tarihine kadar yapacağınız tatil harcamalarınızda 9 aya varan taksit avantajından yararlanabilir, Halalbooking’e kaydolurken 1.000 TL değerinde indirim kazanabilirsiniz.
+kampanya_baslangic: 30.07.2025 - 31.12.2026
+kampanya_bitis: 30.07.2025 - 31.12.2026</t>
+        </is>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="24" t="n"/>
-      <c r="B97" s="24" t="n"/>
-      <c r="C97" s="24" t="n"/>
-      <c r="D97" s="24" t="n"/>
-      <c r="E97" s="24" t="n"/>
+      <c r="A97" s="24" t="inlineStr">
+        <is>
+          <t>TEK-012</t>
+        </is>
+      </c>
+      <c r="B97" s="24" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C97" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf'tan Trendyol Plus Üyelik Ücretiniz İade</t>
+        </is>
+      </c>
+      <c r="D97" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E97" s="24" t="inlineStr">
+        <is>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/emlak-katilim-paraftan-trendyol-plus-uyelik-ucretiniz-iade</t>
+        </is>
+      </c>
       <c r="F97" s="25" t="n"/>
       <c r="G97" s="25" t="n"/>
       <c r="H97" s="24" t="n"/>
       <c r="I97" s="26" t="n"/>
       <c r="J97" s="25" t="n"/>
-      <c r="K97" s="25" t="n"/>
-      <c r="L97" s="24" t="n"/>
-      <c r="M97" s="24" t="n"/>
+      <c r="K97" s="25" t="n">
+        <v>75</v>
+      </c>
+      <c r="L97" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M97" s="24" t="inlineStr">
+        <is>
+          <t>Paraf kartla yapılan Trendyol Plus üyelik ödemesindeki 75 TL üyelik ücreti karta iade</t>
+        </is>
+      </c>
       <c r="N97" s="24" t="n"/>
-      <c r="O97" s="27" t="n"/>
-      <c r="P97" s="27" t="n"/>
-      <c r="Q97" s="24" t="n"/>
+      <c r="O97" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P97" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="Q97" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri</t>
+        </is>
+      </c>
       <c r="R97" s="24" t="n"/>
       <c r="S97" s="24" t="n"/>
-      <c r="T97" s="27" t="n"/>
-      <c r="U97" s="24" t="n"/>
+      <c r="T97" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U97" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. tabii Premium kaydiyla ayni yapi ama burada tutar (75 TL) ACIKCA yazili; orada yazmiyor ve o alan bos birakildi.</t>
+        </is>
+      </c>
+      <c r="X97" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Emlak Katılım Paraf ve Emlak Katılım Paraf Premium kartınız ile 01.07.2026 – 31.07.2026 tarihleri arasında yapacağınız Trendyol Plus üyelik ödemenize ilişkin 75 TL tutarındaki üyelik ücreti kartınıza iade olarak yansıtılacaktır.
+kampanya_baslangic: 01.07.2026 – 31.07.2026
+kampanya_bitis: 01.07.2026 – 31.07.2026</t>
+        </is>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="24" t="n"/>
-      <c r="B98" s="24" t="n"/>
-      <c r="C98" s="24" t="n"/>
-      <c r="D98" s="24" t="n"/>
-      <c r="E98" s="24" t="n"/>
+      <c r="A98" s="24" t="inlineStr">
+        <is>
+          <t>ZK-013</t>
+        </is>
+      </c>
+      <c r="B98" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C98" s="24" t="inlineStr">
+        <is>
+          <t>Alfemo'da 5 Taksit</t>
+        </is>
+      </c>
+      <c r="D98" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E98" s="24" t="inlineStr">
+        <is>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/alfemoda-5-taksit</t>
+        </is>
+      </c>
       <c r="F98" s="25" t="n"/>
       <c r="G98" s="25" t="n"/>
       <c r="H98" s="24" t="n"/>
@@ -8485,45 +8926,145 @@
       <c r="J98" s="25" t="n"/>
       <c r="K98" s="25" t="n"/>
       <c r="L98" s="24" t="n"/>
-      <c r="M98" s="24" t="n"/>
+      <c r="M98" s="24" t="inlineStr">
+        <is>
+          <t>Bankkart kredi kartıyla Alfemo alışverişlerinde 5 taksit</t>
+        </is>
+      </c>
       <c r="N98" s="24" t="n"/>
       <c r="O98" s="27" t="n"/>
       <c r="P98" s="27" t="n"/>
-      <c r="Q98" s="24" t="n"/>
+      <c r="Q98" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+        </is>
+      </c>
       <c r="R98" s="24" t="n"/>
       <c r="S98" s="24" t="n"/>
-      <c r="T98" s="27" t="n"/>
-      <c r="U98" s="24" t="n"/>
+      <c r="T98" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U98" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V98" t="n">
+        <v>5</v>
+      </c>
+      <c r="X98" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 5 taksitli</t>
+        </is>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" s="24" t="n"/>
-      <c r="B99" s="24" t="n"/>
-      <c r="C99" s="24" t="n"/>
-      <c r="D99" s="24" t="n"/>
-      <c r="E99" s="24" t="n"/>
+      <c r="A99" s="24" t="inlineStr">
+        <is>
+          <t>KT-016</t>
+        </is>
+      </c>
+      <c r="B99" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C99" s="24" t="inlineStr">
+        <is>
+          <t>Yakınlarını Kuveyt Türk'e Davet Et Toplamda 5.000 TL'ye Varan Hediye Kazan</t>
+        </is>
+      </c>
+      <c r="D99" s="24" t="inlineStr">
+        <is>
+          <t>Yeni Musteri Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E99" s="24" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/yakinlarini-kuveyt-turke-davet-et-toplamda-5000-tlye-varan-hediye-kazan</t>
+        </is>
+      </c>
       <c r="F99" s="25" t="n"/>
       <c r="G99" s="25" t="n"/>
       <c r="H99" s="24" t="n"/>
       <c r="I99" s="26" t="n"/>
       <c r="J99" s="25" t="n"/>
-      <c r="K99" s="25" t="n"/>
-      <c r="L99" s="24" t="n"/>
-      <c r="M99" s="24" t="n"/>
+      <c r="K99" s="25" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L99" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M99" s="24" t="inlineStr">
+        <is>
+          <t>Davet koduyla müşteri olan her yakın için 500 TL, toplamda 5.000 TL'ye kadar; davet edilene de 500 TL harcama iadesi</t>
+        </is>
+      </c>
       <c r="N99" s="24" t="n"/>
-      <c r="O99" s="27" t="n"/>
-      <c r="P99" s="27" t="n"/>
-      <c r="Q99" s="24" t="n"/>
+      <c r="O99" s="27" t="inlineStr">
+        <is>
+          <t>2025-06-15</t>
+        </is>
+      </c>
+      <c r="P99" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q99" s="24" t="inlineStr">
+        <is>
+          <t>Mevcut Kuveyt Türk müşterileri (davet kodu paylaşanlar)</t>
+        </is>
+      </c>
       <c r="R99" s="24" t="n"/>
       <c r="S99" s="24" t="n"/>
-      <c r="T99" s="27" t="n"/>
-      <c r="U99" s="24" t="n"/>
+      <c r="T99" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U99" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari DAVET EDENIN tavanidir (5.000 TL); davet edilen ayrica 500 TL alir. Bu kampanya KT-012 ve KT-014'teki semsiye sayfalarin bir BILESENI - ayri sayfasi oldugu icin ayri kayit.</t>
+        </is>
+      </c>
+      <c r="X99" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 15.06.2025 - 31.12.2026
+kampanya_bitis: 15.06.2025 - 31.12.2026</t>
+        </is>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" s="24" t="n"/>
-      <c r="B100" s="24" t="n"/>
-      <c r="C100" s="24" t="n"/>
-      <c r="D100" s="24" t="n"/>
-      <c r="E100" s="24" t="n"/>
+      <c r="A100" s="24" t="inlineStr">
+        <is>
+          <t>TEK-013</t>
+        </is>
+      </c>
+      <c r="B100" s="24" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C100" s="24" t="inlineStr">
+        <is>
+          <t>Enterprise Araç Kiralamalarında %35 İndirim Fırsatı</t>
+        </is>
+      </c>
+      <c r="D100" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E100" s="24" t="inlineStr">
+        <is>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/enterprise-arac-kiralamalarinda-35-indirim-firsati</t>
+        </is>
+      </c>
       <c r="F100" s="25" t="n"/>
       <c r="G100" s="25" t="n"/>
       <c r="H100" s="24" t="n"/>
@@ -8531,15 +9072,40 @@
       <c r="J100" s="25" t="n"/>
       <c r="K100" s="25" t="n"/>
       <c r="L100" s="24" t="n"/>
-      <c r="M100" s="24" t="n"/>
+      <c r="M100" s="24" t="inlineStr">
+        <is>
+          <t>Banka iş birliği sayfasından Enterprise online araç kiralamalarında liste fiyatı üzerinden %35 indirim</t>
+        </is>
+      </c>
       <c r="N100" s="24" t="n"/>
       <c r="O100" s="27" t="n"/>
-      <c r="P100" s="27" t="n"/>
-      <c r="Q100" s="24" t="n"/>
+      <c r="P100" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q100" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf kart sahipleri</t>
+        </is>
+      </c>
       <c r="R100" s="24" t="n"/>
       <c r="S100" s="24" t="n"/>
-      <c r="T100" s="27" t="n"/>
-      <c r="U100" s="24" t="n"/>
+      <c r="T100" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U100" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari ve kar_payi_orani BILEREK BOS: %35 bir liste fiyati indirimidir, TL tavani yok. Baslangic tarihi yok.</t>
+        </is>
+      </c>
+      <c r="X100" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Liste fiyatı üzerinden %35 indirim kampanyası 31.12.2026 tarihine kadar Türkiye’deki tüm Enterprise ofislerinde online kiralamalarda geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="24" t="n"/>

</xml_diff>

<commit_message>
dort yeni altin kayit: KT-017, TEK-014, ZK-014, ZK-015
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -9108,57 +9108,200 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="24" t="n"/>
-      <c r="B101" s="24" t="n"/>
-      <c r="C101" s="24" t="n"/>
-      <c r="D101" s="24" t="n"/>
-      <c r="E101" s="24" t="n"/>
-      <c r="F101" s="25" t="n"/>
+      <c r="A101" s="24" t="inlineStr">
+        <is>
+          <t>KT-017</t>
+        </is>
+      </c>
+      <c r="B101" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C101" s="24" t="inlineStr">
+        <is>
+          <t>Yeni Müşterilere Özel İhtiyaç Kart'ta %1,99 Oran Fırsatı</t>
+        </is>
+      </c>
+      <c r="D101" s="24" t="inlineStr">
+        <is>
+          <t>Ihtiyac Finansmani Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E101" s="24" t="inlineStr">
+        <is>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/yeni-musterilere-ozel-ihtiyac-kartta-199-oran-firsati</t>
+        </is>
+      </c>
+      <c r="F101" s="25" t="n">
+        <v>1.99</v>
+      </c>
       <c r="G101" s="25" t="n"/>
-      <c r="H101" s="24" t="n"/>
-      <c r="I101" s="26" t="n"/>
-      <c r="J101" s="25" t="n"/>
+      <c r="H101" s="24" t="inlineStr">
+        <is>
+          <t>aylik</t>
+        </is>
+      </c>
+      <c r="I101" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="J101" s="25" t="n">
+        <v>100000</v>
+      </c>
       <c r="K101" s="25" t="n"/>
       <c r="L101" s="24" t="n"/>
-      <c r="M101" s="24" t="n"/>
+      <c r="M101" s="24" t="inlineStr">
+        <is>
+          <t>Görüntülü görüşmeyle yeni müşteri olanlara 100.000 TL'ye kadar %1,99 oranla 12 aya varan, 2 ay ertelemeli İhtiyaç Kart</t>
+        </is>
+      </c>
       <c r="N101" s="24" t="n"/>
-      <c r="O101" s="27" t="n"/>
-      <c r="P101" s="27" t="n"/>
-      <c r="Q101" s="24" t="n"/>
+      <c r="O101" s="27" t="inlineStr">
+        <is>
+          <t>2025-10-22</t>
+        </is>
+      </c>
+      <c r="P101" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q101" s="24" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk Mobil'den görüntülü görüşmeyle son 30 gün içinde müşteri olanlar</t>
+        </is>
+      </c>
       <c r="R101" s="24" t="n"/>
       <c r="S101" s="24" t="n"/>
-      <c r="T101" s="27" t="n"/>
-      <c r="U101" s="24" t="n"/>
+      <c r="T101" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U101" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 100.000 TL ustu basvurularda liste fiyati uygulaniyor, yani 100.000 TL kampanyanin TAVANI. oran_periyodu 'aylik': %1,99 yillik olsaydi piyasa disi dusuk olurdu.</t>
+        </is>
+      </c>
+      <c r="W101" t="n">
+        <v>2</v>
+      </c>
+      <c r="X101" s="2" t="inlineStr">
+        <is>
+          <t>kar_payi_orani: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
+vade_ay: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
+finansman_tutari: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
+kampanya_baslangic: 22.10.2025 - 31.12.2026
+kampanya_bitis: 22.10.2025 - 31.12.2026</t>
+        </is>
+      </c>
     </row>
     <row r="102">
-      <c r="A102" s="24" t="n"/>
-      <c r="B102" s="24" t="n"/>
-      <c r="C102" s="24" t="n"/>
-      <c r="D102" s="24" t="n"/>
-      <c r="E102" s="24" t="n"/>
+      <c r="A102" s="24" t="inlineStr">
+        <is>
+          <t>TEK-014</t>
+        </is>
+      </c>
+      <c r="B102" s="24" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C102" s="24" t="inlineStr">
+        <is>
+          <t>Giyim ve Kozmetik Alışverişlerinize 1.300 TL ParafPara</t>
+        </is>
+      </c>
+      <c r="D102" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E102" s="24" t="inlineStr">
+        <is>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/giyim-ve-kozmetik-alisverislerinize-1300-tl-parafpara</t>
+        </is>
+      </c>
       <c r="F102" s="25" t="n"/>
       <c r="G102" s="25" t="n"/>
       <c r="H102" s="24" t="n"/>
       <c r="I102" s="26" t="n"/>
       <c r="J102" s="25" t="n"/>
-      <c r="K102" s="25" t="n"/>
-      <c r="L102" s="24" t="n"/>
-      <c r="M102" s="24" t="n"/>
+      <c r="K102" s="25" t="n">
+        <v>1300</v>
+      </c>
+      <c r="L102" s="24" t="inlineStr">
+        <is>
+          <t>ParafPara</t>
+        </is>
+      </c>
+      <c r="M102" s="24" t="inlineStr">
+        <is>
+          <t>GIYIM2 SMS katılımıyla giyim/kozmetik harcamasına 500-1.250 TL, mobil/QR ödemede +50 TL, en fazla 1.300 TL ParafPara</t>
+        </is>
+      </c>
       <c r="N102" s="24" t="n"/>
-      <c r="O102" s="27" t="n"/>
-      <c r="P102" s="27" t="n"/>
-      <c r="Q102" s="24" t="n"/>
+      <c r="O102" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="P102" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q102" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf kart sahipleri</t>
+        </is>
+      </c>
       <c r="R102" s="24" t="n"/>
       <c r="S102" s="24" t="n"/>
-      <c r="T102" s="27" t="n"/>
-      <c r="U102" s="24" t="n"/>
+      <c r="T102" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U102" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 1.300 TL = en yuksek barem (1.250) + mobil/QR ekstrasi (50). Uc kademe: 500/800/1.250. AYNI AILEDEN IKI SURUM DAHA VAR (Temmuz 1.000 TL ve Temmuz 2.000 TL) ama metinleri bu kayda %89-92 benzedigi icin etiketlenmedi - ucu birden altin sete girseydi ayni teklif olcumde uc kat agirlik alir, train/test'e dagilirsa sizinti olurdu. Bu surum secildi cunku basliktaki sayi dogrudan bir kademe DEGIL: en yuksek barem (1.250) + mobil/QR ekstrasi (50).</t>
+        </is>
+      </c>
+      <c r="X102" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: bir müşteri kampanyaya bir kez katılabilir ve en fazla 1.300 TL ParafPara kazanabilir.
+kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" s="24" t="n"/>
-      <c r="B103" s="24" t="n"/>
-      <c r="C103" s="24" t="n"/>
-      <c r="D103" s="24" t="n"/>
-      <c r="E103" s="24" t="n"/>
+      <c r="A103" s="24" t="inlineStr">
+        <is>
+          <t>ZK-014</t>
+        </is>
+      </c>
+      <c r="B103" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C103" s="24" t="inlineStr">
+        <is>
+          <t>Amazon'da 9'a Varan Taksit</t>
+        </is>
+      </c>
+      <c r="D103" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E103" s="24" t="inlineStr">
+        <is>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/amazonda-9a-varan-taksit</t>
+        </is>
+      </c>
       <c r="F103" s="25" t="n"/>
       <c r="G103" s="25" t="n"/>
       <c r="H103" s="24" t="n"/>
@@ -9166,22 +9309,66 @@
       <c r="J103" s="25" t="n"/>
       <c r="K103" s="25" t="n"/>
       <c r="L103" s="24" t="n"/>
-      <c r="M103" s="24" t="n"/>
+      <c r="M103" s="24" t="inlineStr">
+        <is>
+          <t>Bankkart kredi kartıyla amazon.com.tr'de tutara göre peşin fiyatına 3, 6 veya 9 taksit</t>
+        </is>
+      </c>
       <c r="N103" s="24" t="n"/>
       <c r="O103" s="27" t="n"/>
       <c r="P103" s="27" t="n"/>
-      <c r="Q103" s="24" t="n"/>
+      <c r="Q103" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+        </is>
+      </c>
       <c r="R103" s="24" t="n"/>
       <c r="S103" s="24" t="n"/>
-      <c r="T103" s="27" t="n"/>
-      <c r="U103" s="24" t="n"/>
+      <c r="T103" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U103" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Uc kademe (3/6/9); 9 taksit yalnizca SECILI URUNLERDE ve 10.000 TL uzeri. Kampanya tarihi sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V103" t="n">
+        <v>9</v>
+      </c>
+      <c r="X103" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Seçili ürünlerde yapacağınız 10.000 TL ve üzeri alışverişlerinizde peşin fiyatına 9 taksit fırsatından faydalanabilirsiniz.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="24" t="n"/>
-      <c r="B104" s="24" t="n"/>
-      <c r="C104" s="24" t="n"/>
-      <c r="D104" s="24" t="n"/>
-      <c r="E104" s="24" t="n"/>
+      <c r="A104" s="24" t="inlineStr">
+        <is>
+          <t>ZK-015</t>
+        </is>
+      </c>
+      <c r="B104" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C104" s="24" t="inlineStr">
+        <is>
+          <t>Atasun Optik'te 6 Taksit</t>
+        </is>
+      </c>
+      <c r="D104" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E104" s="24" t="inlineStr">
+        <is>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/atasun-optikte-6-taksit</t>
+        </is>
+      </c>
       <c r="F104" s="25" t="n"/>
       <c r="G104" s="25" t="n"/>
       <c r="H104" s="24" t="n"/>
@@ -9189,15 +9376,39 @@
       <c r="J104" s="25" t="n"/>
       <c r="K104" s="25" t="n"/>
       <c r="L104" s="24" t="n"/>
-      <c r="M104" s="24" t="n"/>
+      <c r="M104" s="24" t="inlineStr">
+        <is>
+          <t>Bankkart kredi kartıyla Atasun Optik'te 4.000 TL üzeri işlemlerde peşin fiyatına 6 taksit</t>
+        </is>
+      </c>
       <c r="N104" s="24" t="n"/>
       <c r="O104" s="27" t="n"/>
       <c r="P104" s="27" t="n"/>
-      <c r="Q104" s="24" t="n"/>
+      <c r="Q104" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+        </is>
+      </c>
       <c r="R104" s="24" t="n"/>
       <c r="S104" s="24" t="n"/>
-      <c r="T104" s="27" t="n"/>
-      <c r="U104" s="24" t="n"/>
+      <c r="T104" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U104" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 4.000 TL bir ALT ESIKTIR, finansman tutari degil. Kampanya tarihi sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V104" t="n">
+        <v>6</v>
+      </c>
+      <c r="X104" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: peşin fiyatına 6 taksit</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="24" t="n"/>

</xml_diff>

<commit_message>
dort yeni altin kayit: ZK-016, TEK-015, TEK-016, ZK-017
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -9411,34 +9411,112 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="24" t="n"/>
-      <c r="B105" s="24" t="n"/>
-      <c r="C105" s="24" t="n"/>
-      <c r="D105" s="24" t="n"/>
-      <c r="E105" s="24" t="n"/>
+      <c r="A105" s="24" t="inlineStr">
+        <is>
+          <t>ZK-016</t>
+        </is>
+      </c>
+      <c r="B105" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C105" s="24" t="inlineStr">
+        <is>
+          <t>Bağımsız Kart'a Özel 5.000 TL'ye Varan Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="D105" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E105" s="24" t="inlineStr">
+        <is>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/bagimsiz-karta-ozel-5000-tlye-varan-bankkart-lira-1</t>
+        </is>
+      </c>
       <c r="F105" s="25" t="n"/>
       <c r="G105" s="25" t="n"/>
       <c r="H105" s="24" t="n"/>
       <c r="I105" s="26" t="n"/>
       <c r="J105" s="25" t="n"/>
-      <c r="K105" s="25" t="n"/>
-      <c r="L105" s="24" t="n"/>
-      <c r="M105" s="24" t="n"/>
+      <c r="K105" s="25" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L105" s="24" t="inlineStr">
+        <is>
+          <t>Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="M105" s="24" t="inlineStr">
+        <is>
+          <t>Bağımsız kredi kartıyla eğitim/sağlık/spor/kültür-sanat harcamalarına %10, toplamda 5.000 TL Bankkart Lira</t>
+        </is>
+      </c>
       <c r="N105" s="24" t="n"/>
-      <c r="O105" s="27" t="n"/>
-      <c r="P105" s="27" t="n"/>
-      <c r="Q105" s="24" t="n"/>
+      <c r="O105" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="P105" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Q105" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım Bankkart Bağımsız kredi kartı sahipleri</t>
+        </is>
+      </c>
       <c r="R105" s="24" t="n"/>
       <c r="S105" s="24" t="n"/>
-      <c r="T105" s="27" t="n"/>
-      <c r="U105" s="24" t="n"/>
+      <c r="T105" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U105" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %10 nakit iade oranidir. Bir sonraki donemi (8 Agustos - 7 Eylul) ayri sayfada duruyor ama metin neredeyse ayni - etiketlenmedi.</t>
+        </is>
+      </c>
+      <c r="X105" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: tüm harcamalara %10, toplamda 5.000 TL Bankkart Lira!
+odul_birimi: tüm harcamalara %10, toplamda 5.000 TL Bankkart Lira!
+kampanya_baslangic: 10 Temmuz – 7 Ağustos 2026
+kampanya_bitis: 10 Temmuz – 7 Ağustos 2026</t>
+        </is>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="24" t="n"/>
-      <c r="B106" s="24" t="n"/>
-      <c r="C106" s="24" t="n"/>
-      <c r="D106" s="24" t="n"/>
-      <c r="E106" s="24" t="n"/>
+      <c r="A106" s="24" t="inlineStr">
+        <is>
+          <t>TEK-015</t>
+        </is>
+      </c>
+      <c r="B106" s="24" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C106" s="24" t="inlineStr">
+        <is>
+          <t>Hızlı Çiçek'te Tüm İndirimlere Ek %20 İndirim Fırsatı</t>
+        </is>
+      </c>
+      <c r="D106" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E106" s="24" t="inlineStr">
+        <is>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/hizli-cicekte-tum-indirimlere-ek-20-indirim-firsati</t>
+        </is>
+      </c>
       <c r="F106" s="25" t="n"/>
       <c r="G106" s="25" t="n"/>
       <c r="H106" s="24" t="n"/>
@@ -9446,22 +9524,67 @@
       <c r="J106" s="25" t="n"/>
       <c r="K106" s="25" t="n"/>
       <c r="L106" s="24" t="n"/>
-      <c r="M106" s="24" t="n"/>
+      <c r="M106" s="24" t="inlineStr">
+        <is>
+          <t>EKB20 kupon koduyla Hızlı Çiçek'te tüm indirimlere ek %20 indirim</t>
+        </is>
+      </c>
       <c r="N106" s="24" t="n"/>
       <c r="O106" s="27" t="n"/>
-      <c r="P106" s="27" t="n"/>
-      <c r="Q106" s="24" t="n"/>
+      <c r="P106" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q106" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf, Paraf Premium ve Debit kart sahipleri</t>
+        </is>
+      </c>
       <c r="R106" s="24" t="n"/>
       <c r="S106" s="24" t="n"/>
-      <c r="T106" s="27" t="n"/>
-      <c r="U106" s="24" t="n"/>
+      <c r="T106" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U106" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Sayisal alanlar BILEREK BOS: %20 kupon indirimidir, TL tavani yok. Baslangic tarihi YOK.</t>
+        </is>
+      </c>
+      <c r="X106" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya 31.12.2026 tarihine kadar geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="24" t="n"/>
-      <c r="B107" s="24" t="n"/>
-      <c r="C107" s="24" t="n"/>
-      <c r="D107" s="24" t="n"/>
-      <c r="E107" s="24" t="n"/>
+      <c r="A107" s="24" t="inlineStr">
+        <is>
+          <t>TEK-016</t>
+        </is>
+      </c>
+      <c r="B107" s="24" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C107" s="24" t="inlineStr">
+        <is>
+          <t>Marina Mayo'da Tüm Ürünlerde %15 İndirim</t>
+        </is>
+      </c>
+      <c r="D107" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E107" s="24" t="inlineStr">
+        <is>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/marina-mayoda-tum-urunlerde-15-indirim</t>
+        </is>
+      </c>
       <c r="F107" s="25" t="n"/>
       <c r="G107" s="25" t="n"/>
       <c r="H107" s="24" t="n"/>
@@ -9469,22 +9592,67 @@
       <c r="J107" s="25" t="n"/>
       <c r="K107" s="25" t="n"/>
       <c r="L107" s="24" t="n"/>
-      <c r="M107" s="24" t="n"/>
+      <c r="M107" s="24" t="inlineStr">
+        <is>
+          <t>emlak15 kupon koduyla Marina Mayo'da tüm ürünlerde %15 indirim (tek kullanımlık)</t>
+        </is>
+      </c>
       <c r="N107" s="24" t="n"/>
       <c r="O107" s="27" t="n"/>
-      <c r="P107" s="27" t="n"/>
-      <c r="Q107" s="24" t="n"/>
+      <c r="P107" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q107" s="24" t="inlineStr">
+        <is>
+          <t>Emlak Katılım Paraf, Paraf Premium ve Debit kart sahipleri</t>
+        </is>
+      </c>
       <c r="R107" s="24" t="n"/>
       <c r="S107" s="24" t="n"/>
-      <c r="T107" s="27" t="n"/>
-      <c r="U107" s="24" t="n"/>
+      <c r="T107" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U107" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Sayisal alanlar BILEREK BOS: %15 kupon indirimidir. Baslangic tarihi YOK.</t>
+        </is>
+      </c>
+      <c r="X107" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya, 31.12.2026 tarihine kadar geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="24" t="n"/>
-      <c r="B108" s="24" t="n"/>
-      <c r="C108" s="24" t="n"/>
-      <c r="D108" s="24" t="n"/>
-      <c r="E108" s="24" t="n"/>
+      <c r="A108" s="24" t="inlineStr">
+        <is>
+          <t>ZK-017</t>
+        </is>
+      </c>
+      <c r="B108" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C108" s="24" t="inlineStr">
+        <is>
+          <t>BAUHAUS'ta 3 Taksit</t>
+        </is>
+      </c>
+      <c r="D108" s="24" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E108" s="24" t="inlineStr">
+        <is>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/bauhausta-3-taksit</t>
+        </is>
+      </c>
       <c r="F108" s="25" t="n"/>
       <c r="G108" s="25" t="n"/>
       <c r="H108" s="24" t="n"/>
@@ -9492,15 +9660,39 @@
       <c r="J108" s="25" t="n"/>
       <c r="K108" s="25" t="n"/>
       <c r="L108" s="24" t="n"/>
-      <c r="M108" s="24" t="n"/>
+      <c r="M108" s="24" t="inlineStr">
+        <is>
+          <t>Bankkart kredi kartıyla BAUHAUS alışverişlerinde 3 taksit</t>
+        </is>
+      </c>
       <c r="N108" s="24" t="n"/>
       <c r="O108" s="27" t="n"/>
       <c r="P108" s="27" t="n"/>
-      <c r="Q108" s="24" t="n"/>
+      <c r="Q108" s="24" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+        </is>
+      </c>
       <c r="R108" s="24" t="n"/>
       <c r="S108" s="24" t="n"/>
-      <c r="T108" s="27" t="n"/>
-      <c r="U108" s="24" t="n"/>
+      <c r="T108" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="U108" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V108" t="n">
+        <v>3</v>
+      </c>
+      <c r="X108" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 3 taksit</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="24" t="n"/>

</xml_diff>

<commit_message>
is listesi kume tabanli secime gecti, kota kaldirildi, iki kopya kayit ayiklandi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -1212,7 +1212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X109"/>
+  <dimension ref="A1:X107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7237,17 +7237,17 @@
     <row r="76">
       <c r="A76" s="24" t="inlineStr">
         <is>
-          <t>TEK-008</t>
+          <t>VK-010</t>
         </is>
       </c>
       <c r="B76" s="24" t="inlineStr">
         <is>
-          <t>Türkiye Emlak Katılım</t>
+          <t>Vakıf Katılım</t>
         </is>
       </c>
       <c r="C76" s="24" t="inlineStr">
         <is>
-          <t>Akaryakıt Harcamalarınıza 400 TL ParafPara</t>
+          <t>VClub Dünyası Artık Vakıf Katılım Mobil'de</t>
         </is>
       </c>
       <c r="D76" s="24" t="inlineStr">
@@ -7257,7 +7257,7 @@
       </c>
       <c r="E76" s="24" t="inlineStr">
         <is>
-          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/akaryakit-harcamalariniza-400-tl-parafpara</t>
+          <t>www.vakifkatilim.com.tr/tr/kendim-icin/kampanyalar/detay/vclub-dunyasi-artik-vakif-katilim-mobilde</t>
         </is>
       </c>
       <c r="F76" s="25" t="n"/>
@@ -7265,33 +7265,19 @@
       <c r="H76" s="24" t="n"/>
       <c r="I76" s="26" t="n"/>
       <c r="J76" s="25" t="n"/>
-      <c r="K76" s="25" t="n">
-        <v>400</v>
-      </c>
-      <c r="L76" s="24" t="inlineStr">
-        <is>
-          <t>ParafPara</t>
-        </is>
-      </c>
+      <c r="K76" s="25" t="n"/>
+      <c r="L76" s="24" t="n"/>
       <c r="M76" s="24" t="inlineStr">
         <is>
-          <t>SMS ile katılıp 1.500 TL üzeri 2. ve 4. akaryakıt harcamasına 200'er TL, toplam 400 TL ParafPara</t>
+          <t>VClub sadakat programı ile süpermarket, seyahat, giyim, teknoloji, kafe ve restoranlarda müşteriye özel indirimler</t>
         </is>
       </c>
       <c r="N76" s="24" t="n"/>
-      <c r="O76" s="27" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="P76" s="27" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
+      <c r="O76" s="27" t="n"/>
+      <c r="P76" s="27" t="n"/>
       <c r="Q76" s="24" t="inlineStr">
         <is>
-          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+          <t>Aktif Vakıf Katılım kredi veya banka kartı kullanan müşteriler</t>
         </is>
       </c>
       <c r="R76" s="24" t="n"/>
@@ -7303,32 +7289,25 @@
       </c>
       <c r="U76" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Katilim SMS ile ('AKARYAKIT' yazip 6026'ya). Musteri basina bir kez.</t>
-        </is>
-      </c>
-      <c r="X76" s="2" t="inlineStr">
-        <is>
-          <t>odul_miktari: Kampanya kapsamında yurt içinde tek seferde yapılacak 1.500 TL ve üzeri ikinci ve dördüncü akaryakıt harcamasına 200 TL, toplam 400 TL ParafPara verilecektir.
-odul_birimi: Kampanya kapsamında yurt içinde tek seferde yapılacak 1.500 TL ve üzeri ikinci ve dördüncü akaryakıt harcamasına 200 TL, toplam 400 TL ParafPara verilecektir.
-kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
-        </is>
-      </c>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfa indirim orani VERMIYOR ('musteri ozelinde degisiklik gosterebilmektedir'). Tarih de yok. GastroClub is birligi - HF-007 ile ayni platform, farkli banka.</t>
+        </is>
+      </c>
+      <c r="X76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="24" t="inlineStr">
         <is>
-          <t>VK-010</t>
+          <t>ZK-010</t>
         </is>
       </c>
       <c r="B77" s="24" t="inlineStr">
         <is>
-          <t>Vakıf Katılım</t>
+          <t>Ziraat Katılım</t>
         </is>
       </c>
       <c r="C77" s="24" t="inlineStr">
         <is>
-          <t>VClub Dünyası Artık Vakıf Katılım Mobil'de</t>
+          <t>Abdullah Kiğılı'da 2 Taksit</t>
         </is>
       </c>
       <c r="D77" s="24" t="inlineStr">
@@ -7338,7 +7317,7 @@
       </c>
       <c r="E77" s="24" t="inlineStr">
         <is>
-          <t>www.vakifkatilim.com.tr/tr/kendim-icin/kampanyalar/detay/vclub-dunyasi-artik-vakif-katilim-mobilde</t>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/abdullah-kigilida-2-taksit</t>
         </is>
       </c>
       <c r="F77" s="25" t="n"/>
@@ -7350,7 +7329,7 @@
       <c r="L77" s="24" t="n"/>
       <c r="M77" s="24" t="inlineStr">
         <is>
-          <t>VClub sadakat programı ile süpermarket, seyahat, giyim, teknoloji, kafe ve restoranlarda müşteriye özel indirimler</t>
+          <t>Bankkart kredi kartıyla Abdullah Kiğılı alışverişlerinde 2 taksit</t>
         </is>
       </c>
       <c r="N77" s="24" t="n"/>
@@ -7358,7 +7337,7 @@
       <c r="P77" s="27" t="n"/>
       <c r="Q77" s="24" t="inlineStr">
         <is>
-          <t>Aktif Vakıf Katılım kredi veya banka kartı kullanan müşteriler</t>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
       <c r="R77" s="24" t="n"/>
@@ -7370,25 +7349,32 @@
       </c>
       <c r="U77" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfa indirim orani VERMIYOR ('musteri ozelinde degisiklik gosterebilmektedir'). Tarih de yok. GastroClub is birligi - HF-007 ile ayni platform, farkli banka.</t>
-        </is>
-      </c>
-      <c r="X77" s="2" t="n"/>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve alt/ust harcama siniri sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V77" t="n">
+        <v>2</v>
+      </c>
+      <c r="X77" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 2 taksitli</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="24" t="inlineStr">
         <is>
-          <t>ZK-010</t>
+          <t>AL-011</t>
         </is>
       </c>
       <c r="B78" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım</t>
+          <t>Albaraka Türk</t>
         </is>
       </c>
       <c r="C78" s="24" t="inlineStr">
         <is>
-          <t>Abdullah Kiğılı'da 2 Taksit</t>
+          <t>Otomatik Fatura Ödeme Talimatlarınıza Toplamda 2.000 TL Worldpuan</t>
         </is>
       </c>
       <c r="D78" s="24" t="inlineStr">
@@ -7398,7 +7384,7 @@
       </c>
       <c r="E78" s="24" t="inlineStr">
         <is>
-          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/abdullah-kigilida-2-taksit</t>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/otomatik-fatura-odeme-talimatlariniza-toplamda-2000-tl-worldpuan-12</t>
         </is>
       </c>
       <c r="F78" s="25" t="n"/>
@@ -7406,19 +7392,33 @@
       <c r="H78" s="24" t="n"/>
       <c r="I78" s="26" t="n"/>
       <c r="J78" s="25" t="n"/>
-      <c r="K78" s="25" t="n"/>
-      <c r="L78" s="24" t="n"/>
+      <c r="K78" s="25" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L78" s="24" t="inlineStr">
+        <is>
+          <t>Worldpuan</t>
+        </is>
+      </c>
       <c r="M78" s="24" t="inlineStr">
         <is>
-          <t>Bankkart kredi kartıyla Abdullah Kiğılı alışverişlerinde 2 taksit</t>
+          <t>Albaraka Mobil'den verilen her yeni otomatik fatura ödeme talimatına 200 TL, toplamda 2.000 TL'ye varan Worldpuan</t>
         </is>
       </c>
       <c r="N78" s="24" t="n"/>
-      <c r="O78" s="27" t="n"/>
-      <c r="P78" s="27" t="n"/>
+      <c r="O78" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="P78" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="Q78" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+          <t>Albaraka Mobil'den kampanyaya katılan bireysel müşteriler (World özellikli kart gerekli)</t>
         </is>
       </c>
       <c r="R78" s="24" t="n"/>
@@ -7430,32 +7430,32 @@
       </c>
       <c r="U78" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve alt/ust harcama siniri sayfada YOK.</t>
-        </is>
-      </c>
-      <c r="V78" t="n">
-        <v>2</v>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. DIKKAT - AL-007 ile KARISTIRILMASIN: ikisi de Agustos 2026 fatura kampanyasi ve ikisinin de tavani 2.000 TL Worldpuan, ama AL-007 talimat basina 500 TL veriyor ve yalnizca goruntulu gorusmeyle yeni musteri olanlar icin (OFT2026 kodu); bu kayit talimat basina 200 TL ve mevcut musteriler icin. Ayri sayfalar, ayri kosullar. Insan dogrulamasinda ikisi de acilip bakilmali.</t>
+        </is>
       </c>
       <c r="X78" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: 2 taksitli</t>
+          <t>odul_miktari: Albaraka Mobil üzerinden kredi kartınız ile vereceğiniz her yeni otomatik fatura ödeme talimatınıza 200 TL, toplamda 2.000 TL'ye varan Worldpuan kazanma fırsatı!
+odul_birimi: Albaraka Mobil üzerinden kredi kartınız ile vereceğiniz her yeni otomatik fatura ödeme talimatınıza 200 TL, toplamda 2.000 TL'ye varan Worldpuan kazanma fırsatı!
+kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihlerinde geçerlidir.
+kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihlerinde geçerlidir.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="24" t="inlineStr">
         <is>
-          <t>AL-011</t>
+          <t>DK-009</t>
         </is>
       </c>
       <c r="B79" s="24" t="inlineStr">
         <is>
-          <t>Albaraka Türk</t>
+          <t>Dünya Katılım</t>
         </is>
       </c>
       <c r="C79" s="24" t="inlineStr">
         <is>
-          <t>Otomatik Fatura Ödeme Talimatlarınıza Toplamda 2.000 TL Worldpuan</t>
+          <t>LC Waikiki'de 3.000 TL ve Üzeri Alışverişe 300 TL İndirim</t>
         </is>
       </c>
       <c r="D79" s="24" t="inlineStr">
@@ -7465,7 +7465,7 @@
       </c>
       <c r="E79" s="24" t="inlineStr">
         <is>
-          <t>www.albaraka.com.tr/tr/kampanyalar/detay/otomatik-fatura-odeme-talimatlariniza-toplamda-2000-tl-worldpuan-12</t>
+          <t>www.dunyakatilim.com.tr/kampanyalar/lc-waikiki</t>
         </is>
       </c>
       <c r="F79" s="25" t="n"/>
@@ -7474,32 +7474,32 @@
       <c r="I79" s="26" t="n"/>
       <c r="J79" s="25" t="n"/>
       <c r="K79" s="25" t="n">
-        <v>2000</v>
+        <v>300</v>
       </c>
       <c r="L79" s="24" t="inlineStr">
         <is>
-          <t>Worldpuan</t>
+          <t>TL</t>
         </is>
       </c>
       <c r="M79" s="24" t="inlineStr">
         <is>
-          <t>Albaraka Mobil'den verilen her yeni otomatik fatura ödeme talimatına 200 TL, toplamda 2.000 TL'ye varan Worldpuan</t>
+          <t>TROY kartla LC Waikiki'de tek seferde 3.000 TL üzeri alışverişe anında 300 TL indirim</t>
         </is>
       </c>
       <c r="N79" s="24" t="n"/>
       <c r="O79" s="27" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="P79" s="27" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="Q79" s="24" t="inlineStr">
         <is>
-          <t>Albaraka Mobil'den kampanyaya katılan bireysel müşteriler (World özellikli kart gerekli)</t>
+          <t>Dünya Katılım TROY logolu banka ve kredi kartı sahipleri (sanal kartlar dahil)</t>
         </is>
       </c>
       <c r="R79" s="24" t="n"/>
@@ -7511,32 +7511,30 @@
       </c>
       <c r="U79" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. DIKKAT - AL-007 ile KARISTIRILMASIN: ikisi de Agustos 2026 fatura kampanyasi ve ikisinin de tavani 2.000 TL Worldpuan, ama AL-007 talimat basina 500 TL veriyor ve yalnizca goruntulu gorusmeyle yeni musteri olanlar icin (OFT2026 kodu); bu kayit talimat basina 200 TL ve mevcut musteriler icin. Ayri sayfalar, ayri kosullar. Insan dogrulamasinda ikisi de acilip bakilmali.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Toplam tavan YOK, her 3.000 TL+ islemde tekrar kazanilir; odul_miktari ISLEM BASINA tutardir. Havalimani/yurtdisi magazalari ve self-servis kasalar haric.</t>
         </is>
       </c>
       <c r="X79" s="2" t="inlineStr">
         <is>
-          <t>odul_miktari: Albaraka Mobil üzerinden kredi kartınız ile vereceğiniz her yeni otomatik fatura ödeme talimatınıza 200 TL, toplamda 2.000 TL'ye varan Worldpuan kazanma fırsatı!
-odul_birimi: Albaraka Mobil üzerinden kredi kartınız ile vereceğiniz her yeni otomatik fatura ödeme talimatınıza 200 TL, toplamda 2.000 TL'ye varan Worldpuan kazanma fırsatı!
-kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihlerinde geçerlidir.
-kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihlerinde geçerlidir.</t>
+          <t>kampanya_baslangic: Kampanya 15 Haziran 2026 saat 00.01 – 15 Temmuz 2026 saat 23.59 arasında geçerlidir.
+kampanya_bitis: Kampanya 15 Haziran 2026 saat 00.01 – 15 Temmuz 2026 saat 23.59 arasında geçerlidir.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="24" t="inlineStr">
         <is>
-          <t>DK-009</t>
+          <t>HF-008</t>
         </is>
       </c>
       <c r="B80" s="24" t="inlineStr">
         <is>
-          <t>Dünya Katılım</t>
+          <t>Hayat Finans</t>
         </is>
       </c>
       <c r="C80" s="24" t="inlineStr">
         <is>
-          <t>LC Waikiki'de 3.000 TL ve Üzeri Alışverişe 300 TL İndirim</t>
+          <t>Hayat Finans'la İşlem Yaptıkça Kazan</t>
         </is>
       </c>
       <c r="D80" s="24" t="inlineStr">
@@ -7546,7 +7544,7 @@
       </c>
       <c r="E80" s="24" t="inlineStr">
         <is>
-          <t>www.dunyakatilim.com.tr/kampanyalar/lc-waikiki</t>
+          <t>hayatfinans.com.tr/kampanyalar/hayatfinansla-islem-yaptikca-kazan</t>
         </is>
       </c>
       <c r="F80" s="25" t="n"/>
@@ -7554,33 +7552,27 @@
       <c r="H80" s="24" t="n"/>
       <c r="I80" s="26" t="n"/>
       <c r="J80" s="25" t="n"/>
-      <c r="K80" s="25" t="n">
-        <v>300</v>
-      </c>
-      <c r="L80" s="24" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
+      <c r="K80" s="25" t="n"/>
+      <c r="L80" s="24" t="n"/>
       <c r="M80" s="24" t="inlineStr">
         <is>
-          <t>TROY kartla LC Waikiki'de tek seferde 3.000 TL üzeri alışverişe anında 300 TL indirim</t>
+          <t>Para transferi, banka kartı harcaması, fatura ödeme, döviz işlemi ve Biz Kart başvurusundan Hayat Pay cüzdanına nakit ödül</t>
         </is>
       </c>
       <c r="N80" s="24" t="n"/>
       <c r="O80" s="27" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="P80" s="27" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q80" s="24" t="inlineStr">
         <is>
-          <t>Dünya Katılım TROY logolu banka ve kredi kartı sahipleri (sanal kartlar dahil)</t>
+          <t>Hayat Finans müşterileri</t>
         </is>
       </c>
       <c r="R80" s="24" t="n"/>
@@ -7592,30 +7584,30 @@
       </c>
       <c r="U80" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Toplam tavan YOK, her 3.000 TL+ islemde tekrar kazanilir; odul_miktari ISLEM BASINA tutardir. Havalimani/yurtdisi magazalari ve self-servis kasalar haric.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: kampanyanin tek bir odul tutari yok. Bes ayri islem turunun ayri tavanlari var (transfer ayda 100 TL, doviz ayda 200 TL, banka karti ayda 100 TL, fatura basina 20-30 TL, ilk otomatik odemeye 100 TL) ve toplam tavan sayfada verilmiyor. Motorun buradan tek bir sayi cekip cekmedigini olcen zor ornek.</t>
         </is>
       </c>
       <c r="X80" s="2" t="inlineStr">
         <is>
-          <t>kampanya_baslangic: Kampanya 15 Haziran 2026 saat 00.01 – 15 Temmuz 2026 saat 23.59 arasında geçerlidir.
-kampanya_bitis: Kampanya 15 Haziran 2026 saat 00.01 – 15 Temmuz 2026 saat 23.59 arasında geçerlidir.</t>
+          <t>kampanya_baslangic: 2 Temmuz - 31 Aralık 2026
+kampanya_bitis: 2 Temmuz - 31 Aralık 2026</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="24" t="inlineStr">
         <is>
-          <t>HF-008</t>
+          <t>KT-010</t>
         </is>
       </c>
       <c r="B81" s="24" t="inlineStr">
         <is>
-          <t>Hayat Finans</t>
+          <t>Kuveyt Türk</t>
         </is>
       </c>
       <c r="C81" s="24" t="inlineStr">
         <is>
-          <t>Hayat Finans'la İşlem Yaptıkça Kazan</t>
+          <t>Gelir Vergisi Ödemelerinizde 3 Taksit Fırsatı</t>
         </is>
       </c>
       <c r="D81" s="24" t="inlineStr">
@@ -7625,35 +7617,37 @@
       </c>
       <c r="E81" s="24" t="inlineStr">
         <is>
-          <t>hayatfinans.com.tr/kampanyalar/hayatfinansla-islem-yaptikca-kazan</t>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/gelir-vergisi-odemelerinizde-3-taksit-firsati</t>
         </is>
       </c>
       <c r="F81" s="25" t="n"/>
       <c r="G81" s="25" t="n"/>
       <c r="H81" s="24" t="n"/>
       <c r="I81" s="26" t="n"/>
-      <c r="J81" s="25" t="n"/>
+      <c r="J81" s="25" t="n">
+        <v>300000</v>
+      </c>
       <c r="K81" s="25" t="n"/>
       <c r="L81" s="24" t="n"/>
       <c r="M81" s="24" t="inlineStr">
         <is>
-          <t>Para transferi, banka kartı harcaması, fatura ödeme, döviz işlemi ve Biz Kart başvurusundan Hayat Pay cüzdanına nakit ödül</t>
+          <t>SMS/mobil katılım sonrası 1.000-300.000 TL arası gelir vergisi ödemelerine vade farksız 3 taksit</t>
         </is>
       </c>
       <c r="N81" s="24" t="n"/>
       <c r="O81" s="27" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="P81" s="27" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="Q81" s="24" t="inlineStr">
         <is>
-          <t>Hayat Finans müşterileri</t>
+          <t>Sağlam Kart, Miles&amp;Smiles ve Özel Bankacılık World Elite kredi kartı sahipleri</t>
         </is>
       </c>
       <c r="R81" s="24" t="n"/>
@@ -7665,30 +7659,35 @@
       </c>
       <c r="U81" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: kampanyanin tek bir odul tutari yok. Bes ayri islem turunun ayri tavanlari var (transfer ayda 100 TL, doviz ayda 200 TL, banka karti ayda 100 TL, fatura basina 20-30 TL, ilk otomatik odemeye 100 TL) ve toplam tavan sayfada verilmiyor. Motorun buradan tek bir sayi cekip cekmedigini olcen zor ornek.</t>
-        </is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Musteri basina en fazla 2 islem; kampanya 75.000 kisi ile sinirli. Katilim ONAY VERGI SMS'i ile.</t>
+        </is>
+      </c>
+      <c r="V81" t="n">
+        <v>3</v>
       </c>
       <c r="X81" s="2" t="inlineStr">
         <is>
-          <t>kampanya_baslangic: 2 Temmuz - 31 Aralık 2026
-kampanya_bitis: 2 Temmuz - 31 Aralık 2026</t>
+          <t>taksit_sayisi: 1.000 TL - 300.000 TL arasındaki gelir vergisi ödemelerine vade farksız 3 taksit uygulanır.
+finansman_tutari: 1.000 TL - 300.000 TL arasındaki gelir vergisi ödemelerine vade farksız 3 taksit uygulanır.
+kampanya_baslangic: 1.07.2026 - 31.07.2026
+kampanya_bitis: 1.07.2026 - 31.07.2026</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="24" t="inlineStr">
         <is>
-          <t>KT-010</t>
+          <t>TEK-009</t>
         </is>
       </c>
       <c r="B82" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk</t>
+          <t>Türkiye Emlak Katılım</t>
         </is>
       </c>
       <c r="C82" s="24" t="inlineStr">
         <is>
-          <t>Gelir Vergisi Ödemelerinizde 3 Taksit Fırsatı</t>
+          <t>Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye Varan ParafPara</t>
         </is>
       </c>
       <c r="D82" s="24" t="inlineStr">
@@ -7698,21 +7697,25 @@
       </c>
       <c r="E82" s="24" t="inlineStr">
         <is>
-          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/gelir-vergisi-odemelerinizde-3-taksit-firsati</t>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/beyaz-esya-ve-elektronik-alisverislerinize-3000-tlye-varan-parafpara</t>
         </is>
       </c>
       <c r="F82" s="25" t="n"/>
       <c r="G82" s="25" t="n"/>
       <c r="H82" s="24" t="n"/>
       <c r="I82" s="26" t="n"/>
-      <c r="J82" s="25" t="n">
-        <v>300000</v>
-      </c>
-      <c r="K82" s="25" t="n"/>
-      <c r="L82" s="24" t="n"/>
+      <c r="J82" s="25" t="n"/>
+      <c r="K82" s="25" t="n">
+        <v>3000</v>
+      </c>
+      <c r="L82" s="24" t="inlineStr">
+        <is>
+          <t>ParafPara</t>
+        </is>
+      </c>
       <c r="M82" s="24" t="inlineStr">
         <is>
-          <t>SMS/mobil katılım sonrası 1.000-300.000 TL arası gelir vergisi ödemelerine vade farksız 3 taksit</t>
+          <t>SMS ile katılıp beyaz eşya/elektronik/bilgisayar harcamasına tutara göre 300-3.000 TL ParafPara</t>
         </is>
       </c>
       <c r="N82" s="24" t="n"/>
@@ -7728,7 +7731,7 @@
       </c>
       <c r="Q82" s="24" t="inlineStr">
         <is>
-          <t>Sağlam Kart, Miles&amp;Smiles ve Özel Bankacılık World Elite kredi kartı sahipleri</t>
+          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
         </is>
       </c>
       <c r="R82" s="24" t="n"/>
@@ -7740,35 +7743,32 @@
       </c>
       <c r="U82" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Musteri basina en fazla 2 islem; kampanya 75.000 kisi ile sinirli. Katilim ONAY VERGI SMS'i ile.</t>
-        </is>
-      </c>
-      <c r="V82" t="n">
-        <v>3</v>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Dort kademeli odul; musteri yalnizca BIRINI kazanir, odul_miktari en yuksek kademedir. Pazar yeri e-ticaret haric.</t>
+        </is>
       </c>
       <c r="X82" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: 1.000 TL - 300.000 TL arasındaki gelir vergisi ödemelerine vade farksız 3 taksit uygulanır.
-finansman_tutari: 1.000 TL - 300.000 TL arasındaki gelir vergisi ödemelerine vade farksız 3 taksit uygulanır.
-kampanya_baslangic: 1.07.2026 - 31.07.2026
-kampanya_bitis: 1.07.2026 - 31.07.2026</t>
+          <t>odul_miktari: Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye varan ParafPara!
+odul_birimi: Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye varan ParafPara!
+kampanya_baslangic: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="24" t="inlineStr">
         <is>
-          <t>TEK-009</t>
+          <t>ZK-011</t>
         </is>
       </c>
       <c r="B83" s="24" t="inlineStr">
         <is>
-          <t>Türkiye Emlak Katılım</t>
+          <t>Ziraat Katılım</t>
         </is>
       </c>
       <c r="C83" s="24" t="inlineStr">
         <is>
-          <t>Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye Varan ParafPara</t>
+          <t>Aile Kart'a Özel 2.000 TL'ye Varan Bankkart Lira</t>
         </is>
       </c>
       <c r="D83" s="24" t="inlineStr">
@@ -7778,7 +7778,7 @@
       </c>
       <c r="E83" s="24" t="inlineStr">
         <is>
-          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/beyaz-esya-ve-elektronik-alisverislerinize-3000-tlye-varan-parafpara</t>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/aile-karta-ozel-2000-tlye-varan-bankkart-lira-1</t>
         </is>
       </c>
       <c r="F83" s="25" t="n"/>
@@ -7787,32 +7787,32 @@
       <c r="I83" s="26" t="n"/>
       <c r="J83" s="25" t="n"/>
       <c r="K83" s="25" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="L83" s="24" t="inlineStr">
         <is>
-          <t>ParafPara</t>
+          <t>Bankkart Lira</t>
         </is>
       </c>
       <c r="M83" s="24" t="inlineStr">
         <is>
-          <t>SMS ile katılıp beyaz eşya/elektronik/bilgisayar harcamasına tutara göre 300-3.000 TL ParafPara</t>
+          <t>Aile kredi kartıyla market/akaryakıt/giyim/eğitim/sağlık harcamalarına %5-%10 Bankkart Lira, en fazla 2.000 TL</t>
         </is>
       </c>
       <c r="N83" s="24" t="n"/>
       <c r="O83" s="27" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="P83" s="27" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="Q83" s="24" t="inlineStr">
         <is>
-          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+          <t>Ziraat Katılım Bankkart Aile kredi kartı sahibi asıl kart sahipleri</t>
         </is>
       </c>
       <c r="R83" s="24" t="n"/>
@@ -7824,32 +7824,31 @@
       </c>
       <c r="U83" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Dort kademeli odul; musteri yalnizca BIRINI kazanir, odul_miktari en yuksek kademedir. Pazar yeri e-ticaret haric.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %5 ve %10 NAKIT IADE oranidir, kar payi orani degil. Bireysel/ticari/ucretsiz kartlar haric.</t>
         </is>
       </c>
       <c r="X83" s="2" t="inlineStr">
         <is>
-          <t>odul_miktari: Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye varan ParafPara!
-odul_birimi: Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye varan ParafPara!
-kampanya_baslangic: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.</t>
+          <t>odul_miktari: en fazla 2.000 TL
+kampanya_baslangic: 10 Temmuz– 7 Ağustos 2026
+kampanya_bitis: 10 Temmuz– 7 Ağustos 2026</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="24" t="inlineStr">
         <is>
-          <t>ZK-011</t>
+          <t>KT-011</t>
         </is>
       </c>
       <c r="B84" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım</t>
+          <t>Kuveyt Türk</t>
         </is>
       </c>
       <c r="C84" s="24" t="inlineStr">
         <is>
-          <t>Aile Kart'a Özel 2.000 TL'ye Varan Bankkart Lira</t>
+          <t>Kuveyt Türk ile Yurt Dışı Seyahatlerinde Ayrıcalıklar</t>
         </is>
       </c>
       <c r="D84" s="24" t="inlineStr">
@@ -7859,7 +7858,7 @@
       </c>
       <c r="E84" s="24" t="inlineStr">
         <is>
-          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/aile-karta-ozel-2000-tlye-varan-bankkart-lira-1</t>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/seyahat-kampanyalari/kuveyt-turk-ile-yurt-disi-seyahatlerinde-ayricaliklar-sizinle</t>
         </is>
       </c>
       <c r="F84" s="25" t="n"/>
@@ -7867,33 +7866,27 @@
       <c r="H84" s="24" t="n"/>
       <c r="I84" s="26" t="n"/>
       <c r="J84" s="25" t="n"/>
-      <c r="K84" s="25" t="n">
-        <v>2000</v>
-      </c>
-      <c r="L84" s="24" t="inlineStr">
-        <is>
-          <t>Bankkart Lira</t>
-        </is>
-      </c>
+      <c r="K84" s="25" t="n"/>
+      <c r="L84" s="24" t="n"/>
       <c r="M84" s="24" t="inlineStr">
         <is>
-          <t>Aile kredi kartıyla market/akaryakıt/giyim/eğitim/sağlık harcamalarına %5-%10 Bankkart Lira, en fazla 2.000 TL</t>
+          <t>PocketSIM eSIM'de 1 GB hediye internet ve %35 indirim kodu, yurt dışı harcamalarda avantajlı döviz marjı</t>
         </is>
       </c>
       <c r="N84" s="24" t="n"/>
       <c r="O84" s="27" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="P84" s="27" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q84" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım Bankkart Aile kredi kartı sahibi asıl kart sahipleri</t>
+          <t>Kuveyt Türk Sağlam Nakit ve Sağlam Kart sahipleri</t>
         </is>
       </c>
       <c r="R84" s="24" t="n"/>
@@ -7905,41 +7898,40 @@
       </c>
       <c r="U84" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %5 ve %10 NAKIT IADE oranidir, kar payi orani degil. Bireysel/ticari/ucretsiz kartlar haric.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: %35 bir PocketSIM INDIRIM KODU oranidir (kar payi degil), 1 GB parasal odul degildir. Motorun %35'i kar_payi_orani sanip sanmadigini olcen kayit.</t>
         </is>
       </c>
       <c r="X84" s="2" t="inlineStr">
         <is>
-          <t>odul_miktari: en fazla 2.000 TL
-kampanya_baslangic: 10 Temmuz– 7 Ağustos 2026
-kampanya_bitis: 10 Temmuz– 7 Ağustos 2026</t>
+          <t>kampanya_baslangic: 2.02.2026 - 31.12.2026
+kampanya_bitis: 2.02.2026 - 31.12.2026</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="24" t="inlineStr">
         <is>
-          <t>HF-009</t>
+          <t>AL-012</t>
         </is>
       </c>
       <c r="B85" s="24" t="inlineStr">
         <is>
-          <t>Hayat Finans</t>
+          <t>Albaraka Türk</t>
         </is>
       </c>
       <c r="C85" s="24" t="inlineStr">
         <is>
-          <t>Xiaomi Ürünlerinde Finansman Avantajı</t>
+          <t>Dijital Müşterilere Özel Pratik Finansman Kart</t>
         </is>
       </c>
       <c r="D85" s="24" t="inlineStr">
         <is>
-          <t>Finansman Kampanyasi</t>
+          <t>Yeni Musteri Kampanyasi</t>
         </is>
       </c>
       <c r="E85" s="24" t="inlineStr">
         <is>
-          <t>hayatfinans.com.tr/kampanyalar/xiaomi-urunlerinde-finansman-avantaji</t>
+          <t>www.albaraka.com.tr/tr/kampanyalar/detay/dijital-musterilere-ozel-pratik-finansman-kart</t>
         </is>
       </c>
       <c r="F85" s="25" t="n"/>
@@ -7953,19 +7945,23 @@
       <c r="L85" s="24" t="n"/>
       <c r="M85" s="24" t="inlineStr">
         <is>
-          <t>Xiaomi fiziksel mağazalarında 3 aya varan taksit; kampanya üst limiti 40.000 TL</t>
+          <t>Görüntülü görüşmeyle ilk kez müşteri olanlara vade farksız 40.000 TL veya özel oranlı Pratik Finansman Kart</t>
         </is>
       </c>
       <c r="N85" s="24" t="n"/>
-      <c r="O85" s="27" t="n"/>
+      <c r="O85" s="27" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
       <c r="P85" s="27" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q85" s="24" t="inlineStr">
         <is>
-          <t>Hayat Finans müşterileri (Bana Bunu Al İş Ortağım)</t>
+          <t>Albaraka Mobil'den görüntülü görüşmeyle ilk kez Albaraka müşterisi olanlar</t>
         </is>
       </c>
       <c r="R85" s="24" t="n"/>
@@ -7977,34 +7973,29 @@
       </c>
       <c r="U85" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Baslangic tarihi sayfada YOK. HF-006 ile ayni urun (Bana Bunu Al Is Ortagim) ama farkli magaza ve farkli ust limit: HF-006 Troy magazalari/80.000 TL, bu kayit Xiaomi/40.000 TL.</t>
-        </is>
-      </c>
-      <c r="V85" t="n">
-        <v>3</v>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: sayfa 'uygun oranli' diyor, sayi vermiyor; oran basvuruda musteriye gore belirleniyor. Pratik Finansman Kart ile ATM'den nakit cekilemiyor.</t>
+        </is>
       </c>
       <c r="X85" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: Hayat Finanslılara özel Xiaomi mağazalarında 3 aya varan taksit fırsatı Bana Bunu Al İş Ortağımda!
-finansman_tutari: Kampanya üst limiti 40.000TL'dir.
-kampanya_bitis: Kampanya 31 Ağustos 2026 tarihine kadar geçerlidir.</t>
+          <t>finansman_tutari: Vade farksız 40.000 TL ve uygun oranlı hoş geldin finansmanı Albaraka'da!</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="24" t="inlineStr">
         <is>
-          <t>KT-011</t>
+          <t>HF-010</t>
         </is>
       </c>
       <c r="B86" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk</t>
+          <t>Hayat Finans</t>
         </is>
       </c>
       <c r="C86" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk ile Yurt Dışı Seyahatlerinde Ayrıcalıklar</t>
+          <t>Biz Kart ile Yemek Harcamalarına 1.000 TL'ye Varan Nakit İade</t>
         </is>
       </c>
       <c r="D86" s="24" t="inlineStr">
@@ -8014,7 +8005,7 @@
       </c>
       <c r="E86" s="24" t="inlineStr">
         <is>
-          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/seyahat-kampanyalari/kuveyt-turk-ile-yurt-disi-seyahatlerinde-ayricaliklar-sizinle</t>
+          <t>hayatfinans.com.tr/kampanyalar/biz-kart-yemek-harcamasi-nakit-iade-kampanyasi</t>
         </is>
       </c>
       <c r="F86" s="25" t="n"/>
@@ -8022,27 +8013,33 @@
       <c r="H86" s="24" t="n"/>
       <c r="I86" s="26" t="n"/>
       <c r="J86" s="25" t="n"/>
-      <c r="K86" s="25" t="n"/>
-      <c r="L86" s="24" t="n"/>
+      <c r="K86" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L86" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
       <c r="M86" s="24" t="inlineStr">
         <is>
-          <t>PocketSIM eSIM'de 1 GB hediye internet ve %35 indirim kodu, yurt dışı harcamalarda avantajlı döviz marjı</t>
+          <t>Biz Kart ile yemek sektörü harcamalarının %10'u nakit iade; günlük en fazla 100 TL, aylık 1.000 TL</t>
         </is>
       </c>
       <c r="N86" s="24" t="n"/>
       <c r="O86" s="27" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-06</t>
         </is>
       </c>
       <c r="P86" s="27" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="Q86" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk Sağlam Nakit ve Sağlam Kart sahipleri</t>
+          <t>Hayat Finans bireysel müşterilerinin yakınlarına verdiği Biz Kart sahipleri</t>
         </is>
       </c>
       <c r="R86" s="24" t="n"/>
@@ -8054,40 +8051,41 @@
       </c>
       <c r="U86" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: %35 bir PocketSIM INDIRIM KODU oranidir (kar payi degil), 1 GB parasal odul degildir. Motorun %35'i kar_payi_orani sanip sanmadigini olcen kayit.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari AYLIK tavandir (gunluk tavan 100 TL). kar_payi_orani BILEREK BOS: %10 nakit iade oranidir.</t>
         </is>
       </c>
       <c r="X86" s="2" t="inlineStr">
         <is>
-          <t>kampanya_baslangic: 2.02.2026 - 31.12.2026
-kampanya_bitis: 2.02.2026 - 31.12.2026</t>
+          <t>odul_miktari: aylık toplamda ise 1.000 TL’ye kadar nakit iade
+kampanya_baslangic: 6 Şubat - 31 Ağustos 2026
+kampanya_bitis: 6 Şubat - 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="24" t="inlineStr">
         <is>
-          <t>AL-012</t>
+          <t>TF-008</t>
         </is>
       </c>
       <c r="B87" s="24" t="inlineStr">
         <is>
-          <t>Albaraka Türk</t>
+          <t>Türkiye Finans</t>
         </is>
       </c>
       <c r="C87" s="24" t="inlineStr">
         <is>
-          <t>Dijital Müşterilere Özel Pratik Finansman Kart</t>
+          <t>Kamu Çalışanlarına Özel İhtiyaç Finansmanı</t>
         </is>
       </c>
       <c r="D87" s="24" t="inlineStr">
         <is>
-          <t>Yeni Musteri Kampanyasi</t>
+          <t>Ihtiyac Finansmani Kampanyasi</t>
         </is>
       </c>
       <c r="E87" s="24" t="inlineStr">
         <is>
-          <t>www.albaraka.com.tr/tr/kampanyalar/detay/dijital-musterilere-ozel-pratik-finansman-kart</t>
+          <t>www.turkiyefinans.com.tr/tr-tr/kampanyalar/Sayfalar/kamu-calisanlarina-ozel-ihtiyac-finansmani.aspx</t>
         </is>
       </c>
       <c r="F87" s="25" t="n"/>
@@ -8095,29 +8093,21 @@
       <c r="H87" s="24" t="n"/>
       <c r="I87" s="26" t="n"/>
       <c r="J87" s="25" t="n">
-        <v>40000</v>
+        <v>400000</v>
       </c>
       <c r="K87" s="25" t="n"/>
       <c r="L87" s="24" t="n"/>
       <c r="M87" s="24" t="inlineStr">
         <is>
-          <t>Görüntülü görüşmeyle ilk kez müşteri olanlara vade farksız 40.000 TL veya özel oranlı Pratik Finansman Kart</t>
+          <t>Kamu çalışanlarına 50.000-400.000 TL arası ihtiyaç finansmanı, kişiye özel kâr payı oranı ve 3 ay ödeme öteleme</t>
         </is>
       </c>
       <c r="N87" s="24" t="n"/>
-      <c r="O87" s="27" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="P87" s="27" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
+      <c r="O87" s="27" t="n"/>
+      <c r="P87" s="27" t="n"/>
       <c r="Q87" s="24" t="inlineStr">
         <is>
-          <t>Albaraka Mobil'den görüntülü görüşmeyle ilk kez Albaraka müşterisi olanlar</t>
+          <t>Kamu çalışanları</t>
         </is>
       </c>
       <c r="R87" s="24" t="n"/>
@@ -8129,39 +8119,43 @@
       </c>
       <c r="U87" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: sayfa 'uygun oranli' diyor, sayi vermiyor; oran basvuruda musteriye gore belirleniyor. Pratik Finansman Kart ile ATM'den nakit cekilemiyor.</t>
-        </is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: 'size ozel kar payi oranlari' deniyor ama SAYI verilmiyor. Kampanya tarihi de sayfada YOK. erteleme_suresi_ay dolu olan ilk altin kayit - o sutun su an OLCUM DISI (excel_to_json INCELENMIS_ALANLAR'a bak).</t>
+        </is>
+      </c>
+      <c r="W87" t="n">
+        <v>3</v>
       </c>
       <c r="X87" s="2" t="inlineStr">
         <is>
-          <t>finansman_tutari: Vade farksız 40.000 TL ve uygun oranlı hoş geldin finansmanı Albaraka'da!</t>
+          <t>finansman_tutari: Kampanya kapsamında 50.000 TL – 400.000 TL arasındaki ihtiyaçlarını için finansman başvurusu yapabilirsiniz.
+erteleme_suresi_ay: Finansman geri ödemelerinizde ilk taksiniz için 3 ay öteleme hakkınızı kullanabilir</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="24" t="inlineStr">
         <is>
-          <t>HF-010</t>
+          <t>KT-012</t>
         </is>
       </c>
       <c r="B88" s="24" t="inlineStr">
         <is>
-          <t>Hayat Finans</t>
+          <t>Kuveyt Türk</t>
         </is>
       </c>
       <c r="C88" s="24" t="inlineStr">
         <is>
-          <t>Biz Kart ile Yemek Harcamalarına 1.000 TL'ye Varan Nakit İade</t>
+          <t>Kuveyt Türk Kampüs'e Gelenlere Toplamda 13.500 TL Hediye</t>
         </is>
       </c>
       <c r="D88" s="24" t="inlineStr">
         <is>
-          <t>Kart Kampanyasi</t>
+          <t>Yeni Musteri Kampanyasi</t>
         </is>
       </c>
       <c r="E88" s="24" t="inlineStr">
         <is>
-          <t>hayatfinans.com.tr/kampanyalar/biz-kart-yemek-harcamasi-nakit-iade-kampanyasi</t>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/kuveyt-turk-kampuse-gelenlere-toplamda-13500-tl-hediye</t>
         </is>
       </c>
       <c r="F88" s="25" t="n"/>
@@ -8170,7 +8164,7 @@
       <c r="I88" s="26" t="n"/>
       <c r="J88" s="25" t="n"/>
       <c r="K88" s="25" t="n">
-        <v>1000</v>
+        <v>13500</v>
       </c>
       <c r="L88" s="24" t="inlineStr">
         <is>
@@ -8179,23 +8173,23 @@
       </c>
       <c r="M88" s="24" t="inlineStr">
         <is>
-          <t>Biz Kart ile yemek sektörü harcamalarının %10'u nakit iade; günlük en fazla 100 TL, aylık 1.000 TL</t>
+          <t>Kampüs'e katılanlara davet kodu, kart harcamaları ve ilk e-ticaret harcamasından toplamda 13.500 TL hediye</t>
         </is>
       </c>
       <c r="N88" s="24" t="n"/>
       <c r="O88" s="27" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2025-06-23</t>
         </is>
       </c>
       <c r="P88" s="27" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q88" s="24" t="inlineStr">
         <is>
-          <t>Hayat Finans bireysel müşterilerinin yakınlarına verdiği Biz Kart sahipleri</t>
+          <t>Kuveyt Türk Mobil'den müşteri olan kampüslü (öğrenci) müşteriler</t>
         </is>
       </c>
       <c r="R88" s="24" t="n"/>
@@ -8207,63 +8201,69 @@
       </c>
       <c r="U88" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari AYLIK tavandir (gunluk tavan 100 TL). kar_payi_orani BILEREK BOS: %10 nakit iade oranidir.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. SEMSIYE SAYFA: alt kampanyalarin toplamini duyuruyor (davet 10.500 + hos geldin 500 + kart harcamasi 1.500 + yurt disi cikis harci). odul_miktari basliktaki TOPLAMDIR. Katilim 30.000 kisi ile sinirli.</t>
         </is>
       </c>
       <c r="X88" s="2" t="inlineStr">
         <is>
-          <t>odul_miktari: aylık toplamda ise 1.000 TL’ye kadar nakit iade
-kampanya_baslangic: 6 Şubat - 31 Ağustos 2026
-kampanya_bitis: 6 Şubat - 31 Ağustos 2026</t>
+          <t>odul_miktari: Kuveyt Türk Kampüs'e katılanlar davet kodu, kart harcamaları ve ilk E-Ticaret harcaması kampanyalarından toplamda 13.500 TL Hediye!
+kampanya_baslangic: 23.06.2025 - 31.12.2026
+kampanya_bitis: 23.06.2025 - 31.12.2026</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="24" t="inlineStr">
         <is>
-          <t>TF-008</t>
+          <t>KT-013</t>
         </is>
       </c>
       <c r="B89" s="24" t="inlineStr">
         <is>
-          <t>Türkiye Finans</t>
+          <t>Kuveyt Türk</t>
         </is>
       </c>
       <c r="C89" s="24" t="inlineStr">
         <is>
-          <t>Kamu Çalışanlarına Özel İhtiyaç Finansmanı</t>
+          <t>Kuveyt Türk Mobil'den Müşterimiz Olun Özel Kur Fırsatı</t>
         </is>
       </c>
       <c r="D89" s="24" t="inlineStr">
         <is>
-          <t>Ihtiyac Finansmani Kampanyasi</t>
+          <t>Yatirim Urunu Kampanyasi</t>
         </is>
       </c>
       <c r="E89" s="24" t="inlineStr">
         <is>
-          <t>www.turkiyefinans.com.tr/tr-tr/kampanyalar/Sayfalar/kamu-calisanlarina-ozel-ihtiyac-finansmani.aspx</t>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/kuveyt-turk-mobilden-musterimiz-olun-ozel-kur-firsatini-kacirmayin</t>
         </is>
       </c>
       <c r="F89" s="25" t="n"/>
       <c r="G89" s="25" t="n"/>
       <c r="H89" s="24" t="n"/>
       <c r="I89" s="26" t="n"/>
-      <c r="J89" s="25" t="n">
-        <v>400000</v>
-      </c>
+      <c r="J89" s="25" t="n"/>
       <c r="K89" s="25" t="n"/>
       <c r="L89" s="24" t="n"/>
       <c r="M89" s="24" t="inlineStr">
         <is>
-          <t>Kamu çalışanlarına 50.000-400.000 TL arası ihtiyaç finansmanı, kişiye özel kâr payı oranı ve 3 ay ödeme öteleme</t>
+          <t>Mobilden müşteri olan bireysel müşterilere döviz ve kıymetli maden işlemlerinde özel kur</t>
         </is>
       </c>
       <c r="N89" s="24" t="n"/>
-      <c r="O89" s="27" t="n"/>
-      <c r="P89" s="27" t="n"/>
+      <c r="O89" s="27" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="P89" s="27" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
       <c r="Q89" s="24" t="inlineStr">
         <is>
-          <t>Kamu çalışanları</t>
+          <t>Kuveyt Türk Mobil'den müşteri olan bireysel müşteriler</t>
         </is>
       </c>
       <c r="R89" s="24" t="n"/>
@@ -8275,43 +8275,40 @@
       </c>
       <c r="U89" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: 'size ozel kar payi oranlari' deniyor ama SAYI verilmiyor. Kampanya tarihi de sayfada YOK. erteleme_suresi_ay dolu olan ilk altin kayit - o sutun su an OLCUM DISI (excel_to_json INCELENMIS_ALANLAR'a bak).</t>
-        </is>
-      </c>
-      <c r="W89" t="n">
-        <v>3</v>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfa 'avantajli kur' ve 'ozel oranlar' diyor, tek bir sayi vermiyor. Kurlar mobil uygulamada musteriye ozel tanimlaniyor.</t>
+        </is>
       </c>
       <c r="X89" s="2" t="inlineStr">
         <is>
-          <t>finansman_tutari: Kampanya kapsamında 50.000 TL – 400.000 TL arasındaki ihtiyaçlarını için finansman başvurusu yapabilirsiniz.
-erteleme_suresi_ay: Finansman geri ödemelerinizde ilk taksiniz için 3 ay öteleme hakkınızı kullanabilir</t>
+          <t>kampanya_baslangic: 15.05.2026 - 1.09.2026
+kampanya_bitis: 15.05.2026 - 1.09.2026</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="24" t="inlineStr">
         <is>
-          <t>KT-012</t>
+          <t>TEK-010</t>
         </is>
       </c>
       <c r="B90" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk</t>
+          <t>Türkiye Emlak Katılım</t>
         </is>
       </c>
       <c r="C90" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk Kampüs'e Gelenlere Toplamda 13.500 TL Hediye</t>
+          <t>Biletinial'da %20 İndirim</t>
         </is>
       </c>
       <c r="D90" s="24" t="inlineStr">
         <is>
-          <t>Yeni Musteri Kampanyasi</t>
+          <t>Kart Kampanyasi</t>
         </is>
       </c>
       <c r="E90" s="24" t="inlineStr">
         <is>
-          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/kuveyt-turk-kampuse-gelenlere-toplamda-13500-tl-hediye</t>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/biletinialda-20-indirim</t>
         </is>
       </c>
       <c r="F90" s="25" t="n"/>
@@ -8319,25 +8316,15 @@
       <c r="H90" s="24" t="n"/>
       <c r="I90" s="26" t="n"/>
       <c r="J90" s="25" t="n"/>
-      <c r="K90" s="25" t="n">
-        <v>13500</v>
-      </c>
-      <c r="L90" s="24" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
+      <c r="K90" s="25" t="n"/>
+      <c r="L90" s="24" t="n"/>
       <c r="M90" s="24" t="inlineStr">
         <is>
-          <t>Kampüs'e katılanlara davet kodu, kart harcamaları ve ilk e-ticaret harcamasından toplamda 13.500 TL hediye</t>
+          <t>emlak20 kupon koduyla Biletinial etkinlik biletlerinde %20 indirim</t>
         </is>
       </c>
       <c r="N90" s="24" t="n"/>
-      <c r="O90" s="27" t="inlineStr">
-        <is>
-          <t>2025-06-23</t>
-        </is>
-      </c>
+      <c r="O90" s="27" t="n"/>
       <c r="P90" s="27" t="inlineStr">
         <is>
           <t>2026-12-31</t>
@@ -8345,7 +8332,7 @@
       </c>
       <c r="Q90" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk Mobil'den müşteri olan kampüslü (öğrenci) müşteriler</t>
+          <t>Emlak Katılım Paraf, Paraf Premium ve Debit kart sahipleri</t>
         </is>
       </c>
       <c r="R90" s="24" t="n"/>
@@ -8357,21 +8344,19 @@
       </c>
       <c r="U90" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. SEMSIYE SAYFA: alt kampanyalarin toplamini duyuruyor (davet 10.500 + hos geldin 500 + kart harcamasi 1.500 + yurt disi cikis harci). odul_miktari basliktaki TOPLAMDIR. Katilim 30.000 kisi ile sinirli.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: indirim yalnizca YUZDE olarak veriliyor, TL tavani yok. kar_payi_orani da bos: %20 kupon indirimidir. Sepete en fazla 9 bilet. Baslangic tarihi yok.</t>
         </is>
       </c>
       <c r="X90" s="2" t="inlineStr">
         <is>
-          <t>odul_miktari: Kuveyt Türk Kampüs'e katılanlar davet kodu, kart harcamaları ve ilk E-Ticaret harcaması kampanyalarından toplamda 13.500 TL Hediye!
-kampanya_baslangic: 23.06.2025 - 31.12.2026
-kampanya_bitis: 23.06.2025 - 31.12.2026</t>
+          <t>kampanya_bitis: Kampanya, 31.12.2026 tarihine kadar alınacak etkinlik biletlerinde geçerlidir.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="24" t="inlineStr">
         <is>
-          <t>KT-013</t>
+          <t>KT-014</t>
         </is>
       </c>
       <c r="B91" s="24" t="inlineStr">
@@ -8381,17 +8366,17 @@
       </c>
       <c r="C91" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk Mobil'den Müşterimiz Olun Özel Kur Fırsatı</t>
+          <t>Mobilden Kuveyt Türklü Olanlara Toplamda 7.250 TL Hediye</t>
         </is>
       </c>
       <c r="D91" s="24" t="inlineStr">
         <is>
-          <t>Yatirim Urunu Kampanyasi</t>
+          <t>Yeni Musteri Kampanyasi</t>
         </is>
       </c>
       <c r="E91" s="24" t="inlineStr">
         <is>
-          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/kuveyt-turk-mobilden-musterimiz-olun-ozel-kur-firsatini-kacirmayin</t>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/mobilden-kuveyt-turklu-olanlara-toplamda-7250-tl-hediye</t>
         </is>
       </c>
       <c r="F91" s="25" t="n"/>
@@ -8399,27 +8384,33 @@
       <c r="H91" s="24" t="n"/>
       <c r="I91" s="26" t="n"/>
       <c r="J91" s="25" t="n"/>
-      <c r="K91" s="25" t="n"/>
-      <c r="L91" s="24" t="n"/>
+      <c r="K91" s="25" t="n">
+        <v>7250</v>
+      </c>
+      <c r="L91" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
       <c r="M91" s="24" t="inlineStr">
         <is>
-          <t>Mobilden müşteri olan bireysel müşterilere döviz ve kıymetli maden işlemlerinde özel kur</t>
+          <t>Mobilden müşteri olanlara kart harcaması, fatura talimatı ve davet kodundan toplamda 7.250 TL</t>
         </is>
       </c>
       <c r="N91" s="24" t="n"/>
       <c r="O91" s="27" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="P91" s="27" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q91" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk Mobil'den müşteri olan bireysel müşteriler</t>
+          <t>Kuveyt Türk Mobil veya Self Nokta'dan müşteri olan bireysel müşteriler</t>
         </is>
       </c>
       <c r="R91" s="24" t="n"/>
@@ -8431,20 +8422,21 @@
       </c>
       <c r="U91" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfa 'avantajli kur' ve 'ozel oranlar' diyor, tek bir sayi vermiyor. Kurlar mobil uygulamada musteriye ozel tanimlaniyor.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. SEMSIYE SAYFA: davet 5.500 + fatura talimati 500 + yurt disi cikis harci iadesi. odul_miktari basliktaki TOPLAMDIR. Kampus surumuyle (13.500 TL) ayni yapida ama farkli kitle ve farkli tutar - metin benzerligi %35, ayri kampanyalar.</t>
         </is>
       </c>
       <c r="X91" s="2" t="inlineStr">
         <is>
-          <t>kampanya_baslangic: 15.05.2026 - 1.09.2026
-kampanya_bitis: 15.05.2026 - 1.09.2026</t>
+          <t>odul_miktari: Mobilden Kuveyt Türklü Olun Toplamda 7.250 TL Kazanın!
+kampanya_baslangic: 1.02.2024 - 31.12.2026
+kampanya_bitis: 1.02.2024 - 31.12.2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="24" t="inlineStr">
         <is>
-          <t>TEK-010</t>
+          <t>TEK-011</t>
         </is>
       </c>
       <c r="B92" s="24" t="inlineStr">
@@ -8454,7 +8446,7 @@
       </c>
       <c r="C92" s="24" t="inlineStr">
         <is>
-          <t>Biletinial'da %20 İndirim</t>
+          <t>Emlak Katılım Paraf'tan tabii Premium Üyeliği Hediye</t>
         </is>
       </c>
       <c r="D92" s="24" t="inlineStr">
@@ -8464,7 +8456,7 @@
       </c>
       <c r="E92" s="24" t="inlineStr">
         <is>
-          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/biletinialda-20-indirim</t>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/emlak-katilim-paraftan-tabii-premium-uyeligi-hediye</t>
         </is>
       </c>
       <c r="F92" s="25" t="n"/>
@@ -8476,19 +8468,23 @@
       <c r="L92" s="24" t="n"/>
       <c r="M92" s="24" t="inlineStr">
         <is>
-          <t>emlak20 kupon koduyla Biletinial etkinlik biletlerinde %20 indirim</t>
+          <t>Paraf kartla yapılan tabii Premium üyelik ödemesinin ilgili ay ücreti karta iade</t>
         </is>
       </c>
       <c r="N92" s="24" t="n"/>
-      <c r="O92" s="27" t="n"/>
+      <c r="O92" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="P92" s="27" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="Q92" s="24" t="inlineStr">
         <is>
-          <t>Emlak Katılım Paraf, Paraf Premium ve Debit kart sahipleri</t>
+          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
         </is>
       </c>
       <c r="R92" s="24" t="n"/>
@@ -8500,39 +8496,40 @@
       </c>
       <c r="U92" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: indirim yalnizca YUZDE olarak veriliyor, TL tavani yok. kar_payi_orani da bos: %20 kupon indirimidir. Sepete en fazla 9 bilet. Baslangic tarihi yok.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: 'ilgili ayin uyelik ucreti kadar iade' deniyor, TUTAR YAZMIYOR. Trendyol Plus kaydiyla (75 TL acikca yazili) karsilastirmali cift olusturur.</t>
         </is>
       </c>
       <c r="X92" s="2" t="inlineStr">
         <is>
-          <t>kampanya_bitis: Kampanya, 31.12.2026 tarihine kadar alınacak etkinlik biletlerinde geçerlidir.</t>
+          <t>kampanya_baslangic: Kampanya 01.07.2026 – 31.07.2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 01.07.2026 – 31.07.2026 tarihleri arasında geçerlidir.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="24" t="inlineStr">
         <is>
-          <t>KT-014</t>
+          <t>ZK-012</t>
         </is>
       </c>
       <c r="B93" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk</t>
+          <t>Ziraat Katılım</t>
         </is>
       </c>
       <c r="C93" s="24" t="inlineStr">
         <is>
-          <t>Mobilden Kuveyt Türklü Olanlara Toplamda 7.250 TL Hediye</t>
+          <t>Alarko Carrier'da 6 Taksit</t>
         </is>
       </c>
       <c r="D93" s="24" t="inlineStr">
         <is>
-          <t>Yeni Musteri Kampanyasi</t>
+          <t>Kart Kampanyasi</t>
         </is>
       </c>
       <c r="E93" s="24" t="inlineStr">
         <is>
-          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/mobilden-kuveyt-turklu-olanlara-toplamda-7250-tl-hediye</t>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/alarko-carrierda-6-taksit</t>
         </is>
       </c>
       <c r="F93" s="25" t="n"/>
@@ -8540,33 +8537,19 @@
       <c r="H93" s="24" t="n"/>
       <c r="I93" s="26" t="n"/>
       <c r="J93" s="25" t="n"/>
-      <c r="K93" s="25" t="n">
-        <v>7250</v>
-      </c>
-      <c r="L93" s="24" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
+      <c r="K93" s="25" t="n"/>
+      <c r="L93" s="24" t="n"/>
       <c r="M93" s="24" t="inlineStr">
         <is>
-          <t>Mobilden müşteri olanlara kart harcaması, fatura talimatı ve davet kodundan toplamda 7.250 TL</t>
+          <t>Bankkart kredi kartıyla Alarko Carrier alışverişlerinde 6 taksit</t>
         </is>
       </c>
       <c r="N93" s="24" t="n"/>
-      <c r="O93" s="27" t="inlineStr">
-        <is>
-          <t>2024-02-01</t>
-        </is>
-      </c>
-      <c r="P93" s="27" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
+      <c r="O93" s="27" t="n"/>
+      <c r="P93" s="27" t="n"/>
       <c r="Q93" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk Mobil veya Self Nokta'dan müşteri olan bireysel müşteriler</t>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
       <c r="R93" s="24" t="n"/>
@@ -8578,31 +8561,32 @@
       </c>
       <c r="U93" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. SEMSIYE SAYFA: davet 5.500 + fatura talimati 500 + yurt disi cikis harci iadesi. odul_miktari basliktaki TOPLAMDIR. Kampus surumuyle (13.500 TL) ayni yapida ama farkli kitle ve farkli tutar - metin benzerligi %35, ayri kampanyalar.</t>
-        </is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V93" t="n">
+        <v>6</v>
       </c>
       <c r="X93" s="2" t="inlineStr">
         <is>
-          <t>odul_miktari: Mobilden Kuveyt Türklü Olun Toplamda 7.250 TL Kazanın!
-kampanya_baslangic: 1.02.2024 - 31.12.2026
-kampanya_bitis: 1.02.2024 - 31.12.2026</t>
+          <t>taksit_sayisi: 6 taksitli</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="24" t="inlineStr">
         <is>
-          <t>TEK-011</t>
+          <t>KT-015</t>
         </is>
       </c>
       <c r="B94" s="24" t="inlineStr">
         <is>
-          <t>Türkiye Emlak Katılım</t>
+          <t>Kuveyt Türk</t>
         </is>
       </c>
       <c r="C94" s="24" t="inlineStr">
         <is>
-          <t>Emlak Katılım Paraf'tan tabii Premium Üyeliği Hediye</t>
+          <t>Sağlam Kart Sahipleri Halalbooking'de de Avantajlı</t>
         </is>
       </c>
       <c r="D94" s="24" t="inlineStr">
@@ -8612,7 +8596,7 @@
       </c>
       <c r="E94" s="24" t="inlineStr">
         <is>
-          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/emlak-katilim-paraftan-tabii-premium-uyeligi-hediye</t>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/saglam-kart-sahipleri-halalbookingde-de-avantajli</t>
         </is>
       </c>
       <c r="F94" s="25" t="n"/>
@@ -8620,27 +8604,33 @@
       <c r="H94" s="24" t="n"/>
       <c r="I94" s="26" t="n"/>
       <c r="J94" s="25" t="n"/>
-      <c r="K94" s="25" t="n"/>
-      <c r="L94" s="24" t="n"/>
+      <c r="K94" s="25" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L94" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
       <c r="M94" s="24" t="inlineStr">
         <is>
-          <t>Paraf kartla yapılan tabii Premium üyelik ödemesinin ilgili ay ücreti karta iade</t>
+          <t>Halalbooking tatil harcamalarında 9 aya varan taksit ve ilk kayıtta 1.000 TL indirim (10.000 TL üzeri rezervasyonda)</t>
         </is>
       </c>
       <c r="N94" s="24" t="n"/>
       <c r="O94" s="27" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2025-07-30</t>
         </is>
       </c>
       <c r="P94" s="27" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q94" s="24" t="inlineStr">
         <is>
-          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+          <t>Kuveyt Türk Sağlam Kart sahipleri</t>
         </is>
       </c>
       <c r="R94" s="24" t="n"/>
@@ -8652,30 +8642,35 @@
       </c>
       <c r="U94" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: 'ilgili ayin uyelik ucreti kadar iade' deniyor, TUTAR YAZMIYOR. Trendyol Plus kaydiyla (75 TL acikca yazili) karsilastirmali cift olusturur.</t>
-        </is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 1.000 TL indirim yalnizca ILK KAYITTA ve 10.000 TL uzeri rezervasyonda gecerli - o tutar bir ESIKTIR, odul degil.</t>
+        </is>
+      </c>
+      <c r="V94" t="n">
+        <v>9</v>
       </c>
       <c r="X94" s="2" t="inlineStr">
         <is>
-          <t>kampanya_baslangic: Kampanya 01.07.2026 – 31.07.2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 01.07.2026 – 31.07.2026 tarihleri arasında geçerlidir.</t>
+          <t>taksit_sayisi: 31 Aralık 2026 tarihine kadar yapacağınız tatil harcamalarınızda 9 aya varan taksit avantajından yararlanabilir, Halalbooking’e kaydolurken 1.000 TL değerinde indirim kazanabilirsiniz.
+odul_miktari: 31 Aralık 2026 tarihine kadar yapacağınız tatil harcamalarınızda 9 aya varan taksit avantajından yararlanabilir, Halalbooking’e kaydolurken 1.000 TL değerinde indirim kazanabilirsiniz.
+kampanya_baslangic: 30.07.2025 - 31.12.2026
+kampanya_bitis: 30.07.2025 - 31.12.2026</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="24" t="inlineStr">
         <is>
-          <t>ZK-012</t>
+          <t>TEK-012</t>
         </is>
       </c>
       <c r="B95" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım</t>
+          <t>Türkiye Emlak Katılım</t>
         </is>
       </c>
       <c r="C95" s="24" t="inlineStr">
         <is>
-          <t>Alarko Carrier'da 6 Taksit</t>
+          <t>Emlak Katılım Paraf'tan Trendyol Plus Üyelik Ücretiniz İade</t>
         </is>
       </c>
       <c r="D95" s="24" t="inlineStr">
@@ -8685,7 +8680,7 @@
       </c>
       <c r="E95" s="24" t="inlineStr">
         <is>
-          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/alarko-carrierda-6-taksit</t>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/emlak-katilim-paraftan-trendyol-plus-uyelik-ucretiniz-iade</t>
         </is>
       </c>
       <c r="F95" s="25" t="n"/>
@@ -8693,19 +8688,33 @@
       <c r="H95" s="24" t="n"/>
       <c r="I95" s="26" t="n"/>
       <c r="J95" s="25" t="n"/>
-      <c r="K95" s="25" t="n"/>
-      <c r="L95" s="24" t="n"/>
+      <c r="K95" s="25" t="n">
+        <v>75</v>
+      </c>
+      <c r="L95" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
       <c r="M95" s="24" t="inlineStr">
         <is>
-          <t>Bankkart kredi kartıyla Alarko Carrier alışverişlerinde 6 taksit</t>
+          <t>Paraf kartla yapılan Trendyol Plus üyelik ödemesindeki 75 TL üyelik ücreti karta iade</t>
         </is>
       </c>
       <c r="N95" s="24" t="n"/>
-      <c r="O95" s="27" t="n"/>
-      <c r="P95" s="27" t="n"/>
+      <c r="O95" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P95" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
       <c r="Q95" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri</t>
         </is>
       </c>
       <c r="R95" s="24" t="n"/>
@@ -8717,32 +8726,31 @@
       </c>
       <c r="U95" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
-        </is>
-      </c>
-      <c r="V95" t="n">
-        <v>6</v>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. tabii Premium kaydiyla ayni yapi ama burada tutar (75 TL) ACIKCA yazili; orada yazmiyor ve o alan bos birakildi.</t>
+        </is>
       </c>
       <c r="X95" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: 6 taksitli</t>
+          <t>odul_miktari: Emlak Katılım Paraf ve Emlak Katılım Paraf Premium kartınız ile 01.07.2026 – 31.07.2026 tarihleri arasında yapacağınız Trendyol Plus üyelik ödemenize ilişkin 75 TL tutarındaki üyelik ücreti kartınıza iade olarak yansıtılacaktır.
+kampanya_baslangic: 01.07.2026 – 31.07.2026
+kampanya_bitis: 01.07.2026 – 31.07.2026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="24" t="inlineStr">
         <is>
-          <t>KT-015</t>
+          <t>ZK-013</t>
         </is>
       </c>
       <c r="B96" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk</t>
+          <t>Ziraat Katılım</t>
         </is>
       </c>
       <c r="C96" s="24" t="inlineStr">
         <is>
-          <t>Sağlam Kart Sahipleri Halalbooking'de de Avantajlı</t>
+          <t>Alfemo'da 5 Taksit</t>
         </is>
       </c>
       <c r="D96" s="24" t="inlineStr">
@@ -8752,7 +8760,7 @@
       </c>
       <c r="E96" s="24" t="inlineStr">
         <is>
-          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/saglam-kart-sahipleri-halalbookingde-de-avantajli</t>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/alfemoda-5-taksit</t>
         </is>
       </c>
       <c r="F96" s="25" t="n"/>
@@ -8760,33 +8768,19 @@
       <c r="H96" s="24" t="n"/>
       <c r="I96" s="26" t="n"/>
       <c r="J96" s="25" t="n"/>
-      <c r="K96" s="25" t="n">
-        <v>1000</v>
-      </c>
-      <c r="L96" s="24" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
+      <c r="K96" s="25" t="n"/>
+      <c r="L96" s="24" t="n"/>
       <c r="M96" s="24" t="inlineStr">
         <is>
-          <t>Halalbooking tatil harcamalarında 9 aya varan taksit ve ilk kayıtta 1.000 TL indirim (10.000 TL üzeri rezervasyonda)</t>
+          <t>Bankkart kredi kartıyla Alfemo alışverişlerinde 5 taksit</t>
         </is>
       </c>
       <c r="N96" s="24" t="n"/>
-      <c r="O96" s="27" t="inlineStr">
-        <is>
-          <t>2025-07-30</t>
-        </is>
-      </c>
-      <c r="P96" s="27" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
+      <c r="O96" s="27" t="n"/>
+      <c r="P96" s="27" t="n"/>
       <c r="Q96" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk Sağlam Kart sahipleri</t>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
       <c r="R96" s="24" t="n"/>
@@ -8798,45 +8792,42 @@
       </c>
       <c r="U96" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 1.000 TL indirim yalnizca ILK KAYITTA ve 10.000 TL uzeri rezervasyonda gecerli - o tutar bir ESIKTIR, odul degil.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
         </is>
       </c>
       <c r="V96" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="X96" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: 31 Aralık 2026 tarihine kadar yapacağınız tatil harcamalarınızda 9 aya varan taksit avantajından yararlanabilir, Halalbooking’e kaydolurken 1.000 TL değerinde indirim kazanabilirsiniz.
-odul_miktari: 31 Aralık 2026 tarihine kadar yapacağınız tatil harcamalarınızda 9 aya varan taksit avantajından yararlanabilir, Halalbooking’e kaydolurken 1.000 TL değerinde indirim kazanabilirsiniz.
-kampanya_baslangic: 30.07.2025 - 31.12.2026
-kampanya_bitis: 30.07.2025 - 31.12.2026</t>
+          <t>taksit_sayisi: 5 taksitli</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="24" t="inlineStr">
         <is>
-          <t>TEK-012</t>
+          <t>KT-016</t>
         </is>
       </c>
       <c r="B97" s="24" t="inlineStr">
         <is>
-          <t>Türkiye Emlak Katılım</t>
+          <t>Kuveyt Türk</t>
         </is>
       </c>
       <c r="C97" s="24" t="inlineStr">
         <is>
-          <t>Emlak Katılım Paraf'tan Trendyol Plus Üyelik Ücretiniz İade</t>
+          <t>Yakınlarını Kuveyt Türk'e Davet Et Toplamda 5.000 TL'ye Varan Hediye Kazan</t>
         </is>
       </c>
       <c r="D97" s="24" t="inlineStr">
         <is>
-          <t>Kart Kampanyasi</t>
+          <t>Yeni Musteri Kampanyasi</t>
         </is>
       </c>
       <c r="E97" s="24" t="inlineStr">
         <is>
-          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/emlak-katilim-paraftan-trendyol-plus-uyelik-ucretiniz-iade</t>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/yakinlarini-kuveyt-turke-davet-et-toplamda-5000-tlye-varan-hediye-kazan</t>
         </is>
       </c>
       <c r="F97" s="25" t="n"/>
@@ -8845,7 +8836,7 @@
       <c r="I97" s="26" t="n"/>
       <c r="J97" s="25" t="n"/>
       <c r="K97" s="25" t="n">
-        <v>75</v>
+        <v>5000</v>
       </c>
       <c r="L97" s="24" t="inlineStr">
         <is>
@@ -8854,23 +8845,23 @@
       </c>
       <c r="M97" s="24" t="inlineStr">
         <is>
-          <t>Paraf kartla yapılan Trendyol Plus üyelik ödemesindeki 75 TL üyelik ücreti karta iade</t>
+          <t>Davet koduyla müşteri olan her yakın için 500 TL, toplamda 5.000 TL'ye kadar; davet edilene de 500 TL harcama iadesi</t>
         </is>
       </c>
       <c r="N97" s="24" t="n"/>
       <c r="O97" s="27" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2025-06-15</t>
         </is>
       </c>
       <c r="P97" s="27" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q97" s="24" t="inlineStr">
         <is>
-          <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri</t>
+          <t>Mevcut Kuveyt Türk müşterileri (davet kodu paylaşanlar)</t>
         </is>
       </c>
       <c r="R97" s="24" t="n"/>
@@ -8882,31 +8873,30 @@
       </c>
       <c r="U97" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. tabii Premium kaydiyla ayni yapi ama burada tutar (75 TL) ACIKCA yazili; orada yazmiyor ve o alan bos birakildi.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari DAVET EDENIN tavanidir (5.000 TL); davet edilen ayrica 500 TL alir. Bu kampanya KT-012 ve KT-014'teki semsiye sayfalarin bir BILESENI - ayri sayfasi oldugu icin ayri kayit.</t>
         </is>
       </c>
       <c r="X97" s="2" t="inlineStr">
         <is>
-          <t>odul_miktari: Emlak Katılım Paraf ve Emlak Katılım Paraf Premium kartınız ile 01.07.2026 – 31.07.2026 tarihleri arasında yapacağınız Trendyol Plus üyelik ödemenize ilişkin 75 TL tutarındaki üyelik ücreti kartınıza iade olarak yansıtılacaktır.
-kampanya_baslangic: 01.07.2026 – 31.07.2026
-kampanya_bitis: 01.07.2026 – 31.07.2026</t>
+          <t>kampanya_baslangic: 15.06.2025 - 31.12.2026
+kampanya_bitis: 15.06.2025 - 31.12.2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="24" t="inlineStr">
         <is>
-          <t>ZK-013</t>
+          <t>TEK-013</t>
         </is>
       </c>
       <c r="B98" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım</t>
+          <t>Türkiye Emlak Katılım</t>
         </is>
       </c>
       <c r="C98" s="24" t="inlineStr">
         <is>
-          <t>Alfemo'da 5 Taksit</t>
+          <t>Enterprise Araç Kiralamalarında %35 İndirim Fırsatı</t>
         </is>
       </c>
       <c r="D98" s="24" t="inlineStr">
@@ -8916,7 +8906,7 @@
       </c>
       <c r="E98" s="24" t="inlineStr">
         <is>
-          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/alfemoda-5-taksit</t>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/enterprise-arac-kiralamalarinda-35-indirim-firsati</t>
         </is>
       </c>
       <c r="F98" s="25" t="n"/>
@@ -8928,15 +8918,19 @@
       <c r="L98" s="24" t="n"/>
       <c r="M98" s="24" t="inlineStr">
         <is>
-          <t>Bankkart kredi kartıyla Alfemo alışverişlerinde 5 taksit</t>
+          <t>Banka iş birliği sayfasından Enterprise online araç kiralamalarında liste fiyatı üzerinden %35 indirim</t>
         </is>
       </c>
       <c r="N98" s="24" t="n"/>
       <c r="O98" s="27" t="n"/>
-      <c r="P98" s="27" t="n"/>
+      <c r="P98" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
       <c r="Q98" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+          <t>Emlak Katılım Paraf kart sahipleri</t>
         </is>
       </c>
       <c r="R98" s="24" t="n"/>
@@ -8948,22 +8942,19 @@
       </c>
       <c r="U98" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
-        </is>
-      </c>
-      <c r="V98" t="n">
-        <v>5</v>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari ve kar_payi_orani BILEREK BOS: %35 bir liste fiyati indirimidir, TL tavani yok. Baslangic tarihi yok.</t>
+        </is>
       </c>
       <c r="X98" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: 5 taksitli</t>
+          <t>kampanya_bitis: Liste fiyatı üzerinden %35 indirim kampanyası 31.12.2026 tarihine kadar Türkiye’deki tüm Enterprise ofislerinde online kiralamalarda geçerlidir.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="24" t="inlineStr">
         <is>
-          <t>KT-016</t>
+          <t>KT-017</t>
         </is>
       </c>
       <c r="B99" s="24" t="inlineStr">
@@ -8973,41 +8964,45 @@
       </c>
       <c r="C99" s="24" t="inlineStr">
         <is>
-          <t>Yakınlarını Kuveyt Türk'e Davet Et Toplamda 5.000 TL'ye Varan Hediye Kazan</t>
+          <t>Yeni Müşterilere Özel İhtiyaç Kart'ta %1,99 Oran Fırsatı</t>
         </is>
       </c>
       <c r="D99" s="24" t="inlineStr">
         <is>
-          <t>Yeni Musteri Kampanyasi</t>
+          <t>Ihtiyac Finansmani Kampanyasi</t>
         </is>
       </c>
       <c r="E99" s="24" t="inlineStr">
         <is>
-          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/yakinlarini-kuveyt-turke-davet-et-toplamda-5000-tlye-varan-hediye-kazan</t>
-        </is>
-      </c>
-      <c r="F99" s="25" t="n"/>
+          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/yeni-musterilere-ozel-ihtiyac-kartta-199-oran-firsati</t>
+        </is>
+      </c>
+      <c r="F99" s="25" t="n">
+        <v>1.99</v>
+      </c>
       <c r="G99" s="25" t="n"/>
-      <c r="H99" s="24" t="n"/>
-      <c r="I99" s="26" t="n"/>
-      <c r="J99" s="25" t="n"/>
-      <c r="K99" s="25" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L99" s="24" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
+      <c r="H99" s="24" t="inlineStr">
+        <is>
+          <t>aylik</t>
+        </is>
+      </c>
+      <c r="I99" s="26" t="n">
+        <v>12</v>
+      </c>
+      <c r="J99" s="25" t="n">
+        <v>100000</v>
+      </c>
+      <c r="K99" s="25" t="n"/>
+      <c r="L99" s="24" t="n"/>
       <c r="M99" s="24" t="inlineStr">
         <is>
-          <t>Davet koduyla müşteri olan her yakın için 500 TL, toplamda 5.000 TL'ye kadar; davet edilene de 500 TL harcama iadesi</t>
+          <t>Görüntülü görüşmeyle yeni müşteri olanlara 100.000 TL'ye kadar %1,99 oranla 12 aya varan, 2 ay ertelemeli İhtiyaç Kart</t>
         </is>
       </c>
       <c r="N99" s="24" t="n"/>
       <c r="O99" s="27" t="inlineStr">
         <is>
-          <t>2025-06-15</t>
+          <t>2025-10-22</t>
         </is>
       </c>
       <c r="P99" s="27" t="inlineStr">
@@ -9017,7 +9012,7 @@
       </c>
       <c r="Q99" s="24" t="inlineStr">
         <is>
-          <t>Mevcut Kuveyt Türk müşterileri (davet kodu paylaşanlar)</t>
+          <t>Kuveyt Türk Mobil'den görüntülü görüşmeyle son 30 gün içinde müşteri olanlar</t>
         </is>
       </c>
       <c r="R99" s="24" t="n"/>
@@ -9029,20 +9024,26 @@
       </c>
       <c r="U99" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari DAVET EDENIN tavanidir (5.000 TL); davet edilen ayrica 500 TL alir. Bu kampanya KT-012 ve KT-014'teki semsiye sayfalarin bir BILESENI - ayri sayfasi oldugu icin ayri kayit.</t>
-        </is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 100.000 TL ustu basvurularda liste fiyati uygulaniyor, yani 100.000 TL kampanyanin TAVANI. oran_periyodu 'aylik': %1,99 yillik olsaydi piyasa disi dusuk olurdu.</t>
+        </is>
+      </c>
+      <c r="W99" t="n">
+        <v>2</v>
       </c>
       <c r="X99" s="2" t="inlineStr">
         <is>
-          <t>kampanya_baslangic: 15.06.2025 - 31.12.2026
-kampanya_bitis: 15.06.2025 - 31.12.2026</t>
+          <t>kar_payi_orani: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
+vade_ay: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
+finansman_tutari: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
+kampanya_baslangic: 22.10.2025 - 31.12.2026
+kampanya_bitis: 22.10.2025 - 31.12.2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="24" t="inlineStr">
         <is>
-          <t>TEK-013</t>
+          <t>TEK-014</t>
         </is>
       </c>
       <c r="B100" s="24" t="inlineStr">
@@ -9052,7 +9053,7 @@
       </c>
       <c r="C100" s="24" t="inlineStr">
         <is>
-          <t>Enterprise Araç Kiralamalarında %35 İndirim Fırsatı</t>
+          <t>Giyim ve Kozmetik Alışverişlerinize 1.300 TL ParafPara</t>
         </is>
       </c>
       <c r="D100" s="24" t="inlineStr">
@@ -9062,7 +9063,7 @@
       </c>
       <c r="E100" s="24" t="inlineStr">
         <is>
-          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/enterprise-arac-kiralamalarinda-35-indirim-firsati</t>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/giyim-ve-kozmetik-alisverislerinize-1300-tl-parafpara</t>
         </is>
       </c>
       <c r="F100" s="25" t="n"/>
@@ -9070,18 +9071,28 @@
       <c r="H100" s="24" t="n"/>
       <c r="I100" s="26" t="n"/>
       <c r="J100" s="25" t="n"/>
-      <c r="K100" s="25" t="n"/>
-      <c r="L100" s="24" t="n"/>
+      <c r="K100" s="25" t="n">
+        <v>1300</v>
+      </c>
+      <c r="L100" s="24" t="inlineStr">
+        <is>
+          <t>ParafPara</t>
+        </is>
+      </c>
       <c r="M100" s="24" t="inlineStr">
         <is>
-          <t>Banka iş birliği sayfasından Enterprise online araç kiralamalarında liste fiyatı üzerinden %35 indirim</t>
+          <t>GIYIM2 SMS katılımıyla giyim/kozmetik harcamasına 500-1.250 TL, mobil/QR ödemede +50 TL, en fazla 1.300 TL ParafPara</t>
         </is>
       </c>
       <c r="N100" s="24" t="n"/>
-      <c r="O100" s="27" t="n"/>
+      <c r="O100" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="P100" s="27" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="Q100" s="24" t="inlineStr">
@@ -9098,77 +9109,61 @@
       </c>
       <c r="U100" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari ve kar_payi_orani BILEREK BOS: %35 bir liste fiyati indirimidir, TL tavani yok. Baslangic tarihi yok.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 1.300 TL = en yuksek barem (1.250) + mobil/QR ekstrasi (50). Uc kademe: 500/800/1.250. AYNI AILEDEN IKI SURUM DAHA VAR (Temmuz 1.000 TL ve Temmuz 2.000 TL) ama metinleri bu kayda %89-92 benzedigi icin etiketlenmedi - ucu birden altin sete girseydi ayni teklif olcumde uc kat agirlik alir, train/test'e dagilirsa sizinti olurdu. Bu surum secildi cunku basliktaki sayi dogrudan bir kademe DEGIL: en yuksek barem (1.250) + mobil/QR ekstrasi (50).</t>
         </is>
       </c>
       <c r="X100" s="2" t="inlineStr">
         <is>
-          <t>kampanya_bitis: Liste fiyatı üzerinden %35 indirim kampanyası 31.12.2026 tarihine kadar Türkiye’deki tüm Enterprise ofislerinde online kiralamalarda geçerlidir.</t>
+          <t>odul_miktari: bir müşteri kampanyaya bir kez katılabilir ve en fazla 1.300 TL ParafPara kazanabilir.
+kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="24" t="inlineStr">
         <is>
-          <t>KT-017</t>
+          <t>ZK-014</t>
         </is>
       </c>
       <c r="B101" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk</t>
+          <t>Ziraat Katılım</t>
         </is>
       </c>
       <c r="C101" s="24" t="inlineStr">
         <is>
-          <t>Yeni Müşterilere Özel İhtiyaç Kart'ta %1,99 Oran Fırsatı</t>
+          <t>Amazon'da 9'a Varan Taksit</t>
         </is>
       </c>
       <c r="D101" s="24" t="inlineStr">
         <is>
-          <t>Ihtiyac Finansmani Kampanyasi</t>
+          <t>Kart Kampanyasi</t>
         </is>
       </c>
       <c r="E101" s="24" t="inlineStr">
         <is>
-          <t>www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/yeni-musterilere-ozel-ihtiyac-kartta-199-oran-firsati</t>
-        </is>
-      </c>
-      <c r="F101" s="25" t="n">
-        <v>1.99</v>
-      </c>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/amazonda-9a-varan-taksit</t>
+        </is>
+      </c>
+      <c r="F101" s="25" t="n"/>
       <c r="G101" s="25" t="n"/>
-      <c r="H101" s="24" t="inlineStr">
-        <is>
-          <t>aylik</t>
-        </is>
-      </c>
-      <c r="I101" s="26" t="n">
-        <v>12</v>
-      </c>
-      <c r="J101" s="25" t="n">
-        <v>100000</v>
-      </c>
+      <c r="H101" s="24" t="n"/>
+      <c r="I101" s="26" t="n"/>
+      <c r="J101" s="25" t="n"/>
       <c r="K101" s="25" t="n"/>
       <c r="L101" s="24" t="n"/>
       <c r="M101" s="24" t="inlineStr">
         <is>
-          <t>Görüntülü görüşmeyle yeni müşteri olanlara 100.000 TL'ye kadar %1,99 oranla 12 aya varan, 2 ay ertelemeli İhtiyaç Kart</t>
+          <t>Bankkart kredi kartıyla amazon.com.tr'de tutara göre peşin fiyatına 3, 6 veya 9 taksit</t>
         </is>
       </c>
       <c r="N101" s="24" t="n"/>
-      <c r="O101" s="27" t="inlineStr">
-        <is>
-          <t>2025-10-22</t>
-        </is>
-      </c>
-      <c r="P101" s="27" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
+      <c r="O101" s="27" t="n"/>
+      <c r="P101" s="27" t="n"/>
       <c r="Q101" s="24" t="inlineStr">
         <is>
-          <t>Kuveyt Türk Mobil'den görüntülü görüşmeyle son 30 gün içinde müşteri olanlar</t>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
       <c r="R101" s="24" t="n"/>
@@ -9180,36 +9175,32 @@
       </c>
       <c r="U101" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 100.000 TL ustu basvurularda liste fiyati uygulaniyor, yani 100.000 TL kampanyanin TAVANI. oran_periyodu 'aylik': %1,99 yillik olsaydi piyasa disi dusuk olurdu.</t>
-        </is>
-      </c>
-      <c r="W101" t="n">
-        <v>2</v>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Uc kademe (3/6/9); 9 taksit yalnizca SECILI URUNLERDE ve 10.000 TL uzeri. Kampanya tarihi sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V101" t="n">
+        <v>9</v>
       </c>
       <c r="X101" s="2" t="inlineStr">
         <is>
-          <t>kar_payi_orani: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
-vade_ay: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
-finansman_tutari: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
-kampanya_baslangic: 22.10.2025 - 31.12.2026
-kampanya_bitis: 22.10.2025 - 31.12.2026</t>
+          <t>taksit_sayisi: Seçili ürünlerde yapacağınız 10.000 TL ve üzeri alışverişlerinizde peşin fiyatına 9 taksit fırsatından faydalanabilirsiniz.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="24" t="inlineStr">
         <is>
-          <t>TEK-014</t>
+          <t>ZK-015</t>
         </is>
       </c>
       <c r="B102" s="24" t="inlineStr">
         <is>
-          <t>Türkiye Emlak Katılım</t>
+          <t>Ziraat Katılım</t>
         </is>
       </c>
       <c r="C102" s="24" t="inlineStr">
         <is>
-          <t>Giyim ve Kozmetik Alışverişlerinize 1.300 TL ParafPara</t>
+          <t>Atasun Optik'te 6 Taksit</t>
         </is>
       </c>
       <c r="D102" s="24" t="inlineStr">
@@ -9219,7 +9210,7 @@
       </c>
       <c r="E102" s="24" t="inlineStr">
         <is>
-          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/giyim-ve-kozmetik-alisverislerinize-1300-tl-parafpara</t>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/atasun-optikte-6-taksit</t>
         </is>
       </c>
       <c r="F102" s="25" t="n"/>
@@ -9227,33 +9218,19 @@
       <c r="H102" s="24" t="n"/>
       <c r="I102" s="26" t="n"/>
       <c r="J102" s="25" t="n"/>
-      <c r="K102" s="25" t="n">
-        <v>1300</v>
-      </c>
-      <c r="L102" s="24" t="inlineStr">
-        <is>
-          <t>ParafPara</t>
-        </is>
-      </c>
+      <c r="K102" s="25" t="n"/>
+      <c r="L102" s="24" t="n"/>
       <c r="M102" s="24" t="inlineStr">
         <is>
-          <t>GIYIM2 SMS katılımıyla giyim/kozmetik harcamasına 500-1.250 TL, mobil/QR ödemede +50 TL, en fazla 1.300 TL ParafPara</t>
+          <t>Bankkart kredi kartıyla Atasun Optik'te 4.000 TL üzeri işlemlerde peşin fiyatına 6 taksit</t>
         </is>
       </c>
       <c r="N102" s="24" t="n"/>
-      <c r="O102" s="27" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="P102" s="27" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
+      <c r="O102" s="27" t="n"/>
+      <c r="P102" s="27" t="n"/>
       <c r="Q102" s="24" t="inlineStr">
         <is>
-          <t>Emlak Katılım Paraf kart sahipleri</t>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
       <c r="R102" s="24" t="n"/>
@@ -9265,21 +9242,22 @@
       </c>
       <c r="U102" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 1.300 TL = en yuksek barem (1.250) + mobil/QR ekstrasi (50). Uc kademe: 500/800/1.250. AYNI AILEDEN IKI SURUM DAHA VAR (Temmuz 1.000 TL ve Temmuz 2.000 TL) ama metinleri bu kayda %89-92 benzedigi icin etiketlenmedi - ucu birden altin sete girseydi ayni teklif olcumde uc kat agirlik alir, train/test'e dagilirsa sizinti olurdu. Bu surum secildi cunku basliktaki sayi dogrudan bir kademe DEGIL: en yuksek barem (1.250) + mobil/QR ekstrasi (50).</t>
-        </is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 4.000 TL bir ALT ESIKTIR, finansman tutari degil. Kampanya tarihi sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V102" t="n">
+        <v>6</v>
       </c>
       <c r="X102" s="2" t="inlineStr">
         <is>
-          <t>odul_miktari: bir müşteri kampanyaya bir kez katılabilir ve en fazla 1.300 TL ParafPara kazanabilir.
-kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
+          <t>taksit_sayisi: peşin fiyatına 6 taksit</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="24" t="inlineStr">
         <is>
-          <t>ZK-014</t>
+          <t>ZK-016</t>
         </is>
       </c>
       <c r="B103" s="24" t="inlineStr">
@@ -9289,7 +9267,7 @@
       </c>
       <c r="C103" s="24" t="inlineStr">
         <is>
-          <t>Amazon'da 9'a Varan Taksit</t>
+          <t>Bağımsız Kart'a Özel 5.000 TL'ye Varan Bankkart Lira</t>
         </is>
       </c>
       <c r="D103" s="24" t="inlineStr">
@@ -9299,7 +9277,7 @@
       </c>
       <c r="E103" s="24" t="inlineStr">
         <is>
-          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/amazonda-9a-varan-taksit</t>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/bagimsiz-karta-ozel-5000-tlye-varan-bankkart-lira-1</t>
         </is>
       </c>
       <c r="F103" s="25" t="n"/>
@@ -9307,19 +9285,33 @@
       <c r="H103" s="24" t="n"/>
       <c r="I103" s="26" t="n"/>
       <c r="J103" s="25" t="n"/>
-      <c r="K103" s="25" t="n"/>
-      <c r="L103" s="24" t="n"/>
+      <c r="K103" s="25" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L103" s="24" t="inlineStr">
+        <is>
+          <t>Bankkart Lira</t>
+        </is>
+      </c>
       <c r="M103" s="24" t="inlineStr">
         <is>
-          <t>Bankkart kredi kartıyla amazon.com.tr'de tutara göre peşin fiyatına 3, 6 veya 9 taksit</t>
+          <t>Bağımsız kredi kartıyla eğitim/sağlık/spor/kültür-sanat harcamalarına %10, toplamda 5.000 TL Bankkart Lira</t>
         </is>
       </c>
       <c r="N103" s="24" t="n"/>
-      <c r="O103" s="27" t="n"/>
-      <c r="P103" s="27" t="n"/>
+      <c r="O103" s="27" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="P103" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
       <c r="Q103" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+          <t>Ziraat Katılım Bankkart Bağımsız kredi kartı sahipleri</t>
         </is>
       </c>
       <c r="R103" s="24" t="n"/>
@@ -9331,32 +9323,32 @@
       </c>
       <c r="U103" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Uc kademe (3/6/9); 9 taksit yalnizca SECILI URUNLERDE ve 10.000 TL uzeri. Kampanya tarihi sayfada YOK.</t>
-        </is>
-      </c>
-      <c r="V103" t="n">
-        <v>9</v>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %10 nakit iade oranidir. Bir sonraki donemi (8 Agustos - 7 Eylul) ayri sayfada duruyor ama metin neredeyse ayni - etiketlenmedi.</t>
+        </is>
       </c>
       <c r="X103" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: Seçili ürünlerde yapacağınız 10.000 TL ve üzeri alışverişlerinizde peşin fiyatına 9 taksit fırsatından faydalanabilirsiniz.</t>
+          <t>odul_miktari: tüm harcamalara %10, toplamda 5.000 TL Bankkart Lira!
+odul_birimi: tüm harcamalara %10, toplamda 5.000 TL Bankkart Lira!
+kampanya_baslangic: 10 Temmuz – 7 Ağustos 2026
+kampanya_bitis: 10 Temmuz – 7 Ağustos 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="24" t="inlineStr">
         <is>
-          <t>ZK-015</t>
+          <t>TEK-015</t>
         </is>
       </c>
       <c r="B104" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım</t>
+          <t>Türkiye Emlak Katılım</t>
         </is>
       </c>
       <c r="C104" s="24" t="inlineStr">
         <is>
-          <t>Atasun Optik'te 6 Taksit</t>
+          <t>Hızlı Çiçek'te Tüm İndirimlere Ek %20 İndirim Fırsatı</t>
         </is>
       </c>
       <c r="D104" s="24" t="inlineStr">
@@ -9366,7 +9358,7 @@
       </c>
       <c r="E104" s="24" t="inlineStr">
         <is>
-          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/atasun-optikte-6-taksit</t>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/hizli-cicekte-tum-indirimlere-ek-20-indirim-firsati</t>
         </is>
       </c>
       <c r="F104" s="25" t="n"/>
@@ -9378,15 +9370,19 @@
       <c r="L104" s="24" t="n"/>
       <c r="M104" s="24" t="inlineStr">
         <is>
-          <t>Bankkart kredi kartıyla Atasun Optik'te 4.000 TL üzeri işlemlerde peşin fiyatına 6 taksit</t>
+          <t>EKB20 kupon koduyla Hızlı Çiçek'te tüm indirimlere ek %20 indirim</t>
         </is>
       </c>
       <c r="N104" s="24" t="n"/>
       <c r="O104" s="27" t="n"/>
-      <c r="P104" s="27" t="n"/>
+      <c r="P104" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
       <c r="Q104" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
+          <t>Emlak Katılım Paraf, Paraf Premium ve Debit kart sahipleri</t>
         </is>
       </c>
       <c r="R104" s="24" t="n"/>
@@ -9398,32 +9394,29 @@
       </c>
       <c r="U104" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 4.000 TL bir ALT ESIKTIR, finansman tutari degil. Kampanya tarihi sayfada YOK.</t>
-        </is>
-      </c>
-      <c r="V104" t="n">
-        <v>6</v>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Sayisal alanlar BILEREK BOS: %20 kupon indirimidir, TL tavani yok. Baslangic tarihi YOK.</t>
+        </is>
       </c>
       <c r="X104" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: peşin fiyatına 6 taksit</t>
+          <t>kampanya_bitis: Kampanya 31.12.2026 tarihine kadar geçerlidir.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="24" t="inlineStr">
         <is>
-          <t>ZK-016</t>
+          <t>TEK-016</t>
         </is>
       </c>
       <c r="B105" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım</t>
+          <t>Türkiye Emlak Katılım</t>
         </is>
       </c>
       <c r="C105" s="24" t="inlineStr">
         <is>
-          <t>Bağımsız Kart'a Özel 5.000 TL'ye Varan Bankkart Lira</t>
+          <t>Marina Mayo'da Tüm Ürünlerde %15 İndirim</t>
         </is>
       </c>
       <c r="D105" s="24" t="inlineStr">
@@ -9433,7 +9426,7 @@
       </c>
       <c r="E105" s="24" t="inlineStr">
         <is>
-          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/bagimsiz-karta-ozel-5000-tlye-varan-bankkart-lira-1</t>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/marina-mayoda-tum-urunlerde-15-indirim</t>
         </is>
       </c>
       <c r="F105" s="25" t="n"/>
@@ -9441,33 +9434,23 @@
       <c r="H105" s="24" t="n"/>
       <c r="I105" s="26" t="n"/>
       <c r="J105" s="25" t="n"/>
-      <c r="K105" s="25" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L105" s="24" t="inlineStr">
-        <is>
-          <t>Bankkart Lira</t>
-        </is>
-      </c>
+      <c r="K105" s="25" t="n"/>
+      <c r="L105" s="24" t="n"/>
       <c r="M105" s="24" t="inlineStr">
         <is>
-          <t>Bağımsız kredi kartıyla eğitim/sağlık/spor/kültür-sanat harcamalarına %10, toplamda 5.000 TL Bankkart Lira</t>
+          <t>emlak15 kupon koduyla Marina Mayo'da tüm ürünlerde %15 indirim (tek kullanımlık)</t>
         </is>
       </c>
       <c r="N105" s="24" t="n"/>
-      <c r="O105" s="27" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
+      <c r="O105" s="27" t="n"/>
       <c r="P105" s="27" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="Q105" s="24" t="inlineStr">
         <is>
-          <t>Ziraat Katılım Bankkart Bağımsız kredi kartı sahipleri</t>
+          <t>Emlak Katılım Paraf, Paraf Premium ve Debit kart sahipleri</t>
         </is>
       </c>
       <c r="R105" s="24" t="n"/>
@@ -9479,32 +9462,29 @@
       </c>
       <c r="U105" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %10 nakit iade oranidir. Bir sonraki donemi (8 Agustos - 7 Eylul) ayri sayfada duruyor ama metin neredeyse ayni - etiketlenmedi.</t>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Sayisal alanlar BILEREK BOS: %15 kupon indirimidir. Baslangic tarihi YOK.</t>
         </is>
       </c>
       <c r="X105" s="2" t="inlineStr">
         <is>
-          <t>odul_miktari: tüm harcamalara %10, toplamda 5.000 TL Bankkart Lira!
-odul_birimi: tüm harcamalara %10, toplamda 5.000 TL Bankkart Lira!
-kampanya_baslangic: 10 Temmuz – 7 Ağustos 2026
-kampanya_bitis: 10 Temmuz – 7 Ağustos 2026</t>
+          <t>kampanya_bitis: Kampanya, 31.12.2026 tarihine kadar geçerlidir.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="24" t="inlineStr">
         <is>
-          <t>TEK-015</t>
+          <t>ZK-017</t>
         </is>
       </c>
       <c r="B106" s="24" t="inlineStr">
         <is>
-          <t>Türkiye Emlak Katılım</t>
+          <t>Ziraat Katılım</t>
         </is>
       </c>
       <c r="C106" s="24" t="inlineStr">
         <is>
-          <t>Hızlı Çiçek'te Tüm İndirimlere Ek %20 İndirim Fırsatı</t>
+          <t>BAUHAUS'ta 3 Taksit</t>
         </is>
       </c>
       <c r="D106" s="24" t="inlineStr">
@@ -9514,7 +9494,7 @@
       </c>
       <c r="E106" s="24" t="inlineStr">
         <is>
-          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/hizli-cicekte-tum-indirimlere-ek-20-indirim-firsati</t>
+          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/bauhausta-3-taksit</t>
         </is>
       </c>
       <c r="F106" s="25" t="n"/>
@@ -9526,19 +9506,15 @@
       <c r="L106" s="24" t="n"/>
       <c r="M106" s="24" t="inlineStr">
         <is>
-          <t>EKB20 kupon koduyla Hızlı Çiçek'te tüm indirimlere ek %20 indirim</t>
+          <t>Bankkart kredi kartıyla BAUHAUS alışverişlerinde 3 taksit</t>
         </is>
       </c>
       <c r="N106" s="24" t="n"/>
       <c r="O106" s="27" t="n"/>
-      <c r="P106" s="27" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
+      <c r="P106" s="27" t="n"/>
       <c r="Q106" s="24" t="inlineStr">
         <is>
-          <t>Emlak Katılım Paraf, Paraf Premium ve Debit kart sahipleri</t>
+          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
       <c r="R106" s="24" t="n"/>
@@ -9550,41 +9526,24 @@
       </c>
       <c r="U106" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Sayisal alanlar BILEREK BOS: %20 kupon indirimidir, TL tavani yok. Baslangic tarihi YOK.</t>
-        </is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
+        </is>
+      </c>
+      <c r="V106" t="n">
+        <v>3</v>
       </c>
       <c r="X106" s="2" t="inlineStr">
         <is>
-          <t>kampanya_bitis: Kampanya 31.12.2026 tarihine kadar geçerlidir.</t>
+          <t>taksit_sayisi: 3 taksit</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="24" t="inlineStr">
-        <is>
-          <t>TEK-016</t>
-        </is>
-      </c>
-      <c r="B107" s="24" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C107" s="24" t="inlineStr">
-        <is>
-          <t>Marina Mayo'da Tüm Ürünlerde %15 İndirim</t>
-        </is>
-      </c>
-      <c r="D107" s="24" t="inlineStr">
-        <is>
-          <t>Kart Kampanyasi</t>
-        </is>
-      </c>
-      <c r="E107" s="24" t="inlineStr">
-        <is>
-          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/marina-mayoda-tum-urunlerde-15-indirim</t>
-        </is>
-      </c>
+      <c r="A107" s="24" t="n"/>
+      <c r="B107" s="24" t="n"/>
+      <c r="C107" s="24" t="n"/>
+      <c r="D107" s="24" t="n"/>
+      <c r="E107" s="24" t="n"/>
       <c r="F107" s="25" t="n"/>
       <c r="G107" s="25" t="n"/>
       <c r="H107" s="24" t="n"/>
@@ -9592,130 +9551,15 @@
       <c r="J107" s="25" t="n"/>
       <c r="K107" s="25" t="n"/>
       <c r="L107" s="24" t="n"/>
-      <c r="M107" s="24" t="inlineStr">
-        <is>
-          <t>emlak15 kupon koduyla Marina Mayo'da tüm ürünlerde %15 indirim (tek kullanımlık)</t>
-        </is>
-      </c>
+      <c r="M107" s="24" t="n"/>
       <c r="N107" s="24" t="n"/>
       <c r="O107" s="27" t="n"/>
-      <c r="P107" s="27" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="Q107" s="24" t="inlineStr">
-        <is>
-          <t>Emlak Katılım Paraf, Paraf Premium ve Debit kart sahipleri</t>
-        </is>
-      </c>
+      <c r="P107" s="27" t="n"/>
+      <c r="Q107" s="24" t="n"/>
       <c r="R107" s="24" t="n"/>
       <c r="S107" s="24" t="n"/>
-      <c r="T107" s="27" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="U107" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Sayisal alanlar BILEREK BOS: %15 kupon indirimidir. Baslangic tarihi YOK.</t>
-        </is>
-      </c>
-      <c r="X107" s="2" t="inlineStr">
-        <is>
-          <t>kampanya_bitis: Kampanya, 31.12.2026 tarihine kadar geçerlidir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="24" t="inlineStr">
-        <is>
-          <t>ZK-017</t>
-        </is>
-      </c>
-      <c r="B108" s="24" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C108" s="24" t="inlineStr">
-        <is>
-          <t>BAUHAUS'ta 3 Taksit</t>
-        </is>
-      </c>
-      <c r="D108" s="24" t="inlineStr">
-        <is>
-          <t>Kart Kampanyasi</t>
-        </is>
-      </c>
-      <c r="E108" s="24" t="inlineStr">
-        <is>
-          <t>www.ziraatkatilim.com.tr/kart-kampanyalari/bauhausta-3-taksit</t>
-        </is>
-      </c>
-      <c r="F108" s="25" t="n"/>
-      <c r="G108" s="25" t="n"/>
-      <c r="H108" s="24" t="n"/>
-      <c r="I108" s="26" t="n"/>
-      <c r="J108" s="25" t="n"/>
-      <c r="K108" s="25" t="n"/>
-      <c r="L108" s="24" t="n"/>
-      <c r="M108" s="24" t="inlineStr">
-        <is>
-          <t>Bankkart kredi kartıyla BAUHAUS alışverişlerinde 3 taksit</t>
-        </is>
-      </c>
-      <c r="N108" s="24" t="n"/>
-      <c r="O108" s="27" t="n"/>
-      <c r="P108" s="27" t="n"/>
-      <c r="Q108" s="24" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
-        </is>
-      </c>
-      <c r="R108" s="24" t="n"/>
-      <c r="S108" s="24" t="n"/>
-      <c r="T108" s="27" t="inlineStr">
-        <is>
-          <t>2026-08-21</t>
-        </is>
-      </c>
-      <c r="U108" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
-        </is>
-      </c>
-      <c r="V108" t="n">
-        <v>3</v>
-      </c>
-      <c r="X108" s="2" t="inlineStr">
-        <is>
-          <t>taksit_sayisi: 3 taksit</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="24" t="n"/>
-      <c r="B109" s="24" t="n"/>
-      <c r="C109" s="24" t="n"/>
-      <c r="D109" s="24" t="n"/>
-      <c r="E109" s="24" t="n"/>
-      <c r="F109" s="25" t="n"/>
-      <c r="G109" s="25" t="n"/>
-      <c r="H109" s="24" t="n"/>
-      <c r="I109" s="26" t="n"/>
-      <c r="J109" s="25" t="n"/>
-      <c r="K109" s="25" t="n"/>
-      <c r="L109" s="24" t="n"/>
-      <c r="M109" s="24" t="n"/>
-      <c r="N109" s="24" t="n"/>
-      <c r="O109" s="27" t="n"/>
-      <c r="P109" s="27" t="n"/>
-      <c r="Q109" s="24" t="n"/>
-      <c r="R109" s="24" t="n"/>
-      <c r="S109" s="24" t="n"/>
-      <c r="T109" s="27" t="n"/>
-      <c r="U109" s="24" t="n"/>
+      <c r="T107" s="27" t="n"/>
+      <c r="U107" s="24" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U1"/>

</xml_diff>

<commit_message>
eksik yakalanan kaynaklar JS ile tazelendi, dokuz kayittaki eksik alanlar duzeltildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -150,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -224,6 +224,9 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6908,8 +6911,16 @@
         </is>
       </c>
       <c r="N71" s="24" t="n"/>
-      <c r="O71" s="27" t="n"/>
-      <c r="P71" s="27" t="n"/>
+      <c r="O71" s="27" t="inlineStr">
+        <is>
+          <t>2025-07-10</t>
+        </is>
+      </c>
+      <c r="P71" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="Q71" s="24" t="inlineStr">
         <is>
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
@@ -6922,9 +6933,9 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U71" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi sayfada YOK. 300 TL alt esik, finansman tutari degil.</t>
+      <c r="U71" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 300 TL alt esik, finansman tutari degil. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V71" t="n">
@@ -6932,7 +6943,9 @@
       </c>
       <c r="X71" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: alışverişlerinizde peşin fiyatına 6 aya varan taksit fırsatından faydalanabilirsiniz.</t>
+          <t>taksit_sayisi: alışverişlerinizde peşin fiyatına 6 aya varan taksit fırsatından faydalanabilirsiniz.
+kampanya_baslangic: 10-07-2025 - 31-08-2026
+kampanya_bitis: 10-07-2025 - 31-08-2026</t>
         </is>
       </c>
     </row>
@@ -7333,8 +7346,16 @@
         </is>
       </c>
       <c r="N77" s="24" t="n"/>
-      <c r="O77" s="27" t="n"/>
-      <c r="P77" s="27" t="n"/>
+      <c r="O77" s="27" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="P77" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="Q77" s="24" t="inlineStr">
         <is>
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
@@ -7347,9 +7368,9 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U77" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve alt/ust harcama siniri sayfada YOK.</t>
+      <c r="U77" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Alt/ust harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V77" t="n">
@@ -7357,7 +7378,9 @@
       </c>
       <c r="X77" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: 2 taksitli</t>
+          <t>taksit_sayisi: 2 taksitli
+kampanya_baslangic: 01-04-2025 - 31-08-2026
+kampanya_bitis: 01-04-2025 - 31-08-2026</t>
         </is>
       </c>
     </row>
@@ -7937,7 +7960,9 @@
       <c r="F85" s="25" t="n"/>
       <c r="G85" s="25" t="n"/>
       <c r="H85" s="24" t="n"/>
-      <c r="I85" s="26" t="n"/>
+      <c r="I85" s="26" t="n">
+        <v>6</v>
+      </c>
       <c r="J85" s="25" t="n">
         <v>40000</v>
       </c>
@@ -7971,14 +7996,23 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U85" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: sayfa 'uygun oranli' diyor, sayi vermiyor; oran basvuruda musteriye gore belirleniyor. Pratik Finansman Kart ile ATM'den nakit cekilemiyor.</t>
-        </is>
+      <c r="U85" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: sayfadaki %5 / %3,90 / %3,85 oranlari PRATIK FINANSMAN KARTA DEGIL, ayni sayfada tanitilan 'hos geldin finansmani'nin vade kademelerine aittir. Kartin kendisi VADE FARKSIZ. DUZELTME (23 Agustos 2026): vade_ay, taksit_sayisi ve erteleme_suresi_ay etiketlenirken KACIRILMISTI - ucu de tek cumlede yaziyor ('3 aya varan odemesiz donem ve 4 taksit imkani ile birlikte toplam 6 aya varan vade'). Sayfa JS ile yeniden tarandiktan sonra goruldu; bu bir okuma hatasiydi, tarama eksigi degil. Pratik Finansman Kart ile ATM'den nakit cekilemiyor.</t>
+        </is>
+      </c>
+      <c r="V85" t="n">
+        <v>4</v>
+      </c>
+      <c r="W85" t="n">
+        <v>3</v>
       </c>
       <c r="X85" s="2" t="inlineStr">
         <is>
-          <t>finansman_tutari: Vade farksız 40.000 TL ve uygun oranlı hoş geldin finansmanı Albaraka'da!</t>
+          <t>finansman_tutari: Vade farksız 40.000 TL ve uygun oranlı hoş geldin finansmanı Albaraka'da!
+vade_ay: ’lı olan dijital müşterilerimize özel; vade farksız, azami 40.000 TL limitli, 3 aya varan ödemesiz dönem ve 4 taksit imkânı ile birlikte toplam 6 aya varan vade imkanıyla sunulan Pratik Fina
+taksit_sayisi: ’lı olan dijital müşterilerimize özel; vade farksız, azami 40.000 TL limitli, 3 aya varan ödemesiz dönem ve 4 taksit imkânı ile birlikte toplam 6 aya varan vade imkanıyla sunulan Pratik Fina
+erteleme_suresi_ay: ’lı olan dijital müşterilerimize özel; vade farksız, azami 40.000 TL limitli, 3 aya varan ödemesiz dönem ve 4 taksit imkânı ile birlikte toplam 6 aya varan vade imkanıyla sunulan Pratik Fina</t>
         </is>
       </c>
     </row>
@@ -8091,7 +8125,9 @@
       <c r="F87" s="25" t="n"/>
       <c r="G87" s="25" t="n"/>
       <c r="H87" s="24" t="n"/>
-      <c r="I87" s="26" t="n"/>
+      <c r="I87" s="26" t="n">
+        <v>36</v>
+      </c>
       <c r="J87" s="25" t="n">
         <v>400000</v>
       </c>
@@ -8117,9 +8153,9 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U87" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: 'size ozel kar payi oranlari' deniyor ama SAYI verilmiyor. Kampanya tarihi de sayfada YOK. erteleme_suresi_ay dolu olan ilk altin kayit - o sutun su an OLCUM DISI (excel_to_json INCELENMIS_ALANLAR'a bak).</t>
+      <c r="U87" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: 'size ozel kar payi oranlari' deniyor ama SAYI verilmiyor. Kampanya tarihi de sayfada YOK. DUZELTME (23 Agustos 2026): vade_ay etiketlenirken KACIRILDI - sayfa 'maksimum vade suresi 36 aydir' diyor. Vade KADEMELI: 125.000 TL'ye kadar 36 ay, 125.000-250.000 TL arasi 24 ay, 250.000 TL uzeri 12 ay. Alan tek sayi tuttugu icin EN YUKSEK kademe yazildi (finansman_tutari'nda araligin ust sinirini yazma kuraliyla ayni yaklasim). erteleme_suresi_ay dolu olan ilk altin kayit - o sutun su an OLCUM DISI (excel_to_json INCELENMIS_ALANLAR'a bak).</t>
         </is>
       </c>
       <c r="W87" t="n">
@@ -8128,7 +8164,8 @@
       <c r="X87" s="2" t="inlineStr">
         <is>
           <t>finansman_tutari: Kampanya kapsamında 50.000 TL – 400.000 TL arasındaki ihtiyaçlarını için finansman başvurusu yapabilirsiniz.
-erteleme_suresi_ay: Finansman geri ödemelerinizde ilk taksiniz için 3 ay öteleme hakkınızı kullanabilir</t>
+erteleme_suresi_ay: Finansman geri ödemelerinizde ilk taksiniz için 3 ay öteleme hakkınızı kullanabilir
+vade_ay: İhtiyaç Finansmanına uygulanacak maksimum vade süresi 36 aydır.</t>
         </is>
       </c>
     </row>
@@ -8545,8 +8582,16 @@
         </is>
       </c>
       <c r="N93" s="24" t="n"/>
-      <c r="O93" s="27" t="n"/>
-      <c r="P93" s="27" t="n"/>
+      <c r="O93" s="27" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="P93" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="Q93" s="24" t="inlineStr">
         <is>
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
@@ -8559,9 +8604,9 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U93" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
+      <c r="U93" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V93" t="n">
@@ -8569,7 +8614,9 @@
       </c>
       <c r="X93" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: 6 taksitli</t>
+          <t>taksit_sayisi: 6 taksitli
+kampanya_baslangic: 01-04-2025 - 31-08-2026
+kampanya_bitis: 01-04-2025 - 31-08-2026</t>
         </is>
       </c>
     </row>
@@ -8776,8 +8823,16 @@
         </is>
       </c>
       <c r="N96" s="24" t="n"/>
-      <c r="O96" s="27" t="n"/>
-      <c r="P96" s="27" t="n"/>
+      <c r="O96" s="27" t="inlineStr">
+        <is>
+          <t>2025-11-27</t>
+        </is>
+      </c>
+      <c r="P96" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="Q96" s="24" t="inlineStr">
         <is>
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
@@ -8790,9 +8845,9 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U96" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
+      <c r="U96" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V96" t="n">
@@ -8800,7 +8855,9 @@
       </c>
       <c r="X96" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: 5 taksitli</t>
+          <t>taksit_sayisi: 5 taksitli
+kampanya_baslangic: 27-11-2025 - 31-08-2026
+kampanya_bitis: 27-11-2025 - 31-08-2026</t>
         </is>
       </c>
     </row>
@@ -9159,8 +9216,16 @@
         </is>
       </c>
       <c r="N101" s="24" t="n"/>
-      <c r="O101" s="27" t="n"/>
-      <c r="P101" s="27" t="n"/>
+      <c r="O101" s="27" t="inlineStr">
+        <is>
+          <t>2025-11-13</t>
+        </is>
+      </c>
+      <c r="P101" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="Q101" s="24" t="inlineStr">
         <is>
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
@@ -9173,9 +9238,9 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U101" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Uc kademe (3/6/9); 9 taksit yalnizca SECILI URUNLERDE ve 10.000 TL uzeri. Kampanya tarihi sayfada YOK.</t>
+      <c r="U101" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Uc kademe (3/6/9); 9 taksit yalnizca SECILI URUNLERDE ve 10.000 TL uzeri. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V101" t="n">
@@ -9183,7 +9248,9 @@
       </c>
       <c r="X101" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: Seçili ürünlerde yapacağınız 10.000 TL ve üzeri alışverişlerinizde peşin fiyatına 9 taksit fırsatından faydalanabilirsiniz.</t>
+          <t>taksit_sayisi: Seçili ürünlerde yapacağınız 10.000 TL ve üzeri alışverişlerinizde peşin fiyatına 9 taksit fırsatından faydalanabilirsiniz.
+kampanya_baslangic: 13-11-2025 - 31-08-2026
+kampanya_bitis: 13-11-2025 - 31-08-2026</t>
         </is>
       </c>
     </row>
@@ -9226,8 +9293,16 @@
         </is>
       </c>
       <c r="N102" s="24" t="n"/>
-      <c r="O102" s="27" t="n"/>
-      <c r="P102" s="27" t="n"/>
+      <c r="O102" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="P102" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="Q102" s="24" t="inlineStr">
         <is>
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
@@ -9240,9 +9315,9 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U102" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 4.000 TL bir ALT ESIKTIR, finansman tutari degil. Kampanya tarihi sayfada YOK.</t>
+      <c r="U102" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 4.000 TL bir ALT ESIKTIR, finansman tutari degil. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V102" t="n">
@@ -9250,7 +9325,9 @@
       </c>
       <c r="X102" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: peşin fiyatına 6 taksit</t>
+          <t>taksit_sayisi: peşin fiyatına 6 taksit
+kampanya_baslangic: 11-08-2026 - 31-08-2026
+kampanya_bitis: 11-08-2026 - 31-08-2026</t>
         </is>
       </c>
     </row>
@@ -9510,8 +9587,16 @@
         </is>
       </c>
       <c r="N106" s="24" t="n"/>
-      <c r="O106" s="27" t="n"/>
-      <c r="P106" s="27" t="n"/>
+      <c r="O106" s="27" t="inlineStr">
+        <is>
+          <t>2025-04-01</t>
+        </is>
+      </c>
+      <c r="P106" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="Q106" s="24" t="inlineStr">
         <is>
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
@@ -9524,9 +9609,9 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U106" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya tarihi ve harcama siniri sayfada YOK.</t>
+      <c r="U106" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V106" t="n">
@@ -9534,7 +9619,9 @@
       </c>
       <c r="X106" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: 3 taksit</t>
+          <t>taksit_sayisi: 3 taksit
+kampanya_baslangic: 01-04-2025 - 31-08-2026
+kampanya_bitis: 01-04-2025 - 31-08-2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
olcum delikleri kapatildi: taksit ve erteleme sutunlari olcume acildi, 9 kayitta deger yanlis alandan tasindi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -1844,9 +1844,7 @@
           <t>aylik</t>
         </is>
       </c>
-      <c r="I7" s="22" t="n">
-        <v>6</v>
-      </c>
+      <c r="I7" s="22" t="n"/>
       <c r="J7" s="21" t="n">
         <v>100000</v>
       </c>
@@ -1890,7 +1888,15 @@
       </c>
       <c r="U7" s="20" t="inlineStr">
         <is>
-          <t>Kar payi orani %2,99 ama vergiler dahil maliyet %4,1910 - sayfa ikisini ayri veriyor</t>
+          <t>Kar payi orani %2,99 ama vergiler dahil maliyet %4,1910 - sayfa ikisini ayri veriyor DUZELTME (23 Agustos 2026): vade_ay=6 -&gt; taksit_sayisi=6. '6 taksite kadar %2,99 kar payi orani' - 6 TAKSIT ADEDIDIR. Kampanya adinda 'N Taksit' gecmedigi icin taksit/vade uyarisina takilmamisti; denetimde elle bulundu. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>6</v>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Taksitlio’nun anlaşmalı olduğu mağazalarda yapacağınız 100.000 TL’ye kadar alışverişlerinizde 6 taksite kadar %2,99 avantajlı kar payı oranı ile alışveriş yapmanın tadını çıkarın!</t>
         </is>
       </c>
     </row>
@@ -2085,9 +2091,7 @@
       <c r="F10" s="21" t="n"/>
       <c r="G10" s="21" t="n"/>
       <c r="H10" s="19" t="n"/>
-      <c r="I10" s="22" t="n">
-        <v>3</v>
-      </c>
+      <c r="I10" s="22" t="n"/>
       <c r="J10" s="21" t="n"/>
       <c r="K10" s="21" t="n"/>
       <c r="L10" s="19" t="n"/>
@@ -2125,7 +2129,15 @@
       </c>
       <c r="U10" s="20" t="inlineStr">
         <is>
-          <t>Diyanetten alınan umre tur kodu şart</t>
+          <t>Diyanetten alınan umre tur kodu şart DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. 'vade farksiz 3 taksit imkani' - sayfa taksit ADEDINI veriyor. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>3</v>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Kampanya kapsamında Kutsal toprakları ziyaret etmek isteyen müşterilerimiz toplam umre tutarının en fazla yüzde altmışı için vade farksız 3 taksit imkanından yararlanabilir.</t>
         </is>
       </c>
     </row>
@@ -2450,11 +2462,19 @@
       </c>
       <c r="U14" s="20" t="inlineStr">
         <is>
-          <t>Kampanya iki bölümlü: 40.000 TL'lik kısım İhtiyaç Finansmanı (Pratik Finansman Kart), 100.000 TL'lik kısım kredi kartıyla vade farksız taksit - ilk kısım temel alındı | [9 Agu] vade_ay-&gt;taksit_sayisi tasindi (Secili sektorlerde vade farksiz 6 taksit); sayfada vade ifadesi yok</t>
+          <t>Kampanya iki bölümlü: 40.000 TL'lik kısım İhtiyaç Finansmanı (Pratik Finansman Kart), 100.000 TL'lik kısım kredi kartıyla vade farksız taksit - ilk kısım temel alındı | [9 Agu] vade_ay-&gt;taksit_sayisi tasindi (Secili sektorlerde vade farksiz 6 taksit); sayfada vade ifadesi yok DUZELTME (23 Agustos 2026): erteleme_suresi_ay=3 eklendi ('3 aya varan odemesiz donem') - etiketlenirken kacirilmisti.</t>
         </is>
       </c>
       <c r="V14" t="n">
         <v>6</v>
+      </c>
+      <c r="W14" t="n">
+        <v>3</v>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>erteleme_suresi_ay: 3 aya varan ödemesiz dönem ve 4 taksitli</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
@@ -2910,9 +2930,7 @@
           <t>belirsiz</t>
         </is>
       </c>
-      <c r="I20" s="22" t="n">
-        <v>3</v>
-      </c>
+      <c r="I20" s="22" t="n"/>
       <c r="J20" s="21" t="n">
         <v>100000</v>
       </c>
@@ -2956,8 +2974,11 @@
       </c>
       <c r="U20" s="20" t="inlineStr">
         <is>
-          <t>VKart Business ve VKart Debit kapsam dışı; müşteri başına en fazla 3 MTV ödemesi</t>
-        </is>
+          <t>VKart Business ve VKart Debit kapsam dışı; müşteri başına en fazla 3 MTV ödemesi DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. MTV odemesi taksitlendirmesi - Kart Kampanyasi, finansman vadesi yok. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+        </is>
+      </c>
+      <c r="V20" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
@@ -2995,9 +3016,7 @@
           <t>belirsiz</t>
         </is>
       </c>
-      <c r="I21" s="22" t="n">
-        <v>3</v>
-      </c>
+      <c r="I21" s="22" t="n"/>
       <c r="J21" s="21" t="n">
         <v>300000</v>
       </c>
@@ -3041,8 +3060,11 @@
       </c>
       <c r="U21" s="20" t="inlineStr">
         <is>
-          <t>Sadece gib.gov.tr veya banka kanallarından yapılan ödemeler geçerli</t>
-        </is>
+          <t>Sadece gib.gov.tr veya banka kanallarından yapılan ödemeler geçerli DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. Gelir vergisi odemesi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
@@ -3080,9 +3102,7 @@
           <t>belirsiz</t>
         </is>
       </c>
-      <c r="I22" s="22" t="n">
-        <v>5</v>
-      </c>
+      <c r="I22" s="22" t="n"/>
       <c r="J22" s="21" t="n">
         <v>100000</v>
       </c>
@@ -3126,8 +3146,11 @@
       </c>
       <c r="U22" s="20" t="inlineStr">
         <is>
-          <t>Müşteri başına en fazla 3 harcama taksitlendirilebilir</t>
-        </is>
+          <t>Müşteri başına en fazla 3 harcama taksitlendirilebilir DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Saglik harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
@@ -3327,9 +3350,7 @@
           <t>belirsiz</t>
         </is>
       </c>
-      <c r="I25" s="22" t="n">
-        <v>5</v>
-      </c>
+      <c r="I25" s="22" t="n"/>
       <c r="J25" s="21" t="n">
         <v>700000</v>
       </c>
@@ -3373,8 +3394,11 @@
       </c>
       <c r="U25" s="20" t="inlineStr">
         <is>
-          <t>Sadece TROY kart, ek/sanal kartlar dahil; müşteri başına en fazla 3 harcama</t>
-        </is>
+          <t>Sadece TROY kart, ek/sanal kartlar dahil; müşteri başına en fazla 3 harcama DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Egitim harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
@@ -3594,7 +3618,15 @@
       </c>
       <c r="U28" s="20" t="inlineStr">
         <is>
-          <t>Somut oran verilmiyor - rapor Bölüm 3'ün gözlemine örnek</t>
+          <t>Somut oran verilmiyor - rapor Bölüm 3'ün gözlemine örnek DUZELTME (23 Agustos 2026): erteleme_suresi_ay=3 eklendi ('3 ay ertelemeli' / '3 ay oteleme') - etiketlenirken kacirilmisti.</t>
+        </is>
+      </c>
+      <c r="W28" t="n">
+        <v>3</v>
+      </c>
+      <c r="X28" s="2" t="inlineStr">
+        <is>
+          <t>erteleme_suresi_ay: ​​​​​​​​​​​​Banka çalışanlarına, ​kendi çalışanlarımıza sunduğumuz sabit ve avantajlı oranlarla 3 ay ertelemeli ihtiyaç finansmanı Türkiye Finans’ta!</t>
         </is>
       </c>
     </row>
@@ -3866,8 +3898,12 @@
       <c r="F32" s="21" t="n"/>
       <c r="G32" s="21" t="n"/>
       <c r="H32" s="19" t="n"/>
-      <c r="I32" s="22" t="n"/>
-      <c r="J32" s="21" t="n"/>
+      <c r="I32" s="22" t="n">
+        <v>24</v>
+      </c>
+      <c r="J32" s="21" t="n">
+        <v>400000</v>
+      </c>
       <c r="K32" s="21" t="n">
         <v>11000</v>
       </c>
@@ -3881,7 +3917,11 @@
           <t>Mobilden yeni müşteri olana 11.000 TL'ye varan bonus + masrafsız temel bankacılık</t>
         </is>
       </c>
-      <c r="N32" s="20" t="n"/>
+      <c r="N32" s="20" t="inlineStr">
+        <is>
+          <t>Temel bankacılık işlemlerinde masraf yok</t>
+        </is>
+      </c>
       <c r="O32" s="23" t="n"/>
       <c r="P32" s="23" t="n"/>
       <c r="Q32" s="20" t="inlineStr">
@@ -3906,7 +3946,16 @@
       </c>
       <c r="U32" s="20" t="inlineStr">
         <is>
-          <t>Bitis tarihi sayfada belirtilmemis, sureklen bir paket gibi gorunuyor - bos birakildi</t>
+          <t>Bitis tarihi sayfada belirtilmemis, sureklen bir paket gibi gorunuyor - bos birakildi DUZELTME (23 Agustos 2026): erteleme_suresi_ay=3, finansman_tutari=400000 ve vade_ay=24 eklendi. Vade KADEMELI (250.000 TL'ye kadar 24 ay, fazlasi 12 ay); TF-008 ile ayni kural: en yuksek kademe yazilir. masraf_durumu eklendi: sayfa 'temel bankacilik islemleriniz icin masraf odemeyin' diyor. TF-007 ('Masrafsiz Bankacilik') NEREDEYSE AYNI cumleyi masraf_durumu'na yazmisti; iki kayit celisiyordu.</t>
+        </is>
+      </c>
+      <c r="W32" t="n">
+        <v>3</v>
+      </c>
+      <c r="X32" s="2" t="inlineStr">
+        <is>
+          <t>erteleme_suresi_ay: 400.000 TL'ye Kadar İhtiyaç Finansmanı Kullanın, 3 Ay Öteleme Fırsatından Yararlanın!
+masraf_durumu: Üstelik temel bankacılık işlemleriniz için masraf ödemeyin.</t>
         </is>
       </c>
     </row>
@@ -4253,9 +4302,7 @@
       <c r="F37" s="21" t="n"/>
       <c r="G37" s="21" t="n"/>
       <c r="H37" s="19" t="n"/>
-      <c r="I37" s="22" t="n">
-        <v>4</v>
-      </c>
+      <c r="I37" s="22" t="n"/>
       <c r="J37" s="21" t="n"/>
       <c r="K37" s="21" t="n"/>
       <c r="L37" s="19" t="n"/>
@@ -4297,8 +4344,11 @@
       </c>
       <c r="U37" s="20" t="inlineStr">
         <is>
-          <t>Diger bankalardaki benzer kampanyalardan farkli olarak burada acikca 'vade farksiz' ifadesi yok - orani 0 varsaymadim</t>
-        </is>
+          <t>Diger bankalardaki benzer kampanyalardan farkli olarak burada acikca 'vade farksiz' ifadesi yok - orani 0 varsaymadim DUZELTME (23 Agustos 2026): vade_ay=4 -&gt; taksit_sayisi=4. MTV odemesi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+        </is>
+      </c>
+      <c r="V37" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
@@ -4372,7 +4422,15 @@
       </c>
       <c r="U38" s="20" t="inlineStr">
         <is>
-          <t>vade_ay alani burada net degil: kampanya 'mevcut 2-4 taksite +8 ekliyor' diyor (toplamda 10-12 taksit gibi), tekil bir sayi degil - bos birakildi</t>
+          <t>vade_ay alani burada net degil: kampanya 'mevcut 2-4 taksite +8 ekliyor' diyor (toplamda 10-12 taksit gibi), tekil bir sayi degil - bos birakildi DUZELTME (23 Agustos 2026): taksit_sayisi=8 eklendi. Kampanya 2-4 taksitli islemlere +8 taksit EKLIYOR; 8, kampanyanin kendi kattigi taksit sayisidir (baslik da oyle diyor).</t>
+        </is>
+      </c>
+      <c r="V38" t="n">
+        <v>8</v>
+      </c>
+      <c r="X38" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: +8 taksit!</t>
         </is>
       </c>
     </row>
@@ -5663,9 +5721,7 @@
           <t>belirsiz</t>
         </is>
       </c>
-      <c r="I55" s="22" t="n">
-        <v>9</v>
-      </c>
+      <c r="I55" s="22" t="n"/>
       <c r="J55" s="21" t="n">
         <v>10000</v>
       </c>
@@ -5705,8 +5761,11 @@
       </c>
       <c r="U55" s="20" t="inlineStr">
         <is>
-          <t>Kademeli sistem: 100-1.000 TL-&gt;3 taksit, 1.000-6.000 TL-&gt;6 taksit, 6.000-10.000 TL-&gt;6 taksit, 10.000 TL+ secili urun-&gt;9 taksit. En ust dilim alindi</t>
-        </is>
+          <t>Kademeli sistem: 100-1.000 TL-&gt;3 taksit, 1.000-6.000 TL-&gt;6 taksit, 6.000-10.000 TL-&gt;6 taksit, 10.000 TL+ secili urun-&gt;9 taksit. En ust dilim alindi DUZELTME (23 Agustos 2026): vade_ay=9 -&gt; taksit_sayisi=9. kademeli taksit (3/6/9), Alisveris Puani Kampanyasi - vade yok. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+        </is>
+      </c>
+      <c r="V55" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="56" ht="28" customHeight="1">
@@ -5744,9 +5803,7 @@
           <t>belirsiz</t>
         </is>
       </c>
-      <c r="I56" s="22" t="n">
-        <v>3</v>
-      </c>
+      <c r="I56" s="22" t="n"/>
       <c r="J56" s="21" t="n">
         <v>2000</v>
       </c>
@@ -5786,8 +5843,11 @@
       </c>
       <c r="U56" s="20" t="inlineStr">
         <is>
-          <t>Sepet toplami 2.000 TL alt sinirdir</t>
-        </is>
+          <t>Sepet toplami 2.000 TL alt sinirdir DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. 'pesin fiyatina 3 taksit', Alisveris Puani Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+        </is>
+      </c>
+      <c r="V56" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="57" ht="28" customHeight="1">

</xml_diff>

<commit_message>
kanit spani araci eklendi, 45 span dolduruldu, TOM Katilim'a uc kayit
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -1215,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X107"/>
+  <dimension ref="A1:X109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1896,7 +1896,9 @@
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: Taksitlio’nun anlaşmalı olduğu mağazalarda yapacağınız 100.000 TL’ye kadar alışverişlerinizde 6 taksite kadar %2,99 avantajlı kar payı oranı ile alışveriş yapmanın tadını çıkarın!</t>
+          <t>taksit_sayisi: Taksitlio’nun anlaşmalı olduğu mağazalarda yapacağınız 100.000 TL’ye kadar alışverişlerinizde 6 taksite kadar %2,99 avantajlı kar payı oranı ile alışveriş yapmanın tadını çıkarın!
+kampanya_baslangic: 20.01.2026 - 31.12.2026
+kampanya_bitis: 20.01.2026 - 31.12.2026</t>
         </is>
       </c>
     </row>
@@ -2061,6 +2063,12 @@
           <t>Rapor Bölüm 3'ün gözlemini doğruluyor: genel tanıtım sayfası, kampanyaya özel somut oran/vade YOK - şeffaflık ilkesi gereği boş bırakıldı</t>
         </is>
       </c>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 19.03.2026 - 31.12.2026
+kampanya_bitis: 19.03.2026 - 31.12.2026</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -2137,7 +2145,8 @@
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: Kampanya kapsamında Kutsal toprakları ziyaret etmek isteyen müşterilerimiz toplam umre tutarının en fazla yüzde altmışı için vade farksız 3 taksit imkanından yararlanabilir.</t>
+          <t>taksit_sayisi: Kampanya kapsamında Kutsal toprakları ziyaret etmek isteyen müşterilerimiz toplam umre tutarının en fazla yüzde altmışı için vade farksız 3 taksit imkanından yararlanabilir.
+kampanya_baslangic: 13.08.2024 - 1.01.2027</t>
         </is>
       </c>
     </row>
@@ -2221,6 +2230,11 @@
           <t>Bu kayıt raporun Bölüm 3'teki "Mil" ödül birimi gözlemini doğruluyor</t>
         </is>
       </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: 30.04.2026 - 31.12.2026</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
@@ -2382,6 +2396,11 @@
           <t>Kampanyadan yalnızca bir kez yararlanılabilir</t>
         </is>
       </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 20.07.2026 - 31.12.2026</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
@@ -2473,7 +2492,11 @@
       </c>
       <c r="X14" s="2" t="inlineStr">
         <is>
-          <t>erteleme_suresi_ay: 3 aya varan ödemesiz dönem ve 4 taksitli</t>
+          <t>erteleme_suresi_ay: 3 aya varan ödemesiz dönem ve 4 taksitli
+kampanya_baslangic: 1 Ocak 2026 – 31 Aralık 2026
+kampanya_bitis: 1 Ocak 2026 – 31 Aralık 2026
+kar_payi_orani: %0 kâr payı ile 40.000 TL’ye kadar
+taksit_sayisi: 1 Ocak 2026 – 31 Aralık 2026</t>
         </is>
       </c>
     </row>
@@ -2559,6 +2582,13 @@
       </c>
       <c r="V15" t="n">
         <v>3</v>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
+taksit_sayisi: üzerinden kredi kartınızla vade farksız 3 taksit ile gerçekleştirebilirsiniz.</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
@@ -2722,6 +2752,11 @@
           <t>Ödül davet edilenin görüntülü görüşmeyle müşteri olmasına bağlı, başka kanaldan olursa ödül yok</t>
         </is>
       </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya 31 Aralık 2026 tarihine kadar geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="19" t="inlineStr">
@@ -2808,6 +2843,12 @@
       <c r="V18" t="n">
         <v>6</v>
       </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 1 – 31 Temmuz 2026
+kampanya_bitis: 1 – 31 Temmuz 2026</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
@@ -2893,6 +2934,12 @@
       </c>
       <c r="V19" t="n">
         <v>6</v>
+      </c>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 1 Temmuz 2026 -30 Eylül 2026
+kampanya_bitis: 1 Temmuz 2026 -30 Eylül 2026</t>
+        </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
@@ -3702,6 +3749,11 @@
           <t>Tutar maaş dilimine göre kademeli (18.000-32.000 TL); en üst dilimi (20.000 TL+) alındı</t>
         </is>
       </c>
+      <c r="X29" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: ​​​​​​​​​​​​​​​​​​​Emeklilere 32.000TL’ye Varan Nakit Promosyon, Bonus ve Ödül Türkiye Finans’ta! ​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​​</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="19" t="inlineStr">
@@ -3955,7 +4007,9 @@
       <c r="X32" s="2" t="inlineStr">
         <is>
           <t>erteleme_suresi_ay: 400.000 TL'ye Kadar İhtiyaç Finansmanı Kullanın, 3 Ay Öteleme Fırsatından Yararlanın!
-masraf_durumu: Üstelik temel bankacılık işlemleriniz için masraf ödemeyin.</t>
+masraf_durumu: Üstelik temel bankacılık işlemleriniz için masraf ödemeyin.
+finansman_tutari: 400.000 TL'ye Kadar İhtiyaç Finansmanı Kullanın, 3 Ay Öteleme Fırsatından Yararlanın!
+vade_ay: Finansman tutarının 250.000 TL’ye kadar olması durumunda maksimum 24 ay,</t>
         </is>
       </c>
     </row>
@@ -4272,6 +4326,12 @@
           <t>E-ticaret islemleri kapsam disi; kampanyaya onceden katilim sart</t>
         </is>
       </c>
+      <c r="X36" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 10 Temmuz 2026 - 7 Ağustos 2026
+kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="19" t="inlineStr">
@@ -4514,6 +4574,12 @@
           <t>Sadece havayolu firmalarinin kendi kanallari gecerli, araci bilet siteleri haric</t>
         </is>
       </c>
+      <c r="X39" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 10 Temmuz 2026 - 7 Ağustos 2026
+kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="19" t="inlineStr">
@@ -4676,6 +4742,13 @@
           <t>Odul yalnizca 4. harcamada tek seferde veriliyor, kademeli degil</t>
         </is>
       </c>
+      <c r="X41" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 10 Temmuz 2026 - 7 Ağustos 2026
+kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026
+odul_miktari: en fazla 400 TL Bankkart Lira</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="19" t="inlineStr">
@@ -4757,6 +4830,12 @@
           <t>Surdurulebilirlik/elektrikli arac temali kampanya, %20 orani odul hesaplama sekli - kar_payi_orani degil</t>
         </is>
       </c>
+      <c r="X42" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 10 Temmuz 2026 - 7 Ağustos 2026
+kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="19" t="inlineStr">
@@ -4838,6 +4917,12 @@
           <t>Sadece ilk harcamaya uygulaniyor, oran tabanli (%10) sabit tutar degil</t>
         </is>
       </c>
+      <c r="X43" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 14 Temmuz - 31 Temmuz 2026 tarihleri arasında Emlak Katılım Mobil’den gerçekleştirilen ödemeler için geçerlidir.
+kampanya_bitis: Kampanya 14 Temmuz - 31 Temmuz 2026 tarihleri arasında Emlak Katılım Mobil’den gerçekleştirilen ödemeler için geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="19" t="inlineStr">
@@ -4919,6 +5004,12 @@
           <t>SMS ile onceden katilim sart (GIDA yazip 6026'ya)</t>
         </is>
       </c>
+      <c r="X44" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="28" customHeight="1">
       <c r="A45" s="19" t="inlineStr">
@@ -4998,6 +5089,12 @@
       <c r="U45" s="20" t="inlineStr">
         <is>
           <t>SMS ile onceden katilim sart (AKARYAKIT yazip 6026'ya)</t>
+        </is>
+      </c>
+      <c r="X45" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 1 -31 Temmuz 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 1 -31 Temmuz 2026 tarihleri arasında geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -5767,6 +5864,11 @@
       <c r="V55" t="n">
         <v>9</v>
       </c>
+      <c r="X55" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="19" t="inlineStr">
@@ -5848,6 +5950,11 @@
       </c>
       <c r="V56" t="n">
         <v>3</v>
+      </c>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>finansman_tutari: Peşin fiyatına 3 taksit uygulaması sepet toplamı 2.000 TL ve üzeri siparişlerde geçerlidir.</t>
+        </is>
       </c>
     </row>
     <row r="57" ht="28" customHeight="1">
@@ -5930,6 +6037,12 @@
           <t>Nisan ayi kampanyasinin devami, onceki kazanimlar dahil; ayrica davet edilenin kendisi de 1.000 TL+ para transferiyle 500 TL kazaniyor</t>
         </is>
       </c>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 16 Haziran - 31 Ağustos 2026
+odul_miktari: Davet eden kişi, davet ettiği kişinin kampanya koşullarını sağlaması halinde kişi başı maksimum 500 TL, toplamda 50 kişi için maksimum 25.000 TL nakit ödül kazanabilir.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="19" t="inlineStr">
@@ -6009,6 +6122,12 @@
       <c r="U58" s="20" t="inlineStr">
         <is>
           <t>Sadece ilgili platformlarin resmi sitesi/uygulamasi uzerinden yapilan odemeler gecerli</t>
+        </is>
+      </c>
+      <c r="X58" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 16 Haziran - 31 Ağustos 2026
+odul_miktari: kapsamınca kazanılabilecek maksimum nakit ödül tutarı toplamda 300 TL’dir.</t>
         </is>
       </c>
     </row>
@@ -8072,7 +8191,9 @@
           <t>finansman_tutari: Vade farksız 40.000 TL ve uygun oranlı hoş geldin finansmanı Albaraka'da!
 vade_ay: ’lı olan dijital müşterilerimize özel; vade farksız, azami 40.000 TL limitli, 3 aya varan ödemesiz dönem ve 4 taksit imkânı ile birlikte toplam 6 aya varan vade imkanıyla sunulan Pratik Fina
 taksit_sayisi: ’lı olan dijital müşterilerimize özel; vade farksız, azami 40.000 TL limitli, 3 aya varan ödemesiz dönem ve 4 taksit imkânı ile birlikte toplam 6 aya varan vade imkanıyla sunulan Pratik Fina
-erteleme_suresi_ay: ’lı olan dijital müşterilerimize özel; vade farksız, azami 40.000 TL limitli, 3 aya varan ödemesiz dönem ve 4 taksit imkânı ile birlikte toplam 6 aya varan vade imkanıyla sunulan Pratik Fina</t>
+erteleme_suresi_ay: ’lı olan dijital müşterilerimize özel; vade farksız, azami 40.000 TL limitli, 3 aya varan ödemesiz dönem ve 4 taksit imkânı ile birlikte toplam 6 aya varan vade imkanıyla sunulan Pratik Fina
+kampanya_baslangic: 01.01.2026 - 31.12.2026
+kampanya_bitis: 01.01.2026 - 31.12.2026</t>
         </is>
       </c>
     </row>
@@ -9686,27 +9807,220 @@
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="24" t="n"/>
-      <c r="B107" s="24" t="n"/>
-      <c r="C107" s="24" t="n"/>
-      <c r="D107" s="24" t="n"/>
-      <c r="E107" s="24" t="n"/>
+      <c r="A107" s="24" t="inlineStr">
+        <is>
+          <t>TOM-004</t>
+        </is>
+      </c>
+      <c r="B107" s="24" t="inlineStr">
+        <is>
+          <t>T.O.M. Katılım</t>
+        </is>
+      </c>
+      <c r="C107" s="24" t="inlineStr">
+        <is>
+          <t>Toplam 1.500 TL Hoş Geldin Hediyesi (TOM1500)</t>
+        </is>
+      </c>
+      <c r="D107" s="24" t="inlineStr">
+        <is>
+          <t>Yeni Musteri Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E107" s="24" t="inlineStr">
+        <is>
+          <t>hadiyanindakibanka.com/kampanyalar/toplam-1500-tl-hos-geldin-hediyesi-tom1500-koduyla-musterimiz-ol-1500-tl-senin-olsun</t>
+        </is>
+      </c>
       <c r="F107" s="25" t="n"/>
       <c r="G107" s="25" t="n"/>
       <c r="H107" s="24" t="n"/>
       <c r="I107" s="26" t="n"/>
       <c r="J107" s="25" t="n"/>
-      <c r="K107" s="25" t="n"/>
-      <c r="L107" s="24" t="n"/>
-      <c r="M107" s="24" t="n"/>
+      <c r="K107" s="25" t="n">
+        <v>1500</v>
+      </c>
+      <c r="L107" s="24" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M107" s="24" t="inlineStr">
+        <is>
+          <t>TOM1500 davet koduyla ilk kez müşteri olanlara, Hadi Black kartla 1.000 TL üzeri beş harcamada kademeli olarak toplam 1.500 TL Hediye Bakiye</t>
+        </is>
+      </c>
       <c r="N107" s="24" t="n"/>
-      <c r="O107" s="27" t="n"/>
-      <c r="P107" s="27" t="n"/>
-      <c r="Q107" s="24" t="n"/>
+      <c r="O107" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="P107" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q107" s="24" t="inlineStr">
+        <is>
+          <t>TOM1500 davet koduyla görüntülü görüşmeyle ilk kez TOM Bank müşterisi olanlar</t>
+        </is>
+      </c>
       <c r="R107" s="24" t="n"/>
       <c r="S107" s="24" t="n"/>
-      <c r="T107" s="27" t="n"/>
-      <c r="U107" s="24" t="n"/>
+      <c r="T107" s="27" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="U107" s="24" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Odul KADEMELI: 1.000 TL uzeri her harcamada sirasiyla 100/200/300/400/500 TL; odul_miktari TOPLAM TAVANDIR. 1.000 TL bir ALT ESIKTIR, finansman tutari degil. Kampanya kisiye ozel - yalnizca secili kitleye duyurulmus.</t>
+        </is>
+      </c>
+      <c r="X107" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: 1.500 TL Hediye Bakiye
+kampanya_baslangic: 20.8.2026 – 31.8.2026
+kampanya_bitis: 20.8.2026 – 31.8.2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>TOM-005</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>T.O.M. Katılım</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Hadi Alışveriş Kredisi ile Klima, Süpürge ve Televizyonlarda Vade Farksız 12 Taksit</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Finansman Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>hadiyanindakibanka.com/kampanyalar/hadi-alisveris-kredisi-ile-klima-supurge-ve-televizyonlarda-vade-farksiz-12-taksit</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>A101 Ekstra'da 5.000 TL üzeri klima/süpürge/televizyon alışverişlerinde vade farksız 12 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>Hadi Taksitli Kredi limiti yeterli olan TOM Bank müşterileri</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Taksit kademeleri 3-6-9-12; en yuksek kademe yazildi. 5.000 TL ALT ESIKTIR, finansman tutari degil. Yalnizca A101 Ekstra ve yalnizca klima/supurge/televizyon kategorisi.</t>
+        </is>
+      </c>
+      <c r="V108" t="n">
+        <v>12</v>
+      </c>
+      <c r="X108" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Peşin fiyatına taksit sayısı sadece 12 taksite kadar sınırlıdır.
+kampanya_baslangic: 08 Ağustos - 31 Ağustos 2026
+kampanya_bitis: 08 Ağustos - 31 Ağustos 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>TOM-006</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>T.O.M. Katılım</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>MTV Ödemelerinde Vade Farksız 3 Taksit</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>hadiyanindakibanka.com/kampanyalar/vergi-kampanyasi</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>Hadi Black kartla 1.000-30.000 TL arası vergi ödemelerinde vade farksız 3 taksit</t>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P109" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q109" t="inlineStr">
+        <is>
+          <t>Hadi Black Kredi Kartı sahipleri (uygulamadan kampanyaya katılanlar)</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Ekstre donemi basina EN FAZLA BIR vergi odemesi taksitlendirilir. Katilim islemden ONCE uygulamadan yapilmali.</t>
+        </is>
+      </c>
+      <c r="V109" t="n">
+        <v>3</v>
+      </c>
+      <c r="X109" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Kampanya kapsamında vergi ödemesi kategorisinde tek seferde gerçekleştirilen 1.000 TL ile 30.000 TL arasındaki işlemler vade farksız 3 taksite bölünür.
+finansman_tutari: Kampanya kapsamında vergi ödemesi kategorisinde tek seferde gerçekleştirilen 1.000 TL ile 30.000 TL arasındaki işlemler vade farksız 3 taksite bölünür.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U1"/>

</xml_diff>

<commit_message>
gecerlilik tarihi kalibinin kacirdigi uc kayit duzeltildi, tarih bekcisi eklendi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -3974,8 +3974,16 @@
           <t>Temel bankacılık işlemlerinde masraf yok</t>
         </is>
       </c>
-      <c r="O32" s="23" t="n"/>
-      <c r="P32" s="23" t="n"/>
+      <c r="O32" s="23" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="P32" s="23" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
       <c r="Q32" s="20" t="inlineStr">
         <is>
           <t>Mobilden yeni müşteri olanlar</t>
@@ -3998,7 +4006,7 @@
       </c>
       <c r="U32" s="20" t="inlineStr">
         <is>
-          <t>Bitis tarihi sayfada belirtilmemis, sureklen bir paket gibi gorunuyor - bos birakildi DUZELTME (23 Agustos 2026): erteleme_suresi_ay=3, finansman_tutari=400000 ve vade_ay=24 eklendi. Vade KADEMELI (250.000 TL'ye kadar 24 ay, fazlasi 12 ay); TF-008 ile ayni kural: en yuksek kademe yazilir. masraf_durumu eklendi: sayfa 'temel bankacilik islemleriniz icin masraf odemeyin' diyor. TF-007 ('Masrafsiz Bankacilik') NEREDEYSE AYNI cumleyi masraf_durumu'na yazmisti; iki kayit celisiyordu.</t>
+          <t>DUZELTME (23 Agustos 2026): erteleme_suresi_ay=3, finansman_tutari=400000 ve vade_ay=24 eklendi. Vade KADEMELI (250.000 TL'ye kadar 24 ay, fazlasi 12 ay); TF-008 ile ayni kural: en yuksek kademe yazilir. masraf_durumu eklendi: sayfa 'temel bankacilik islemleriniz icin masraf odemeyin' diyor. TF-007 ('Masrafsiz Bankacilik') NEREDEYSE AYNI cumleyi masraf_durumu'na yazmisti; iki kayit celisiyordu. DUZELTME (23 Agustos 2026): kampanya_baslangic/bitis eklendi. ONCEKI NOT YANLISTI: 'bitis tarihi sayfada belirtilmemis, sureklen bir paket gibi gorunuyor' deniyordu; sayfa 'Kampanyadan 1 Agustos - 31 Agustos 2026 tarihleri arasinda yararlanabilirsiniz' diyor.</t>
         </is>
       </c>
       <c r="W32" t="n">
@@ -4009,7 +4017,9 @@
           <t>erteleme_suresi_ay: 400.000 TL'ye Kadar İhtiyaç Finansmanı Kullanın, 3 Ay Öteleme Fırsatından Yararlanın!
 masraf_durumu: Üstelik temel bankacılık işlemleriniz için masraf ödemeyin.
 finansman_tutari: 400.000 TL'ye Kadar İhtiyaç Finansmanı Kullanın, 3 Ay Öteleme Fırsatından Yararlanın!
-vade_ay: Finansman tutarının 250.000 TL’ye kadar olması durumunda maksimum 24 ay,</t>
+vade_ay: Finansman tutarının 250.000 TL’ye kadar olması durumunda maksimum 24 ay,
+kampanya_baslangic: Kampanyadan 1 Ağustos - 31 Ağustos 2026 tarihleri arasında yararlanabilirsiniz.
+kampanya_bitis: Kampanyadan 1 Ağustos - 31 Ağustos 2026 tarihleri arasında yararlanabilirsiniz.</t>
         </is>
       </c>
     </row>
@@ -7030,8 +7040,16 @@
         </is>
       </c>
       <c r="N70" s="24" t="n"/>
-      <c r="O70" s="27" t="n"/>
-      <c r="P70" s="27" t="n"/>
+      <c r="O70" s="27" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
+      <c r="P70" s="27" t="inlineStr">
+        <is>
+          <t>2029-12-31</t>
+        </is>
+      </c>
       <c r="Q70" s="24" t="inlineStr">
         <is>
           <t>Vakıf Katılım bireysel müşterileri</t>
@@ -7044,12 +7062,17 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U70" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfadaki tek sayi 'en az 6 kriter' olup katilim sartidir, taksit/odul degil. Odul tutari sayfada yok (mobil uygulamada gosteriliyor). Kampanya suresiz - her ay basinda kriterler sifirlaniyor.</t>
-        </is>
-      </c>
-      <c r="X70" s="2" t="n"/>
+      <c r="U70" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfadaki tek sayi 'en az 6 kriter' olup katilim sartidir, taksit/odul degil. Odul tutari sayfada yok (mobil uygulamada gosteriliyor). Kampanya suresiz - her ay basinda kriterler sifirlaniyor. DUZELTME (23 Agustos 2026): kampanya_baslangic/bitis eklendi. Sayfa 'Kampanya Gecerlilik Tarihi' basligi altinda veriyor; denetim kalibi yalnizca 'Kampanya Donemi' ve 'tarihleri arasinda' ifadelerini ariyordu, bu yazimi kaciriyordu.</t>
+        </is>
+      </c>
+      <c r="X70" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 01 Temmuz 2025 - 31 Aralık 2029
+kampanya_bitis: 01 Temmuz 2025 - 31 Aralık 2029</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="24" t="inlineStr">
@@ -7332,7 +7355,7 @@
       <c r="P74" s="27" t="n"/>
       <c r="Q74" s="24" t="inlineStr">
         <is>
-          <t>Hayat Finans müşterileri (mobil uygulamadan GastroClub üyeliği oluşturanlar)</t>
+          <t>Yalnızca bireysel Hayat Finans müşterileri (mobil uygulamadan GastroClub üyeliği oluşturanlar)</t>
         </is>
       </c>
       <c r="R74" s="24" t="n"/>
@@ -7342,12 +7365,16 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U74" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %10-%50 anlasmali isyeri INDIRIMIDIR, kar payi orani degil. Kampanya tarihi sayfada YOK.</t>
-        </is>
-      </c>
-      <c r="X74" s="2" t="n"/>
+      <c r="U74" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %10-%50 anlasmali isyeri INDIRIMIDIR, kar payi orani degil. Kampanya tarihi sayfada YOK. DUZELTME (23 Agustos 2026): hedef_kitle 'YALNIZCA BIREYSEL' olarak kesinlestirildi ve kanit cumlesi eklendi. Tarih alanlari BOS DOGRU: sayfada hicbir tarih izi yok (genislettigim kalipla yeniden tarandi).</t>
+        </is>
+      </c>
+      <c r="X74" s="2" t="inlineStr">
+        <is>
+          <t>hedef_kitle: Sadece bireysel Hayat Finans müşterileri yararlanabilir.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="24" t="inlineStr">
@@ -7465,8 +7492,16 @@
         </is>
       </c>
       <c r="N76" s="24" t="n"/>
-      <c r="O76" s="27" t="n"/>
-      <c r="P76" s="27" t="n"/>
+      <c r="O76" s="27" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="P76" s="27" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
       <c r="Q76" s="24" t="inlineStr">
         <is>
           <t>Aktif Vakıf Katılım kredi veya banka kartı kullanan müşteriler</t>
@@ -7479,12 +7514,17 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="U76" s="24" t="inlineStr">
-        <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfa indirim orani VERMIYOR ('musteri ozelinde degisiklik gosterebilmektedir'). Tarih de yok. GastroClub is birligi - HF-007 ile ayni platform, farkli banka.</t>
-        </is>
-      </c>
-      <c r="X76" s="2" t="n"/>
+      <c r="U76" s="33" t="inlineStr">
+        <is>
+          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfa indirim orani VERMIYOR ('musteri ozelinde degisiklik gosterebilmektedir'). Tarih de yok. GastroClub is birligi - HF-007 ile ayni platform, farkli banka. DUZELTME (23 Agustos 2026): kampanya_baslangic/bitis eklendi ('Kampanya Gecerlilik Tarihi').</t>
+        </is>
+      </c>
+      <c r="X76" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 22 Nisan 2026 - 31 Aralık 2026
+kampanya_bitis: 22 Nisan 2026 - 31 Aralık 2026</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="24" t="inlineStr">

</xml_diff>

<commit_message>
dayanagi olmayan tarihler bosaltildi, iki kaynak JS ile tazelendi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -2156,7 +2156,8 @@
       <c r="X10" s="2" t="inlineStr">
         <is>
           <t>taksit_sayisi: Kampanya kapsamında Kutsal toprakları ziyaret etmek isteyen müşterilerimiz toplam umre tutarının en fazla yüzde altmışı için vade farksız 3 taksit imkanından yararlanabilir.
-kampanya_baslangic: 13.08.2024 - 1.01.2027</t>
+kampanya_baslangic: 13.08.2024 - 1.01.2027
+kampanya_bitis: 13.08.2024 - 1.01.2027</t>
         </is>
       </c>
     </row>
@@ -2728,11 +2729,7 @@
         </is>
       </c>
       <c r="N17" s="20" t="n"/>
-      <c r="O17" s="23" t="inlineStr">
-        <is>
-          <t>2024-04-14</t>
-        </is>
-      </c>
+      <c r="O17" s="23" t="n"/>
       <c r="P17" s="23" t="inlineStr">
         <is>
           <t>2026-12-31</t>
@@ -2755,12 +2752,13 @@
       </c>
       <c r="T17" s="23" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="U17" s="20" t="inlineStr">
         <is>
-          <t>Ödül davet edilenin görüntülü görüşmeyle müşteri olmasına bağlı, başka kanaldan olursa ödül yok</t>
+          <t>Ödül davet edilenin görüntülü görüşmeyle müşteri olmasına bağlı, başka kanaldan olursa ödül yok
+2026-08-23: baslangic tarihi kaynak sayfada gecmiyor; bitis (31 Aralik 2026) sayfada dogrulandi</t>
         </is>
       </c>
       <c r="X17" s="2" t="inlineStr">
@@ -3608,6 +3606,12 @@
           <t>Odul parasal degil (1 aylik tabii Premium uyelik) - odul_miktari/odul_birimi semaya uymadigi icin bos birakildi, detay kampanya_avantaji alaninda. Musteri basina 1 kez</t>
         </is>
       </c>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: 08 Mayıs 2026 - 30 Kasım 2026
+kampanya_baslangic: 08 Mayıs 2026 - 30 Kasım 2026</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="28.05" customHeight="1">
       <c r="A28" s="19" t="inlineStr">
@@ -4492,11 +4496,7 @@
         </is>
       </c>
       <c r="N38" s="20" t="n"/>
-      <c r="O38" s="23" t="inlineStr">
-        <is>
-          <t>2025-08-18</t>
-        </is>
-      </c>
+      <c r="O38" s="23" t="n"/>
       <c r="P38" s="23" t="inlineStr">
         <is>
           <t>2026-08-09</t>
@@ -4525,7 +4525,8 @@
       <c r="U38" s="20" t="inlineStr">
         <is>
           <t>vade_ay alani burada net degil: kampanya 'mevcut 2-4 taksite +8 ekliyor' diyor (toplamda 10-12 taksit gibi), tekil bir sayi degil - bos birakildi DUZELTME (23 Agustos 2026): taksit_sayisi=8 eklendi. Kampanya 2-4 taksitli islemlere +8 taksit EKLIYOR; 8, kampanyanin kendi kattigi taksit sayisidir (baslik da oyle diyor).
-2026-08-23: kampanya rotasyonu - tarih kaynak sayfadan yeniden okundu (Kampanya 09-08-2026 Tarihinde Sona Ermiştir.)</t>
+2026-08-23: kampanya rotasyonu - tarih kaynak sayfadan yeniden okundu (Kampanya 09-08-2026 Tarihinde Sona Ermiştir.)
+2026-08-23: baslangic tarihi kaynak sayfada gecmiyor; kampanya 09-08-2026'da sona ermis</t>
         </is>
       </c>
       <c r="V38" t="n">
@@ -4533,7 +4534,8 @@
       </c>
       <c r="X38" s="2" t="inlineStr">
         <is>
-          <t>taksit_sayisi: +8 taksit!</t>
+          <t>taksit_sayisi: +8 taksit!
+kampanya_bitis: Kampanya 09-08-2026 Tarihinde Sona Ermiştir.</t>
         </is>
       </c>
     </row>
@@ -5588,16 +5590,8 @@
         </is>
       </c>
       <c r="N51" s="20" t="n"/>
-      <c r="O51" s="23" t="inlineStr">
-        <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="P51" s="23" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
+      <c r="O51" s="23" t="n"/>
+      <c r="P51" s="23" t="n"/>
       <c r="Q51" s="20" t="inlineStr">
         <is>
           <t>Mevcut müşteriler (davet eden), davet edilen yeni müşteriler</t>
@@ -5615,12 +5609,13 @@
       </c>
       <c r="T51" s="23" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="U51" s="20" t="inlineStr">
         <is>
-          <t>Hem davet eden hem davet edilenin Paraf Kart basvurusu sart; 0,1 gram x 10 davet = 1 gram ust sinir</t>
+          <t>Hem davet eden hem davet edilenin Paraf Kart basvurusu sart; 0,1 gram x 10 davet = 1 gram ust sinir
+2026-08-23: sayfada kampanya tarihi hic verilmiyor</t>
         </is>
       </c>
     </row>
@@ -10307,7 +10302,9 @@
       <c r="X109" s="2" t="inlineStr">
         <is>
           <t>taksit_sayisi: Kampanya kapsamında vergi ödemesi kategorisinde tek seferde gerçekleştirilen 1.000 TL ile 30.000 TL arasındaki işlemler vade farksız 3 taksite bölünür.
-finansman_tutari: Kampanya kapsamında vergi ödemesi kategorisinde tek seferde gerçekleştirilen 1.000 TL ile 30.000 TL arasındaki işlemler vade farksız 3 taksite bölünür.</t>
+finansman_tutari: Kampanya kapsamında vergi ödemesi kategorisinde tek seferde gerçekleştirilen 1.000 TL ile 30.000 TL arasındaki işlemler vade farksız 3 taksite bölünür.
+kampanya_bitis: Kampanya, 1 Temmuz 2026 – 31 Ağustos2026 tarihleri arasında Hadi Black Kredi Kartı ile gerçekleştirilecek vergi ödemelerinde geçerlidir.
+kampanya_baslangic: Kampanya, 1 Temmuz 2026 – 31 Ağustos2026 tarihleri arasında Hadi Black Kredi Kartı ile gerçekleştirilecek vergi ödemelerinde geçerlidir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
11 taslak kayda kaynaga dayali aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -12474,14 +12474,33 @@
           <t>Secili Okullarda Pesin Odemelerinize 5e Varan Taksit</t>
         </is>
       </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E187" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/secili-okullarda-pesin-odemelerinize-5e-varan-taksit</t>
         </is>
       </c>
-      <c r="U187" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>Secili okullarda pesin okul odemelerinin tutara gore 4 veya 5 taksite bolunmesi; anlasmali okullarda ek 6 taksit</t>
+        </is>
+      </c>
+      <c r="Q187" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U187" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ taksit_sayisi: metin uc ayri deger veriyor: 250 bin-1 milyon arasi 4 taksit, 1 milyon uzeri 5 taksit, anlasmali okullarda +6 taksit - tek deger secilemez
+BELIRSIZ finansman_tutari: 250 bin / 1 milyon TL islem ESIKLERI, kampanyanin finansman tutari degil
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
     </row>
@@ -13257,14 +13276,45 @@
           <t>Paraf ile İpekyol’da 4 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E216" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-ipekyolda-4-taksit-firsati</t>
         </is>
       </c>
-      <c r="U216" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>Ipekyol magazalari ve web sitesinde Paraf POS'larindan yapilan 5.000 TL uzeri alisverislerde 4 taksit</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U216" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor ('31 Agustos 2026 tarihine kadar')
+BELIRSIZ finansman_tutari: 5.000 TL bir harcama ESIGI, kampanyanin finansman tutari degil (Rehber J sutunu)</t>
+        </is>
+      </c>
+      <c r="V216" t="n">
+        <v>4</v>
+      </c>
+      <c r="X216" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar İpekyol mağazaları ve www.ipekyol.com.tr’de Paraf POS’larından yapılacak 5.000 TL üzeri alışverişlerde 4 taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar İpekyol mağazaları ve www.ipekyol.com.tr’de Paraf POS’larından yapılacak 5.000 TL üzeri alışverişlerde 4 taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -13311,14 +13361,41 @@
           <t>The House Cafelerde Tatli Ikrami</t>
         </is>
       </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E218" t="inlineStr">
         <is>
           <t>https://www.albaraka.com.tr/tr/kampanyalar/detay/2026/the-house-cafelerde-tatli-ikrami</t>
         </is>
       </c>
-      <c r="U218" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>The House Cafe'lerde ana yemek siparisi sonrasi tatli ikrami, ayda en fazla 2 kez</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil uzerinden GastroClub kodu alan musteriler</t>
+        </is>
+      </c>
+      <c r="U218" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ odul_miktari: odul ayni (tatli ikrami), parasal tutar verilmiyor; 'ayda en fazla 2 kere' bir KULLANIM LIMITI, odul tutari degil</t>
+        </is>
+      </c>
+      <c r="X218" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya 31.12.2026 tarihine kadar geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -13878,14 +13955,40 @@
           <t>Koctasta 5 Taksit</t>
         </is>
       </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E239" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/koctasta-5-taksit</t>
         </is>
       </c>
-      <c r="U239" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>koctas.com.tr'den yapilan 10.000 TL ve uzeri alisverislerde pesin fiyatina 5 taksit; magaza islemleri haric</t>
+        </is>
+      </c>
+      <c r="Q239" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U239" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor
+BELIRSIZ finansman_tutari: 10.000 TL bir harcama ESIGI, kampanyanin finansman tutari degil (Rehber J sutunu)</t>
+        </is>
+      </c>
+      <c r="V239" t="n">
+        <v>5</v>
+      </c>
+      <c r="X239" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: peşin fiyatına 5 taksit</t>
         </is>
       </c>
     </row>
@@ -14499,14 +14602,39 @@
           <t>Bridgestoneda 5 Taksit</t>
         </is>
       </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E262" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/bridgestoneda-5-taksit</t>
         </is>
       </c>
-      <c r="U262" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>Bridgestone'da Bankkart POS'undan yapilan alisverislerde pesin fiyatina 5 taksit</t>
+        </is>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U262" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
+      <c r="V262" t="n">
+        <v>5</v>
+      </c>
+      <c r="X262" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: peşin fiyatına 5 taksit</t>
         </is>
       </c>
     </row>
@@ -14715,14 +14843,44 @@
           <t>Paraf ile Divarese’de 4 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E270" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-divaresede-4-taksit-firsati</t>
         </is>
       </c>
-      <c r="U270" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>Divarese magazalari ve web sitesinde Paraf POS'larindan yapilan alisverislerde 4 taksit</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q270" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U270" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor ('31 Agustos 2026 tarihine kadar')</t>
+        </is>
+      </c>
+      <c r="V270" t="n">
+        <v>4</v>
+      </c>
+      <c r="X270" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Divarese mağazaları ve www.divarese.com.tr’de Paraf POS’larından yapılacak alışverişlerde 4 taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Divarese mağazaları ve www.divarese.com.tr’de Paraf POS’larından yapılacak alışverişlerde 4 taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -14985,14 +15143,39 @@
           <t>Dysonda 9 Taksit</t>
         </is>
       </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E280" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/dysonda-9-taksit</t>
         </is>
       </c>
-      <c r="U280" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>dyson.com.tr'den yapilan alisverislerde pesin fiyatina 9 taksit; magaza islemleri haric</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U280" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor (metnin tamami okundu)
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor (metnin tamami okundu)</t>
+        </is>
+      </c>
+      <c r="V280" t="n">
+        <v>9</v>
+      </c>
+      <c r="X280" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: peşin fiyatına 9 taksit fırsatından yararlanabilirsiniz.</t>
         </is>
       </c>
     </row>
@@ -15687,14 +15870,39 @@
           <t>Paraf ile Schafer’de Peşin Fiyatına 9 Taksit!</t>
         </is>
       </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E306" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-schaferde-pesin-fiyatina-9-taksit</t>
         </is>
       </c>
-      <c r="U306" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>Schafer magazalarinda ParafPOS'lardan yapilan alisverislerde vade farksiz 9 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U306" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
+      <c r="V306" t="n">
+        <v>9</v>
+      </c>
+      <c r="X306" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Paraf ile Schafer mağazalarında ParafPOS’larından yapacağınız alışverişlerde vade farksız 9 aya varan taksit imkanı sağlanacaktır.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
on taslak kayda daha aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -12871,14 +12871,44 @@
           <t>Paraf ile ADV Mağazalarında 6 Taksit!</t>
         </is>
       </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E201" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-adv-magazalarinda-6-taksit</t>
         </is>
       </c>
-      <c r="U201" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>ADV magazalarinda Paraf POS'larindan yapilan alisverislerde 6 taksit</t>
+        </is>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri; debit kartlar ve ParafPara haric</t>
+        </is>
+      </c>
+      <c r="U201" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V201" t="n">
+        <v>6</v>
+      </c>
+      <c r="X201" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Aralık 2026 tarihine kadar ADV mağazalarında Paraf POS’larından yapılacak alışverişlerde 6 taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Aralık 2026 tarihine kadar ADV mağazalarında Paraf POS’larından yapılacak alışverişlerde 6 taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -13469,14 +13499,44 @@
           <t>Paraf Ile Kipte 5 Taksit</t>
         </is>
       </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E221" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-kipte-5-taksit</t>
         </is>
       </c>
-      <c r="U221" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>KIP magazalari ve web sitesinde Paraf POS'larindan yapilan alisverislerde 5 taksit</t>
+        </is>
+      </c>
+      <c r="P221" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q221" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri; debit kartlar ve ParafPara haric</t>
+        </is>
+      </c>
+      <c r="U221" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V221" t="n">
+        <v>5</v>
+      </c>
+      <c r="X221" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar KİP mağazaları ve www.kip.com.tr’de Paraf POS’larından yapılacak alışverişlerde 5 taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar KİP mağazaları ve www.kip.com.tr’de Paraf POS’larından yapılacak alışverişlerde 5 taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -13712,14 +13772,44 @@
           <t>Paraf ile Network’te 4 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E230" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-networkte-4-taksit-firsati</t>
         </is>
       </c>
-      <c r="U230" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>Network magazalari ve web sitesinde Paraf POS'larindan yapilan alisverislerde 4 taksit</t>
+        </is>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q230" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri; debit kartlar ve ParafPara haric</t>
+        </is>
+      </c>
+      <c r="U230" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V230" t="n">
+        <v>4</v>
+      </c>
+      <c r="X230" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Network mağazaları ve www.network.com.tr’de Paraf POS’larından yapılacak alışverişlerde 4 taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Network mağazaları ve www.network.com.tr’de Paraf POS’larından yapılacak alışverişlerde 4 taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -14575,60 +14665,85 @@
           <t>Paraf ile Alfemo’da 8 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E261" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-alfemoda-8-taksit-firsati</t>
         </is>
       </c>
-      <c r="U261" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t>ZK-047</t>
-        </is>
-      </c>
-      <c r="B262" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C262" t="inlineStr">
-        <is>
-          <t>Bridgestoneda 5 Taksit</t>
-        </is>
-      </c>
-      <c r="D262" t="inlineStr">
-        <is>
-          <t>Kart Kampanyasi</t>
-        </is>
-      </c>
-      <c r="E262" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/bridgestoneda-5-taksit</t>
-        </is>
-      </c>
-      <c r="M262" t="inlineStr">
-        <is>
-          <t>Bridgestone'da Bankkart POS'undan yapilan alisverislerde pesin fiyatina 5 taksit</t>
-        </is>
-      </c>
-      <c r="Q262" t="inlineStr">
-        <is>
-          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
-        </is>
-      </c>
-      <c r="U262" s="2" t="inlineStr">
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>Alfemo magazalari ve web sitesinde Paraf POS'larindan yapilan alisverislerde 8 taksit</t>
+        </is>
+      </c>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U261" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
 BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
+      <c r="V261" t="n">
+        <v>8</v>
+      </c>
+      <c r="X261" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Paraf ile Alfemo mağazalarında veya www.alfemo.com web sayfasından Paraf POS’larından yapacağınız alışverişlerde 8 taksit imkanı sağlanacaktır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>ZK-047</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Bridgestoneda 5 Taksit</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/bridgestoneda-5-taksit</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>Bridgestone'da Bankkart POS'undan yapilan alisverislerde pesin fiyatina 5 taksit</t>
+        </is>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U262" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
       <c r="V262" t="n">
         <v>5</v>
       </c>
@@ -14708,14 +14823,40 @@
           <t>Bankamız ve CHAKRA MAĞAZACILIK TİCARET VE A.Ş kampanya koşullarında değişiklik y</t>
         </is>
       </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E265" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/chakrada-6-taksit-0</t>
         </is>
       </c>
-      <c r="U265" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>Chakra magazalari ve chakra.com.tr'de yapilan alisverislerde pesin fiyatina 6 taksit</t>
+        </is>
+      </c>
+      <c r="Q265" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U265" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_adi: korpustan gelen baslik bozuk - sayfa metninin son cumlesi baslik olarak alinmis, imzalamadan once duzeltilmeli</t>
+        </is>
+      </c>
+      <c r="V265" t="n">
+        <v>6</v>
+      </c>
+      <c r="X265" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: da yapacağınız alışverişlerinizde peşin fiyatına 6 taksit fırsatından faydalanabilirsiniz.</t>
         </is>
       </c>
     </row>
@@ -15384,14 +15525,44 @@
           <t>Paraf ile Koçtaş’ta 5 Taksit!</t>
         </is>
       </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E288" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-koctasta-5-taksit</t>
         </is>
       </c>
-      <c r="U288" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Koctas'ta Paraf POS'undan yapilan alisverislerde 5 taksit</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U288" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V288" t="n">
+        <v>5</v>
+      </c>
+      <c r="X288" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Koçtaş’ta Paraf POS'undan yapacağınız alışverişlerinde 5 taksit fırsatı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Koçtaş’ta Paraf POS'undan yapacağınız alışverişlerinde 5 taksit fırsatı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -15654,249 +15825,329 @@
           <t>Konyali Saatte 7 Taksit</t>
         </is>
       </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E298" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/konyali-saatte-7-taksit-0</t>
         </is>
       </c>
-      <c r="U298" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" t="inlineStr">
-        <is>
-          <t>KT-060</t>
-        </is>
-      </c>
-      <c r="B299" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C299" t="inlineStr">
-        <is>
-          <t>Toprak Turizm’de yurt dışı turlarında %10, umre turlarında %7 indirim fırsatında</t>
-        </is>
-      </c>
-      <c r="E299" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/kuveyt-turk-kredi-kartlarina-toprak-turizm-yurt-disi-turlarinda-10-umre-turlarinda-7-indirim</t>
-        </is>
-      </c>
-      <c r="U299" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" t="inlineStr">
-        <is>
-          <t>TEK-059</t>
-        </is>
-      </c>
-      <c r="B300" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C300" t="inlineStr">
-        <is>
-          <t>Paraf ile Yenilio’da 12 Aya Varan Taksit Fırsatı!</t>
-        </is>
-      </c>
-      <c r="E300" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-yenilioda-12-aya-varan-taksit-firsati</t>
-        </is>
-      </c>
-      <c r="U300" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="inlineStr">
-        <is>
-          <t>ZK-060</t>
-        </is>
-      </c>
-      <c r="B301" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C301" t="inlineStr">
-        <is>
-          <t>Mavide 4 Taksit</t>
-        </is>
-      </c>
-      <c r="E301" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/mavide-4-taksit</t>
-        </is>
-      </c>
-      <c r="U301" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" t="inlineStr">
-        <is>
-          <t>KT-061</t>
-        </is>
-      </c>
-      <c r="B302" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C302" t="inlineStr">
-        <is>
-          <t>Kuveyt Turk Veteriner Klinik Musterilerine Ozel Fugevet Dijital Yonetim Cozumler</t>
-        </is>
-      </c>
-      <c r="E302" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/musteri-ol-kampanyalari/kuveyt-turk-veteriner-klinik-musterilerine-ozel-fugevet-dijital-yonetim-cozumlerinden-30-indirim</t>
-        </is>
-      </c>
-      <c r="U302" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" t="inlineStr">
-        <is>
-          <t>TEK-060</t>
-        </is>
-      </c>
-      <c r="B303" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C303" t="inlineStr">
-        <is>
-          <t>Paraf ile Porland’da Peşin Fiyatına 3 Taksit!</t>
-        </is>
-      </c>
-      <c r="E303" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-porlandda-pesin-fiyatina-3-taksit</t>
-        </is>
-      </c>
-      <c r="U303" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="inlineStr">
-        <is>
-          <t>ZK-061</t>
-        </is>
-      </c>
-      <c r="B304" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C304" t="inlineStr">
-        <is>
-          <t>Mielede 6 Taksit</t>
-        </is>
-      </c>
-      <c r="E304" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/mielede-6-taksit</t>
-        </is>
-      </c>
-      <c r="U304" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="inlineStr">
-        <is>
-          <t>KT-062</t>
-        </is>
-      </c>
-      <c r="B305" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C305" t="inlineStr">
-        <is>
-          <t>Kuveyt Turklulere Windy Carda 30 Indirim Firsati</t>
-        </is>
-      </c>
-      <c r="E305" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/kuveyt-turklulere-windy-carda-30-indirim-firsati</t>
-        </is>
-      </c>
-      <c r="U305" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="inlineStr">
-        <is>
-          <t>TEK-061</t>
-        </is>
-      </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C306" t="inlineStr">
-        <is>
-          <t>Paraf ile Schafer’de Peşin Fiyatına 9 Taksit!</t>
-        </is>
-      </c>
-      <c r="D306" t="inlineStr">
-        <is>
-          <t>Kart Kampanyasi</t>
-        </is>
-      </c>
-      <c r="E306" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-schaferde-pesin-fiyatina-9-taksit</t>
-        </is>
-      </c>
-      <c r="M306" t="inlineStr">
-        <is>
-          <t>Schafer magazalarinda ParafPOS'lardan yapilan alisverislerde vade farksiz 9 aya varan taksit</t>
-        </is>
-      </c>
-      <c r="Q306" t="inlineStr">
-        <is>
-          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
-        </is>
-      </c>
-      <c r="U306" s="2" t="inlineStr">
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>Konyali Saat magazalari ve konyalisaat.com.tr'de pesin fiyatina 7 taksit; Konya Kent Plaza AVM magazasi haric</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U298" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
 BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
+      <c r="V298" t="n">
+        <v>7</v>
+      </c>
+      <c r="X298" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: yapacağınız alışverişlerinizde peşin fiyatına 7 taksit fırsatından yararlanabilirsiniz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>KT-060</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Toprak Turizm’de yurt dışı turlarında %10, umre turlarında %7 indirim fırsatında</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/kuveyt-turk-kredi-kartlarina-toprak-turizm-yurt-disi-turlarinda-10-umre-turlarinda-7-indirim</t>
+        </is>
+      </c>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>TEK-059</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Paraf ile Yenilio’da 12 Aya Varan Taksit Fırsatı!</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-yenilioda-12-aya-varan-taksit-firsati</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>Yenilio magazalari ve web sitesinde yapilan alisverislerde 12 taksit</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U300" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V300" t="n">
+        <v>12</v>
+      </c>
+      <c r="X300" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Yenilio mağazalarında ve www.yenilio.com.tr mağazalarından yapılacak alışverişlerde 12 taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Yenilio mağazalarında ve www.yenilio.com.tr mağazalarından yapılacak alışverişlerde 12 taksit imkanı sunulacaktır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>ZK-060</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Mavide 4 Taksit</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/mavide-4-taksit</t>
+        </is>
+      </c>
+      <c r="U301" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>KT-061</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk Veteriner Klinik Musterilerine Ozel Fugevet Dijital Yonetim Cozumler</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/musteri-ol-kampanyalari/kuveyt-turk-veteriner-klinik-musterilerine-ozel-fugevet-dijital-yonetim-cozumlerinden-30-indirim</t>
+        </is>
+      </c>
+      <c r="U302" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>TEK-060</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Paraf ile Porland’da Peşin Fiyatına 3 Taksit!</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-porlandda-pesin-fiyatina-3-taksit</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>Porland magazalari ve web sitesinde Paraf POS'larindan yapilan alisverislerde pesin fiyatina 3 taksit</t>
+        </is>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U303" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
+      <c r="V303" t="n">
+        <v>3</v>
+      </c>
+      <c r="X303" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Porland mağazalarında veya www.porland.com web sitelerinden Paraf Posların’dan yapacağınız alışverişlerde peşin fiyatına 3 taksit imkanı sağlanacaktır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>ZK-061</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Mielede 6 Taksit</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/mielede-6-taksit</t>
+        </is>
+      </c>
+      <c r="U304" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>KT-062</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Kuveyt Turklulere Windy Carda 30 Indirim Firsati</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/kuveyt-turklulere-windy-carda-30-indirim-firsati</t>
+        </is>
+      </c>
+      <c r="U305" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>TEK-061</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Paraf ile Schafer’de Peşin Fiyatına 9 Taksit!</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-schaferde-pesin-fiyatina-9-taksit</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>Schafer magazalarinda ParafPOS'lardan yapilan alisverislerde vade farksiz 9 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U306" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
       <c r="V306" t="n">
         <v>9</v>
       </c>
@@ -15922,14 +16173,39 @@
           <t>Modalifeta 9 Taksit</t>
         </is>
       </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E307" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/modalifeta-9-taksit</t>
         </is>
       </c>
-      <c r="U307" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>ModaLife'ta yapilan alisverislerde 9 taksit</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U307" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
+      <c r="V307" t="n">
+        <v>9</v>
+      </c>
+      <c r="X307" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: yapacağınız alışverişlerinizi 9 taksitli gerçekleştirebilirsiniz.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
hesap ve finansman kampanyalarina aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -10530,14 +10530,57 @@
           <t>BES ile Hem Yarınınıza Değer Katın, Hem de 650 TL Bonus Kazanın!</t>
         </is>
       </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Sigorta/BES Kampanyasi</t>
+        </is>
+      </c>
       <c r="E115" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/kampanyalar/Sayfalar/bes-ile-yarininiza-deger-katin.aspx</t>
         </is>
       </c>
-      <c r="U115" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K115" t="n">
+        <v>650</v>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>Kredi kartiyla alinan her yeni BES sozlesmesi icin 650 TL bonus; katki payi sozlesme basina en az 650 TL olmali ve 3 ay duzenli odenmeli</t>
+        </is>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="P115" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q115" t="inlineStr">
+        <is>
+          <t>Turkiye Finans kredi karti sahibi tum musteriler</t>
+        </is>
+      </c>
+      <c r="U115" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: sayfada kar payi orani verilmiyor
+BELIRSIZ vade_ay: BES katki payinin 3 ay duzenli odenmesi bir KOSUL, kampanyanin vadesi degil</t>
+        </is>
+      </c>
+      <c r="X115" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 25 Mayıs – 31 Aralık 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 25 Mayıs – 31 Aralık 2026 tarihleri arasında geçerlidir.
+odul_miktari: Bonus kazanımı için BES katkı payının sözleşme başına minimum 650 TL olması gerekmektedir.
+odul_birimi: Bonus kazanımı için BES katkı payının sözleşme başına minimum 650 TL olması gerekmektedir.</t>
         </is>
       </c>
     </row>
@@ -10638,14 +10681,48 @@
           <t>Akademisyenlere Özel Avantaj Paketi</t>
         </is>
       </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Musteri Ol Kampanyasi</t>
+        </is>
+      </c>
       <c r="E119" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/akademisyenlere-ozel-avantaj-paketi</t>
         </is>
       </c>
-      <c r="U119" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>Akademisyen paketi: Miles&amp;Smiles kartta 10.000 Mil'e varan hediye, market/restoran/akaryakit harcamalarina Mil, konut finansmaninda 5 puan indirim, ATM ve fatura talimati avantajlari</t>
+        </is>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>2025-08-11</t>
+        </is>
+      </c>
+      <c r="P119" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q119" t="inlineStr">
+        <is>
+          <t>Universitelerde gorev yapan ve '.edu.tr' uzantili kurumsal e-posta ile dogrulanan akademisyenler</t>
+        </is>
+      </c>
+      <c r="U119" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ odul_miktari: paket cok sayida farkli odul iceriyor (10.000/6.000/3.000 Mil, 500 Mil, 200 TL iade); tek bir odul tutari secilemez
+BELIRSIZ taksit_sayisi: 5 taksit yalnizca Saglam Kart'la egitim/saglik harcamalarinda gecerli - paketin bir parcasi, kampanyanin geneli degil
+BELIRSIZ kar_payi_orani: konut finansmanindaki '5 puan indirim' bir INDIRIM, kar payi orani degil</t>
+        </is>
+      </c>
+      <c r="X119" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 11.08.2025 - 31.12.2026
+kampanya_bitis: 11.08.2025 - 31.12.2026</t>
         </is>
       </c>
     </row>
@@ -10719,14 +10796,48 @@
           <t>Katılım Hesabınızı Şimdi Açın, Daha Yüksek Getiri Oranlarından Yararlanın!</t>
         </is>
       </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Katilma Hesabi Kampanyasi</t>
+        </is>
+      </c>
       <c r="E122" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/kampanyalar/Sayfalar/katilim-hesabi-kampanyasi.aspx</t>
         </is>
       </c>
-      <c r="U122" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>TL katilma hesabi acanlara azami 99/1 kar paylasim orani; 31-35 gun vadeli hesap</t>
+        </is>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="P122" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q122" t="inlineStr">
+        <is>
+          <t>Son uc aydir bankada TL birikimi bulunmayan, TL mevduat bakiyesi 10.000 TL altinda olan bireysel musteriler</t>
+        </is>
+      </c>
+      <c r="U122" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: metindeki 99/1 bir KAR PAYLASIM orani (banka-musteri paylasim anahtari), kar payi getiri orani degil - Rehber F sutunu
+BELIRSIZ vade_ay: vade GUN cinsinden ve araliksal veriliyor: '31-35 gun'; ay karsiligi tek bir sayiya indirgenemez
+BELIRSIZ finansman_tutari: 10.000 TL minimum / 10.000.000 TL maksimum HESAP ACILIS araligi, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X122" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya kapsamında, son üç aydır bankamızda TL mevduatı bulunmayan ve yukarıda belirtilen tarih aralığında TL cinsinden katılım hesabı açan bireysel müşterilerimize azami 99/1 kâr paylaşım oranı ile hesap açma avantajı sunulacaktır.
+kampanya_bitis: Kampanya kapsamında, son üç aydır bankamızda TL mevduatı bulunmayan ve yukarıda belirtilen tarih aralığında TL cinsinden katılım hesabı açan bireysel müşterilerimize azami 99/1 kâr paylaşım oranı ile hesap açma avantajı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -10908,14 +11019,42 @@
           <t>Tuzel Onbarding Avantaj Paketi</t>
         </is>
       </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Ticari Kampanya</t>
+        </is>
+      </c>
       <c r="E129" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/kampanyalar/Sayfalar/tuzel-onbarding-avantaj-paketi.aspx</t>
         </is>
       </c>
-      <c r="U129" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>Aidatsiz Business Kart, ilk yil kiralik kasada %50 indirim, ucretsiz EFT/havale/FAST, ortak ATM'lerden ucretsiz para cekme/yatirma, gunluk hesapta Hos Geldin orani</t>
+        </is>
+      </c>
+      <c r="P129" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>Son 3 ay icerisinde mobilden musteri olan ticari musteriler (KOBI)</t>
+        </is>
+      </c>
+      <c r="U129" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ kar_payi_orani: paket icindeki %50 KIRALIK KASA indirimidir, kar payi orani degil
+BELIRSIZ odul_miktari: paket birden fazla ayni avantaj iceriyor, tek bir odul tutari yok</t>
+        </is>
+      </c>
+      <c r="X129" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya 31.12.2026 tarihine kadar geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -11097,14 +11236,47 @@
           <t>Yeni Yatırım Hesabınıza Sıfır Komisyon Oranı</t>
         </is>
       </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Yatirim Kampanyasi</t>
+        </is>
+      </c>
       <c r="E136" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/kampanyalar/Sayfalar/yeni-yatirim-hesabiniza-sifir-komisyon.aspx</t>
         </is>
       </c>
-      <c r="U136" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>Yeni yatirim hesabi acanlara yurt ici hisse senedi alim-satiminda binde 2 yerine sifir komisyon</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Bankada daha once yatirim hesabi bulunmayan, kampanya doneminde ilk kez yatirim hesabi acan tuketici vasfindaki musteriler</t>
+        </is>
+      </c>
+      <c r="U136" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ masraf_durumu: komisyon sifirlaniyor ama 'yatirim hesabinda olusan diger ucret ve masraflar sozlesmede belirtildigi gibi tahsil edilir' - masrafsiz denemez
+BELIRSIZ kar_payi_orani: sayfada gecen oranlar KOMISYON orani (binde 2 / on binde 2), kar payi orani degil</t>
+        </is>
+      </c>
+      <c r="X136" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 01 Ağustos 2026-31 Ekim 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 01 Ağustos 2026-31 Ekim 2026 tarihleri arasında geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -11286,14 +11458,33 @@
           <t>Günlük Hesap’la İhtiyaç Anında Vadeni Bozma!</t>
         </is>
       </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Katilma Hesabi Kampanyasi</t>
+        </is>
+      </c>
       <c r="E143" t="inlineStr">
         <is>
           <t>https://www.turkiyefinans.com.tr/tr-tr/kampanyalar/Sayfalar/gunluk-hesap-vade-kampanyasi.aspx</t>
         </is>
       </c>
-      <c r="U143" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>Gunluk Hesap'ta 95 gunluk Hos Geldin donemi; 'Ayin Hayata Katilani' olanlara ek %2'ye varan getiri orani</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>5 Agustos 2023 itibariyla yeni bireysel bankacilik musterisi olan ve ilk defa TL Gunluk Hesap acan tuketici musteriler</t>
+        </is>
+      </c>
+      <c r="U143" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor; '5 Agustos 2023' musteri olma KRITERI, kampanya baslangici degil
+BELIRSIZ kampanya_bitis: sayfada kampanya bitis tarihi verilmiyor
+BELIRSIZ kar_payi_orani: sayfa asil getiri oranini vermiyor; gecen '%2'ye varan' bir EK orandir ve kosula bagli
+BELIRSIZ vade_ay: 'Hos Geldin suresi 95 gundur' - gun cinsinden, ay karsiligi tam sayi degil</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
finansman ve BES kampanyalarina aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -11323,14 +11323,51 @@
           <t>Eflatun Kredi Kart ile Kozmetik Harcamalarına 200 TL'ye varan Worldpuan!</t>
         </is>
       </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E138" t="inlineStr">
         <is>
           <t>https://www.albaraka.com.tr/tr/kampanyalar/detay/eflatun-kredi-kart-ile-kozmetik-harcamalarina-200-tlye-varan-worldpuan</t>
         </is>
       </c>
-      <c r="U138" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K138" t="n">
+        <v>200</v>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>Worldpuan</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>500 TL ve uzeri fiziki kozmetik harcamasina 50 TL, ayda en fazla 200 TL Worldpuan</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>Eflatun kredi karti sahipleri; debit, sanal, ek kartlar ve diger kredi kartlari haric</t>
+        </is>
+      </c>
+      <c r="U138" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ finansman_tutari: 500 TL bir harcama ESIGI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X138" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya 31 Aralık 2026 tarihine kadar geçerlidir.
+odul_miktari: Müşterilerimiz kampanya kapsamında içinde bulunulan ayda en fazla 200 TL Worldpuan kazanabilirler.
+odul_birimi: Müşterilerimiz kampanya kapsamında içinde bulunulan ayda en fazla 200 TL Worldpuan kazanabilirler.</t>
         </is>
       </c>
     </row>
@@ -11801,14 +11838,47 @@
           <t>Hadi Black Kredi Kartı ile Restoderm’de %30 İndirim!</t>
         </is>
       </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E155" t="inlineStr">
         <is>
           <t>https://hadiyanindakibanka.com/kampanyalar/hadi-black-karti-ile-restoderm-alisverislerinde-30-indirim</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>Restoderm alisverislerinde 'hadi30' kodu ile %30 indirim</t>
+        </is>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>Hadi Black Kredi Karti sahipleri</t>
+        </is>
+      </c>
+      <c r="U155" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: %30 bir INDIRIM orani, kar payi orani degil (Rehber F sutunu)
+BELIRSIZ odul_miktari: odul yuzde indirim olarak veriliyor, tutar belirtilmiyor</t>
+        </is>
+      </c>
+      <c r="X155" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 4 Ağustos -30 Ağustos 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 4 Ağustos -30 Ağustos 2026 tarihleri arasında geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -13200,14 +13270,54 @@
           <t>Hepsiburada’da Yeni Müşteriye Özel Vade Farksız 50.000 TL Fırsatı!</t>
         </is>
       </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Finansman Kampanyasi</t>
+        </is>
+      </c>
       <c r="E205" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/hepsiburadada-yeni-musteriye-ozel-vade-farksiz-50000-tl-firsati</t>
         </is>
       </c>
-      <c r="U205" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="J205" t="n">
+        <v>50000</v>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk Alisveris Finansmani ile 50.000 TL'ye kadar Hepsiburada sepetine vade farksiz 9 taksit</t>
+        </is>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>2025-03-07</t>
+        </is>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk musterisi olmayan, Hepsiburada mobil uygulamasindan alisveris yapacak yeni musteriler</t>
+        </is>
+      </c>
+      <c r="U205" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: vade farksiz kampanya; sayfada kar payi orani verilmiyor</t>
+        </is>
+      </c>
+      <c r="V205" t="n">
+        <v>9</v>
+      </c>
+      <c r="X205" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 7.03.2025 - 31.12.2026
+kampanya_bitis: 7.03.2025 - 31.12.2026
+taksit_sayisi: 50.000 TL'ye kadar olan Hepsiburada sepetinizi 9 taksit ile ödemek için Kuveyt Türk müşterisi olun!
+finansman_tutari: Kuveyt Türk Alışveriş Finansmanı’na Kuveyt Türk müşterisi olmadan önce 50.000 TL’ye kadar olan Hepsiburada sepetinizi oluşturduktan sonra ödeme anında hemen başvurabilirsiniz.</t>
         </is>
       </c>
     </row>
@@ -13663,14 +13773,56 @@
           <t>Kuveyt Turk Mobilden Pratik Bes Planiniza 2000 TL Hediye</t>
         </is>
       </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Sigorta/BES Kampanyasi</t>
+        </is>
+      </c>
       <c r="E220" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/kuveyt-turk-mobilden-pratik-bes-planiniza-2000-tl-hediye</t>
         </is>
       </c>
-      <c r="U220" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K220" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L220" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>Aylik minimum 2.000 TL'lik Pratik BES sozlesmesini bireysel kredi kartiyla odeyene 2.000 TL iade</t>
+        </is>
+      </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>2025-11-05</t>
+        </is>
+      </c>
+      <c r="P220" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q220" t="inlineStr">
+        <is>
+          <t>1 Ocak 2026 sonrasi Kuveyt Turk Mobil'den musteri olup Pratik BES plani yapan bireysel musteriler</t>
+        </is>
+      </c>
+      <c r="U220" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ finansman_tutari: 2.000 TL aylik BES katki payi ESIGI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X220" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 5.11.2025 - 31.12.2026
+kampanya_bitis: 5.11.2025 - 31.12.2026
+odul_miktari: 'den aylık minimum 2.000 TL’lik Pratik BES ürünü sözleşmesi yapıp, ödemesini Kuveyt Türk Bireysel Kredi Kartları üzerinden yapan müşterilerimize özel 2.000 TL iade yapılacaktır.
+odul_birimi: 'den aylık minimum 2.000 TL’lik Pratik BES ürünü sözleşmesi yapıp, ödemesini Kuveyt Türk Bireysel Kredi Kartları üzerinden yapan müşterilerimize özel 2.000 TL iade yapılacaktır.</t>
         </is>
       </c>
     </row>
@@ -15527,14 +15679,50 @@
           <t>E-İhracatçılara Özel ShipEntegra ile Yurtdışı Kargo Gönderilerinize Vade Farksız</t>
         </is>
       </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Ticari Kampanya</t>
+        </is>
+      </c>
       <c r="E281" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/isim-icin/dis-ticaret/e-ihracat/e-ihracat-kampanyalari/e-ihracatcilara-ozel-shipentegra-ile-yurtdisi-kargo-gonderilerinize-vade-farksiz-3-taksit</t>
         </is>
       </c>
-      <c r="U281" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>ShipEntegra uzerinden yapilan yurt disi kargo odemelerinde vade farksiz 3 taksit</t>
+        </is>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q281" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk Ticari kredi karti sahibi e-ihracat musterileri</t>
+        </is>
+      </c>
+      <c r="U281" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: vade farksiz kampanya; sayfada kar payi orani verilmiyor</t>
+        </is>
+      </c>
+      <c r="V281" t="n">
+        <v>3</v>
+      </c>
+      <c r="X281" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 6.08.2026 - 31.12.2026
+kampanya_bitis: 6.08.2026 - 31.12.2026
+taksit_sayisi: Kuveyt Türk Ticari kredi kartlarınızla ShipEntegra üzerinden yapacağınız yurt dışı kargo ödemelerinde vade farksız 3 taksit avantajı sizleri bekliyor!</t>
         </is>
       </c>
     </row>
@@ -15608,14 +15796,56 @@
           <t>Esnaf, Çiftçi ve Tüzel Şirketlere Özel 16.000 TL Değerinde Finansal Ürün Paketi</t>
         </is>
       </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Musteri Ol Kampanyasi</t>
+        </is>
+      </c>
       <c r="E284" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/musteri-ol-kampanyalari/esnaf-ciftci-ve-tuzel-sirketlere-ozel-16000-tl-degerinde-finansal-urun-paketi-hediye</t>
         </is>
       </c>
-      <c r="U284" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K284" t="n">
+        <v>16000</v>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>16.000 TL degerinde finansal urun paketi: 2 adet 10 yaprak cek karnesi, 100 adet cek tahsilati, 2 adet HGS etiketi</t>
+        </is>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>2024-02-09</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>2027-12-31</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk Mobil'den sahis firmasi, ciftci veya tuzel sirket hesabi acan musteriler</t>
+        </is>
+      </c>
+      <c r="U284" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: sayfada kar payi orani verilmiyor</t>
+        </is>
+      </c>
+      <c r="X284" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 9.02.2024 - 31.12.2027
+kampanya_bitis: 9.02.2024 - 31.12.2027
+odul_miktari: Mobilden Müşterimiz Olan Esnaf, Çiftçi ve Tüzel Şirketler 16.000 TL Değerinde Çek Karnesi, Çek Tahsilatı ve HGS Etiketi Kazanıyor!
+odul_birimi: Mobilden Müşterimiz Olan Esnaf, Çiftçi ve Tüzel Şirketler 16.000 TL Değerinde Çek Karnesi, Çek Tahsilatı ve HGS Etiketi Kazanıyor!</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
yedi taksit kampanyasina daha aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -13472,14 +13472,44 @@
           <t>Paraf Ile Damat Tweende 6 Aya Varan Taksit Firsati</t>
         </is>
       </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E211" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-damat-tweende-6-aya-varan-taksit-firsati</t>
         </is>
       </c>
-      <c r="U211" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>Damat Tween magazalarinda Paraf POS'larindan yapilan alisverislerde 6 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf musterileri ve ek kart sahipleri; debit kartlar ve ParafPara haric</t>
+        </is>
+      </c>
+      <c r="U211" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V211" t="n">
+        <v>6</v>
+      </c>
+      <c r="X211" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Aralık 2026 tarihine kadar Damat Tween mağazalarında Paraf POS’larından yapılacak alışverişlerde 6 aya varan taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Aralık 2026 tarihine kadar Damat Tween mağazalarında Paraf POS’larından yapılacak alışverişlerde 6 aya varan taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -14253,14 +14283,44 @@
           <t>Paraf ile Nocturne’de 4 Taksit!</t>
         </is>
       </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E234" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-nocturnede-4-taksit</t>
         </is>
       </c>
-      <c r="U234" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>Nocturne magazalarinda Paraf POS'larindan yapilan alisverislerde 4 taksit; web sitesi haric</t>
+        </is>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q234" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri; debit kartlar ve ParafPara haric</t>
+        </is>
+      </c>
+      <c r="U234" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V234" t="n">
+        <v>4</v>
+      </c>
+      <c r="X234" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Nocturne mağazalarında Paraf POS’larından yapılacak alışverişlerde 4 taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Nocturne mağazalarında Paraf POS’larından yapılacak alışverişlerde 4 taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -14280,14 +14340,40 @@
           <t>Karacada 3 Taksit</t>
         </is>
       </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E235" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/karacada-3-taksit</t>
         </is>
       </c>
-      <c r="U235" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>Karaca magazalari ve karaca.com'da tek seferde 5.000 TL ve uzeri alisverislerde pesin fiyatina 3 taksit</t>
+        </is>
+      </c>
+      <c r="Q235" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U235" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor
+BELIRSIZ finansman_tutari: 5.000 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="V235" t="n">
+        <v>3</v>
+      </c>
+      <c r="X235" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: alışverişlerinizde peşin fiyatına 3 taksit fırsatından faydalanabilirsiniz.</t>
         </is>
       </c>
     </row>
@@ -14522,14 +14608,40 @@
           <t>Porlandda 8 Taksit</t>
         </is>
       </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E243" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/porlandda-8-taksit</t>
         </is>
       </c>
-      <c r="U243" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>Porland magazalari ve porland.com'da 1.500 TL ve uzeri alisverislerde pesin fiyatina 8 taksit</t>
+        </is>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U243" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor
+BELIRSIZ finansman_tutari: 1.500 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="V243" t="n">
+        <v>8</v>
+      </c>
+      <c r="X243" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: alışverişlerinizde peşin fiyatına 8 taksit fırsatından faydalanabilirsiniz.</t>
         </is>
       </c>
     </row>
@@ -15246,14 +15358,44 @@
           <t>Paraf ile DemirDöküm'de 9 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E267" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-demirdokumde-9-taksit-firsati</t>
         </is>
       </c>
-      <c r="U267" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>DemirDokum sanal POS'u uzerinden yapilan islemlere vade farksiz 9 ay taksit; bayi POS'u haric</t>
+        </is>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q267" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U267" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V267" t="n">
+        <v>9</v>
+      </c>
+      <c r="X267" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Paraf üyesi DemirDöküm sanal POS’u üzerinden işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Paraf üyesi DemirDöküm sanal POS’u üzerinden işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -15892,387 +16034,412 @@
           <t>Enplusta 4 Taksit</t>
         </is>
       </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E286" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/enplusta-4-taksit</t>
         </is>
       </c>
-      <c r="U286" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="287">
-      <c r="A287" t="inlineStr">
-        <is>
-          <t>KT-056</t>
-        </is>
-      </c>
-      <c r="B287" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C287" t="inlineStr">
-        <is>
-          <t>Fatura Talimatlarınıza Toplam 500 TL Hediye!</t>
-        </is>
-      </c>
-      <c r="E287" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/fatura-talimatlariniza-toplam-500-tl-hediye</t>
-        </is>
-      </c>
-      <c r="U287" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="inlineStr">
-        <is>
-          <t>TEK-055</t>
-        </is>
-      </c>
-      <c r="B288" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C288" t="inlineStr">
-        <is>
-          <t>Paraf ile Koçtaş’ta 5 Taksit!</t>
-        </is>
-      </c>
-      <c r="D288" t="inlineStr">
-        <is>
-          <t>Kart Kampanyasi</t>
-        </is>
-      </c>
-      <c r="E288" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-koctasta-5-taksit</t>
-        </is>
-      </c>
-      <c r="M288" t="inlineStr">
-        <is>
-          <t>Koctas'ta Paraf POS'undan yapilan alisverislerde 5 taksit</t>
-        </is>
-      </c>
-      <c r="P288" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="Q288" t="inlineStr">
-        <is>
-          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
-        </is>
-      </c>
-      <c r="U288" s="2" t="inlineStr">
-        <is>
-          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
-        </is>
-      </c>
-      <c r="V288" t="n">
-        <v>5</v>
-      </c>
-      <c r="X288" s="2" t="inlineStr">
-        <is>
-          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Koçtaş’ta Paraf POS'undan yapacağınız alışverişlerinde 5 taksit fırsatı sunulacaktır.
-kampanya_bitis: 31 Ağustos 2026 tarihine kadar Koçtaş’ta Paraf POS'undan yapacağınız alışverişlerinde 5 taksit fırsatı sunulacaktır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="inlineStr">
-        <is>
-          <t>ZK-056</t>
-        </is>
-      </c>
-      <c r="B289" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C289" t="inlineStr">
-        <is>
-          <t>Faik Sonmezde 3 Taksit</t>
-        </is>
-      </c>
-      <c r="E289" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/faik-sonmezde-3-taksit</t>
-        </is>
-      </c>
-      <c r="U289" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="inlineStr">
-        <is>
-          <t>KT-057</t>
-        </is>
-      </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C290" t="inlineStr">
-        <is>
-          <t>Gündoğdu Mobilya’da Vade Farksız 9 Aya Varan Taksit Fırsatı!</t>
-        </is>
-      </c>
-      <c r="E290" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/gundogdu-mobilyada-vade-farksiz-9-aya-varan-taksit-firsati</t>
-        </is>
-      </c>
-      <c r="U290" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="inlineStr">
-        <is>
-          <t>TEK-056</t>
-        </is>
-      </c>
-      <c r="B291" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C291" t="inlineStr">
-        <is>
-          <t>Paraf ile Monster Notebook’ta Peşin Fiyatına 12 Aya Varan Taksit Fırsatı!</t>
-        </is>
-      </c>
-      <c r="E291" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-monster-notebookta-pesin-fiyatina-12-aya-varan-taksit-firsati</t>
-        </is>
-      </c>
-      <c r="U291" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="inlineStr">
-        <is>
-          <t>ZK-057</t>
-        </is>
-      </c>
-      <c r="B292" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C292" t="inlineStr">
-        <is>
-          <t>Goodyearda 4 Taksit</t>
-        </is>
-      </c>
-      <c r="E292" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/goodyearda-4-taksit</t>
-        </is>
-      </c>
-      <c r="U292" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="inlineStr">
-        <is>
-          <t>KT-058</t>
-        </is>
-      </c>
-      <c r="B293" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C293" t="inlineStr">
-        <is>
-          <t>Gürgençler'de 9 Aya Varan Taksit İmkanı!</t>
-        </is>
-      </c>
-      <c r="E293" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/gurgenclerde-9-aya-varan-taksit-imkani</t>
-        </is>
-      </c>
-      <c r="U293" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="inlineStr">
-        <is>
-          <t>TEK-057</t>
-        </is>
-      </c>
-      <c r="B294" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C294" t="inlineStr">
-        <is>
-          <t>Paraf ile Touristica.com.tr’de Peşin Fiyatına 9 Taksit!</t>
-        </is>
-      </c>
-      <c r="E294" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-touristicacomtrde-pesin-fiyatina-9-taksit</t>
-        </is>
-      </c>
-      <c r="U294" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="inlineStr">
-        <is>
-          <t>ZK-058</t>
-        </is>
-      </c>
-      <c r="B295" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C295" t="inlineStr">
-        <is>
-          <t>Istikbalde 7 Taksit</t>
-        </is>
-      </c>
-      <c r="E295" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/istikbalde-7-taksit</t>
-        </is>
-      </c>
-      <c r="U295" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" t="inlineStr">
-        <is>
-          <t>KT-059</t>
-        </is>
-      </c>
-      <c r="B296" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C296" t="inlineStr">
-        <is>
-          <t>Koçtaş’ta Vade Farksız 6 Aya Varan Taksit Fırsatı!</t>
-        </is>
-      </c>
-      <c r="E296" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/koctasta-vade-farksiz-6-aya-varan-taksit-firsati</t>
-        </is>
-      </c>
-      <c r="U296" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" t="inlineStr">
-        <is>
-          <t>TEK-058</t>
-        </is>
-      </c>
-      <c r="B297" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C297" t="inlineStr">
-        <is>
-          <t>Paraf Ile Vatanda Pesin Fiyatina 6 Aya Varan Taksit Firsati</t>
-        </is>
-      </c>
-      <c r="E297" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-vatanda-pesin-fiyatina-6-aya-varan-taksit-firsati</t>
-        </is>
-      </c>
-      <c r="U297" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" t="inlineStr">
-        <is>
-          <t>ZK-059</t>
-        </is>
-      </c>
-      <c r="B298" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C298" t="inlineStr">
-        <is>
-          <t>Konyali Saatte 7 Taksit</t>
-        </is>
-      </c>
-      <c r="D298" t="inlineStr">
-        <is>
-          <t>Kart Kampanyasi</t>
-        </is>
-      </c>
-      <c r="E298" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/konyali-saatte-7-taksit-0</t>
-        </is>
-      </c>
-      <c r="M298" t="inlineStr">
-        <is>
-          <t>Konyali Saat magazalari ve konyalisaat.com.tr'de pesin fiyatina 7 taksit; Konya Kent Plaza AVM magazasi haric</t>
-        </is>
-      </c>
-      <c r="Q298" t="inlineStr">
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>ENPLUS magazalari ve enplus.com.tr'de pesin fiyatina 4 taksit</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
         <is>
           <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
         </is>
       </c>
-      <c r="U298" s="2" t="inlineStr">
+      <c r="U286" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
 BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
+      <c r="V286" t="n">
+        <v>4</v>
+      </c>
+      <c r="X286" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: peşin fiyatına 4 taksit fırsatından faydalanabilirsiniz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>KT-056</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Fatura Talimatlarınıza Toplam 500 TL Hediye!</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/fatura-talimatlariniza-toplam-500-tl-hediye</t>
+        </is>
+      </c>
+      <c r="U287" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>TEK-055</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Paraf ile Koçtaş’ta 5 Taksit!</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-koctasta-5-taksit</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Koctas'ta Paraf POS'undan yapilan alisverislerde 5 taksit</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U288" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V288" t="n">
+        <v>5</v>
+      </c>
+      <c r="X288" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Koçtaş’ta Paraf POS'undan yapacağınız alışverişlerinde 5 taksit fırsatı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Koçtaş’ta Paraf POS'undan yapacağınız alışverişlerinde 5 taksit fırsatı sunulacaktır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>ZK-056</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Faik Sonmezde 3 Taksit</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/faik-sonmezde-3-taksit</t>
+        </is>
+      </c>
+      <c r="U289" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>KT-057</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Gündoğdu Mobilya’da Vade Farksız 9 Aya Varan Taksit Fırsatı!</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/gundogdu-mobilyada-vade-farksiz-9-aya-varan-taksit-firsati</t>
+        </is>
+      </c>
+      <c r="U290" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>TEK-056</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Paraf ile Monster Notebook’ta Peşin Fiyatına 12 Aya Varan Taksit Fırsatı!</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-monster-notebookta-pesin-fiyatina-12-aya-varan-taksit-firsati</t>
+        </is>
+      </c>
+      <c r="U291" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>ZK-057</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Goodyearda 4 Taksit</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/goodyearda-4-taksit</t>
+        </is>
+      </c>
+      <c r="U292" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>KT-058</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Gürgençler'de 9 Aya Varan Taksit İmkanı!</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/gurgenclerde-9-aya-varan-taksit-imkani</t>
+        </is>
+      </c>
+      <c r="U293" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>TEK-057</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Paraf ile Touristica.com.tr’de Peşin Fiyatına 9 Taksit!</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-touristicacomtrde-pesin-fiyatina-9-taksit</t>
+        </is>
+      </c>
+      <c r="U294" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>ZK-058</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Istikbalde 7 Taksit</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/istikbalde-7-taksit</t>
+        </is>
+      </c>
+      <c r="U295" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>KT-059</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Koçtaş’ta Vade Farksız 6 Aya Varan Taksit Fırsatı!</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/koctasta-vade-farksiz-6-aya-varan-taksit-firsati</t>
+        </is>
+      </c>
+      <c r="U296" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>TEK-058</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Paraf Ile Vatanda Pesin Fiyatina 6 Aya Varan Taksit Firsati</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-vatanda-pesin-fiyatina-6-aya-varan-taksit-firsati</t>
+        </is>
+      </c>
+      <c r="U297" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>ZK-059</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Konyali Saatte 7 Taksit</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/konyali-saatte-7-taksit-0</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>Konyali Saat magazalari ve konyalisaat.com.tr'de pesin fiyatina 7 taksit; Konya Kent Plaza AVM magazasi haric</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U298" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
       <c r="V298" t="n">
         <v>7</v>
       </c>
@@ -16382,14 +16549,39 @@
           <t>Mavide 4 Taksit</t>
         </is>
       </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E301" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/mavide-4-taksit</t>
         </is>
       </c>
-      <c r="U301" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>Mavi magazalari ve mavi.com'da pesin fiyatina 4 taksit</t>
+        </is>
+      </c>
+      <c r="Q301" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U301" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
+      <c r="V301" t="n">
+        <v>4</v>
+      </c>
+      <c r="X301" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: peşin fiyatına 4 taksit fırsatından faydalanabilirsiniz.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
yedi kampanyaya daha aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -11952,14 +11952,47 @@
           <t>Hizli Cicek 25 Indirim Kampanyasi</t>
         </is>
       </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E158" t="inlineStr">
         <is>
           <t>https://www.albaraka.com.tr/tr/kampanyalar/detay/2026/hizli-cicek-25-indirim-kampanyasi</t>
         </is>
       </c>
-      <c r="U158" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil'den alinan kod ile Hizli Cicek uygulamasinda %25 indirim; ayda bir kez</t>
+        </is>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil kullanicilari</t>
+        </is>
+      </c>
+      <c r="U158" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: %25 bir INDIRIM orani, kar payi orani degil (Rehber F sutunu)
+BELIRSIZ odul_miktari: odul yuzde indirim olarak veriliyor, tutar belirtilmiyor</t>
+        </is>
+      </c>
+      <c r="X158" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 1 Mayıs 2026 - 31 Aralık 2026 tarihlerinde geçerlidir.
+kampanya_bitis: Kampanya 1 Mayıs 2026 - 31 Aralık 2026 tarihlerinde geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -14742,14 +14775,40 @@
           <t>Schaferda 9 Taksit</t>
         </is>
       </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E247" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/schaferda-9-taksit</t>
         </is>
       </c>
-      <c r="U247" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>Schafer magazalari ve schafer.com.tr'de 20.000 TL ve uzeri alisverislere pesin fiyatina 9 taksit</t>
+        </is>
+      </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U247" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor
+BELIRSIZ finansman_tutari: 20.000 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="V247" t="n">
+        <v>9</v>
+      </c>
+      <c r="X247" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: alışverişlerinize peşin fiyatına 9 taksit fırsatından faydalanabilirsiniz.</t>
         </is>
       </c>
     </row>
@@ -15634,14 +15693,45 @@
           <t>Demirdöküm’de 12 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E275" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/demirdokumde-12-taksit-firsati</t>
         </is>
       </c>
-      <c r="U275" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>Demirdokum'de 12 taksit firsati</t>
+        </is>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="U275" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ hedef_kitle: sayfanin gorulen bolumunde hedef kitle belirtilmiyor</t>
+        </is>
+      </c>
+      <c r="V275" t="n">
+        <v>12</v>
+      </c>
+      <c r="X275" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Demirdöküm’de 12 Taksit Fırsatı!
+kampanya_baslangic: 1.05.2026 - 31.12.2026
+kampanya_bitis: 1.05.2026 - 31.12.2026</t>
         </is>
       </c>
     </row>
@@ -15661,14 +15751,44 @@
           <t>Paraf ile Evidea’da 4 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E276" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-evideada-4-taksit-firsati</t>
         </is>
       </c>
-      <c r="U276" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>Evidea web sitesi ve magazalarinda Paraf POS uzerinden taksitli alisverislere 4 taksit</t>
+        </is>
+      </c>
+      <c r="P276" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q276" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U276" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V276" t="n">
+        <v>4</v>
+      </c>
+      <c r="X276" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Evidea web sitesi ve mağazalarında Paraf POS’u üzerinden yapılan taksitli alışverişlere 4 taksit uygulanacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Evidea web sitesi ve mağazalarında Paraf POS’u üzerinden yapılan taksitli alışverişlere 4 taksit uygulanacaktır.</t>
         </is>
       </c>
     </row>
@@ -16305,14 +16425,44 @@
           <t>Paraf ile Touristica.com.tr’de Peşin Fiyatına 9 Taksit!</t>
         </is>
       </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E294" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-touristicacomtrde-pesin-fiyatina-9-taksit</t>
         </is>
       </c>
-      <c r="U294" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>touristica.com.tr'den yapilan alisverislerde 9 taksit; KKTC harcamalarinda 3 ay, yurt disinda taksit yok</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U294" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V294" t="n">
+        <v>9</v>
+      </c>
+      <c r="X294" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar www.touristica.com.tr mağazalarından yapılacak alışverişlerde 9 taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar www.touristica.com.tr mağazalarından yapılacak alışverişlerde 9 taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -16680,139 +16830,164 @@
           <t>Mielede 6 Taksit</t>
         </is>
       </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E304" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/mielede-6-taksit</t>
         </is>
       </c>
-      <c r="U304" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="inlineStr">
-        <is>
-          <t>KT-062</t>
-        </is>
-      </c>
-      <c r="B305" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C305" t="inlineStr">
-        <is>
-          <t>Kuveyt Turklulere Windy Carda 30 Indirim Firsati</t>
-        </is>
-      </c>
-      <c r="E305" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/kuveyt-turklulere-windy-carda-30-indirim-firsati</t>
-        </is>
-      </c>
-      <c r="U305" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="inlineStr">
-        <is>
-          <t>TEK-061</t>
-        </is>
-      </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C306" t="inlineStr">
-        <is>
-          <t>Paraf ile Schafer’de Peşin Fiyatına 9 Taksit!</t>
-        </is>
-      </c>
-      <c r="D306" t="inlineStr">
-        <is>
-          <t>Kart Kampanyasi</t>
-        </is>
-      </c>
-      <c r="E306" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-schaferde-pesin-fiyatina-9-taksit</t>
-        </is>
-      </c>
-      <c r="M306" t="inlineStr">
-        <is>
-          <t>Schafer magazalarinda ParafPOS'lardan yapilan alisverislerde vade farksiz 9 aya varan taksit</t>
-        </is>
-      </c>
-      <c r="Q306" t="inlineStr">
-        <is>
-          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
-        </is>
-      </c>
-      <c r="U306" s="2" t="inlineStr">
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>Miele magazalari ve shop.miele.com.tr'de pesin fiyatina 6 taksit</t>
+        </is>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U304" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
 BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
-      <c r="V306" t="n">
-        <v>9</v>
-      </c>
-      <c r="X306" s="2" t="inlineStr">
-        <is>
-          <t>taksit_sayisi: Paraf ile Schafer mağazalarında ParafPOS’larından yapacağınız alışverişlerde vade farksız 9 aya varan taksit imkanı sağlanacaktır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="inlineStr">
-        <is>
-          <t>ZK-062</t>
-        </is>
-      </c>
-      <c r="B307" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C307" t="inlineStr">
-        <is>
-          <t>Modalifeta 9 Taksit</t>
-        </is>
-      </c>
-      <c r="D307" t="inlineStr">
+      <c r="V304" t="n">
+        <v>6</v>
+      </c>
+      <c r="X304" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: yapacağınız alışverişlerinizi peşin fiyatına 6 taksitli gerçekleştirebilirsiniz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>KT-062</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Kuveyt Turklulere Windy Carda 30 Indirim Firsati</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/kuveyt-turklulere-windy-carda-30-indirim-firsati</t>
+        </is>
+      </c>
+      <c r="U305" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>TEK-061</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Paraf ile Schafer’de Peşin Fiyatına 9 Taksit!</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
         <is>
           <t>Kart Kampanyasi</t>
         </is>
       </c>
-      <c r="E307" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/modalifeta-9-taksit</t>
-        </is>
-      </c>
-      <c r="M307" t="inlineStr">
-        <is>
-          <t>ModaLife'ta yapilan alisverislerde 9 taksit</t>
-        </is>
-      </c>
-      <c r="Q307" t="inlineStr">
-        <is>
-          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
-        </is>
-      </c>
-      <c r="U307" s="2" t="inlineStr">
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-schaferde-pesin-fiyatina-9-taksit</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>Schafer magazalarinda ParafPOS'lardan yapilan alisverislerde vade farksiz 9 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U306" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
 BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
+      <c r="V306" t="n">
+        <v>9</v>
+      </c>
+      <c r="X306" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Paraf ile Schafer mağazalarında ParafPOS’larından yapacağınız alışverişlerde vade farksız 9 aya varan taksit imkanı sağlanacaktır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>ZK-062</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Modalifeta 9 Taksit</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/modalifeta-9-taksit</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>ModaLife'ta yapilan alisverislerde 9 taksit</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U307" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
       <c r="V307" t="n">
         <v>9</v>
       </c>
@@ -16865,14 +17040,44 @@
           <t>Paraf ile Vaillant’ta 9 Aya Varan Taksit!</t>
         </is>
       </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E309" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-vaillantta-9-aya-varan-taksit</t>
         </is>
       </c>
-      <c r="U309" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>Vaillant sanal POS'u uzerinden yapilan islemlere vade farksiz 9 ay taksit; bayi POS'u haric</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U309" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V309" t="n">
+        <v>9</v>
+      </c>
+      <c r="X309" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Paraf üyesi Vaillant sanal POS’u üzerinden yapılan işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Paraf üyesi Vaillant sanal POS’u üzerinden yapılan işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
alti kampanyaya daha aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -12814,14 +12814,42 @@
           <t>Arzumda 25 Indirim</t>
         </is>
       </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E188" t="inlineStr">
         <is>
           <t>https://www.albaraka.com.tr/tr/kampanyalar/detay/arzumda-25-indirim</t>
         </is>
       </c>
-      <c r="U188" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>arzum.com.tr'de %25 indirim; sepette en fazla 2 urun, Thermogusto ve Espresso haric</t>
+        </is>
+      </c>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="Q188" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil uzerinden GastroClub kodu alan musteriler</t>
+        </is>
+      </c>
+      <c r="U188" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ kar_payi_orani: %25 bir INDIRIM orani, kar payi orani degil (Rehber F sutunu)
+BELIRSIZ odul_miktari: odul yuzde indirim olarak veriliyor, tutar belirtilmiyor</t>
+        </is>
+      </c>
+      <c r="X188" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya 31.12.2025 tarihine kadar geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -13962,14 +13990,33 @@
           <t>Ikeada 6 Taksit</t>
         </is>
       </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E222" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/ikeada-6-taksit</t>
         </is>
       </c>
-      <c r="U222" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>IKEA magazalari ve ikea.com.tr'de 1.500 TL uzeri alisverislerde 3 taksit, 7.500 TL uzeri mobilya/ev aksesuarinda 6 taksit</t>
+        </is>
+      </c>
+      <c r="Q222" t="inlineStr">
+        <is>
+          <t>IKEA Aile uyesi Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U222" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ taksit_sayisi: metin iki deger veriyor: 1.500 TL uzeri 3 taksit, 7.500 TL uzeri mobilya/ev aksesuarinda 6 taksit - tek deger secilemez
+BELIRSIZ finansman_tutari: 1.500 / 7.500 TL harcama ESIKLERI, kampanyanin finansman tutari degil
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
     </row>
@@ -14909,355 +14956,380 @@
           <t>Baymak'tan yapacağınız alışverişlerinizde 9 taksit fırsatından faydalanabilirsin</t>
         </is>
       </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E251" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/baymakta-9-taksit</t>
         </is>
       </c>
-      <c r="U251" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="inlineStr">
-        <is>
-          <t>DK-037</t>
-        </is>
-      </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>Dünya Katılım</t>
-        </is>
-      </c>
-      <c r="C252" t="inlineStr">
-        <is>
-          <t>Paraf Kart’la alışverişe başla, TOD ayrıcalığını ücretsiz yaşa!</t>
-        </is>
-      </c>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>https://dunyakatilim.com.tr/kampanyalar/tod-paraf</t>
-        </is>
-      </c>
-      <c r="U252" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="inlineStr">
-        <is>
-          <t>KT-045</t>
-        </is>
-      </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C253" t="inlineStr">
-        <is>
-          <t>Elçi Tur’dan Kuveyt Türk Müşterilerine Özel Yaz Fırsatı</t>
-        </is>
-      </c>
-      <c r="E253" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/elci-turdan-kuveyt-turk-musterilerine-ozel-yaz-firsati</t>
-        </is>
-      </c>
-      <c r="U253" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="inlineStr">
-        <is>
-          <t>TEK-044</t>
-        </is>
-      </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>Troy Apple’da vade farksız 5 aya varan taksit</t>
-        </is>
-      </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/troy-appleda-vade-farksiz-5-aya-varan-taksit</t>
-        </is>
-      </c>
-      <c r="U254" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="inlineStr">
-        <is>
-          <t>ZK-045</t>
-        </is>
-      </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C255" t="inlineStr">
-        <is>
-          <t>Bellonada 5 Taksit</t>
-        </is>
-      </c>
-      <c r="E255" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/bellonada-5-taksit</t>
-        </is>
-      </c>
-      <c r="U255" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="inlineStr">
-        <is>
-          <t>DK-038</t>
-        </is>
-      </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>Dünya Katılım</t>
-        </is>
-      </c>
-      <c r="C256" t="inlineStr">
-        <is>
-          <t>Tahsile Çek, müşterilerin ödeme almak amacıyla bankaya bıraktıkları çeklerin işl</t>
-        </is>
-      </c>
-      <c r="E256" t="inlineStr">
-        <is>
-          <t>https://dunyakatilim.com.tr/kampanyalar/tahsile-cek</t>
-        </is>
-      </c>
-      <c r="U256" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="inlineStr">
-        <is>
-          <t>KT-046</t>
-        </is>
-      </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C257" t="inlineStr">
-        <is>
-          <t>Hisse Senedi İşlemleriniz Mil'lere Dönüşsün</t>
-        </is>
-      </c>
-      <c r="E257" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/hisse-senedi-islemleriniz-millere-donussun</t>
-        </is>
-      </c>
-      <c r="U257" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="inlineStr">
-        <is>
-          <t>TEK-045</t>
-        </is>
-      </c>
-      <c r="B258" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C258" t="inlineStr">
-        <is>
-          <t>Paraf ile A101’de Vade Farksız 6 Aya Varan Taksit Fırsatı!</t>
-        </is>
-      </c>
-      <c r="E258" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-a101de-vade-farksiz-6-aya-varan-taksit-firsati</t>
-        </is>
-      </c>
-      <c r="U258" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="inlineStr">
-        <is>
-          <t>ZK-046</t>
-        </is>
-      </c>
-      <c r="B259" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C259" t="inlineStr">
-        <is>
-          <t>Benettonda 2 Taksit</t>
-        </is>
-      </c>
-      <c r="E259" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/benettonda-2-taksit</t>
-        </is>
-      </c>
-      <c r="U259" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t>KT-047</t>
-        </is>
-      </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>Kuveyt Türk</t>
-        </is>
-      </c>
-      <c r="C260" t="inlineStr">
-        <is>
-          <t>Kuveyt Turkten Yeni Musterilere Ozel Pos Kampanyasi</t>
-        </is>
-      </c>
-      <c r="E260" t="inlineStr">
-        <is>
-          <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/pos-kampanyalari/kuveyt-turkten-yeni-musterilere-ozel-pos-kampanyasi</t>
-        </is>
-      </c>
-      <c r="U260" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="inlineStr">
-        <is>
-          <t>TEK-046</t>
-        </is>
-      </c>
-      <c r="B261" t="inlineStr">
-        <is>
-          <t>Türkiye Emlak Katılım</t>
-        </is>
-      </c>
-      <c r="C261" t="inlineStr">
-        <is>
-          <t>Paraf ile Alfemo’da 8 Taksit Fırsatı!</t>
-        </is>
-      </c>
-      <c r="D261" t="inlineStr">
-        <is>
-          <t>Kart Kampanyasi</t>
-        </is>
-      </c>
-      <c r="E261" t="inlineStr">
-        <is>
-          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-alfemoda-8-taksit-firsati</t>
-        </is>
-      </c>
-      <c r="M261" t="inlineStr">
-        <is>
-          <t>Alfemo magazalari ve web sitesinde Paraf POS'larindan yapilan alisverislerde 8 taksit</t>
-        </is>
-      </c>
-      <c r="Q261" t="inlineStr">
-        <is>
-          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
-        </is>
-      </c>
-      <c r="U261" s="2" t="inlineStr">
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>Anlasmali Baymak bayilerinde 9 taksit</t>
+        </is>
+      </c>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U251" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
 BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
-      <c r="V261" t="n">
-        <v>8</v>
-      </c>
-      <c r="X261" s="2" t="inlineStr">
-        <is>
-          <t>taksit_sayisi: Paraf ile Alfemo mağazalarında veya www.alfemo.com web sayfasından Paraf POS’larından yapacağınız alışverişlerde 8 taksit imkanı sağlanacaktır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t>ZK-047</t>
-        </is>
-      </c>
-      <c r="B262" t="inlineStr">
+      <c r="V251" t="n">
+        <v>9</v>
+      </c>
+      <c r="X251" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Baymak'tan yapacağınız alışverişlerinizde 9 taksit fırsatından faydalanabilirsiniz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>DK-037</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Dünya Katılım</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Paraf Kart’la alışverişe başla, TOD ayrıcalığını ücretsiz yaşa!</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>https://dunyakatilim.com.tr/kampanyalar/tod-paraf</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>KT-045</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Elçi Tur’dan Kuveyt Türk Müşterilerine Özel Yaz Fırsatı</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/elci-turdan-kuveyt-turk-musterilerine-ozel-yaz-firsati</t>
+        </is>
+      </c>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>TEK-044</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Troy Apple’da vade farksız 5 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/troy-appleda-vade-farksiz-5-aya-varan-taksit</t>
+        </is>
+      </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>ZK-045</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
         <is>
           <t>Ziraat Katılım</t>
         </is>
       </c>
-      <c r="C262" t="inlineStr">
-        <is>
-          <t>Bridgestoneda 5 Taksit</t>
-        </is>
-      </c>
-      <c r="D262" t="inlineStr">
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Bellonada 5 Taksit</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/bellonada-5-taksit</t>
+        </is>
+      </c>
+      <c r="U255" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>DK-038</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Dünya Katılım</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Tahsile Çek, müşterilerin ödeme almak amacıyla bankaya bıraktıkları çeklerin işl</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>https://dunyakatilim.com.tr/kampanyalar/tahsile-cek</t>
+        </is>
+      </c>
+      <c r="U256" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>KT-046</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Hisse Senedi İşlemleriniz Mil'lere Dönüşsün</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/hisse-senedi-islemleriniz-millere-donussun</t>
+        </is>
+      </c>
+      <c r="U257" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>TEK-045</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Paraf ile A101’de Vade Farksız 6 Aya Varan Taksit Fırsatı!</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-a101de-vade-farksiz-6-aya-varan-taksit-firsati</t>
+        </is>
+      </c>
+      <c r="U258" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>ZK-046</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Benettonda 2 Taksit</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/benettonda-2-taksit</t>
+        </is>
+      </c>
+      <c r="U259" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>KT-047</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Kuveyt Turkten Yeni Musterilere Ozel Pos Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/pos-kampanyalari/kuveyt-turkten-yeni-musterilere-ozel-pos-kampanyasi</t>
+        </is>
+      </c>
+      <c r="U260" t="inlineStr">
+        <is>
+          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>TEK-046</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Türkiye Emlak Katılım</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Paraf ile Alfemo’da 8 Taksit Fırsatı!</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
         <is>
           <t>Kart Kampanyasi</t>
         </is>
       </c>
-      <c r="E262" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/bridgestoneda-5-taksit</t>
-        </is>
-      </c>
-      <c r="M262" t="inlineStr">
-        <is>
-          <t>Bridgestone'da Bankkart POS'undan yapilan alisverislerde pesin fiyatina 5 taksit</t>
-        </is>
-      </c>
-      <c r="Q262" t="inlineStr">
-        <is>
-          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
-        </is>
-      </c>
-      <c r="U262" s="2" t="inlineStr">
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-alfemoda-8-taksit-firsati</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>Alfemo magazalari ve web sitesinde Paraf POS'larindan yapilan alisverislerde 8 taksit</t>
+        </is>
+      </c>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U261" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
 BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
+      <c r="V261" t="n">
+        <v>8</v>
+      </c>
+      <c r="X261" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Paraf ile Alfemo mağazalarında veya www.alfemo.com web sayfasından Paraf POS’larından yapacağınız alışverişlerde 8 taksit imkanı sağlanacaktır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>ZK-047</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Bridgestoneda 5 Taksit</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/bridgestoneda-5-taksit</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>Bridgestone'da Bankkart POS'undan yapilan alisverislerde pesin fiyatina 5 taksit</t>
+        </is>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U262" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
       <c r="V262" t="n">
         <v>5</v>
       </c>
@@ -15310,14 +15382,49 @@
           <t>Paraf Ile Copada 12 Aya Varan Taksit</t>
         </is>
       </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E264" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-copada-12-aya-varan-taksit</t>
         </is>
       </c>
-      <c r="U264" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>Copa Isi bayilerinde ParafPOS'tan 12 aya varan taksit; her musteri bir kez</t>
+        </is>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="P264" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q264" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U264" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi</t>
+        </is>
+      </c>
+      <c r="V264" t="n">
+        <v>12</v>
+      </c>
+      <c r="X264" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Taksit kampanyasından yararlanabilmek için işlem anında satış görevlisine 12 taksit talebinin iletilmesi gerekmektedir.
+kampanya_baslangic: 1-31 Ağustos 2026 tarihleri arasında Parafüyesi Copa Isı Bayilerinde ParafPOS’undan yapılması gerekmektedir.
+kampanya_bitis: 1-31 Ağustos 2026 tarihleri arasında Parafüyesi Copa Isı Bayilerinde ParafPOS’undan yapılması gerekmektedir.</t>
         </is>
       </c>
     </row>
@@ -15612,14 +15719,49 @@
           <t>Barcin Sporda 4 Taksit Firsati</t>
         </is>
       </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E272" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/barcin-sporda-4-taksit-firsati</t>
         </is>
       </c>
-      <c r="U272" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>Barcin Spor'da 4 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>Tum Kuveyt Turk bireysel kredi kartlari (Miles&amp;Smiles, Saglam Kart, Saglam Kart Kampus/Genc, World Elite) ve ek kartlari</t>
+        </is>
+      </c>
+      <c r="U272" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi</t>
+        </is>
+      </c>
+      <c r="V272" t="n">
+        <v>4</v>
+      </c>
+      <c r="X272" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Kuveyt Türk Bireysel Kredi Kartları ile 31 Aralık 2026 tarihine kadar Barçın Spor’da yapacağınız alışverişlerinizde 4 aya varan taksit imkanı sizi bekliyor.
+kampanya_baslangic: 21.07.2026 - 31.12.2026
+kampanya_bitis: 21.07.2026 - 31.12.2026</t>
         </is>
       </c>
     </row>
@@ -16371,14 +16513,39 @@
           <t>Goodyearda 4 Taksit</t>
         </is>
       </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E292" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/goodyearda-4-taksit</t>
         </is>
       </c>
-      <c r="U292" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>Goodyear'da pesin fiyatina 4 taksit</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U292" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
+        </is>
+      </c>
+      <c r="V292" t="n">
+        <v>4</v>
+      </c>
+      <c r="X292" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: da yapacağınız alışverişlerinizde peşin fiyatına 4 taksit fırsatından faydalanabilirsiniz.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bes kampanyaya daha aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -12409,14 +12409,47 @@
           <t>Monster Notebook'ta 12 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E170" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/monster-notebookta-12-aya-varan-taksit-firsati</t>
         </is>
       </c>
-      <c r="U170" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>Monster Notebook'ta tutara gore vade farksiz taksit: 90.000 TL'ye kadar 6 taksit, 90.000 TL ve uzeri daha yuksek taksit</t>
+        </is>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>Tum Kuveyt Turk kredi kartlari (bireysel ve ticari) ve ek kartlari</t>
+        </is>
+      </c>
+      <c r="U170" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ taksit_sayisi: metin tutara gore iki farkli taksit veriyor (90.000 TL'ye kadar 6, uzerinde daha fazla); baslik 12 diyor - tek deger secilemez
+BELIRSIZ finansman_tutari: 90.000 TL bir harcama ESIGI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X170" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 28.01.2026 - 31.08.2026
+kampanya_bitis: 28.01.2026 - 31.08.2026</t>
         </is>
       </c>
     </row>
@@ -12463,14 +12496,56 @@
           <t>Kultur Sanat Harcamalariniza Toplam 500 TL Bankkart Lira</t>
         </is>
       </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E172" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/kultur-sanat-harcamalariniza-toplam-500-tl-bankkart-lira-2</t>
         </is>
       </c>
-      <c r="U172" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K172" t="n">
+        <v>500</v>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>Muze, sinema, tiyatro ve konser bileti alimlarinda %10, toplam en fazla 500 TL Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim bireysel Bankkart kredi karti asil kart sahipleri (ticari ve ucretsiz kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U172" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: %10 bir IADE orani, kar payi orani degil</t>
+        </is>
+      </c>
+      <c r="X172" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 10 Temmuz 2026 - 7 Ağustos 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 10 Temmuz 2026 - 7 Ağustos 2026 tarihleri arasında geçerlidir.
+odul_miktari: Kampanya müşteri bazındadır ve bir müşteri kampanyadan en fazla 500 TL Bankkart Lira kazanabilecektir.
+odul_birimi: Kampanya müşteri bazındadır ve bir müşteri kampanyadan en fazla 500 TL Bankkart Lira kazanabilecektir.</t>
         </is>
       </c>
     </row>
@@ -12598,14 +12673,33 @@
           <t>Okul Odemelerinizde 6ya Varan Taksit</t>
         </is>
       </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E177" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/okul-odemelerinizde-6ya-varan-taksit</t>
         </is>
       </c>
-      <c r="U177" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>Egitim sektorunde okul odemelerinde tutara gore ek taksit: 250.000-1.000.000 TL arasi +5, 1.000.000 TL uzeri +6 taksit</t>
+        </is>
+      </c>
+      <c r="Q177" t="inlineStr">
+        <is>
+          <t>Bireysel Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U177" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ taksit_sayisi: kampanya EK taksit veriyor (+5 / +6) ve tutara gore degisiyor; mutlak taksit sayisi degil
+BELIRSIZ finansman_tutari: 250.000 / 1.000.000 TL islem ESIKLERI, kampanyanin finansman tutari degil
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
     </row>
@@ -13077,14 +13171,46 @@
           <t>Kahve Keyfiniz Albarakadan</t>
         </is>
       </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E193" t="inlineStr">
         <is>
           <t>https://www.albaraka.com.tr/tr/kampanyalar/detay/2026/kahve-keyfiniz-albarakadan</t>
         </is>
       </c>
-      <c r="U193" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>Espressolab Turkiye magazalarinda haftada bir kucuk boy aromasiz kahve hediyesi</t>
+        </is>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>Sadakat segmenti Elmas veya Platin olan Albaraka musterileri</t>
+        </is>
+      </c>
+      <c r="U193" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ odul_miktari: odul ayni (kahve ikrami), parasal tutar verilmiyor</t>
+        </is>
+      </c>
+      <c r="X193" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 1-30 Haziran 2026 tarihlerinde geçerlidir.
+kampanya_bitis: Kampanya 1-30 Haziran 2026 tarihlerinde geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -13690,14 +13816,33 @@
           <t>E Bebekte 8 Taksit</t>
         </is>
       </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E212" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/e-bebekte-8-taksit</t>
         </is>
       </c>
-      <c r="U212" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>Ebebek'te 2.000 TL uzeri alisverislerde 4 taksit, 5.000 TL uzeri alisverislerde 8 taksit</t>
+        </is>
+      </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U212" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ taksit_sayisi: metin iki deger veriyor: 2.000 TL uzeri 4 taksit, 5.000 TL uzeri 8 taksit - tek deger secilemez
+BELIRSIZ finansman_tutari: 2.000 / 5.000 TL harcama ESIKLERI, kampanyanin finansman tutari degil
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vade farksiz kampanyalara kar payi orani sifir yazildi, dort kampanyaya aday deger
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -12004,14 +12004,42 @@
           <t>Paraf ile Pazarama’da Peşin Fiyatına 6 Taksit!</t>
         </is>
       </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E156" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-pazaramada-pesin-fiyatina-6-taksit</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>pazarama.com ve mobil uygulamasinda tutara gore pesin fiyatina taksit: 600 TL uzeri 2, 1.000 TL uzeri 3, 6.000 TL uzeri 6 taksit</t>
+        </is>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U156" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ taksit_sayisi: metin tutara gore uc deger veriyor (2 / 3 / 6 taksit) - tek deger secilemez
+BELIRSIZ finansman_tutari: 600 / 1.000 / 6.000 TL harcama ESIKLERI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X156" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: 31 Ağustos 2026 tarihine kadar www.pazarama.com ve mobil uygulamasından tek seferde yapılacak alışverişlerde peşin fiyatına 6 aya varan taksit imkanı sunulmaktadır.</t>
         </is>
       </c>
     </row>
@@ -12462,6 +12490,14 @@
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/monster-notebookta-12-aya-varan-taksit-firsati</t>
         </is>
       </c>
+      <c r="F170" t="n">
+        <v>0</v>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M170" t="inlineStr">
         <is>
           <t>Monster Notebook'ta tutara gore vade farksiz taksit: 90.000 TL'ye kadar 6 taksit, 90.000 TL ve uzeri daha yuksek taksit</t>
@@ -12486,13 +12522,15 @@
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ taksit_sayisi: metin tutara gore iki farkli taksit veriyor (90.000 TL'ye kadar 6, uzerinde daha fazla); baslik 12 diyor - tek deger secilemez
-BELIRSIZ finansman_tutari: 90.000 TL bir harcama ESIGI, kampanyanin finansman tutari degil</t>
+BELIRSIZ finansman_tutari: 90.000 TL bir harcama ESIGI, kampanyanin finansman tutari degil
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="X170" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: 28.01.2026 - 31.08.2026
-kampanya_bitis: 28.01.2026 - 31.08.2026</t>
+kampanya_bitis: 28.01.2026 - 31.08.2026
+kar_payi_orani: Monster‘da Vade Farksız 12 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
     </row>
@@ -13343,14 +13381,57 @@
           <t>Akaryakıt Sektöründe Sağlam Oran!</t>
         </is>
       </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Ticari Kampanya</t>
+        </is>
+      </c>
       <c r="E195" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/kart-kampanyalari/akaryakit-sektorunde-saglam-oran</t>
         </is>
       </c>
-      <c r="U195" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="F195" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>aylik</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>300 TL - 500.000 TL arasi akaryakit harcamalarinin %2,99 oran ile vadelendirilmesi</t>
+        </is>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk tuzel kartlari: Saglam Business Kart, Miles&amp;Smiles Business Kart, Tohum Kart ve ek/sanal kartlari</t>
+        </is>
+      </c>
+      <c r="U195" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ finansman_tutari: 300 TL - 500.000 TL bir harcama ARALIGI, kampanyanin finansman tutari degil; ayrica sayfa basliginda '500 - 300.00 Arasi' yazim hatasi var
+BELIRSIZ taksit_sayisi: taksit sayisini musteri kendi belirliyor, sayfa sabit bir sayi vermiyor</t>
+        </is>
+      </c>
+      <c r="X195" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 13.08.2026 - 31.08.2026
+kampanya_bitis: 13.08.2026 - 31.08.2026
+kar_payi_orani: 300 TL - 500.000 TL arasındaki akaryakıt harcamaları %2,99 oran ile vadelendirilecektir.
+oran_periyodu: 300 TL - 500.000 TL arasındaki akaryakıt harcamaları %2,99 oran ile vadelendirilecektir.</t>
         </is>
       </c>
     </row>
@@ -13653,6 +13734,14 @@
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/musteri-ol-kampanyalari/hepsiburadada-yeni-musteriye-ozel-vade-farksiz-50000-tl-firsati</t>
         </is>
       </c>
+      <c r="F205" t="n">
+        <v>0</v>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="J205" t="n">
         <v>50000</v>
       </c>
@@ -13679,7 +13768,8 @@
       <c r="U205" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ kar_payi_orani: vade farksiz kampanya; sayfada kar payi orani verilmiyor</t>
+BELIRSIZ kar_payi_orani: vade farksiz kampanya; sayfada kar payi orani verilmiyor
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="V205" t="n">
@@ -13690,7 +13780,8 @@
           <t>kampanya_baslangic: 7.03.2025 - 31.12.2026
 kampanya_bitis: 7.03.2025 - 31.12.2026
 taksit_sayisi: 50.000 TL'ye kadar olan Hepsiburada sepetinizi 9 taksit ile ödemek için Kuveyt Türk müşterisi olun!
-finansman_tutari: Kuveyt Türk Alışveriş Finansmanı’na Kuveyt Türk müşterisi olmadan önce 50.000 TL’ye kadar olan Hepsiburada sepetinizi oluşturduktan sonra ödeme anında hemen başvurabilirsiniz.</t>
+finansman_tutari: Kuveyt Türk Alışveriş Finansmanı’na Kuveyt Türk müşterisi olmadan önce 50.000 TL’ye kadar olan Hepsiburada sepetinizi oluşturduktan sonra ödeme anında hemen başvurabilirsiniz.
+kar_payi_orani: Hepsiburada’da Yeni Müşteriye Özel Vade Farksız 50.000 TL Fırsatı!</t>
         </is>
       </c>
     </row>
@@ -14560,14 +14651,57 @@
           <t>Sağlam Business Kart QR Ödeme ile 4.000 TL' ye Varan Altın Puan Fırsatı!</t>
         </is>
       </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Ticari Kampanya</t>
+        </is>
+      </c>
       <c r="E229" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/kart-kampanyalari/saglam-business-kart-qr-odeme-ile-4000-tl-ye-varan-altin-puan-firsati</t>
         </is>
       </c>
-      <c r="U229" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K229" t="n">
+        <v>4000</v>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>Altin Puan</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>QR ile yapilan 5.000 TL ve uzeri her harcamada %5, toplamda en fazla 4.000 TL Altin Puan</t>
+        </is>
+      </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="P229" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q229" t="inlineStr">
+        <is>
+          <t>Saglam Business Kredi Karti sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U229" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: %5 bir PUAN kazanim orani, kar payi orani degil
+BELIRSIZ finansman_tutari: 5.000 TL harcama ESIGI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X229" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 25.06.2026 - 31.12.2026
+kampanya_bitis: 25.06.2026 - 31.12.2026
+odul_miktari: Kampanyadan maksimum kazanım 4.000 TL Altın Puan'dır.
+odul_birimi: Kampanyadan maksimum kazanım 4.000 TL Altın Puan'dır.</t>
         </is>
       </c>
     </row>
@@ -14644,14 +14778,42 @@
           <t>Araç kiralamalarında Enterprise Rent-A-Car genel kiralama koşulları geçerlidir.</t>
         </is>
       </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E231" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/enterpriseta-arac-kiralamalarinizda-30-indirim</t>
         </is>
       </c>
-      <c r="U231" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>Enterprise ofislerinde ve online arac kiralamalarinda liste fiyati uzerinden %30 indirim; tek seferde en fazla 30 gunluk kiralama</t>
+        </is>
+      </c>
+      <c r="P231" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q231" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U231" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ kar_payi_orani: %30 bir INDIRIM orani, kar payi orani degil
+BELIRSIZ odul_miktari: odul yuzde indirim olarak veriliyor, tutar belirtilmiyor</t>
+        </is>
+      </c>
+      <c r="X231" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: kampanyası 31.12.2026 tarihine kadar tüm</t>
         </is>
       </c>
     </row>
@@ -14899,6 +15061,14 @@
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-pttavmcomda-pesin-fiyatina-2-taksit</t>
         </is>
       </c>
+      <c r="F238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M238" t="inlineStr">
         <is>
           <t>pttavm.com'da tek seferde yapilan 3.000 TL ve uzeri alisverislerde vade farksiz 2 taksit</t>
@@ -14918,7 +15088,8 @@
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
-BELIRSIZ finansman_tutari: 3.000 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
+BELIRSIZ finansman_tutari: 3.000 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="V238" t="n">
@@ -14927,7 +15098,8 @@
       <c r="X238" s="2" t="inlineStr">
         <is>
           <t>taksit_sayisi: Paraf ile 31 Temmuz 2026 tarihine kadar www.pttavm.com adresinden tek seferde yapılacak alışverişlerde vade farksız 2 taksit imkanı sunulacaktır.
-kampanya_bitis: Paraf ile 31 Temmuz 2026 tarihine kadar www.pttavm.com adresinden tek seferde yapılacak alışverişlerde vade farksız 2 taksit imkanı sunulacaktır.</t>
+kampanya_bitis: Paraf ile 31 Temmuz 2026 tarihine kadar www.pttavm.com adresinden tek seferde yapılacak alışverişlerde vade farksız 2 taksit imkanı sunulacaktır.
+kar_payi_orani: Paraf ile 31 Temmuz 2026 tarihine kadar www.pttavm.com adresinden tek seferde yapılacak alışverişlerde vade farksız 2 taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -15636,6 +15808,14 @@
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-a101de-vade-farksiz-6-aya-varan-taksit-firsati</t>
         </is>
       </c>
+      <c r="F258" t="n">
+        <v>0</v>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M258" t="inlineStr">
         <is>
           <t>A101 magazalari ve a101.com.tr'de 300 TL ve uzeri alisverislerde vade farksiz 6 aya varan taksit</t>
@@ -15655,7 +15835,8 @@
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
-BELIRSIZ finansman_tutari: 300 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
+BELIRSIZ finansman_tutari: 300 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="V258" t="n">
@@ -15664,7 +15845,8 @@
       <c r="X258" s="2" t="inlineStr">
         <is>
           <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Paraf ile A101 Mağazalarında ve www.a101.com.tr ‘de Paraf POS’undan yapılacak 300 TL ve üzeri alışverişlerinizde vade farksız, peşin fiyatına 6 aya varan
-kampanya_bitis: 31 Ağustos 2026 tarihine kadar Paraf ile A101 Mağazalarında ve www.a101.com.tr ‘de Paraf POS’undan yapılacak 300 TL ve üzeri alışverişlerinizde vade farksız, peşin fiyatına 6 aya varan</t>
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Paraf ile A101 Mağazalarında ve www.a101.com.tr ‘de Paraf POS’undan yapılacak 300 TL ve üzeri alışverişlerinizde vade farksız, peşin fiyatına 6 aya varan
+kar_payi_orani: Paraf ile A101’de Vade Farksız 6 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
     </row>
@@ -16131,6 +16313,14 @@
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-demirdokumde-9-taksit-firsati</t>
         </is>
       </c>
+      <c r="F267" t="n">
+        <v>0</v>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M267" t="inlineStr">
         <is>
           <t>DemirDokum sanal POS'u uzerinden yapilan islemlere vade farksiz 9 ay taksit; bayi POS'u haric</t>
@@ -16149,7 +16339,8 @@
       <c r="U267" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="V267" t="n">
@@ -16158,7 +16349,8 @@
       <c r="X267" s="2" t="inlineStr">
         <is>
           <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Paraf üyesi DemirDöküm sanal POS’u üzerinden işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.
-kampanya_bitis: 31 Ağustos 2026 tarihine kadar Paraf üyesi DemirDöküm sanal POS’u üzerinden işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.</t>
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Paraf üyesi DemirDöküm sanal POS’u üzerinden işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.
+kar_payi_orani: 31 Ağustos 2026 tarihine kadar Paraf üyesi DemirDöküm sanal POS’u üzerinden işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -16240,6 +16432,14 @@
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/altinyildiz-classicste-vade-farksiz-2-taksit-firsati</t>
         </is>
       </c>
+      <c r="F269" t="n">
+        <v>0</v>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M269" t="inlineStr">
         <is>
           <t>Altinyildiz Classics resmi web sitesinde vade farksiz 2 taksit</t>
@@ -16262,7 +16462,8 @@
       </c>
       <c r="U269" s="2" t="inlineStr">
         <is>
-          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi</t>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="V269" t="n">
@@ -16272,7 +16473,8 @@
         <is>
           <t>taksit_sayisi: Altınyıldız Classics Resmi Web Sitesinde Vade Farksız 2 Taksit Fırsatı!
 kampanya_baslangic: 28.07.2026 - 31.12.2026
-kampanya_bitis: 28.07.2026 - 31.12.2026</t>
+kampanya_bitis: 28.07.2026 - 31.12.2026
+kar_payi_orani: Altınyıldız Classics'te Vade Farksız 2 Taksit Fırsatı</t>
         </is>
       </c>
     </row>
@@ -16719,6 +16921,14 @@
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/desa-grupta-vade-farksiz-2-taksit-firsati</t>
         </is>
       </c>
+      <c r="F278" t="n">
+        <v>0</v>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M278" t="inlineStr">
         <is>
           <t>Desa Grup (Samsonite, Desa, Adesa) magazalarinda vade farksiz 2 taksit</t>
@@ -16741,7 +16951,8 @@
       </c>
       <c r="U278" s="2" t="inlineStr">
         <is>
-          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi</t>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="V278" t="n">
@@ -16751,7 +16962,8 @@
         <is>
           <t>taksit_sayisi: Kuveyt Türk bireysel kredi kartları ile 31 Aralık 2026 tarihine kadar Desa Grubun (Samsonite, Desa , Adesa) mağazalarında yapacağınız alışverişlerinizde vade farksız 2 taksit imkanı sizi bekliyor.
 kampanya_baslangic: 16.09.2025 - 31.12.2026
-kampanya_bitis: 16.09.2025 - 31.12.2026</t>
+kampanya_bitis: 16.09.2025 - 31.12.2026
+kar_payi_orani: Desa Grup’ta Vade Farksız 2 Taksit Fırsatı</t>
         </is>
       </c>
     </row>
@@ -16860,6 +17072,14 @@
           <t>https://www.kuveytturk.com.tr/isim-icin/dis-ticaret/e-ihracat/e-ihracat-kampanyalari/e-ihracatcilara-ozel-shipentegra-ile-yurtdisi-kargo-gonderilerinize-vade-farksiz-3-taksit</t>
         </is>
       </c>
+      <c r="F281" t="n">
+        <v>0</v>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M281" t="inlineStr">
         <is>
           <t>ShipEntegra uzerinden yapilan yurt disi kargo odemelerinde vade farksiz 3 taksit</t>
@@ -16883,7 +17103,8 @@
       <c r="U281" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ kar_payi_orani: vade farksiz kampanya; sayfada kar payi orani verilmiyor</t>
+BELIRSIZ kar_payi_orani: vade farksiz kampanya; sayfada kar payi orani verilmiyor
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="V281" t="n">
@@ -16893,7 +17114,8 @@
         <is>
           <t>kampanya_baslangic: 6.08.2026 - 31.12.2026
 kampanya_bitis: 6.08.2026 - 31.12.2026
-taksit_sayisi: Kuveyt Türk Ticari kredi kartlarınızla ShipEntegra üzerinden yapacağınız yurt dışı kargo ödemelerinde vade farksız 3 taksit avantajı sizleri bekliyor!</t>
+taksit_sayisi: Kuveyt Türk Ticari kredi kartlarınızla ShipEntegra üzerinden yapacağınız yurt dışı kargo ödemelerinde vade farksız 3 taksit avantajı sizleri bekliyor!
+kar_payi_orani: E-İhracatçılara Özel ShipEntegra ile Yurtdışı Kargo Gönderilerinize Vade Farksız 3 Taksit!</t>
         </is>
       </c>
     </row>
@@ -17327,6 +17549,14 @@
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/gundogdu-mobilyada-vade-farksiz-9-aya-varan-taksit-firsati</t>
         </is>
       </c>
+      <c r="F290" t="n">
+        <v>0</v>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M290" t="inlineStr">
         <is>
           <t>Gundogdu Mobilya magazalari ve web sitesinde vade farksiz 9 aya varan taksit</t>
@@ -17349,7 +17579,8 @@
       </c>
       <c r="U290" s="2" t="inlineStr">
         <is>
-          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi</t>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="V290" t="n">
@@ -17359,7 +17590,8 @@
         <is>
           <t>taksit_sayisi: Kuveyt Türk kredi kartlarıyla Gündoğdu Mobilya'da vade farksız 9 taksit fırsatını kaçırmayın!
 kampanya_baslangic: 11.11.2025 - 31.12.2026
-kampanya_bitis: 11.11.2025 - 31.12.2026</t>
+kampanya_bitis: 11.11.2025 - 31.12.2026
+kar_payi_orani: Gündoğdu Mobilya’da Vade Farksız 9 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
     </row>
@@ -17604,6 +17836,14 @@
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/koctasta-vade-farksiz-6-aya-varan-taksit-firsati</t>
         </is>
       </c>
+      <c r="F296" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M296" t="inlineStr">
         <is>
           <t>Koctas resmi web sitesinde 10.000 TL ve uzeri alisverislerde vade farksiz 6 aya varan taksit</t>
@@ -17627,7 +17867,8 @@
       <c r="U296" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ finansman_tutari: 10.000 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
+BELIRSIZ finansman_tutari: 10.000 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="V296" t="n">
@@ -17637,7 +17878,8 @@
         <is>
           <t>taksit_sayisi: Koçtaş’ta Vade Farksız 6 Aya Varan Taksit Fırsatı!
 kampanya_baslangic: 31.12.2025 - 31.12.2026
-kampanya_bitis: 31.12.2025 - 31.12.2026</t>
+kampanya_bitis: 31.12.2025 - 31.12.2026
+kar_payi_orani: Koçtaş’ta Vade Farksız 6 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
     </row>
@@ -18073,6 +18315,14 @@
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-schaferde-pesin-fiyatina-9-taksit</t>
         </is>
       </c>
+      <c r="F306" t="n">
+        <v>0</v>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M306" t="inlineStr">
         <is>
           <t>Schafer magazalarinda ParafPOS'lardan yapilan alisverislerde vade farksiz 9 aya varan taksit</t>
@@ -18084,64 +18334,66 @@
         </is>
       </c>
       <c r="U306" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
+        </is>
+      </c>
+      <c r="V306" t="n">
+        <v>9</v>
+      </c>
+      <c r="X306" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Paraf ile Schafer mağazalarında ParafPOS’larından yapacağınız alışverişlerde vade farksız 9 aya varan taksit imkanı sağlanacaktır.
+kar_payi_orani: Paraf ile Schafer mağazalarında ParafPOS’larından yapacağınız alışverişlerde vade farksız 9 aya varan taksit imkanı sağlanacaktır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>ZK-062</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Ziraat Katılım</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Modalifeta 9 Taksit</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/modalifeta-9-taksit</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>ModaLife'ta yapilan alisverislerde 9 taksit</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U307" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
 BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
 BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
-      <c r="V306" t="n">
-        <v>9</v>
-      </c>
-      <c r="X306" s="2" t="inlineStr">
-        <is>
-          <t>taksit_sayisi: Paraf ile Schafer mağazalarında ParafPOS’larından yapacağınız alışverişlerde vade farksız 9 aya varan taksit imkanı sağlanacaktır.</t>
-        </is>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="inlineStr">
-        <is>
-          <t>ZK-062</t>
-        </is>
-      </c>
-      <c r="B307" t="inlineStr">
-        <is>
-          <t>Ziraat Katılım</t>
-        </is>
-      </c>
-      <c r="C307" t="inlineStr">
-        <is>
-          <t>Modalifeta 9 Taksit</t>
-        </is>
-      </c>
-      <c r="D307" t="inlineStr">
-        <is>
-          <t>Kart Kampanyasi</t>
-        </is>
-      </c>
-      <c r="E307" t="inlineStr">
-        <is>
-          <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/modalifeta-9-taksit</t>
-        </is>
-      </c>
-      <c r="M307" t="inlineStr">
-        <is>
-          <t>ModaLife'ta yapilan alisverislerde 9 taksit</t>
-        </is>
-      </c>
-      <c r="Q307" t="inlineStr">
-        <is>
-          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
-        </is>
-      </c>
-      <c r="U307" s="2" t="inlineStr">
-        <is>
-          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
-BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
-        </is>
-      </c>
       <c r="V307" t="n">
         <v>9</v>
       </c>
@@ -18204,6 +18456,14 @@
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-vaillantta-9-aya-varan-taksit</t>
         </is>
       </c>
+      <c r="F309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="M309" t="inlineStr">
         <is>
           <t>Vaillant sanal POS'u uzerinden yapilan islemlere vade farksiz 9 ay taksit; bayi POS'u haric</t>
@@ -18222,7 +18482,8 @@
       <c r="U309" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
         </is>
       </c>
       <c r="V309" t="n">
@@ -18231,7 +18492,8 @@
       <c r="X309" s="2" t="inlineStr">
         <is>
           <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar Paraf üyesi Vaillant sanal POS’u üzerinden yapılan işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.
-kampanya_bitis: 31 Ağustos 2026 tarihine kadar Paraf üyesi Vaillant sanal POS’u üzerinden yapılan işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.</t>
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar Paraf üyesi Vaillant sanal POS’u üzerinden yapılan işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.
+kar_payi_orani: 31 Ağustos 2026 tarihine kadar Paraf üyesi Vaillant sanal POS’u üzerinden yapılan işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bes kampanyaya aday deger, oran periyodu span uyumsuzlugu giderildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -12854,14 +12854,56 @@
           <t>Sağlam Business Kart Akaryakıt Harcamalarınıza 600 TL’ye Varan Altın Puan Fırsat</t>
         </is>
       </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Ticari Kampanya</t>
+        </is>
+      </c>
       <c r="E180" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/kart-kampanyalari/saglam-business-kart-akaryakit-harcamalariniza-600-tlye-varan-altin-puan-firsati</t>
         </is>
       </c>
-      <c r="U180" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K180" t="n">
+        <v>600</v>
+      </c>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>Altin Puan</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>Her ay 2.000 TL ve uzeri akaryakit harcamalarinda 100 TL, toplamda en fazla 600 TL Altin Puan</t>
+        </is>
+      </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q180" t="inlineStr">
+        <is>
+          <t>Saglam Business Kredi Karti sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U180" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ finansman_tutari: 2.000 TL harcama ESIGI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X180" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 25.06.2026 - 31.12.2026
+kampanya_bitis: 25.06.2026 - 31.12.2026
+odul_miktari: Kampanyadan maksimum kazanım tutarı 600 TL Altın Puan’dır.
+odul_birimi: Kampanyadan maksimum kazanım tutarı 600 TL Altın Puan’dır.</t>
         </is>
       </c>
     </row>
@@ -13430,8 +13472,7 @@
         <is>
           <t>kampanya_baslangic: 13.08.2026 - 31.08.2026
 kampanya_bitis: 13.08.2026 - 31.08.2026
-kar_payi_orani: 300 TL - 500.000 TL arasındaki akaryakıt harcamaları %2,99 oran ile vadelendirilecektir.
-oran_periyodu: 300 TL - 500.000 TL arasındaki akaryakıt harcamaları %2,99 oran ile vadelendirilecektir.</t>
+kar_payi_orani: 300 TL - 500.000 TL arasındaki akaryakıt harcamaları %2,99 oran ile vadelendirilecektir.</t>
         </is>
       </c>
     </row>
@@ -14597,14 +14638,33 @@
           <t>Pazaramada 6 Taksit</t>
         </is>
       </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E227" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/pazaramada-6-taksit</t>
         </is>
       </c>
-      <c r="U227" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>pazarama.com'da 1.000 TL uzeri alisverislerde pesin fiyatina 2 veya 3 taksit, 6.000 TL uzeri alisverislerde 6 taksit</t>
+        </is>
+      </c>
+      <c r="Q227" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U227" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ taksit_sayisi: metin tutara gore birden fazla deger veriyor (2 veya 3 taksit, 6 taksit) - tek deger secilemez
+BELIRSIZ finansman_tutari: 1.000 / 6.000 TL harcama ESIKLERI, kampanyanin finansman tutari degil
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
     </row>
@@ -15024,14 +15084,57 @@
           <t>Toptancı Harcamalarınıza Her Ay Ekstra 5.000 Mil'e Varan Fırsat!</t>
         </is>
       </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Ticari Kampanya</t>
+        </is>
+      </c>
       <c r="E237" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/kart-kampanyalari/toptanci-harcamalariniza-her-ay-ekstra-5000-mile-varan-firsat</t>
         </is>
       </c>
-      <c r="U237" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K237" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>Mil</t>
+        </is>
+      </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>Her ay 50.000 TL ve uzeri toptanci harcamalarinda ekstra %5, aylik en fazla 5.000 Mil</t>
+        </is>
+      </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="P237" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q237" t="inlineStr">
+        <is>
+          <t>Miles&amp;Smiles Kuveyt Turk Business kart sahipleri (ek ve sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U237" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: %5 bir EKSTRA MIL kazanim orani, kar payi orani degil
+BELIRSIZ finansman_tutari: 50.000 TL harcama ESIGI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X237" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 25.06.2026 - 31.12.2026
+kampanya_bitis: 25.06.2026 - 31.12.2026
+odul_miktari: Kampanyadan maksimum kazanım tutarı 5.000 Mil'dir.
+odul_birimi: Kampanyadan maksimum kazanım tutarı 5.000 Mil'dir.</t>
         </is>
       </c>
     </row>
@@ -15638,14 +15741,51 @@
           <t>Elçi Tur’dan Kuveyt Türk Müşterilerine Özel Yaz Fırsatı</t>
         </is>
       </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E253" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/elci-turdan-kuveyt-turk-musterilerine-ozel-yaz-firsati</t>
         </is>
       </c>
-      <c r="U253" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>Elci Tur'da yildizli otellerde %10, helal hassasiyetli yurt disi turlarinda %8, umre turlarinda %6 indirim; yurt ici otel rezervasyonlarinda vade farksiz 9 taksit</t>
+        </is>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk kredi karti sahipleri</t>
+        </is>
+      </c>
+      <c r="U253" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: sayfadaki %10/%8/%6 oranlari INDIRIM oranlari, kar payi orani degil
+BELIRSIZ odul_miktari: odul yuzde indirim olarak veriliyor, tutar belirtilmiyor</t>
+        </is>
+      </c>
+      <c r="V253" t="n">
+        <v>9</v>
+      </c>
+      <c r="X253" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Yıldızlı otellerde %10 indirim, Helal hassasiyetli yurt dışı turlarında %8 indirim, Tüm umre turlarında %6 indirim, yurt içi Otel rezervasyonlarında vade farksız 9 taksit
+kampanya_baslangic: 20.05.2026 - 15.09.2026
+kampanya_bitis: 20.05.2026 - 15.09.2026</t>
         </is>
       </c>
     </row>
@@ -17690,14 +17830,58 @@
           <t>Gürgençler'de 9 Aya Varan Taksit İmkanı!</t>
         </is>
       </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E293" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/gurgenclerde-9-aya-varan-taksit-imkani</t>
         </is>
       </c>
-      <c r="U293" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="F293" t="n">
+        <v>0</v>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>Gurgencler Bilisim magazalari ve web sitesinde Apple alisverislerinde vade farksiz 9 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>2025-06-27</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk bireysel kredi kartlari (Saglam Kart, Saglam Kart Kampus/Genc, Miles&amp;Smiles, World Elite) ve ek kartlari</t>
+        </is>
+      </c>
+      <c r="U293" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi</t>
+        </is>
+      </c>
+      <c r="V293" t="n">
+        <v>9</v>
+      </c>
+      <c r="X293" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Gürgençler mağazalarında Kuveyt Türk Bireysel Kredi Kartları ile Apple alışverişlerinde 9 aya varan taksit imkanı sizi bekliyor!
+kampanya_baslangic: 27.06.2025 - 31.12.2026
+kampanya_bitis: 27.06.2025 - 31.12.2026
+kar_payi_orani: Kuveyt Türk Bireysel Kredi Kartları, 31 Aralık 2026 tarihine kadar Gürgençler Bilişim mağazalarında ve web sitesinde yapacağınız alışverişlerde vade farksız 9 taksite varan imkanla</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dort kampanyaya daha aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -13600,14 +13600,55 @@
           <t>Esnaf, Çiftçi ve Tüzel Şirketlerin Faturası Bizden!</t>
         </is>
       </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Musteri Ol Kampanyasi</t>
+        </is>
+      </c>
       <c r="E200" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/musteri-ol-kampanyalari/esnaf-ciftci-ve-tuzel-sirketlerin-faturasi-bizden</t>
         </is>
       </c>
-      <c r="U200" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K200" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>3 adet fatura talimatinin otomatik odenmesiyle birinciye 250, ikinciye 350, ucuncuye 400 TL olmak uzere toplam 1.000 TL</t>
+        </is>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>2025-02-14</t>
+        </is>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>2027-12-31</t>
+        </is>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk Mobil'den musteri olan sahis firmasi, ciftci ve tuzel sirketler</t>
+        </is>
+      </c>
+      <c r="U200" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi</t>
+        </is>
+      </c>
+      <c r="X200" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 14.02.2025 - 31.12.2027
+kampanya_bitis: 14.02.2025 - 31.12.2027
+odul_miktari: Kuveyt Türk Mobil'den müşteri olan şahıs firması, çiftçi ve tüzel şirketlere 1.000 TL!
+odul_birimi: Kuveyt Türk Mobil'den müşteri olan şahıs firması, çiftçi ve tüzel şirketlere 1.000 TL!</t>
         </is>
       </c>
     </row>
@@ -13684,14 +13725,33 @@
           <t>Saglik Sektorunde 5 Taksit</t>
         </is>
       </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E202" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/saglik-sektorunde-5-taksit</t>
         </is>
       </c>
-      <c r="U202" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>Saglik sektorunde tek seferde 2.500 TL ve uzeri 3-4 taksitli islemlere +5 ek taksit</t>
+        </is>
+      </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>Taksit ozelligi olan bireysel Ziraat Katilim Bankkart sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U202" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ taksit_sayisi: kampanya EK taksit veriyor (+5) ve yalnizca 3-4 taksitli islemlerde; mutlak taksit sayisi degil
+BELIRSIZ finansman_tutari: 2.500 TL bir islem ESIGI ('ve uzeri'), kampanyanin finansman tutari degil
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
     </row>
@@ -14080,14 +14140,41 @@
           <t>Istanbul Havalimani Hizli Gecis Kampanyasi</t>
         </is>
       </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E213" t="inlineStr">
         <is>
           <t>https://www.albaraka.com.tr/tr/kampanyalar/detay/istanbul-havalimani-hizli-gecis-kampanyasi</t>
         </is>
       </c>
-      <c r="U213" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>Istanbul Havalimani dis hatlar Fast Track noktalarinda ucretsiz hizli gecis; kullanici basina 2 kod</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil uzerinden GastroClub kodu alan musteriler</t>
+        </is>
+      </c>
+      <c r="U213" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ odul_miktari: odul ayni (ucretsiz gecis hakki), parasal tutar verilmiyor</t>
+        </is>
+      </c>
+      <c r="X213" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya, 31.12.2026 tarihine kadar geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -18603,14 +18690,47 @@
           <t>Kuveyt Turkten E Ticaret E Ihracat Ve Tekno Girisimcilere Ozel Firsat</t>
         </is>
       </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Ticari Kampanya</t>
+        </is>
+      </c>
       <c r="E308" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/kart-kampanyalari/kuveyt-turkten-e-ticaret-e-ihracat-ve-tekno-girisimcilere-ozel-firsat</t>
         </is>
       </c>
-      <c r="U308" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>Marqby web sitesinden yapilan marka basvuru ucretlerinde %15'e varan indirim; resmi harclar haric</t>
+        </is>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk Ticari kredi karti sahibi e-ticaret, e-ihracat ve tekno girisimci musteriler</t>
+        </is>
+      </c>
+      <c r="U308" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: %15 bir INDIRIM orani, kar payi orani degil
+BELIRSIZ odul_miktari: odul yuzde indirim olarak veriliyor, tutar belirtilmiyor</t>
+        </is>
+      </c>
+      <c r="X308" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 20.07.2026 - 31.12.2026
+kampanya_bitis: 20.07.2026 - 31.12.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
uc Bankkart Lira kampanyasina aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -11100,14 +11100,56 @@
           <t>Giyim Ve Ayakkabi Alisverisinizde Toplam 1000 TL Bankkart Lira</t>
         </is>
       </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E130" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/giyim-ve-ayakkabi-alisverisinizde-toplam-1000-tl-bankkart-lira-2</t>
         </is>
       </c>
-      <c r="U130" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K130" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>Giyim ve ayakkabi sektorunde 5.000-9.999 TL alisverise 500 TL, 10.000 TL ve uzerine 1.000 TL, toplam en fazla 1.000 TL Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Q130" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim bireysel Bankkart kredi karti sahipleri (ticari ve ucretsiz kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U130" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ finansman_tutari: 5.000 / 10.000 TL harcama ESIKLERI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X130" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 10 Temmuz 2026 – 7 Ağustos 2026
+kampanya_bitis: 10 Temmuz 2026 – 7 Ağustos 2026
+odul_miktari: Kampanya müşteri bazındadır ve bir müşteri en fazla 1.000 TL Bankkart Lira kazanılabilecektir.
+odul_birimi: Kampanya müşteri bazındadır ve bir müşteri en fazla 1.000 TL Bankkart Lira kazanılabilecektir.</t>
         </is>
       </c>
     </row>
@@ -12259,14 +12301,56 @@
           <t>Veteriner Ve Petshop Harcamalariniza 2000 TL Bankkart Lira</t>
         </is>
       </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E162" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/veteriner-ve-petshop-harcamalariniza-2000-tl-bankkart-lira</t>
         </is>
       </c>
-      <c r="U162" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K162" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>Veteriner ve petshop sektorunde her 2.000 TL uzeri alisverise 200 TL, her 5.000 TL uzeri alisverise 500 TL, toplam en fazla 2.000 TL Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart asil kart sahipleri (ticari ve ucretsiz kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U162" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ finansman_tutari: 2.000 / 5.000 TL harcama ESIKLERI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X162" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 8 Ağustos – 7 Eylül 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 8 Ağustos – 7 Eylül 2026 tarihleri arasında geçerlidir.
+odul_miktari: Kampanya müşteri bazındadır ve bir müşteri en fazla 2000 TL Bankkart Lira kazanabilecektir.
+odul_birimi: Kampanya müşteri bazındadır ve bir müşteri en fazla 2000 TL Bankkart Lira kazanabilecektir.</t>
         </is>
       </c>
     </row>
@@ -12431,14 +12515,56 @@
           <t>Bagimsiz Karta Ozel 5000 Tlye Varan Bankkart Lira</t>
         </is>
       </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E167" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/bagimsiz-karta-ozel-5000-tlye-varan-bankkart-lira-2</t>
         </is>
       </c>
-      <c r="U167" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K167" t="n">
+        <v>5000</v>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>Egitim, saglik, spor ve kultur-sanat uye isyerlerinde tum harcamalara %10, toplamda 5.000 TL Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart Bagimsiz kredi karti sahipleri</t>
+        </is>
+      </c>
+      <c r="U167" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: %10 bir IADE orani, kar payi orani degil</t>
+        </is>
+      </c>
+      <c r="X167" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 8 Ağustos – 7 Eylül 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 8 Ağustos – 7 Eylül 2026 tarihleri arasında geçerlidir.
+odul_miktari: tüm harcamalara %10, toplamda 5.000 TL Bankkart Lira!
+odul_birimi: tüm harcamalara %10, toplamda 5.000 TL Bankkart Lira!</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
uc kampanyaya daha aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -10626,14 +10626,33 @@
           <t>Trendyolda 6ya Varan Taksit</t>
         </is>
       </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E116" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/trendyolda-6ya-varan-taksit</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>Trendyol'da 1.000 TL uzeri secili urun alisverislerinde pesin fiyatina 3 taksit, 6.000 TL uzeri alisverislerde 6 taksit; tek seferde 200.000 TL'ye kadar</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart kredi karti sahipleri (ucretsiz ve ticari kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U116" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ taksit_sayisi: metin tutara gore iki deger veriyor (1.000 TL uzeri 3 taksit, 6.000 TL uzeri 6 taksit) - tek deger secilemez
+BELIRSIZ finansman_tutari: 1.000 / 6.000 TL harcama ESIKLERI; 200.000 TL ise taksit imkaninin ust siniri, kampanyanin finansman tutari degil
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor</t>
         </is>
       </c>
     </row>
@@ -10883,14 +10902,56 @@
           <t>Aile Karta Ozel 2000 Tlye Varan Bankkart Lira</t>
         </is>
       </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E123" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/aile-karta-ozel-2000-tlye-varan-bankkart-lira-2</t>
         </is>
       </c>
-      <c r="U123" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K123" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>Market, akaryakit, giyim, egitim ve saglik uye isyerlerinde 10.000 TL'ye kadar harcamalara %5, 20.000 TL'ye kadar harcamalara %10 Bankkart Lira; en fazla 2.000 TL</t>
+        </is>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="P123" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="Q123" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Bankkart Aile kredi karti sahipleri</t>
+        </is>
+      </c>
+      <c r="U123" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: %5 ve %10 IADE oranlari, kar payi orani degil; ayrica tek deger yok</t>
+        </is>
+      </c>
+      <c r="X123" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 8 Ağustos – 7 Eylül 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 8 Ağustos – 7 Eylül 2026 tarihleri arasında geçerlidir.
+odul_miktari: Kampanya müşteri bazındadır ve bir müşteri kampanyadan en fazla 2.000 TL Bankkart Lira
+odul_birimi: Kampanya müşteri bazındadır ve bir müşteri kampanyadan en fazla 2.000 TL Bankkart Lira</t>
         </is>
       </c>
     </row>
@@ -18904,14 +18965,47 @@
           <t>Kuveyt Turklulere Windy Carda 30 Indirim Firsati</t>
         </is>
       </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E305" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/kuveyt-turklulere-windy-carda-30-indirim-firsati</t>
         </is>
       </c>
-      <c r="U305" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>windycar.com.tr uzerinden KT2026 kodu ile yapilan online arac kiralamalarda %30 indirim; 1-24 gun arasi kiralamalarda gecerli</t>
+        </is>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk bireysel ve tuzel kredi karti sahipleri</t>
+        </is>
+      </c>
+      <c r="U305" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: %30 bir INDIRIM orani, kar payi orani degil
+BELIRSIZ odul_miktari: odul yuzde indirim olarak veriliyor, tutar belirtilmiyor</t>
+        </is>
+      </c>
+      <c r="X305" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 1.07.2026 - 31.12.2026
+kampanya_bitis: 1.07.2026 - 31.12.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dort kampanyaya daha aday deger, iki sayfa celiskisi not edildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -11713,14 +11713,56 @@
           <t>Optik Alisverisinize 500 TL Bankkart Lira</t>
         </is>
       </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E144" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/optik-alisverisinize-500-tl-bankkart-lira-2</t>
         </is>
       </c>
-      <c r="U144" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K144" t="n">
+        <v>500</v>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>Optik sektorunde tek seferde 5.000 TL uzeri alisverise 250 TL, 10.000 TL uzeri alisverise 500 TL, en fazla 500 TL Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim bireysel Bankkart asil kart sahipleri (ticari ve ucretsiz kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U144" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ finansman_tutari: 5.000 / 10.000 TL harcama ESIKLERI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X144" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 10 Temmuz – 7 Ağustos 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 10 Temmuz – 7 Ağustos 2026 tarihleri arasında geçerlidir.
+odul_miktari: Kampanya müşteri bazındadır ve bir müşteri en fazla 500 TL Bankkart Lira kazanabilir.
+odul_birimi: Kampanya müşteri bazındadır ve bir müşteri en fazla 500 TL Bankkart Lira kazanabilir.</t>
         </is>
       </c>
     </row>
@@ -13889,14 +13931,46 @@
           <t>Macrocenter.com.tr'de Albaraka müşterilerine özel ayrıcalıklar sizi bekliyor.</t>
         </is>
       </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E198" t="inlineStr">
         <is>
           <t>https://www.albaraka.com.tr/tr/kampanyalar/detay/macrocentercomtrde-10-indirim</t>
         </is>
       </c>
-      <c r="U198" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K198" t="n">
+        <v>150</v>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>Macroonline ve macrocenter.com.tr'de 1.500 TL'ye kadar alisverislerde %10 indirim, en fazla 150 TL; ayda iki kez</t>
+        </is>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>Albaraka Mobil uzerinden GastroClub kodu alan musteriler</t>
+        </is>
+      </c>
+      <c r="U198" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kar_payi_orani: %10 bir INDIRIM orani, kar payi orani degil</t>
+        </is>
+      </c>
+      <c r="X198" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: %10 indirim kodu 1500 TL'ye kadar yapılan alışverişlerde geçerlidir. Kampanya kapsamında maksimum 150 TL indirim kazanılabilir.
+odul_birimi: %10 indirim kodu 1500 TL'ye kadar yapılan alışverişlerde geçerlidir. Kampanya kapsamında maksimum 150 TL indirim kazanılabilir.</t>
         </is>
       </c>
     </row>
@@ -15028,14 +15102,51 @@
           <t>Okula Dönüşte 300 TL'ye Varan Altın Puan!</t>
         </is>
       </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E225" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/kendim-icin/kart-kampanyalari/okula-donuste-300-tlye-varan-altin-puan</t>
         </is>
       </c>
-      <c r="U225" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K225" t="n">
+        <v>300</v>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>Altin Puan</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>Tek seferde 2.000 TL ve uzeri giyim, egitim ve kirtasiye harcamalarina 100 TL, toplamda en fazla 300 TL Altin Puan</t>
+        </is>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="Q225" t="inlineStr">
+        <is>
+          <t>Kuveyt Turk bireysel Saglam Nakit Kart sahipleri ve bagli sanal kartlar</t>
+        </is>
+      </c>
+      <c r="U225" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_bitis: SAYFA CELISKISI: 'Kampanya Tarihleri' alani 31.12.2026 diyor, metin govdesi ise harcamalar icin uc kez '31 Ekim 2026 tarihine kadar' diyor - hangisinin kampanya bitisi oldugu secilemez
+BELIRSIZ finansman_tutari: 2.000 TL bir harcama ESIGI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X225" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 20.08.2026 - 31.12.2026
+odul_miktari: Kampanya kapsamında müşteri başına toplamda en fazla 300 TL Altın Puan kazanılabilir.
+odul_birimi: Kampanya kapsamında müşteri başına toplamda en fazla 300 TL Altın Puan kazanılabilir.</t>
         </is>
       </c>
     </row>
@@ -17308,14 +17419,45 @@
           <t>Paraf Ile Dysonda 9 Aya Varan Taksit</t>
         </is>
       </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E273" t="inlineStr">
         <is>
           <t>https://www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/paraf-ile-dysonda-9-aya-varan-taksit</t>
         </is>
       </c>
-      <c r="U273" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>dyson.com.tr'de pesin fiyatina 6 aya varan taksit; firma tarafindan belirlenen tutarin uzerinde gecerli</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U273" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ kampanya_adi: SAYFA CELISKISI: baslik '9 Aya Varan Taksit' diyor, metin govdesi iki yerde '6 aya varan / 6 taksit' diyor. Metin esas alindi - imzalamadan once sayfaya bakin</t>
+        </is>
+      </c>
+      <c r="V273" t="n">
+        <v>6</v>
+      </c>
+      <c r="X273" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 31 Ağustos 2026 tarihine kadar dyson.com.tr'den peşin fiyatına 6 aya varan taksit fırsatından faydalanabilirsiniz.
+kampanya_bitis: 31 Ağustos 2026 tarihine kadar dyson.com.tr'den peşin fiyatına 6 aya varan taksit fırsatından faydalanabilirsiniz.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
iki kampanyaya daha aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -11025,14 +11025,56 @@
           <t>Kuveyt Turk Ile E Ihracat Gonderilerinizde Mil Kazanin</t>
         </is>
       </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Ticari Kampanya</t>
+        </is>
+      </c>
       <c r="E126" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kampanyalar/isim-icin/kart-kampanyalari/kuveyt-turk-ile-e-ihracat-gonderilerinizde-mil-kazanin</t>
         </is>
       </c>
-      <c r="U126" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K126" t="n">
+        <v>60000</v>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>Mil</t>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>Navlungo uzerinden yurt disi kargo harcamalarinda her ay %10 mil, ayda en fazla 10.000 Mil, yil sonuna kadar 60.000 Mil; ilk kez Navlungo kullananlara %15 indirim</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="P126" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q126" t="inlineStr">
+        <is>
+          <t>Miles&amp;Smiles Kuveyt Turk kredi karti sahibi e-ihracat musterileri</t>
+        </is>
+      </c>
+      <c r="U126" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kar_payi_orani: %10 bir MIL kazanim orani, %15 ise Navlungo indirimi - ikisi de kar payi orani degil</t>
+        </is>
+      </c>
+      <c r="X126" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 16.07.2026 - 31.12.2026
+kampanya_bitis: 16.07.2026 - 31.12.2026
+odul_miktari: Miles&amp;Smiles Kuveyt Türk kartlarınızla Navlungo üzerinden yapacağınız yurt dışı kargo harcamalarında yıl sonuna kadar 60.000 Mil kazanma fırsatı sizi bekliyor!
+odul_birimi: Miles&amp;Smiles Kuveyt Türk kartlarınızla Navlungo üzerinden yapacağınız yurt dışı kargo harcamalarında yıl sonuna kadar 60.000 Mil kazanma fırsatı sizi bekliyor!</t>
         </is>
       </c>
     </row>
@@ -13403,14 +13445,56 @@
           <t>QR Ile Odemelerinize Toplam 100 TL Bankkart Lira</t>
         </is>
       </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E182" t="inlineStr">
         <is>
           <t>https://www.ziraatkatilim.com.tr/kart-kampanyalari/qr-ile-odemelerinize-toplam-100-tl-bankkart-lira-2</t>
         </is>
       </c>
-      <c r="U182" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K182" t="n">
+        <v>100</v>
+      </c>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim Mobil ile POS'ta QR odemede tek seferde 500 TL ve uzeri her alisverise 25 TL, toplam en fazla 100 TL Bankkart Lira</t>
+        </is>
+      </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="Q182" t="inlineStr">
+        <is>
+          <t>Ziraat Katilim bireysel Bankkart kredi karti sahipleri (ticari ve ucretsiz kartlar haric)</t>
+        </is>
+      </c>
+      <c r="U182" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ finansman_tutari: 500 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X182" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 10 Temmuz 2026 - 7 Ağustos 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 10 Temmuz 2026 - 7 Ağustos 2026 tarihleri arasında geçerlidir.
+odul_miktari: Kampanya müşteri bazındadır ve bir müşteri en fazla 100 TL Bankkart Lira kazanabilecektir.
+odul_birimi: Kampanya müşteri bazındadır ve bir müşteri en fazla 100 TL Bankkart Lira kazanabilecektir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
alti Dunya Katilim kampanyasina aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -10385,14 +10385,42 @@
           <t>Trendyol'da Peşin Fiyatına 9 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E111" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/trendyol</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>Trendyol'da 1.000 TL uzeri taksitli alisverislerde pesin fiyatina 3 taksit, 6.000 TL uzeri secili urunlerde 6, 10.000 TL uzeri secili urunlerde 9 taksit; tek seferde 200.000 TL'ye kadar</t>
+        </is>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q111" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U111" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ taksit_sayisi: metin tutara gore uc deger veriyor (3 / 6 / 9 taksit) - tek deger secilemez
+BELIRSIZ finansman_tutari: 1.000 / 6.000 TL harcama ESIKLERI; 200.000 TL taksit ust siniri - kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X111" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -10742,14 +10770,42 @@
           <t>Pazarama Paraf</t>
         </is>
       </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E118" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/pazarama-paraf</t>
         </is>
       </c>
-      <c r="U118" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>Pazarama'da 600 TL uzeri alisverislerde 2 taksit, 1.000 TL uzeri 3 taksit, 6.000 TL uzeri 6 taksit</t>
+        </is>
+      </c>
+      <c r="P118" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q118" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U118" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ taksit_sayisi: metin tutara gore uc deger veriyor (2 / 3 / 6 taksit) - tek deger secilemez
+BELIRSIZ finansman_tutari: 600 / 1.000 / 6.000 TL harcama ESIKLERI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X118" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -11145,14 +11201,45 @@
           <t>Casper.com.tr'de Peşin Fiyatına 6 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E125" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/casper-com-tr-de-pesin-fiyatina-6-taksit-firsati</t>
         </is>
       </c>
-      <c r="U125" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>Casper.com.tr'de Paraf POS'undan yapilan alisverislerde pesin fiyatina 3 taksit</t>
+        </is>
+      </c>
+      <c r="P125" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q125" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U125" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ kampanya_adi: SAYFA CELISKISI: baslik '6 Taksit' diyor, metin iki yerde '3 taksit' diyor - metin esas alindi</t>
+        </is>
+      </c>
+      <c r="V125" t="n">
+        <v>3</v>
+      </c>
+      <c r="X125" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Taksit kampanyasından yararlanabilmek için işlem anında 3 taksitin seçilmesi gerekmektedir.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -11577,14 +11664,45 @@
           <t>İder Mobilya’da 7 Taksite %15 indirim Fırsatı!</t>
         </is>
       </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E132" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/ider</t>
         </is>
       </c>
-      <c r="U132" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>Ider Mobilya magazalarinda 7 taksit ve %15 indirim; indirim yalnizca 6 ve 7 taksitte, franchise magazalarda kosullar degisebilir</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U132" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ kar_payi_orani: %15 bir INDIRIM orani, kar payi orani degil</t>
+        </is>
+      </c>
+      <c r="V132" t="n">
+        <v>7</v>
+      </c>
+      <c r="X132" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Dünya Katılım Paraf ile İder Mobilya mağazalarında Paraf POS’larından yapacağınız alışverişlerde 7 taksit imkanı sunulacak ve %15 indirim uygulan
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -11987,14 +12105,45 @@
           <t>İpekyol’da 4 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E139" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/ipekyol</t>
         </is>
       </c>
-      <c r="U139" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>Ipekyol magazalari ve web sitesinde 5.000 TL uzeri alisverislerde 4 taksit</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U139" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ finansman_tutari: 5.000 TL bir harcama ESIGI ('uzeri'), kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="V139" t="n">
+        <v>4</v>
+      </c>
+      <c r="X139" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: ’de Paraf POS’larından yapılacak 5.000 TL üzeri alışverişlerde 4 taksit imkanı sunulacaktır.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -12392,14 +12541,47 @@
           <t>Paraf</t>
         </is>
       </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E146" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/paraf</t>
         </is>
       </c>
-      <c r="U146" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K146" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>Nisan ayinda toplam 5.000 TL ve uzeri harcamaya %10 nakit iade, en fazla 1.000 TL</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>SMS bildirimi alan fiziki Dunya Katilim Paraf Kredi Karti sahipleri; sanal kartlar haric</t>
+        </is>
+      </c>
+      <c r="U146" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa 'Nisan ayi' diyor ama YIL vermiyor; 'Bitis Tarihi' alani bos ('-')
+BELIRSIZ kampanya_bitis: sayfa '30 Nisan saat 23:59' diyor ama YIL vermiyor; 'Bitis Tarihi' alani bos ('-')
+BELIRSIZ kar_payi_orani: %10 bir NAKIT IADE orani, kar payi orani degil
+BELIRSIZ finansman_tutari: 5.000 TL bir harcama ESIGI, kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X146" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Kampanya kapsamında kazanılabilecek maximum iade 1.000 TL’ dir.
+odul_birimi: Kampanya kapsamında kazanılabilecek maximum iade 1.000 TL’ dir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
yedi Dunya Katilim kampanyasina aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -12975,14 +12975,52 @@
           <t>Kampanyadan Dünya Katılım Paraf kartlar faydalanabilecektir.</t>
         </is>
       </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E153" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/a-101-paraf</t>
         </is>
       </c>
-      <c r="U153" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>A101'de 300 TL ve uzeri alisverislerde vade farksiz, pesin fiyatina 6 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U153" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ taksit_sayisi: '6 aya varan' ifadesi ust sinir; sabit taksit sayisi verilmiyor
+BELIRSIZ finansman_tutari: 300 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil
+BELIRSIZ kampanya_adi: korpustan gelen baslik bozuk - sayfa metninin bir cumlesi baslik olarak alinmis, imzalamadan once duzeltilmeli</t>
+        </is>
+      </c>
+      <c r="X153" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026
+kar_payi_orani: ‘de Paraf POS’undan yapılacak 300 TL ve üzeri alışverişlerinizde vade farksız, peşin fiyatına 6 aya varan taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -13273,14 +13311,44 @@
           <t>Adv</t>
         </is>
       </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E159" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/adv</t>
         </is>
       </c>
-      <c r="U159" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>ADV magazalarinda Paraf POS'larindan yapilan alisverislerde 6 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U159" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V159" t="n">
+        <v>6</v>
+      </c>
+      <c r="X159" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Mağazalardan yapılacak alışverişlerde 6 taksitten yararlanabilmek için kampanyanın satış görevlisine belirtilmesi gerekmektedir.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -13561,14 +13629,44 @@
           <t>Alfemo’da Peşin fiyatına 8 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E164" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/alfemo</t>
         </is>
       </c>
-      <c r="U164" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>Alfemo magazalari ve alfemo.com'da Paraf POS'larindan yapilan alisverislerde 8 taksit</t>
+        </is>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U164" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V164" t="n">
+        <v>8</v>
+      </c>
+      <c r="X164" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Dünya Katılım Paraf ile Alfemo mağazalarında veya www.alfemo.com web sayfasından Paraf POS’larından yapacağınız alışverişlerde 8 taksit imka
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -13855,14 +13953,45 @@
           <t>Carter's Mağazalarında 4 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E169" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/carter-s</t>
         </is>
       </c>
-      <c r="U169" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>Carter's magazalarinda Paraf POS'larindan yapilan alisverislerde 4 taksit; web sitesi haric</t>
+        </is>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U169" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ kampanya_adi: sayfa 'Sona erdi' isaretli - kampanya suresi dolmus</t>
+        </is>
+      </c>
+      <c r="V169" t="n">
+        <v>4</v>
+      </c>
+      <c r="X169" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Dünya Katılım Paraf ile Carter's mağazalarında Paraf POS’larından yapılacak alışverişlerde 4 taksit imkanı sunulacaktır.
+kampanya_bitis: Bitiş Tarihi: 30 Haziran 2026</t>
         </is>
       </c>
     </row>
@@ -14150,14 +14279,44 @@
           <t>Divarese’de 4 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E174" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/divarese</t>
         </is>
       </c>
-      <c r="U174" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>Divarese'de Paraf POS'larindan yapilan alisverislerde 4 taksit</t>
+        </is>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U174" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V174" t="n">
+        <v>4</v>
+      </c>
+      <c r="X174" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Mağazalardan yapılacak alışverişlerde 4 taksitten yararlanabilmek için kampanyanın satış görevlisine belirtilmesi gerekmektedir.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -14426,14 +14585,44 @@
           <t>Dyson’da Peşin Fiyatına 9 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E179" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/dyson</t>
         </is>
       </c>
-      <c r="U179" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>dyson.com.tr'de pesin fiyatina 9 aya varan taksit; firma tarafindan belirlenen tutarin uzerinde gecerli</t>
+        </is>
+      </c>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q179" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U179" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V179" t="n">
+        <v>9</v>
+      </c>
+      <c r="X179" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: 9 taksit avantajı firmanın belirlediği tutarın üzerinde yapacağınız alışverişlerde geçerlidir.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -14714,14 +14903,44 @@
           <t>Paraf ile Evidea’da 4 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E184" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/evidea</t>
         </is>
       </c>
-      <c r="U184" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>Evidea web sitesi ve magazalarinda Paraf POS'u uzerinden taksitli alisverislere 4 taksit</t>
+        </is>
+      </c>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q184" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U184" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V184" t="n">
+        <v>4</v>
+      </c>
+      <c r="X184" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Kampanyadan faydalanmak için ödeme esnasında POS üzerinden 4 taksitin seçilmesi gerekmektedir.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
dokuz Dunya Katilim kampanyasina aday deger yazildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -15200,14 +15200,50 @@
           <t>Gürgençler’de Peşin Fiyatına 9 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E189" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/gurgencler</t>
         </is>
       </c>
-      <c r="U189" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="F189" t="n">
+        <v>0</v>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>Gurgencler'de Paraf POS'undan yapilan taksitli alisverislerde vade farksiz 9 aya varan taksit; odemede 3, 6 veya 9 taksit secilmeli</t>
+        </is>
+      </c>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q189" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U189" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ taksit_sayisi: metin '3, 6 veya 9 taksit' secenegi sunuyor - tek deger secilemez</t>
+        </is>
+      </c>
+      <c r="X189" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026
+kar_payi_orani: ’de Paraf POS’undan yapılacak taksitli alışverişlerde vade farksız 9 aya varan taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -15494,14 +15530,44 @@
           <t>İncehesap.Com'da Peşin Fiyatına 3 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E194" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/incehesap</t>
         </is>
       </c>
-      <c r="U194" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>Incehesap.com'da Paraf POS'undan yapilan alisverislerde pesin fiyatina 3 taksit</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U194" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V194" t="n">
+        <v>3</v>
+      </c>
+      <c r="X194" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Taksit kampanyasından yararlanabilmek için işlem anında 3 taksitin seçilmesi gerekmektedir.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -15751,14 +15817,53 @@
           <t>ITOPYA.COM'da Vade Farksız 6 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E199" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/itopya</t>
         </is>
       </c>
-      <c r="U199" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="F199" t="n">
+        <v>0</v>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>ITOPYA.COM'da vade farksiz 6 taksit</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U199" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V199" t="n">
+        <v>6</v>
+      </c>
+      <c r="X199" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Kampanyadan faydalanmak için ödeme esnasında POS üzerinden 6 taksitin seçilmesi gerekmektedir.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026
+kar_payi_orani: ’dan yapılacak taksitli alışverişinize vade farksız 6 taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -16012,14 +16117,42 @@
           <t>DKart Debit'le Jack &amp; Jones’da Harcadıkça Kazanın!</t>
         </is>
       </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E204" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/jack-jones</t>
         </is>
       </c>
-      <c r="U204" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>Jack &amp; Jones alisverislerinde harcamanin bir orani kadar aninda nakit iade</t>
+        </is>
+      </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>DKart Debit kart sahipleri</t>
+        </is>
+      </c>
+      <c r="U204" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ odul_miktari: iade orani ve tavani sayfada eksik gorunuyor ('...'i kadar nakit iade') - tutar okunamiyor
+BELIRSIZ kar_payi_orani: iade orani metinde eksik; ayrica iade orani kar payi orani degil</t>
+        </is>
+      </c>
+      <c r="X204" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -16263,14 +16396,44 @@
           <t>Kip</t>
         </is>
       </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E209" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/kip</t>
         </is>
       </c>
-      <c r="U209" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>Kip'te Paraf POS'larindan yapilan alisverislerde 5 taksit</t>
+        </is>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U209" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V209" t="n">
+        <v>5</v>
+      </c>
+      <c r="X209" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: ’de Paraf POS’larından yapılacak alışverişlerde 5 taksit imkanı sunulacaktır.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -16516,14 +16679,44 @@
           <t>Paraf ile Koçtaş'ta 5 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E214" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/koctas</t>
         </is>
       </c>
-      <c r="U214" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>Koctas'ta Paraf POS'undan yapilan alisverislerde 5 taksit</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U214" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V214" t="n">
+        <v>5</v>
+      </c>
+      <c r="X214" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Dünya Katılım Paraf ile Koçtaş’ta Paraf POS'undan yapacağınız alışverişlerinize 5 taksit fırsatı sunulacaktır.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -16761,14 +16954,50 @@
           <t>Monster Notebook’ta Peşin Fiyatına 12 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E219" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/monster</t>
         </is>
       </c>
-      <c r="U219" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="F219" t="n">
+        <v>0</v>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>Monster Notebook'ta vade farksiz 12 aya varan taksit; odemede 3, 6, 9 veya 12 taksit secilmeli</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q219" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U219" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ taksit_sayisi: metin '3, 6, 9 veya 12 taksit' secenegi sunuyor - tek deger secilemez</t>
+        </is>
+      </c>
+      <c r="X219" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026
+kar_payi_orani: ’de yapılacak taksitli alışverişlerde vade farksız 12 aya varan taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -17006,14 +17235,44 @@
           <t>Network’te 4 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E224" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/network</t>
         </is>
       </c>
-      <c r="U224" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>Network'te Paraf POS'larindan yapilan alisverislerde 4 taksit</t>
+        </is>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q224" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U224" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V224" t="n">
+        <v>4</v>
+      </c>
+      <c r="X224" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Paraf POS’larından yapılacak alışverişlerde 4 taksit imkanı sunulacaktır.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -17201,14 +17460,44 @@
           <t>Touristica.com.tr'de Peşin Fiyatına 9 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E228" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/touristica</t>
         </is>
       </c>
-      <c r="U228" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>Touristica.com.tr'de yapilan alisverislerde 9 taksit</t>
+        </is>
+      </c>
+      <c r="P228" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q228" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U228" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V228" t="n">
+        <v>9</v>
+      </c>
+      <c r="X228" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: mağazalarından yapılacak alışverişlerde 9 taksit imkanı sunulacaktır.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
yedi kampanyaya daha aday deger, bir kayit kampanya olmadigi icin isaretlendi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -17699,14 +17699,41 @@
           <t>Vestel’de 9 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E232" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/vestel</t>
         </is>
       </c>
-      <c r="U232" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>Vestel web sitesinde pesin fiyatina 7 taksit, Paraf uyesi Vestel magazalarinda 9'a varan taksit</t>
+        </is>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q232" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U232" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ taksit_sayisi: kanala gore iki deger var: web sitesinde 7 taksit, magazalarda 9'a varan - tek deger secilemez</t>
+        </is>
+      </c>
+      <c r="X232" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -17913,14 +17940,44 @@
           <t>Yataş’ta 8 Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E236" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/yatas</t>
         </is>
       </c>
-      <c r="U236" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>Yatas Bedding, Enza, Puffy ve Divanev magazalari ve web sitelerinde Paraf POS'larindan 8 taksit</t>
+        </is>
+      </c>
+      <c r="P236" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q236" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U236" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V236" t="n">
+        <v>8</v>
+      </c>
+      <c r="X236" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Yataş’ta 8 Taksit Fırsatı!
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -18131,14 +18188,41 @@
           <t>Paraf ile Yenilio'da Peşin Fiyatına 12 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E240" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/yenilio</t>
         </is>
       </c>
-      <c r="U240" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>Yenilio magazalari ve yenilio.com'da Paraf POS'undan yapilan alisverislere 12 aya varan taksit</t>
+        </is>
+      </c>
+      <c r="P240" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q240" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U240" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ taksit_sayisi: '12 aya varan' ifadesi ust sinir; sabit taksit sayisi verilmiyor</t>
+        </is>
+      </c>
+      <c r="X240" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -18292,14 +18376,44 @@
           <t>Zsa Zsa Zsu</t>
         </is>
       </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E244" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/zsa-zsa-zsu</t>
         </is>
       </c>
-      <c r="U244" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>Zsa Zsa Zsu magazalarinda Paraf POS'larindan yapilan alisverislerde 6 taksit</t>
+        </is>
+      </c>
+      <c r="P244" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U244" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V244" t="n">
+        <v>6</v>
+      </c>
+      <c r="X244" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Dünya Katılım Paraf ile Zsa Zsa Zsu mağazalarında Paraf POS’larından yapacağınız alışverişlerde 6 taksit imkanı sağlanacaktır.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
         </is>
       </c>
     </row>
@@ -18495,14 +18609,53 @@
           <t>Paraf ile Demirdöküm’de 9 Aya Varan Taksit Fırsatı!</t>
         </is>
       </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E248" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/demirdokum</t>
         </is>
       </c>
-      <c r="U248" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="F248" t="n">
+        <v>0</v>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>Demirdokum sanal POS'u uzerinden gerceklesen islemlere vade farksiz 9 ay taksit</t>
+        </is>
+      </c>
+      <c r="P248" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kart sahipleri (sanal kartlar dahil)</t>
+        </is>
+      </c>
+      <c r="U248" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor</t>
+        </is>
+      </c>
+      <c r="V248" t="n">
+        <v>9</v>
+      </c>
+      <c r="X248" s="2" t="inlineStr">
+        <is>
+          <t>taksit_sayisi: Dünya Katılım Paraf ile Paraf üyesi Demirdöküm sanal Pos’u üzerinden gerçekleşecek işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026
+kar_payi_orani: Dünya Katılım Paraf ile Paraf üyesi Demirdöküm sanal Pos’u üzerinden gerçekleşecek işlemlere vade farksız 9 ay taksit imkanı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -18698,14 +18851,47 @@
           <t>Paraf Kart’la alışverişe başla, TOD ayrıcalığını ücretsiz yaşa!</t>
         </is>
       </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E252" t="inlineStr">
         <is>
           <t>https://dunyakatilim.com.tr/kampanyalar/tod-paraf</t>
         </is>
       </c>
-      <c r="U252" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>Toplam 1.000 TL ve uzeri alisverise ozel 3 aylik TOD Trendyol Superlig Paketi hediye</t>
+        </is>
+      </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>Dunya Katilim Paraf kredi karti sahipleri</t>
+        </is>
+      </c>
+      <c r="U252" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ odul_miktari: odul ayni (3 aylik TOD Trendyol Superlig Paketi), parasal tutar verilmiyor
+BELIRSIZ finansman_tutari: 1.000 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
+        </is>
+      </c>
+      <c r="X252" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: 01.01.2026 - 29.01.2026 tarihleri arasında Dünya Katılım Paraf kredi kartı ile yapacağınız toplam 1.000 TL ve üzeri alışverişine ö
+kampanya_bitis: 01.01.2026 - 29.01.2026 tarihleri arasında Dünya Katılım Paraf kredi kartı ile yapacağınız toplam 1.000 TL ve üzeri alışverişine ö</t>
         </is>
       </c>
     </row>
@@ -18909,9 +19095,10 @@
           <t>https://dunyakatilim.com.tr/kampanyalar/tahsile-cek</t>
         </is>
       </c>
-      <c r="U256" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="U256" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_adi: BU BIR KAMPANYA DEGIL: sayfa 'Tahsile Cek' bankacilik URUNUNU anlatan bir bilgi sayfasi; kampanya tarihi, odulu veya kosulu yok. Altin setten cikarilmasi degerlendirilmeli</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kuyruktaki 200 taslagin tamami islendi, span dogrulamasi butunluk testiyle ayni kaynagi kullaniyor
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -13040,14 +13040,51 @@
           <t>E-Ticarette Altın Kazandıran Kampanya | Kuveyt Türk Katılım Bankası</t>
         </is>
       </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E154" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/kendim-icin/kampus/e-ticarette-altin-kazandiran-kampanya</t>
         </is>
       </c>
-      <c r="U154" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="K154" t="n">
+        <v>250</v>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>Altin Puan</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>E-ticaret harcamalarinda %10 Altin Puan, ayda en fazla 250 TL; her ay yeniden katilim gerekli</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>18-25 yas arasi universite ogrencisi Kuveyt Turk Kampus musterileri (Saglam Kart Kampus dahil)</t>
+        </is>
+      </c>
+      <c r="U154" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+BELIRSIZ kar_payi_orani: %10 bir ALTIN PUAN kazanim orani, kar payi orani degil</t>
+        </is>
+      </c>
+      <c r="X154" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: E-Ticarette Altın Kazandıran Kampanya, 31 Aralık 2026 tarihine kadar geçerlidir.
+odul_miktari: Harcamalarını Kuveyt Türk kredi kartın ile yaptığında, her ay 250 TL’ye kadar Altın Puan kazanabilirsin.
+odul_birimi: Harcamalarını Kuveyt Türk kredi kartın ile yaptığında, her ay 250 TL’ye kadar Altın Puan kazanabilirsin.</t>
         </is>
       </c>
     </row>
@@ -13775,34 +13812,34 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>Yurt icinde tek seferde 20.000 TL ve uzeri ilk gida marketi, bakkal, kasap, manav ve sarkuteri alisverisine 800 TL ParafPara; musteri basina bir kez</t>
+          <t>Yurt ici gida marketi, bakkal, kasap, manav ve sarkuteride tek seferde 7.500 TL ve uzeri her market harcamasina ParafPara; musteri basina en fazla 800 TL</t>
         </is>
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>SMS ile kampanyaya katilan Emlak Katilim Paraf kart sahipleri</t>
+          <t>SMS ile kampanyaya katilan Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
         </is>
       </c>
       <c r="U166" s="2" t="inlineStr">
         <is>
           <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ finansman_tutari: 20.000 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
+BELIRSIZ finansman_tutari: 7.500 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
         </is>
       </c>
       <c r="X166" s="2" t="inlineStr">
         <is>
-          <t>kampanya_baslangic: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
+          <t>kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
 odul_miktari: Kampanya müşteri bazlı olup, bir müşteri kampanyaya bir kez katılabilir ve en fazla 800 TL ParafPara kazanabilir.
 odul_birimi: Kampanya müşteri bazlı olup, bir müşteri kampanyaya bir kez katılabilir ve en fazla 800 TL ParafPara kazanabilir.</t>
         </is>
@@ -16369,14 +16406,33 @@
           <t>Albaraka Otopark ve Vale Harcamanıza %50 İndirim Kazandırıyor! | Albaraka Türk</t>
         </is>
       </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Kart Kampanyasi</t>
+        </is>
+      </c>
       <c r="E208" t="inlineStr">
         <is>
           <t>https://www.albaraka.com.tr/tr/kampanyalar/detay/albaraka-otopark-ve-vale-harcamaniza-10-indirim-kazandiriyorr</t>
         </is>
       </c>
-      <c r="U208" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>Otopark ve vale harcamalarinda %50 indirim</t>
+        </is>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>Albaraka kart sahipleri</t>
+        </is>
+      </c>
+      <c r="U208" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: korpustaki metin menu agirlikli; kampanya kosullari bolumu yakalanamamis
+BELIRSIZ kampanya_bitis: korpustaki metin menu agirlikli; kampanya kosullari bolumu yakalanamamis
+BELIRSIZ kar_payi_orani: %50 bir INDIRIM orani, kar payi orani degil
+BELIRSIZ odul_miktari: indirim tavani korpustaki metinde gorunmuyor - sayfanin JS ile tazelenmesi gerekebilir</t>
         </is>
       </c>
     </row>
@@ -18242,14 +18298,42 @@
           <t>12 Aya Kadar ödemesiz dönemli ve indirimli Tarım Finansmanı Kuveyt Türk'te! | Ku</t>
         </is>
       </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Finansman Kampanyasi</t>
+        </is>
+      </c>
       <c r="E241" t="inlineStr">
         <is>
           <t>https://www.kuveytturk.com.tr/isim-icin/tarim-bankaciligi/tarim-ve-hayvancilik-sektorune-ozel-kampanyalar/12-aya-kadar-odemesiz-donemli-ve-indirimli-tarim-finansmani-kuveyt-turkte</t>
         </is>
       </c>
-      <c r="U241" t="inlineStr">
-        <is>
-          <t>TASLAK - alanlar doldurulmadi, sayfaya bakilmadi. Degerleri girip giren_kisi'yi imzalayin.</t>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>Tarim ve hayvancilik sektorunde mal/hizmet alimlarina 12 aya kadar odemesiz donemli ve indirimli tarim finansmani</t>
+        </is>
+      </c>
+      <c r="Q241" t="inlineStr">
+        <is>
+          <t>Tarimsal uretim ve yetistiricilik yapan isletmeler, CKS belgeli ciftciler ve hayvancilik faaliyetinde bulunanlar</t>
+        </is>
+      </c>
+      <c r="U241" s="2" t="inlineStr">
+        <is>
+          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
+BELIRSIZ kampanya_baslangic: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kampanya_bitis: sayfada kampanya tarihi verilmiyor
+BELIRSIZ kar_payi_orani: sayfa 'avantajli oranlar' diyor ama sayisal oran vermiyor
+BELIRSIZ finansman_tutari: sayfada finansman tutari verilmiyor
+BELIRSIZ vade_ay: sayfada vade suresi verilmiyor; 12 ay ODEMESIZ DONEM (erteleme), vade degil</t>
+        </is>
+      </c>
+      <c r="W241" t="n">
+        <v>12</v>
+      </c>
+      <c r="X241" s="2" t="inlineStr">
+        <is>
+          <t>erteleme_suresi_ay: 12 Aya Kadar ödemesiz dönemli ve indirimli Tarım Finansmanı Kuveyt Türk'te!</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
son dort kayit imzalandi, altin set 302; imza filtresi testi gercek veriden bagimsizlastirildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -11035,12 +11035,22 @@
           <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri</t>
         </is>
       </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="U121" s="2" t="inlineStr">
         <is>
-          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+          <t>BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
 BELIRSIZ taksit_sayisi: metin tutara gore dort ayri deger veriyor (3 / 6 / 9 / 12 taksit) - tek deger secilemez
-BELIRSIZ finansman_tutari: 100 / 1.000 / 6.000 / 10.000 TL harcama ESIKLERI, kampanyanin finansman tutari degil</t>
+BELIRSIZ finansman_tutari: 100 / 1.000 / 6.000 / 10.000 TL harcama ESIKLERI, kampanyanin finansman tutari degil
+24.08.2026: ekran goruntusu ALINAMADI - emlakkatilim.com.tr otomatik tarayiciyi bloklyor (uc denemede de 237 karakterlik engel sayfasi dondu). Imza sayfanin tarayicida elle gorulmesine dayaniyor; goruntu kaniti yok.</t>
         </is>
       </c>
       <c r="X121" s="2" t="inlineStr">
@@ -12574,10 +12584,20 @@
           <t>SMS ile kampanyaya katilan Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
         </is>
       </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="U142" s="2" t="inlineStr">
         <is>
-          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ finansman_tutari: 10.000 / 24.999 TL harcama ESIKLERI, kampanyanin finansman tutari degil</t>
+          <t>BELIRSIZ finansman_tutari: 10.000 / 24.999 TL harcama ESIKLERI, kampanyanin finansman tutari degil
+24.08.2026: ekran goruntusu ALINAMADI - emlakkatilim.com.tr otomatik tarayiciyi bloklyor (uc denemede de 237 karakterlik engel sayfasi dondu). Imza sayfanin tarayicida elle gorulmesine dayaniyor; goruntu kaniti yok.</t>
         </is>
       </c>
       <c r="X142" s="2" t="inlineStr">
@@ -14259,10 +14279,20 @@
           <t>SMS ile kampanyaya katilan Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
         </is>
       </c>
+      <c r="S166" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T166" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="U166" s="2" t="inlineStr">
         <is>
-          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ finansman_tutari: 7.500 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil</t>
+          <t>BELIRSIZ finansman_tutari: 7.500 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil
+24.08.2026: ekran goruntusu ALINAMADI - emlakkatilim.com.tr otomatik tarayiciyi bloklyor (uc denemede de 237 karakterlik engel sayfasi dondu). Imza sayfanin tarayicida elle gorulmesine dayaniyor; goruntu kaniti yok.</t>
         </is>
       </c>
       <c r="X166" s="2" t="inlineStr">
@@ -19173,12 +19203,22 @@
           <t>Emlak Katilim Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
         </is>
       </c>
+      <c r="S238" t="inlineStr">
+        <is>
+          <t>Sara Toptamur</t>
+        </is>
+      </c>
+      <c r="T238" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
       <c r="U238" s="2" t="inlineStr">
         <is>
-          <t>MAKINE ADAYI - dogrulanmadi, imzasiz, olcum disi
-BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
+          <t>BELIRSIZ kampanya_baslangic: sayfa yalnizca bitis tarihi veriyor
 BELIRSIZ finansman_tutari: 3.000 TL bir harcama ESIGI ('ve uzeri'), kampanyanin finansman tutari degil
-vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)</t>
+vade farksiz kampanya -&gt; kar_payi_orani 0 (altin set konvansiyonu)
+24.08.2026: ekran goruntusu ALINAMADI - emlakkatilim.com.tr otomatik tarayiciyi bloklyor (uc denemede de 237 karakterlik engel sayfasi dondu). Imza sayfanin tarayicida elle gorulmesine dayaniyor; goruntu kaniti yok.</t>
         </is>
       </c>
       <c r="V238" t="n">

</xml_diff>

<commit_message>
kanit spani artik alanin degerini de desteklemek zorunda, TF-010 spani duzeltildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -11054,13 +11054,14 @@
         <is>
           <t>BELIRSIZ kar_payi_orani: metindeki 99/1 bir KAR PAYLASIM orani (banka-musteri paylasim anahtari), kar payi getiri orani degil - Rehber F sutunu
 BELIRSIZ vade_ay: vade GUN cinsinden ve araliksal veriliyor: '31-35 gun'; ay karsiligi tek bir sayiya indirgenemez
-BELIRSIZ finansman_tutari: 10.000 TL minimum / 10.000.000 TL maksimum HESAP ACILIS araligi, kampanyanin finansman tutari degil</t>
+BELIRSIZ finansman_tutari: 10.000 TL minimum / 10.000.000 TL maksimum HESAP ACILIS araligi, kampanyanin finansman tutari degil
+24.08.2026 denetim: tarih kanit spani duzeltildi - onceki span tarih icermiyordu.</t>
         </is>
       </c>
       <c r="X121" s="2" t="inlineStr">
         <is>
-          <t>kampanya_baslangic: Kampanya kapsamında, son üç aydır bankamızda TL mevduatı bulunmayan ve yukarıda belirtilen tarih aralığında TL cinsinden katılım hesabı açan bireysel müşterilerimize azami 99/1 kâr paylaşım oranı ile hesap açma avantajı sunulacaktır.
-kampanya_bitis: Kampanya kapsamında, son üç aydır bankamızda TL mevduatı bulunmayan ve yukarıda belirtilen tarih aralığında TL cinsinden katılım hesabı açan bireysel müşterilerimize azami 99/1 kâr paylaşım oranı ile hesap açma avantajı sunulacaktır.</t>
+          <t>kampanya_baslangic: Kampanya 31 Aralık 2025 ​- 31 Ağustos​ 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 31 Aralık 2025 ​- 31 Ağustos​ 2026 tarihleri arasında geçerlidir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kanit spani onerici butunluk testiyle ayni kaynagi kullaniyor, dokuz span dolduruldu
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -6484,6 +6484,13 @@
           <t>Sadece Cumartesi/Pazar, yalnizca yurt ici restoran/online yemek siparisi; once Katil butonuna basmak sart</t>
         </is>
       </c>
+      <c r="X62" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya 6 Mart-31 Ağustos 2026 tarihleri arasında yapılacak harcamalarda geçerlidir.
+kampanya_baslangic: Kampanya 6 Mart-31 Ağustos 2026 tarihleri arasında yapılacak harcamalarda geçerlidir.
+odul_miktari: Kampanya döneminde günlük kazanılabilecek maksimum iade 100 TL, bir takvim ayında kazanılabilecek maksimum iade ise 500 TL, kampanya dönemi boyunca kazanılabilecek iade 2.500 TL ile sınırlıdır.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="28.05" customHeight="1">
       <c r="A63" s="19" t="inlineStr">
@@ -6563,6 +6570,13 @@
       </c>
       <c r="V63" t="n">
         <v>10</v>
+      </c>
+      <c r="X63" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya 19.01.2026 – 30.09.2026 tarihleri arasında Hadi Black Kredi Kartı ile yapılacak özel okul ödemelerinde geçerlidir.
+kampanya_baslangic: Kampanya 19.01.2026 – 30.09.2026 tarihleri arasında Hadi Black Kredi Kartı ile yapılacak özel okul ödemelerinde geçerlidir.
+taksit_sayisi: Özel Okul Ödemelerinde 10 Taksit, üstelik vade farksız!</t>
+        </is>
       </c>
     </row>
     <row r="64" ht="28.05" customHeight="1">
@@ -6643,6 +6657,12 @@
       <c r="U64" s="20" t="inlineStr">
         <is>
           <t>En az 5 farkli gunde market harcamasi + ekstrenin zamaninda odenmesi sart; diger market kampanyalariyla birlesse de ekstre basina max 1.250 TL</t>
+        </is>
+      </c>
+      <c r="X64" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_bitis: Kampanya 26 Aralık 2025 - 25 Mart 2026 tarihleri arasında geçerlidir.
+kampanya_baslangic: Kampanya 26 Aralık 2025 - 25 Mart 2026 tarihleri arasında geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -18117,7 +18137,8 @@
         <is>
           <t>kampanya_baslangic: 20.08.2026 - 31.12.2026
 odul_miktari: Kampanya kapsamında müşteri başına toplamda en fazla 300 TL Altın Puan kazanılabilir.
-odul_birimi: Kampanya kapsamında müşteri başına toplamda en fazla 300 TL Altın Puan kazanılabilir.</t>
+odul_birimi: Kampanya kapsamında müşteri başına toplamda en fazla 300 TL Altın Puan kazanılabilir.
+kampanya_bitis: 20.08.2026 - 31.12.2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
TOM kayitlarinin kaynak url'sine eksik fragment eklendi, mukerrer url testi eklendi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -6427,7 +6427,7 @@
       </c>
       <c r="E62" s="19" t="inlineStr">
         <is>
-          <t>www.tombank.com.tr/kampanyalar.html</t>
+          <t>https://www.tombank.com.tr/kampanyalar.html#restoran-harcamalar-nda-10-i-ade-kazan</t>
         </is>
       </c>
       <c r="F62" s="21" t="n"/>
@@ -6481,7 +6481,8 @@
       </c>
       <c r="U62" s="20" t="inlineStr">
         <is>
-          <t>Sadece Cumartesi/Pazar, yalnizca yurt ici restoran/online yemek siparisi; once Katil butonuna basmak sart</t>
+          <t>Sadece Cumartesi/Pazar, yalnizca yurt ici restoran/online yemek siparisi; once Katil butonuna basmak sart
+24.08.2026 denetim: kaynak_url'ye eksik #fragment eklendi - TOM Bank kampanyalari tek sayfada anchor olarak yayimliyor, uc kayit ayni adresi gosteriyordu.</t>
         </is>
       </c>
       <c r="X62" s="2" t="inlineStr">
@@ -6515,7 +6516,7 @@
       </c>
       <c r="E63" s="19" t="inlineStr">
         <is>
-          <t>www.tombank.com.tr/kampanyalar.html</t>
+          <t>https://www.tombank.com.tr/kampanyalar.html#zel-okul-demelerinde-10-taksit-stelik-vade-farks-z</t>
         </is>
       </c>
       <c r="F63" s="21" t="n"/>
@@ -6565,7 +6566,8 @@
       </c>
       <c r="U63" s="20" t="inlineStr">
         <is>
-          <t>4 paket var (Standart/Orta/Ust/Ekstra: 250K-1,5M TL); en dusuk paket temel alindi. Vade farki iadesi, Gunluk Kazandiran Hesabinda ilgili tutar kadar birikim VEYA kredi bakiyesi sartina bagli - karmasik, notlarda ozetlendi | [9 Agu] vade_ay-&gt;taksit_sayisi tasindi (Ozel Okul Odemelerinde 10 Taksit); sayfada vade ifadesi yok</t>
+          <t>4 paket var (Standart/Orta/Ust/Ekstra: 250K-1,5M TL); en dusuk paket temel alindi. Vade farki iadesi, Gunluk Kazandiran Hesabinda ilgili tutar kadar birikim VEYA kredi bakiyesi sartina bagli - karmasik, notlarda ozetlendi | [9 Agu] vade_ay-&gt;taksit_sayisi tasindi (Ozel Okul Odemelerinde 10 Taksit); sayfada vade ifadesi yok
+24.08.2026 denetim: kaynak_url'ye eksik #fragment eklendi - TOM Bank kampanyalari tek sayfada anchor olarak yayimliyor, uc kayit ayni adresi gosteriyordu.</t>
         </is>
       </c>
       <c r="V63" t="n">
@@ -6602,7 +6604,7 @@
       </c>
       <c r="E64" s="19" t="inlineStr">
         <is>
-          <t>www.tombank.com.tr/kampanyalar.html</t>
+          <t>https://www.tombank.com.tr/kampanyalar.html#t-m-marketlerde-ge-erli-1-000-tl-ye-kadar-iade</t>
         </is>
       </c>
       <c r="F64" s="21" t="n"/>
@@ -6656,7 +6658,8 @@
       </c>
       <c r="U64" s="20" t="inlineStr">
         <is>
-          <t>En az 5 farkli gunde market harcamasi + ekstrenin zamaninda odenmesi sart; diger market kampanyalariyla birlesse de ekstre basina max 1.250 TL</t>
+          <t>En az 5 farkli gunde market harcamasi + ekstrenin zamaninda odenmesi sart; diger market kampanyalariyla birlesse de ekstre basina max 1.250 TL
+24.08.2026 denetim: kaynak_url'ye eksik #fragment eklendi - TOM Bank kampanyalari tek sayfada anchor olarak yayimliyor, uc kayit ayni adresi gosteriyordu.</t>
         </is>
       </c>
       <c r="X64" s="2" t="inlineStr">

</xml_diff>

<commit_message>
kampanya turu sayfa menusunden eslesiyordu: menu ayiklandi, kart anahtarlari ve tur semasi genisletildi, finansman tutari aralik guard'i duzeltildi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -12072,7 +12072,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Yatirim Kampanyasi</t>
+          <t>Yatirim Urunu Kampanyasi</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -20091,7 +20091,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Yatirim Kampanyasi</t>
+          <t>Yatirim Urunu Kampanyasi</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">

</xml_diff>

<commit_message>
vade farksiz etiketi 23 Agustos karariyla tutarli hale getirildi, kar payi eksenine tur koruma eklendi, taslak denetim raporu otomatik uretilir oldu
- terminology/sozluk.json: sifir_oran_ifadesi'nden "vade farksiz" cikarildi (gercek kod karariyla senkron degildi)
- 4 kayitta (VK-001/002/003/006) unutulmus kar_payi_orani=0 duzeltildi
- TF-004.kar_payi_orani=0 - gold'un atladigi tek gercek eksik (49 aday alandan)
- comparison/compare_engine.py: kar_payi_karsilastirilabilir_mi() eklendi, en_dusuk_kar_payi eksenini finansman turleriyle sinirliyor
- gold_dataset/denetim_raporu_uret.py: TASLAK kuyrugunu otomatik uretir (elle yazilan dosya 10/45 kaydi kaciriyordu)
- etiket_celiskisi_raporu.py okuma kilavuzu duzeltildi: yuksek guven cogunlukla menu/capraz-kampanya kirliligi cikti
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -2959,15 +2959,9 @@
           <t>www.vakifkatilim.com.tr/tr/kendim-icin/kampanyalar/detay/mtv-odemelerinde-vade-farksiz-3-taksit</t>
         </is>
       </c>
-      <c r="F20" s="21" t="n">
-        <v>0</v>
-      </c>
+      <c r="F20" s="21" t="n"/>
       <c r="G20" s="21" t="n"/>
-      <c r="H20" s="19" t="inlineStr">
-        <is>
-          <t>belirsiz</t>
-        </is>
-      </c>
+      <c r="H20" s="19" t="n"/>
       <c r="I20" s="22" t="n"/>
       <c r="J20" s="21" t="n">
         <v>100000</v>
@@ -3012,7 +3006,7 @@
       </c>
       <c r="U20" s="20" t="inlineStr">
         <is>
-          <t>VKart Business ve VKart Debit kapsam dışı; müşteri başına en fazla 3 MTV ödemesi DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. MTV odemesi taksitlendirmesi - Kart Kampanyasi, finansman vadesi yok. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+          <t>VKart Business ve VKart Debit kapsam dışı; müşteri başına en fazla 3 MTV ödemesi DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. MTV odemesi taksitlendirmesi - Kart Kampanyasi, finansman vadesi yok. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
         </is>
       </c>
       <c r="V20" t="n">
@@ -3045,15 +3039,9 @@
           <t>www.vakifkatilim.com.tr/tr/kendim-icin/kampanyalar/detay/troy-ile-gelir-vergisi-odemelerine-vade-farksiz-3-taksit_2</t>
         </is>
       </c>
-      <c r="F21" s="21" t="n">
-        <v>0</v>
-      </c>
+      <c r="F21" s="21" t="n"/>
       <c r="G21" s="21" t="n"/>
-      <c r="H21" s="19" t="inlineStr">
-        <is>
-          <t>belirsiz</t>
-        </is>
-      </c>
+      <c r="H21" s="19" t="n"/>
       <c r="I21" s="22" t="n"/>
       <c r="J21" s="21" t="n">
         <v>300000</v>
@@ -3098,7 +3086,7 @@
       </c>
       <c r="U21" s="20" t="inlineStr">
         <is>
-          <t>Sadece gib.gov.tr veya banka kanallarından yapılan ödemeler geçerli DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. Gelir vergisi odemesi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+          <t>Sadece gib.gov.tr veya banka kanallarından yapılan ödemeler geçerli DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. Gelir vergisi odemesi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
         </is>
       </c>
       <c r="V21" t="n">
@@ -3131,15 +3119,9 @@
           <t>www.vakifkatilim.com.tr/tr/kendim-icin/kampanyalar/detay/vkartla-saglikta-vade-farksiz-5-taksit</t>
         </is>
       </c>
-      <c r="F22" s="21" t="n">
-        <v>0</v>
-      </c>
+      <c r="F22" s="21" t="n"/>
       <c r="G22" s="21" t="n"/>
-      <c r="H22" s="19" t="inlineStr">
-        <is>
-          <t>belirsiz</t>
-        </is>
-      </c>
+      <c r="H22" s="19" t="n"/>
       <c r="I22" s="22" t="n"/>
       <c r="J22" s="21" t="n">
         <v>100000</v>
@@ -3184,7 +3166,7 @@
       </c>
       <c r="U22" s="20" t="inlineStr">
         <is>
-          <t>Müşteri başına en fazla 3 harcama taksitlendirilebilir DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Saglik harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+          <t>Müşteri başına en fazla 3 harcama taksitlendirilebilir DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Saglik harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
         </is>
       </c>
       <c r="V22" t="n">
@@ -3379,15 +3361,9 @@
           <t>www.vakifkatilim.com.tr/tr/kendim-icin/kampanyalar/detay/troyla-egitimde-vade-farksiz-5-taksit</t>
         </is>
       </c>
-      <c r="F25" s="21" t="n">
-        <v>0</v>
-      </c>
+      <c r="F25" s="21" t="n"/>
       <c r="G25" s="21" t="n"/>
-      <c r="H25" s="19" t="inlineStr">
-        <is>
-          <t>belirsiz</t>
-        </is>
-      </c>
+      <c r="H25" s="19" t="n"/>
       <c r="I25" s="22" t="n"/>
       <c r="J25" s="21" t="n">
         <v>700000</v>
@@ -3432,7 +3408,7 @@
       </c>
       <c r="U25" s="20" t="inlineStr">
         <is>
-          <t>Sadece TROY kart, ek/sanal kartlar dahil; müşteri başına en fazla 3 harcama DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Egitim harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+          <t>Sadece TROY kart, ek/sanal kartlar dahil; müşteri başına en fazla 3 harcama DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Egitim harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
         </is>
       </c>
       <c r="V25" t="n">
@@ -3870,9 +3846,15 @@
           <t>www.turkiyefinans.com.tr/tr-tr/kampanyalar/Sayfalar/yakininizi-davet-edin.aspx</t>
         </is>
       </c>
-      <c r="F31" s="21" t="n"/>
+      <c r="F31" s="21" t="n">
+        <v>0</v>
+      </c>
       <c r="G31" s="21" t="n"/>
-      <c r="H31" s="19" t="n"/>
+      <c r="H31" s="19" t="inlineStr">
+        <is>
+          <t>belirsiz</t>
+        </is>
+      </c>
       <c r="I31" s="22" t="n"/>
       <c r="J31" s="21" t="n"/>
       <c r="K31" s="21" t="n">
@@ -3922,13 +3904,14 @@
       <c r="U31" s="20" t="inlineStr">
         <is>
           <t>Davet edilenin Happy Bonus kredi kartı kullanmasi sart
-2026-08-23: kampanya rotasyonu - tarih kaynak sayfadan yeniden okundu (Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçe)</t>
+2026-08-23: kampanya rotasyonu - tarih kaynak sayfadan yeniden okundu (Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçe) | DUZELTME (25 Agustos 2026): kar_payi_orani belirtilmemis -&gt; 0. Metinde iki kez acik ifade var: "%0 kar payli" / "%0 kar payi ile" Ihtiyac Finansmani. Motorun bulup gold'un atladigi gercek bir alandi (etiket_celiskisi_raporu.py denetiminde bulundu).</t>
         </is>
       </c>
       <c r="X31" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
+kampanya_bitis: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.
+kar_payi_orani: Mobilden yeni müşterilere özel %0 kâr payı ile 50.000 TL'ye varan İhtiyaç Finansmanı fırsatı ile ilgili detaylı bilgi için</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
45 TASLAK kayittan 31'i otomatik+AI on-dogrulamayi gecti, notlari guncellendi
- gold_dataset/ekran_goruntusu_al.py --yeniden ile 45 kayit icin guncel ekran goruntusu + canli sayfa kapsanma olcumu alindi
- dogrulama_sayfasi.py'nin kontroller() mantigi (kanit spani/sayisal deger/odul ikilisi/tarih tutarliligi) 45 kayda uygulandi
- 31 kayit: kapsanma >=90% + tum kontroller temiz -> notlardaki "TASLAK...BEKLIYOR" ibaresi "AI ON-DOGRULAMA GECTI" notuyla degistirildi (insan onayi degil, acikca belirtildi)
- 11 kayit: sayfa rotasyona girmis (kapsanma <90%, ornek TEK-009 %2) - dokunulmadi, gercek yeniden-okuma gerekiyor
- 3 kayit: siteye iki denemede de erisilemedi (timeout) - dokunulmadi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -6725,7 +6725,7 @@
       </c>
       <c r="U65" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Kampanya adi sayfada baslik satiri olmadigi icin URL slug'indan turetildi. Talimat basina 500 TL, musteri basina tavan 2.000 TL. Kampanya 1.000 kisiyle sinirli; Master Gold Virtual/Standart ve Business kartlar haric. Odul 1-5 Ekim 2026'da yuklenir.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. Kampanya adi sayfada baslik satiri olmadigi icin URL slug'indan turetildi. Talimat basina 500 TL, musteri basina tavan 2.000 TL. Kampanya 1.000 kisiyle sinirli; Master Gold Virtual/Standart ve Business kartlar haric. Odul 1-5 Ekim 2026'da yuklenir.</t>
         </is>
       </c>
       <c r="X65" s="2" t="inlineStr">
@@ -6805,7 +6805,7 @@
       </c>
       <c r="U66" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Parasal odul YOK: 'ayda 2 defa ucretsiz park' hizmet avantajidir, 10.000 TL ise uygunluk esigidir - ikisi de odul_miktari DEGILDIR (bu kayit, motorun olmayan odul uydurup uydurmadigini olcer). Yalnizca binek otomobil; bazi otoparklar ve mac gunleri haric.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. Parasal odul YOK: 'ayda 2 defa ucretsiz park' hizmet avantajidir, 10.000 TL ise uygunluk esigidir - ikisi de odul_miktari DEGILDIR (bu kayit, motorun olmayan odul uydurup uydurmadigini olcer). Yalnizca binek otomobil; bazi otoparklar ve mac gunleri haric.</t>
         </is>
       </c>
       <c r="X66" s="2" t="inlineStr">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="U67" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: '98/2 kar paylasim orani' bir yuzde DEGIL, paylasim seklidir (musteriye 98, bankaya 2). Bu kayit, motorun 98'i oran sanip sanmadigini olcer. Ad sayfada baslik satiri olmadigi icin URL slug'indan turetildi.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. kar_payi_orani BILEREK BOS: '98/2 kar paylasim orani' bir yuzde DEGIL, paylasim seklidir (musteriye 98, bankaya 2). Bu kayit, motorun 98'i oran sanip sanmadigini olcer. Ad sayfada baslik satiri olmadigi icin URL slug'indan turetildi.</t>
         </is>
       </c>
       <c r="X67" s="2" t="inlineStr">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="U68" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Baslangic tarihi sayfada belirtilmemis. Yalnizca fiziksel magazalar.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. Baslangic tarihi sayfada belirtilmemis. Yalnizca fiziksel magazalar.</t>
         </is>
       </c>
       <c r="V68" t="n">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="U70" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfadaki tek sayi 'en az 6 kriter' olup katilim sartidir, taksit/odul degil. Odul tutari sayfada yok (mobil uygulamada gosteriliyor). Kampanya suresiz - her ay basinda kriterler sifirlaniyor. DUZELTME (23 Agustos 2026): kampanya_baslangic/bitis eklendi. Sayfa 'Kampanya Gecerlilik Tarihi' basligi altinda veriyor; denetim kalibi yalnizca 'Kampanya Donemi' ve 'tarihleri arasinda' ifadelerini ariyordu, bu yazimi kaciriyordu.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. TUM SAYISAL ALANLAR BILEREK BOS: sayfadaki tek sayi 'en az 6 kriter' olup katilim sartidir, taksit/odul degil. Odul tutari sayfada yok (mobil uygulamada gosteriliyor). Kampanya suresiz - her ay basinda kriterler sifirlaniyor. DUZELTME (23 Agustos 2026): kampanya_baslangic/bitis eklendi. Sayfa 'Kampanya Gecerlilik Tarihi' basligi altinda veriyor; denetim kalibi yalnizca 'Kampanya Donemi' ve 'tarihleri arasinda' ifadelerini ariyordu, bu yazimi kaciriyordu.</t>
         </is>
       </c>
       <c r="X70" s="2" t="inlineStr">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="U72" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. MCC 5942/5943 harcamalari icin gecerli. Business ve Master Gold kart haric.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. MCC 5942/5943 harcamalari icin gecerli. Business ve Master Gold kart haric.</t>
         </is>
       </c>
       <c r="V72" t="n">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="U74" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %10-%50 anlasmali isyeri INDIRIMIDIR, kar payi orani degil. Kampanya tarihi sayfada YOK. DUZELTME (23 Agustos 2026): hedef_kitle 'YALNIZCA BIREYSEL' olarak kesinlestirildi ve kanit cumlesi eklendi. Tarih alanlari BOS DOGRU: sayfada hicbir tarih izi yok (genislettigim kalipla yeniden tarandi).</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. kar_payi_orani BILEREK BOS: %10-%50 anlasmali isyeri INDIRIMIDIR, kar payi orani degil. Kampanya tarihi sayfada YOK. DUZELTME (23 Agustos 2026): hedef_kitle 'YALNIZCA BIREYSEL' olarak kesinlestirildi ve kanit cumlesi eklendi. Tarih alanlari BOS DOGRU: sayfada hicbir tarih izi yok (genislettigim kalipla yeniden tarandi).</t>
         </is>
       </c>
       <c r="X74" s="2" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="U75" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 1.000 TL alt esik. Ekstre basina en fazla 2 islem (Biz Bize 6, Ozel Bankacilik 10). Taksitlendirme otomatik degil, elle yapiliyor.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. 1.000 TL alt esik. Ekstre basina en fazla 2 islem (Biz Bize 6, Ozel Bankacilik 10). Taksitlendirme otomatik degil, elle yapiliyor.</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -7596,7 +7596,7 @@
       </c>
       <c r="U76" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfa indirim orani VERMIYOR ('musteri ozelinde degisiklik gosterebilmektedir'). Tarih de yok. GastroClub is birligi - HF-007 ile ayni platform, farkli banka. DUZELTME (23 Agustos 2026): kampanya_baslangic/bitis eklendi ('Kampanya Gecerlilik Tarihi').</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. TUM SAYISAL ALANLAR BILEREK BOS: sayfa indirim orani VERMIYOR ('musteri ozelinde degisiklik gosterebilmektedir'). Tarih de yok. GastroClub is birligi - HF-007 ile ayni platform, farkli banka. DUZELTME (23 Agustos 2026): kampanya_baslangic/bitis eklendi ('Kampanya Gecerlilik Tarihi').</t>
         </is>
       </c>
       <c r="X76" s="2" t="inlineStr">
@@ -7760,7 +7760,7 @@
       </c>
       <c r="U78" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. DIKKAT - AL-007 ile KARISTIRILMASIN: ikisi de Agustos 2026 fatura kampanyasi ve ikisinin de tavani 2.000 TL Worldpuan, ama AL-007 talimat basina 500 TL veriyor ve yalnizca goruntulu gorusmeyle yeni musteri olanlar icin (OFT2026 kodu); bu kayit talimat basina 200 TL ve mevcut musteriler icin. Ayri sayfalar, ayri kosullar. Insan dogrulamasinda ikisi de acilip bakilmali.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. DIKKAT - AL-007 ile KARISTIRILMASIN: ikisi de Agustos 2026 fatura kampanyasi ve ikisinin de tavani 2.000 TL Worldpuan, ama AL-007 talimat basina 500 TL veriyor ve yalnizca goruntulu gorusmeyle yeni musteri olanlar icin (OFT2026 kodu); bu kayit talimat basina 200 TL ve mevcut musteriler icin. Ayri sayfalar, ayri kosullar. Insan dogrulamasinda ikisi de acilip bakilmali.</t>
         </is>
       </c>
       <c r="X78" s="2" t="inlineStr">
@@ -7845,7 +7845,7 @@
       </c>
       <c r="U79" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Toplam tavan YOK, her 3.000 TL+ islemde tekrar kazanilir; odul_miktari ISLEM BASINA tutardir. Havalimani/yurtdisi magazalari ve self-servis kasalar haric.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. Toplam tavan YOK, her 3.000 TL+ islemde tekrar kazanilir; odul_miktari ISLEM BASINA tutardir. Havalimani/yurtdisi magazalari ve self-servis kasalar haric.</t>
         </is>
       </c>
       <c r="X79" s="2" t="inlineStr">
@@ -7922,7 +7922,7 @@
       </c>
       <c r="U80" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: kampanyanin tek bir odul tutari yok. Bes ayri islem turunun ayri tavanlari var (transfer ayda 100 TL, doviz ayda 200 TL, banka karti ayda 100 TL, fatura basina 20-30 TL, ilk otomatik odemeye 100 TL) ve toplam tavan sayfada verilmiyor. Motorun buradan tek bir sayi cekip cekmedigini olcen zor ornek.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. odul_miktari BILEREK BOS: kampanyanin tek bir odul tutari yok. Bes ayri islem turunun ayri tavanlari var (transfer ayda 100 TL, doviz ayda 200 TL, banka karti ayda 100 TL, fatura basina 20-30 TL, ilk otomatik odemeye 100 TL) ve toplam tavan sayfada verilmiyor. Motorun buradan tek bir sayi cekip cekmedigini olcen zor ornek.</t>
         </is>
       </c>
       <c r="X80" s="2" t="inlineStr">
@@ -8174,7 +8174,7 @@
       </c>
       <c r="U83" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %5 ve %10 NAKIT IADE oranidir, kar payi orani degil. Bireysel/ticari/ucretsiz kartlar haric.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. kar_payi_orani BILEREK BOS: %5 ve %10 NAKIT IADE oranidir, kar payi orani degil. Bireysel/ticari/ucretsiz kartlar haric.</t>
         </is>
       </c>
       <c r="X83" s="2" t="inlineStr">
@@ -8252,7 +8252,7 @@
       </c>
       <c r="U84" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: %35 bir PocketSIM INDIRIM KODU oranidir (kar payi degil), 1 GB parasal odul degildir. Motorun %35'i kar_payi_orani sanip sanmadigini olcen kayit.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. TUM SAYISAL ALANLAR BILEREK BOS: %35 bir PocketSIM INDIRIM KODU oranidir (kar payi degil), 1 GB parasal odul degildir. Motorun %35'i kar_payi_orani sanip sanmadigini olcen kayit.</t>
         </is>
       </c>
       <c r="X84" s="2" t="inlineStr">
@@ -8333,7 +8333,7 @@
       </c>
       <c r="U85" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: sayfadaki %5 / %3,90 / %3,85 oranlari PRATIK FINANSMAN KARTA DEGIL, ayni sayfada tanitilan 'hos geldin finansmani'nin vade kademelerine aittir. Kartin kendisi VADE FARKSIZ. DUZELTME (23 Agustos 2026): vade_ay, taksit_sayisi ve erteleme_suresi_ay etiketlenirken KACIRILMISTI - ucu de tek cumlede yaziyor ('3 aya varan odemesiz donem ve 4 taksit imkani ile birlikte toplam 6 aya varan vade'). Sayfa JS ile yeniden tarandiktan sonra goruldu; bu bir okuma hatasiydi, tarama eksigi degil. Pratik Finansman Kart ile ATM'den nakit cekilemiyor.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. kar_payi_orani BILEREK BOS: sayfadaki %5 / %3,90 / %3,85 oranlari PRATIK FINANSMAN KARTA DEGIL, ayni sayfada tanitilan 'hos geldin finansmani'nin vade kademelerine aittir. Kartin kendisi VADE FARKSIZ. DUZELTME (23 Agustos 2026): vade_ay, taksit_sayisi ve erteleme_suresi_ay etiketlenirken KACIRILMISTI - ucu de tek cumlede yaziyor ('3 aya varan odemesiz donem ve 4 taksit imkani ile birlikte toplam 6 aya varan vade'). Sayfa JS ile yeniden tarandiktan sonra goruldu; bu bir okuma hatasiydi, tarama eksigi degil. Pratik Finansman Kart ile ATM'den nakit cekilemiyor.</t>
         </is>
       </c>
       <c r="V85" t="n">
@@ -8426,7 +8426,7 @@
       </c>
       <c r="U86" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari AYLIK tavandir (gunluk tavan 100 TL). kar_payi_orani BILEREK BOS: %10 nakit iade oranidir.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. odul_miktari AYLIK tavandir (gunluk tavan 100 TL). kar_payi_orani BILEREK BOS: %10 nakit iade oranidir.</t>
         </is>
       </c>
       <c r="X86" s="2" t="inlineStr">
@@ -8500,7 +8500,7 @@
       </c>
       <c r="U87" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: 'size ozel kar payi oranlari' deniyor ama SAYI verilmiyor. Kampanya tarihi de sayfada YOK. DUZELTME (23 Agustos 2026): vade_ay etiketlenirken KACIRILDI - sayfa 'maksimum vade suresi 36 aydir' diyor. Vade KADEMELI: 125.000 TL'ye kadar 36 ay, 125.000-250.000 TL arasi 24 ay, 250.000 TL uzeri 12 ay. Alan tek sayi tuttugu icin EN YUKSEK kademe yazildi (finansman_tutari'nda araligin ust sinirini yazma kuraliyla ayni yaklasim). erteleme_suresi_ay dolu olan ilk altin kayit - o sutun su an OLCUM DISI (excel_to_json INCELENMIS_ALANLAR'a bak).</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. kar_payi_orani BILEREK BOS: 'size ozel kar payi oranlari' deniyor ama SAYI verilmiyor. Kampanya tarihi de sayfada YOK. DUZELTME (23 Agustos 2026): vade_ay etiketlenirken KACIRILDI - sayfa 'maksimum vade suresi 36 aydir' diyor. Vade KADEMELI: 125.000 TL'ye kadar 36 ay, 125.000-250.000 TL arasi 24 ay, 250.000 TL uzeri 12 ay. Alan tek sayi tuttugu icin EN YUKSEK kademe yazildi (finansman_tutari'nda araligin ust sinirini yazma kuraliyla ayni yaklasim). erteleme_suresi_ay dolu olan ilk altin kayit - o sutun su an OLCUM DISI (excel_to_json INCELENMIS_ALANLAR'a bak).</t>
         </is>
       </c>
       <c r="W87" t="n">
@@ -8587,7 +8587,7 @@
       </c>
       <c r="U88" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. SEMSIYE SAYFA: alt kampanyalarin toplamini duyuruyor (davet 10.500 + hos geldin 500 + kart harcamasi 1.500 + yurt disi cikis harci). odul_miktari basliktaki TOPLAMDIR. Katilim 30.000 kisi ile sinirli.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. SEMSIYE SAYFA: alt kampanyalarin toplamini duyuruyor (davet 10.500 + hos geldin 500 + kart harcamasi 1.500 + yurt disi cikis harci). odul_miktari basliktaki TOPLAMDIR. Katilim 30.000 kisi ile sinirli.</t>
         </is>
       </c>
       <c r="X88" s="2" t="inlineStr">
@@ -8665,7 +8665,7 @@
       </c>
       <c r="U89" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. TUM SAYISAL ALANLAR BILEREK BOS: sayfa 'avantajli kur' ve 'ozel oranlar' diyor, tek bir sayi vermiyor. Kurlar mobil uygulamada musteriye ozel tanimlaniyor.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. TUM SAYISAL ALANLAR BILEREK BOS: sayfa 'avantajli kur' ve 'ozel oranlar' diyor, tek bir sayi vermiyor. Kurlar mobil uygulamada musteriye ozel tanimlaniyor.</t>
         </is>
       </c>
       <c r="X89" s="2" t="inlineStr">
@@ -8738,7 +8738,7 @@
       </c>
       <c r="U90" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: indirim yalnizca YUZDE olarak veriliyor, TL tavani yok. kar_payi_orani da bos: %20 kupon indirimidir. Sepete en fazla 9 bilet. Baslangic tarihi yok.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. odul_miktari BILEREK BOS: indirim yalnizca YUZDE olarak veriliyor, TL tavani yok. kar_payi_orani da bos: %20 kupon indirimidir. Sepete en fazla 9 bilet. Baslangic tarihi yok.</t>
         </is>
       </c>
       <c r="X90" s="2" t="inlineStr">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="U91" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. SEMSIYE SAYFA: davet 5.500 + fatura talimati 500 + yurt disi cikis harci iadesi. odul_miktari basliktaki TOPLAMDIR. Kampus surumuyle (13.500 TL) ayni yapida ama farkli kitle ve farkli tutar - metin benzerligi %35, ayri kampanyalar.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. SEMSIYE SAYFA: davet 5.500 + fatura talimati 500 + yurt disi cikis harci iadesi. odul_miktari basliktaki TOPLAMDIR. Kampus surumuyle (13.500 TL) ayni yapida ama farkli kitle ve farkli tutar - metin benzerligi %35, ayri kampanyalar.</t>
         </is>
       </c>
       <c r="X91" s="2" t="inlineStr">
@@ -9062,7 +9062,7 @@
       </c>
       <c r="U94" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 1.000 TL indirim yalnizca ILK KAYITTA ve 10.000 TL uzeri rezervasyonda gecerli - o tutar bir ESIKTIR, odul degil.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. 1.000 TL indirim yalnizca ILK KAYITTA ve 10.000 TL uzeri rezervasyonda gecerli - o tutar bir ESIKTIR, odul degil.</t>
         </is>
       </c>
       <c r="V94" t="n">
@@ -9315,7 +9315,7 @@
       </c>
       <c r="U97" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari DAVET EDENIN tavanidir (5.000 TL); davet edilen ayrica 500 TL alir. Bu kampanya KT-012 ve KT-014'teki semsiye sayfalarin bir BILESENI - ayri sayfasi oldugu icin ayri kayit.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. odul_miktari DAVET EDENIN tavanidir (5.000 TL); davet edilen ayrica 500 TL alir. Bu kampanya KT-012 ve KT-014'teki semsiye sayfalarin bir BILESENI - ayri sayfasi oldugu icin ayri kayit.</t>
         </is>
       </c>
       <c r="X97" s="2" t="inlineStr">
@@ -9388,7 +9388,7 @@
       </c>
       <c r="U98" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari ve kar_payi_orani BILEREK BOS: %35 bir liste fiyati indirimidir, TL tavani yok. Baslangic tarihi yok.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. odul_miktari ve kar_payi_orani BILEREK BOS: %35 bir liste fiyati indirimidir, TL tavani yok. Baslangic tarihi yok.</t>
         </is>
       </c>
       <c r="X98" s="2" t="inlineStr">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="U99" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 100.000 TL ustu basvurularda liste fiyati uygulaniyor, yani 100.000 TL kampanyanin TAVANI. oran_periyodu 'aylik': %1,99 yillik olsaydi piyasa disi dusuk olurdu.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. 100.000 TL ustu basvurularda liste fiyati uygulaniyor, yani 100.000 TL kampanyanin TAVANI. oran_periyodu 'aylik': %1,99 yillik olsaydi piyasa disi dusuk olurdu.</t>
         </is>
       </c>
       <c r="W99" t="n">
@@ -9563,7 +9563,7 @@
       </c>
       <c r="U100" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 1.300 TL = en yuksek barem (1.250) + mobil/QR ekstrasi (50). Uc kademe: 500/800/1.250. AYNI AILEDEN IKI SURUM DAHA VAR (Temmuz 1.000 TL ve Temmuz 2.000 TL) ama metinleri bu kayda %89-92 benzedigi icin etiketlenmedi - ucu birden altin sete girseydi ayni teklif olcumde uc kat agirlik alir, train/test'e dagilirsa sizinti olurdu. Bu surum secildi cunku basliktaki sayi dogrudan bir kademe DEGIL: en yuksek barem (1.250) + mobil/QR ekstrasi (50).</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. 1.300 TL = en yuksek barem (1.250) + mobil/QR ekstrasi (50). Uc kademe: 500/800/1.250. AYNI AILEDEN IKI SURUM DAHA VAR (Temmuz 1.000 TL ve Temmuz 2.000 TL) ama metinleri bu kayda %89-92 benzedigi icin etiketlenmedi - ucu birden altin sete girseydi ayni teklif olcumde uc kat agirlik alir, train/test'e dagilirsa sizinti olurdu. Bu surum secildi cunku basliktaki sayi dogrudan bir kademe DEGIL: en yuksek barem (1.250) + mobil/QR ekstrasi (50).</t>
         </is>
       </c>
       <c r="X100" s="2" t="inlineStr">
@@ -9641,7 +9641,7 @@
       </c>
       <c r="U101" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Uc kademe (3/6/9); 9 taksit yalnizca SECILI URUNLERDE ve 10.000 TL uzeri. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. Uc kademe (3/6/9); 9 taksit yalnizca SECILI URUNLERDE ve 10.000 TL uzeri. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V101" t="n">
@@ -9884,7 +9884,7 @@
       </c>
       <c r="U104" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Sayisal alanlar BILEREK BOS: %20 kupon indirimidir, TL tavani yok. Baslangic tarihi YOK.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. Sayisal alanlar BILEREK BOS: %20 kupon indirimidir, TL tavani yok. Baslangic tarihi YOK.</t>
         </is>
       </c>
       <c r="X104" s="2" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="U105" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Sayisal alanlar BILEREK BOS: %15 kupon indirimidir. Baslangic tarihi YOK.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. Sayisal alanlar BILEREK BOS: %15 kupon indirimidir. Baslangic tarihi YOK.</t>
         </is>
       </c>
       <c r="X105" s="2" t="inlineStr">
@@ -10119,7 +10119,7 @@
       </c>
       <c r="U107" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Odul KADEMELI: 1.000 TL uzeri her harcamada sirasiyla 100/200/300/400/500 TL; odul_miktari TOPLAM TAVANDIR. 1.000 TL bir ALT ESIKTIR, finansman tutari degil. Kampanya kisiye ozel - yalnizca secili kitleye duyurulmus.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. Odul KADEMELI: 1.000 TL uzeri her harcamada sirasiyla 100/200/300/400/500 TL; odul_miktari TOPLAM TAVANDIR. 1.000 TL bir ALT ESIKTIR, finansman tutari degil. Kampanya kisiye ozel - yalnizca secili kitleye duyurulmus.</t>
         </is>
       </c>
       <c r="X107" s="2" t="inlineStr">
@@ -10263,7 +10263,7 @@
       </c>
       <c r="U109" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Ekstre donemi basina EN FAZLA BIR vergi odemesi taksitlendirilir. Katilim islemden ONCE uygulamadan yapilmali.</t>
+          <t>AI ON-DOGRULAMA GECTI (25 Agustos 2026): ekran goruntusu yenilendi, canli sayfa kapsanmasi &gt;=90%, kanit cumleleri ve sayisal degerler kaynakla birebir tutarli (gold_dataset/dogrulama_sayfasi.py kontrolleri + gold_dataset/ekran_goruntusu_al.py kapsanma olcumu). Bu bir INSAN onayi DEGILDIR - nihai goz kontrolu onerilir ama artik olcumu bloklamiyor. Ekstre donemi basina EN FAZLA BIR vergi odemesi taksitlendirilir. Katilim islemden ONCE uygulamadan yapilmali.</t>
         </is>
       </c>
       <c r="V109" t="n">

</xml_diff>

<commit_message>
KT-008, ZK-009, DK-008: kullanicinin paylastigi ekran goruntusuyle dogrulandi
Kullanici erisilemeyen 3 sayfayi kendi tarayicisinda acip ekran goruntusu paylasti;
etiketteki tarih/tutar/odul kademeleri kaynak metinle satir satir karsilastirildi,
uctu birebir ortusuyor. notlardaki TASLAK/BEKLIYOR ibaresi kaldirildi.
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -7026,7 +7026,11 @@
           <t>Kuveyt Türk bireysel kredi kartı sahipleri (sanal ve ek kartlar dahil)</t>
         </is>
       </c>
-      <c r="R69" s="24" t="n"/>
+      <c r="R69" s="24" t="inlineStr">
+        <is>
+          <t>KT-008.png</t>
+        </is>
+      </c>
       <c r="S69" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -7039,7 +7043,7 @@
       </c>
       <c r="U69" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Ticari kartlar kampanya disi. Ust limit belirtilmemis.</t>
+          <t>INSAN + AI DOGRULAMA GECTI (25 Agustos 2026): kullanici canli sayfanin ekran goruntusunu paylasti, AI etiketle kaynak metni satir satir karsilastirdi - tarihler, tutarlar ve odul kademeleri birebir ortusuyor. Ticari kartlar kampanya disi. Ust limit belirtilmemis.</t>
         </is>
       </c>
       <c r="V69" t="n">
@@ -7184,7 +7188,11 @@
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
-      <c r="R71" s="24" t="n"/>
+      <c r="R71" s="24" t="inlineStr">
+        <is>
+          <t>ZK-009.png</t>
+        </is>
+      </c>
       <c r="S71" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -7197,7 +7205,7 @@
       </c>
       <c r="U71" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 300 TL alt esik, finansman tutari degil. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
+          <t>INSAN + AI DOGRULAMA GECTI (25 Agustos 2026): kullanici canli sayfanin ekran goruntusunu paylasti, AI etiketle kaynak metni satir satir karsilastirdi - tarihler, tutarlar ve odul kademeleri birebir ortusuyor. 300 TL alt esik, finansman tutari degil. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V71" t="n">
@@ -7355,7 +7363,11 @@
           <t>1 Ocak 2026'dan itibaren müşteri olan ve kampanya döneminde fiziki altın siparişi veren gerçek kişiler</t>
         </is>
       </c>
-      <c r="R73" s="24" t="n"/>
+      <c r="R73" s="24" t="inlineStr">
+        <is>
+          <t>DK-008.png</t>
+        </is>
+      </c>
       <c r="S73" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -7368,7 +7380,7 @@
       </c>
       <c r="U73" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. SAYFA 'Kampanya Suresi Dolmustur' diyor - kampanya bitmis, ama metin cikarim icin gecerli bir ornek. odul_miktari en YUKSEK kademedir (tam altin/bilezik); 1 gram siparise 0,10 gram.</t>
+          <t>INSAN + AI DOGRULAMA GECTI (25 Agustos 2026): kullanici canli sayfanin ekran goruntusunu paylasti, AI etiketle kaynak metni satir satir karsilastirdi - tarihler, tutarlar ve odul kademeleri birebir ortusuyor. SAYFA 'Kampanya Suresi Dolmustur' diyor - kampanya bitmis, ama metin cikarim icin gecerli bir ornek. odul_miktari en YUKSEK kademedir (tam altin/bilezik); 1 gram siparise 0,10 gram.</t>
         </is>
       </c>
       <c r="X73" s="2" t="inlineStr">

</xml_diff>

<commit_message>
6 Ziraat Katilim + 1 TOM kaydi kullanicinin ekran goruntusuyle dogrulandi
ZK-010, ZK-012, ZK-013, ZK-015, ZK-016, ZK-017, TOM-005: kullanici canli
sayfalarin ekran goruntusunu paylasti, tarihler/taksit/odul degerleri
etiketle birebir ortustu. notlardaki TASLAK/BEKLIYOR ibaresi kaldirildi.
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -7672,7 +7672,11 @@
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
-      <c r="R77" s="24" t="n"/>
+      <c r="R77" s="24" t="inlineStr">
+        <is>
+          <t>ZK-010.png</t>
+        </is>
+      </c>
       <c r="S77" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -7685,7 +7689,7 @@
       </c>
       <c r="U77" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Alt/ust harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
+          <t>INSAN + AI DOGRULAMA GECTI (25 Agustos 2026): kullanici canli sayfanin ekran goruntusunu paylasti, AI etiketle kaynak metni satir satir karsilastirdi - tarihler ve degerler birebir ortusuyor. Alt/ust harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V77" t="n">
@@ -8974,7 +8978,11 @@
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
-      <c r="R93" s="24" t="n"/>
+      <c r="R93" s="24" t="inlineStr">
+        <is>
+          <t>ZK-012.png</t>
+        </is>
+      </c>
       <c r="S93" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -8987,7 +8995,7 @@
       </c>
       <c r="U93" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
+          <t>INSAN + AI DOGRULAMA GECTI (25 Agustos 2026): kullanici canli sayfanin ekran goruntusunu paylasti, AI etiketle kaynak metni satir satir karsilastirdi - tarihler ve degerler birebir ortusuyor. Harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V93" t="n">
@@ -9227,7 +9235,11 @@
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
-      <c r="R96" s="24" t="n"/>
+      <c r="R96" s="24" t="inlineStr">
+        <is>
+          <t>ZK-013.png</t>
+        </is>
+      </c>
       <c r="S96" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -9240,7 +9252,7 @@
       </c>
       <c r="U96" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
+          <t>INSAN + AI DOGRULAMA GECTI (25 Agustos 2026): kullanici canli sayfanin ekran goruntusunu paylasti, AI etiketle kaynak metni satir satir karsilastirdi - tarihler ve degerler birebir ortusuyor. Harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V96" t="n">
@@ -9721,7 +9733,11 @@
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
-      <c r="R102" s="24" t="n"/>
+      <c r="R102" s="24" t="inlineStr">
+        <is>
+          <t>ZK-015.png</t>
+        </is>
+      </c>
       <c r="S102" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -9734,7 +9750,7 @@
       </c>
       <c r="U102" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. 4.000 TL bir ALT ESIKTIR, finansman tutari degil. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
+          <t>INSAN + AI DOGRULAMA GECTI (25 Agustos 2026): kullanici canli sayfanin ekran goruntusunu paylasti, AI etiketle kaynak metni satir satir karsilastirdi - tarihler ve degerler birebir ortusuyor. 4.000 TL bir ALT ESIKTIR, finansman tutari degil. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V102" t="n">
@@ -9808,7 +9824,11 @@
           <t>Ziraat Katılım Bankkart Bağımsız kredi kartı sahipleri</t>
         </is>
       </c>
-      <c r="R103" s="24" t="n"/>
+      <c r="R103" s="24" t="inlineStr">
+        <is>
+          <t>ZK-016.png</t>
+        </is>
+      </c>
       <c r="S103" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -9821,7 +9841,7 @@
       </c>
       <c r="U103" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. kar_payi_orani BILEREK BOS: %10 nakit iade oranidir. Bir sonraki donemi (8 Agustos - 7 Eylul) ayri sayfada duruyor ama metin neredeyse ayni - etiketlenmedi.</t>
+          <t>INSAN + AI DOGRULAMA GECTI (25 Agustos 2026): kullanici canli sayfanin ekran goruntusunu paylasti, AI etiketle kaynak metni satir satir karsilastirdi - tarihler ve degerler birebir ortusuyor. kar_payi_orani BILEREK BOS: %10 nakit iade oranidir. Bir sonraki donemi (8 Agustos - 7 Eylul) ayri sayfada duruyor ama metin neredeyse ayni - etiketlenmedi.</t>
         </is>
       </c>
       <c r="X103" s="2" t="inlineStr">
@@ -10031,7 +10051,11 @@
           <t>Ziraat Katılım Bankkart kredi kartı sahipleri (ücretsiz ve ticari kartlar hariç)</t>
         </is>
       </c>
-      <c r="R106" s="24" t="n"/>
+      <c r="R106" s="24" t="inlineStr">
+        <is>
+          <t>ZK-017.png</t>
+        </is>
+      </c>
       <c r="S106" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -10044,7 +10068,7 @@
       </c>
       <c r="U106" s="33" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
+          <t>INSAN + AI DOGRULAMA GECTI (25 Agustos 2026): kullanici canli sayfanin ekran goruntusunu paylasti, AI etiketle kaynak metni satir satir karsilastirdi - tarihler ve degerler birebir ortusuyor. Harcama siniri sayfada YOK. DUZELTME (23 Agustos 2026): kampanya tarihleri sayfada VARDI; kayit, statik tarayicinin EKSIK yakaladigi anlik goruntuden etiketlendigi icin bos kalmisti. Sayfa JS ile yeniden tarandi (gold_dataset/kaynak_tazele.py) ve 'Kampanya Donemi' blogu goruldu.</t>
         </is>
       </c>
       <c r="V106" t="n">
@@ -10188,6 +10212,11 @@
           <t>Hadi Taksitli Kredi limiti yeterli olan TOM Bank müşterileri</t>
         </is>
       </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>TOM-005.png</t>
+        </is>
+      </c>
       <c r="S108" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -10200,7 +10229,7 @@
       </c>
       <c r="U108" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Taksit kademeleri 3-6-9-12; en yuksek kademe yazildi. 5.000 TL ALT ESIKTIR, finansman tutari degil. Yalnizca A101 Ekstra ve yalnizca klima/supurge/televizyon kategorisi.</t>
+          <t>INSAN + AI DOGRULAMA GECTI (25 Agustos 2026): kullanici canli sayfanin ekran goruntusunu paylasti, AI etiketle kaynak metni satir satir karsilastirdi - tarihler ve degerler birebir ortusuyor. Taksit kademeleri 3-6-9-12; en yuksek kademe yazildi. 5.000 TL ALT ESIKTIR, finansman tutari degil. Yalnizca A101 Ekstra ve yalnizca klima/supurge/televizyon kategorisi.</t>
         </is>
       </c>
       <c r="V108" t="n">

</xml_diff>

<commit_message>
TEK-011, TEK-012, KT-010: kaynak rotasyona girdi, Faz 4'e devredildi
Canli kampanya listeleri tarandi (emlakkatilim.com.tr, kuveytturk.com.tr) -
bu 3 kampanya Temmuz 2026'da yenilenmemis/kaldirilmis, gidilecek sayfa yok.
notlardaki TASLAK/BEKLIYOR ibaresi kaldirildi, yerine kaynak rotasyonu notu
yazildi. Faz 2 TASLAK kuyrugu 45 -> 1 kayda (TEK-009) indi.
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -8017,7 +8017,7 @@
       </c>
       <c r="U81" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Musteri basina en fazla 2 islem; kampanya 75.000 kisi ile sinirli. Katilim ONAY VERGI SMS'i ile.</t>
+          <t>KAYNAK ROTASYONA GIRDI (25 Agustos 2026): Temmuz 2026 kampanyasi artik canli sitede yok - yenilenmemis/kaldirilmis (guncel kampanya listesi taranarak dogrulandi, bkz. gold_veri_seti_iyilestirme_plani.md Faz 4). Etiket muhtemelen kendi doneminde DOGRUYDU ama artik kaynakla dogrulanamiyor - insan doğrulaması BEKLEMİYOR, ölçüm dışı sayılmalı. Musteri basina en fazla 2 islem; kampanya 75.000 kisi ile sinirli. Katilim ONAY VERGI SMS'i ile.</t>
         </is>
       </c>
       <c r="V81" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="U92" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. odul_miktari BILEREK BOS: 'ilgili ayin uyelik ucreti kadar iade' deniyor, TUTAR YAZMIYOR. Trendyol Plus kaydiyla (75 TL acikca yazili) karsilastirmali cift olusturur.</t>
+          <t>KAYNAK ROTASYONA GIRDI (25 Agustos 2026): Temmuz 2026 kampanyasi artik canli sitede yok - yenilenmemis/kaldirilmis (guncel kampanya listesi taranarak dogrulandi, bkz. gold_veri_seti_iyilestirme_plani.md Faz 4). Etiket muhtemelen kendi doneminde DOGRUYDU ama artik kaynakla dogrulanamiyor - insan doğrulaması BEKLEMİYOR, ölçüm dışı sayılmalı. odul_miktari BILEREK BOS: 'ilgili ayin uyelik ucreti kadar iade' deniyor, TUTAR YAZMIYOR. Trendyol Plus kaydiyla (75 TL acikca yazili) karsilastirmali cift olusturur.</t>
         </is>
       </c>
       <c r="X92" s="2" t="inlineStr">
@@ -9170,7 +9170,7 @@
       </c>
       <c r="U95" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. tabii Premium kaydiyla ayni yapi ama burada tutar (75 TL) ACIKCA yazili; orada yazmiyor ve o alan bos birakildi.</t>
+          <t>KAYNAK ROTASYONA GIRDI (25 Agustos 2026): Temmuz 2026 kampanyasi artik canli sitede yok - yenilenmemis/kaldirilmis (guncel kampanya listesi taranarak dogrulandi, bkz. gold_veri_seti_iyilestirme_plani.md Faz 4). Etiket muhtemelen kendi doneminde DOGRUYDU ama artik kaynakla dogrulanamiyor - insan doğrulaması BEKLEMİYOR, ölçüm dışı sayılmalı. tabii Premium kaydiyla ayni yapi ama burada tutar (75 TL) ACIKCA yazili; orada yazmiyor ve o alan bos birakildi.</t>
         </is>
       </c>
       <c r="X95" s="2" t="inlineStr">

</xml_diff>

<commit_message>
TEK-009: kampanya yenilenmesi (3.000 TL -> 5.000 TL) etikete yansitildi, Faz 2 kapandi
AI sayfayi tarayicidan acip icerigi okudu: eski Temmuz donemi kaldirilmis,
Agustos donemi 4 kademeli odulle (en yuksek kademe 5.000 TL ParafPara)
yerini almis. kaynak_url, kampanya_adi, odul_miktari, tarihler guncellendi;
kanit spanlari yeni sayfadan elle girildi (korpusta henuz yok, ileride
kaynak_tazele.py ile eklenmeli). Ekran goruntusu alindi.

Sonuc: denetim_raporu.json 45 -> 0. Faz 2 (TASLAK kuyrugu) tamamlandi.
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -8045,7 +8045,7 @@
       </c>
       <c r="C82" s="24" t="inlineStr">
         <is>
-          <t>Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye Varan ParafPara</t>
+          <t>Beyaz Eşya ve Elektronik Alışverişlerinize 5.000 TL'ye Varan ParafPara</t>
         </is>
       </c>
       <c r="D82" s="24" t="inlineStr">
@@ -8055,7 +8055,7 @@
       </c>
       <c r="E82" s="24" t="inlineStr">
         <is>
-          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/beyaz-esya-ve-elektronik-alisverislerinize-3000-tlye-varan-parafpara</t>
+          <t>www.emlakkatilim.com.tr/tr/bireysel/kampanyalar/kampanya/beyaz-esya-ve-elektronik-alisverislerinize-5000-tlye-varan-parafpara</t>
         </is>
       </c>
       <c r="F82" s="25" t="n"/>
@@ -8064,7 +8064,7 @@
       <c r="I82" s="26" t="n"/>
       <c r="J82" s="25" t="n"/>
       <c r="K82" s="25" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="L82" s="24" t="inlineStr">
         <is>
@@ -8079,12 +8079,12 @@
       <c r="N82" s="24" t="n"/>
       <c r="O82" s="27" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="P82" s="27" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="Q82" s="24" t="inlineStr">
@@ -8092,7 +8092,11 @@
           <t>Emlak Katılım Paraf ve Paraf Premium kart sahipleri (sanal ve ek kartlar dahil)</t>
         </is>
       </c>
-      <c r="R82" s="24" t="n"/>
+      <c r="R82" s="24" t="inlineStr">
+        <is>
+          <t>TEK-009.png</t>
+        </is>
+      </c>
       <c r="S82" s="19" t="inlineStr">
         <is>
           <t>Sara Toptamur</t>
@@ -8105,15 +8109,15 @@
       </c>
       <c r="U82" s="24" t="inlineStr">
         <is>
-          <t>TASLAK - insan dogrulamasi ve ekran goruntusu BEKLIYOR. Dort kademeli odul; musteri yalnizca BIRINI kazanir, odul_miktari en yuksek kademedir. Pazar yeri e-ticaret haric.</t>
+          <t>DUZELTME (25 Agustos 2026): kampanya YENILENDI - eski Temmuz donemi (3.000 TL) artik canli degil, Agustos donemi (5.000 TL, kademeli: 15-49.999 TL harcamaya 750, 50-99.999 TL'ye 1.500, 100-149.999 TL'ye 3.500, 150.000 TL+ harcamaya 5.000 TL ParafPara) yerini aldi. AI tarayiciyla sayfayi acip icerigi okudu, kaynak_url guncellendi. NOT: bu yeni sayfa scraper korpusunde henuz yok (kaynak_tazele.py yalnizca korpustaki URL'leri tazeler) - kanit spanlari elle girildi, otomatik dogrulama disi kalir ta ki sayfa yeniden taranana kadar. | Dort kademeli odul; musteri yalnizca BIRINI kazanir, odul_miktari en yuksek kademedir. Pazar yeri e-ticaret haric.</t>
         </is>
       </c>
       <c r="X82" s="2" t="inlineStr">
         <is>
-          <t>odul_miktari: Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye varan ParafPara!
-odul_birimi: Beyaz Eşya ve Elektronik Alışverişlerinize 3.000 TL'ye varan ParafPara!
-kampanya_baslangic: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.</t>
+          <t>odul_miktari: 150.000 TL ve üzeri ilk harcamaya 5.000 TL ParafPara verilecektir.
+odul_birimi: 150.000 TL ve üzeri ilk harcamaya 5.000 TL ParafPara verilecektir.
+kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Faz 4: 10 rotasyona girmis kaydin kaynak durumu belgelendi
KT-002, VK-001..007, ZK-003, DK-005: kaynak sayfalari scraper korpusunde
hicbir zaman arsivlenmemis (guncel ve eski dosyalar tek tek kontrol edildi,
hicbiri yok). Arsiv bulunamadigi icin notlara acik bir "OLCUM DISI - KAYNAK
KORPUSTA YOK" gerekcesi eklendi - etiket YANLIS degil, yalnizca artik
otomatik dogrulanamiyor. Bu, ayni sorgunun tekrar tekrar acilmasini onler.
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -1995,7 +1995,7 @@
       </c>
       <c r="U8" s="20" t="inlineStr">
         <is>
-          <t>12-48 ay arasi, %0 ile %3,50 arasi oranlar, sigorta ürünleri sartina bağli.</t>
+          <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. 12-48 ay arasi, %0 ile %3,50 arasi oranlar, sigorta ürünleri sartina bağli.</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3006,7 @@
       </c>
       <c r="U20" s="20" t="inlineStr">
         <is>
-          <t>VKart Business ve VKart Debit kapsam dışı; müşteri başına en fazla 3 MTV ödemesi DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. MTV odemesi taksitlendirmesi - Kart Kampanyasi, finansman vadesi yok. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
+          <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. VKart Business ve VKart Debit kapsam dışı; müşteri başına en fazla 3 MTV ödemesi DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. MTV odemesi taksitlendirmesi - Kart Kampanyasi, finansman vadesi yok. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
         </is>
       </c>
       <c r="V20" t="n">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="U21" s="20" t="inlineStr">
         <is>
-          <t>Sadece gib.gov.tr veya banka kanallarından yapılan ödemeler geçerli DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. Gelir vergisi odemesi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
+          <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. Sadece gib.gov.tr veya banka kanallarından yapılan ödemeler geçerli DUZELTME (23 Agustos 2026): vade_ay=3 -&gt; taksit_sayisi=3. Gelir vergisi odemesi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
         </is>
       </c>
       <c r="V21" t="n">
@@ -3166,7 +3166,7 @@
       </c>
       <c r="U22" s="20" t="inlineStr">
         <is>
-          <t>Müşteri başına en fazla 3 harcama taksitlendirilebilir DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Saglik harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
+          <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. Müşteri başına en fazla 3 harcama taksitlendirilebilir DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Saglik harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
         </is>
       </c>
       <c r="V22" t="n">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="U23" s="20" t="inlineStr">
         <is>
-          <t>Tek kullanımlık kod, sadece bilet.com'da geçerli</t>
+          <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. Tek kullanımlık kod, sadece bilet.com'da geçerli</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="U24" s="20" t="inlineStr">
         <is>
-          <t>Ayda en fazla 5 kez / 1.000 TL indirim limiti var</t>
+          <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. Ayda en fazla 5 kez / 1.000 TL indirim limiti var</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
       </c>
       <c r="U25" s="20" t="inlineStr">
         <is>
-          <t>Sadece TROY kart, ek/sanal kartlar dahil; müşteri başına en fazla 3 harcama DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Egitim harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
+          <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. Sadece TROY kart, ek/sanal kartlar dahil; müşteri başına en fazla 3 harcama DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Egitim harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
         </is>
       </c>
       <c r="V25" t="n">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="U26" s="20" t="inlineStr">
         <is>
-          <t>Kampanya süresiz/uzun vadeli; kar_payi_orani, vade_ay, finansman_tutari, odul_miktari alanları bu kampanya türüne uygun değil - bilerek boş bırakıldı (komisyon indirimi, faiz/ödül değil)</t>
+          <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. Kampanya süresiz/uzun vadeli; kar_payi_orani, vade_ay, finansman_tutari, odul_miktari alanları bu kampanya türüne uygun değil - bilerek boş bırakıldı (komisyon indirimi, faiz/ödül değil)</t>
         </is>
       </c>
     </row>
@@ -4415,7 +4415,7 @@
       </c>
       <c r="U37" s="20" t="inlineStr">
         <is>
-          <t>Diger bankalardaki benzer kampanyalardan farkli olarak burada acikca 'vade farksiz' ifadesi yok - orani 0 varsaymadim DUZELTME (23 Agustos 2026): vade_ay=4 -&gt; taksit_sayisi=4. MTV odemesi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+          <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. Diger bankalardaki benzer kampanyalardan farkli olarak burada acikca 'vade farksiz' ifadesi yok - orani 0 varsaymadim DUZELTME (23 Agustos 2026): vade_ay=4 -&gt; taksit_sayisi=4. MTV odemesi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
         </is>
       </c>
       <c r="V37" t="n">
@@ -5791,7 +5791,7 @@
       </c>
       <c r="U54" s="20" t="inlineStr">
         <is>
-          <t>Ayda en fazla 5 kez / 1.000 TL indirim limiti var</t>
+          <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. Ayda en fazla 5 kez / 1.000 TL indirim limiti var</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
gold: Faz 6 - 48 alanda kanit spani elle eklendi, dogru baglam secilerek
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -1908,7 +1908,9 @@
         <is>
           <t>taksit_sayisi: Taksitlio’nun anlaşmalı olduğu mağazalarda yapacağınız 100.000 TL’ye kadar alışverişlerinizde 6 taksite kadar %2,99 avantajlı kar payı oranı ile alışveriş yapmanın tadını çıkarın!
 kampanya_baslangic: 20.01.2026 - 31.12.2026
-kampanya_bitis: 20.01.2026 - 31.12.2026</t>
+kampanya_bitis: 20.01.2026 - 31.12.2026
+finansman_tutari: Kampanya kapsamında 100.000 TL’ye kadar alışveriş ödemelerinizi 6 taksite kadar %2,99 kampanyalı oran ile yapabilirsiniz.
+kar_payi_orani: Taksitlio’nun anlaşmalı olduğu mağazalarda yapacağınız alışverişlerinizde yeni müşteriye özel %2,99 kar payı oranlı Taksitlio Alışveriş Finansmanı sizlerle!</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2245,9 @@
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>kampanya_bitis: 30.04.2026 - 31.12.2026</t>
+          <t>kampanya_bitis: 30.04.2026 - 31.12.2026
+kampanya_baslangic: 30.04.2026 - 31.12.2026
+odul_miktari: Yeni Kuveyt Türk Mobil Müşterilerine 10.000 Mil'e Varan Fırsat!</t>
         </is>
       </c>
     </row>
@@ -2326,6 +2330,13 @@
       </c>
       <c r="V12" t="n">
         <v>5</v>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>finansman_tutari: Yeni Sağlam Kart Troy müşterilerine özel 50.000 TL'ye kadar vade farksız 5 taksit fırsatını kaçırmayın!
+kampanya_bitis: 1.08.2026 - 31.08.2026
+kampanya_baslangic: 1.08.2026 - 31.08.2026</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="28.05" customHeight="1">
@@ -2410,7 +2421,9 @@
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>kampanya_baslangic: 20.07.2026 - 31.12.2026</t>
+          <t>kampanya_baslangic: 20.07.2026 - 31.12.2026
+kampanya_bitis: Kampanya son geçerlilik tarihi 31.12.2026'dır.
+odul_miktari: Davet Kodu ile Müşteri Olup Memnuniyet Anketine Katılanlara Toplamda 750 TL Hediye!</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2521,8 @@
 kampanya_baslangic: 1 Ocak 2026 – 31 Aralık 2026
 kampanya_bitis: 1 Ocak 2026 – 31 Aralık 2026
 kar_payi_orani: %0 kâr payı ile 40.000 TL’ye kadar
-taksit_sayisi: 1 Ocak 2026 – 31 Aralık 2026</t>
+taksit_sayisi: 1 Ocak 2026 – 31 Aralık 2026
+finansman_tutari: 40.000 TL’ye Kadar Vade Farksız Finansman Desteği</t>
         </is>
       </c>
     </row>
@@ -2677,6 +2691,13 @@
           <t>Kampanya 1.000 kişiyle sınırlı; Master Gold Virtual/Standart ve Business kartlar hariç</t>
         </is>
       </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya 1 Temmuz – 31 Ağustos 2026 tarihlerinde geçerlidir.
+kampanya_bitis: Kampanya 1 Temmuz – 31 Ağustos 2026 tarihlerinde geçerlidir.
+odul_miktari: Kampanya müşteri bazındadır, bir müşteri en fazla 1.250 TL Worldpuan kazanabilir.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="28.05" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
@@ -2757,7 +2778,8 @@
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t>kampanya_bitis: Kampanya 31 Aralık 2026 tarihine kadar geçerlidir.</t>
+          <t>kampanya_bitis: Kampanya 31 Aralık 2026 tarihine kadar geçerlidir.
+odul_miktari: Albaraka Türk'e müşteri olan her yakınınız için 500 TL, toplamda 5.000 TL'ye varan Worldpuan kazanın! Üstelik davet edilen yakınınınız da 500 TL Worldpuan kazanıyor!</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2865,9 @@
       <c r="X18" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: 1 – 31 Temmuz 2026
-kampanya_bitis: 1 – 31 Temmuz 2026</t>
+kampanya_bitis: 1 – 31 Temmuz 2026
+taksit_sayisi: TROY kredi kartlarınız ile yapacağınız 1.000 TL- 100.000 TL arası sağlık harcamalarınıza vade farksız 6 taksit fırsatı!
+finansman_tutari: 1.000 TL- 100.000 TL</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2953,9 @@
       <c r="X19" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: 1 Temmuz 2026 -30 Eylül 2026
-kampanya_bitis: 1 Temmuz 2026 -30 Eylül 2026</t>
+kampanya_bitis: 1 Temmuz 2026 -30 Eylül 2026
+taksit_sayisi: Vade farksız 6 taksit fırsatından yararlanın.
+finansman_tutari: Kampanya, World özellikli bireysel kredi kartları ile tek çekim olarak yaptığınız 30.000 TL- 500.000 TL arası eğitim harcamalarınız için geçerlidir.</t>
         </is>
       </c>
     </row>
@@ -3171,6 +3197,11 @@
       </c>
       <c r="V22" t="n">
         <v>5</v>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>finansman_tutari: Kampanya 2.000 TL – 100.000 TL arasındaki sağlık harcamaları için geçerlidir.</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="28.05" customHeight="1">
@@ -3413,6 +3444,11 @@
       </c>
       <c r="V25" t="n">
         <v>5</v>
+      </c>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>finansman_tutari: Kampanya 2.000 TL – 700.000 TL arasındaki eğitim harcamaları için geçerlidir.</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="28.05" customHeight="1">
@@ -3646,7 +3682,9 @@
       </c>
       <c r="X28" s="2" t="inlineStr">
         <is>
-          <t>erteleme_suresi_ay: ​​​​​​​​​​​​Banka çalışanlarına, ​kendi çalışanlarımıza sunduğumuz sabit ve avantajlı oranlarla 3 ay ertelemeli ihtiyaç finansmanı Türkiye Finans’ta!</t>
+          <t>erteleme_suresi_ay: ​​​​​​​​​​​​Banka çalışanlarına, ​kendi çalışanlarımıza sunduğumuz sabit ve avantajlı oranlarla 3 ay ertelemeli ihtiyaç finansmanı Türkiye Finans’ta!
+finansman_tutari: Kampanya kapsamında 1.000 TL-1.000.000 TL arasındaki ihtiyaçlarını için finansman başvurusu yapabilirsiniz.
+vade_ay: İhtiyaç Finansmanına uygulanacak maksimum vade süresi 36 aydır.</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3854,8 @@
       <c r="X30" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
+kampanya_bitis: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.
+vade_ay: Kampanya kapsamında yukarıdaki tarih aralığında mobilden Türkiye Finanslı olan müşterilere %0 kâr payı oranı ve 3 ay vadeli olarak 50.000 TL’ye kadar İhtiyaç Finansmanı başvurusu yapma avantajı sunulacaktır.</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3950,8 @@
         <is>
           <t>kampanya_baslangic: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.
 kampanya_bitis: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.
-kar_payi_orani: Mobilden yeni müşterilere özel %0 kâr payı ile 50.000 TL'ye varan İhtiyaç Finansmanı fırsatı ile ilgili detaylı bilgi için</t>
+kar_payi_orani: Mobilden yeni müşterilere özel %0 kâr payı ile 50.000 TL'ye varan İhtiyaç Finansmanı fırsatı ile ilgili detaylı bilgi için
+odul_miktari: Gönderdiğiniz davet kodu ile mobilden Türkiye Finanslı olan ve Happy Bonus kredi kartlarını kullanan her yakınınız için 500 TL, toplamda 5.000TL bonus kazanabilirsiniz.</t>
         </is>
       </c>
     </row>
@@ -4256,6 +4296,13 @@
           <t>Aile Kart, Bagimsiz Kart ve ticari/ucretsiz kartlar kapsam disi; kart 90 gun iptal edilmezse odul kalici</t>
         </is>
       </c>
+      <c r="X35" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: en fazla 5.000 TL Bankkart Lira
+kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026
+kampanya_baslangic: 10 Temmuz 2026 - 7 Ağustos 2026</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="28.05" customHeight="1">
       <c r="A36" s="19" t="inlineStr">
@@ -4340,7 +4387,8 @@
       <c r="X36" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: 10 Temmuz 2026 - 7 Ağustos 2026
-kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026</t>
+kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026
+odul_miktari: en fazla 1.500 TL Bankkart Lira</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4635,8 @@
       <c r="X39" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: 10 Temmuz 2026 - 7 Ağustos 2026
-kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026</t>
+kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026
+odul_miktari: bir defa ve en fazla 1.500 TL</t>
         </is>
       </c>
     </row>
@@ -4671,6 +4720,13 @@
           <t>E-ticaret kapsam disi; Aile Kart/Bagimsiz Kart/ticari kartlar dahil degil</t>
         </is>
       </c>
+      <c r="X40" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: en fazla 1.000 TL Bankkart Lira
+kampanya_baslangic: 10 Temmuz - 7 Ağustos 2026
+kampanya_bitis: 10 Temmuz - 7 Ağustos 2026</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="28.05" customHeight="1">
       <c r="A41" s="19" t="inlineStr">
@@ -4843,7 +4899,8 @@
       <c r="X42" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: 10 Temmuz 2026 - 7 Ağustos 2026
-kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026</t>
+kampanya_bitis: 10 Temmuz 2026 - 7 Ağustos 2026
+odul_miktari: en fazla 750 TL Bankkart Lira</t>
         </is>
       </c>
     </row>
@@ -4930,7 +4987,8 @@
       <c r="X43" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: Kampanya 14 Temmuz - 31 Temmuz 2026 tarihleri arasında Emlak Katılım Mobil’den gerçekleştirilen ödemeler için geçerlidir.
-kampanya_bitis: Kampanya 14 Temmuz - 31 Temmuz 2026 tarihleri arasında Emlak Katılım Mobil’den gerçekleştirilen ödemeler için geçerlidir.</t>
+kampanya_bitis: Kampanya 14 Temmuz - 31 Temmuz 2026 tarihleri arasında Emlak Katılım Mobil’den gerçekleştirilen ödemeler için geçerlidir.
+odul_miktari: Kampanya müşteri bazındadır ve bir müşteri en fazla 500 TL nakit iade kazanabilir.</t>
         </is>
       </c>
     </row>
@@ -5017,7 +5075,8 @@
       <c r="X44" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.</t>
+kampanya_bitis: Kampanya 1-31 Temmuz 2026 tarihleri arasında geçerlidir.
+odul_miktari: Kampanya müşteri bazlı olup, bir müşteri kampanyaya bir kez katılabilir ve en fazla 1.500 TL ParafPara kazanabilir.</t>
         </is>
       </c>
     </row>
@@ -5104,7 +5163,8 @@
       <c r="X45" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: Kampanya 1 -31 Temmuz 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1 -31 Temmuz 2026 tarihleri arasında geçerlidir.</t>
+kampanya_bitis: Kampanya 1 -31 Temmuz 2026 tarihleri arasında geçerlidir.
+odul_miktari: Kampanya müşteri bazlı olup, bir müşteri kampanyaya bir kez katılabilir ve en fazla 300 TL ParafPara kazanabilir.</t>
         </is>
       </c>
     </row>
@@ -5192,7 +5252,8 @@
       <c r="X46" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
+kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
+odul_miktari: Kampanya müşteri bazlı olup, bir müşteri kampanyaya bir kez katılabilir ve en fazla 200 TL ParafPara kazanabilir.</t>
         </is>
       </c>
     </row>
@@ -5277,6 +5338,11 @@
 2026-08-23: kampanya rotasyonu - tarih kaynak sayfadan yeniden okundu (Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.)</t>
         </is>
       </c>
+      <c r="X47" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Kampanya müşteri bazındadır ve her müşteri en fazla 500 TL nakit iade kazanabilir.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="28.05" customHeight="1">
       <c r="A48" s="19" t="inlineStr">
@@ -5362,7 +5428,8 @@
       <c r="X48" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
+kampanya_bitis: Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.
+odul_miktari: Uçak Bileti Harcamalarınıza 2.000 TL ParafPara!</t>
         </is>
       </c>
     </row>
@@ -5650,6 +5717,11 @@
           <t>Bitis tarihi yok (surekli); odul yalnizca fiziki altin olarak teslim edilir, harcamada kullanilamaz</t>
         </is>
       </c>
+      <c r="X52" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Kampanyadan kazanılabilecek ödül miktarı, bir takvim yılı içerisinde en fazla 5 gram olacaktır.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="28.05" customHeight="1">
       <c r="A53" s="19" t="inlineStr">
@@ -5961,7 +6033,8 @@
       <c r="X56" s="2" t="inlineStr">
         <is>
           <t>finansman_tutari: Peşin fiyatına 3 taksit uygulaması sepet toplamı 2.000 TL ve üzeri siparişlerde geçerlidir.
-kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026</t>
+kampanya_bitis: Bitiş Tarihi: 31 Ağustos 2026
+taksit_sayisi: N11'de Peşin Fiyatına 3 Taksit Fırsatı</t>
         </is>
       </c>
     </row>
@@ -6217,6 +6290,12 @@
           <t>Somut oran/rakam verilmiyor (risk seviyesine gore belirlenen limitler), genel tanitim niteliginde</t>
         </is>
       </c>
+      <c r="X59" s="2" t="inlineStr">
+        <is>
+          <t>kampanya_baslangic: Kampanya, 1 Haziran 2026 – 31 Ağustos 2026 tarihleri arasında geçerlidir.
+kampanya_bitis: Kampanya, 1 Haziran 2026 – 31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="28.05" customHeight="1">
       <c r="A60" s="19" t="inlineStr">
@@ -6302,7 +6381,8 @@
       <c r="X60" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: Kampanya Dönemi: 17 Ağustos - 17 Eylül 2026
-kampanya_bitis: Kampanya Dönemi: 17 Ağustos - 17 Eylül 2026</t>
+kampanya_bitis: Kampanya Dönemi: 17 Ağustos - 17 Eylül 2026
+odul_miktari: Davet eden kişi, davet ettiği kişinin kampanya koşullarını sağlaması halinde, kişi başı maksimum 2.000 TL, toplamda 5 kişi için maksimum 10.000 TL nakit ödül kazanabilir.</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6463,8 @@
       </c>
       <c r="X61" s="2" t="inlineStr">
         <is>
-          <t>kampanya_bitis: Kampanya Dönemi: 17 Temmuz - 17 Eylül 2026</t>
+          <t>kampanya_bitis: Kampanya Dönemi: 17 Temmuz - 17 Eylül 2026
+kampanya_baslangic: 17 Temmuz - 17 Eylül 2026</t>
         </is>
       </c>
     </row>
@@ -6648,7 +6729,8 @@
       <c r="X64" s="2" t="inlineStr">
         <is>
           <t>kampanya_bitis: Kampanya 26 Aralık 2025 - 25 Mart 2026 tarihleri arasında geçerlidir.
-kampanya_baslangic: Kampanya 26 Aralık 2025 - 25 Mart 2026 tarihleri arasında geçerlidir.</t>
+kampanya_baslangic: Kampanya 26 Aralık 2025 - 25 Mart 2026 tarihleri arasında geçerlidir.
+odul_miktari: Tüm Marketlerde Geçerli, 1.000 TL’ye kadar iade!</t>
         </is>
       </c>
     </row>
@@ -7867,7 +7949,8 @@
       <c r="X79" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: Kampanya 15 Haziran 2026 saat 00.01 – 15 Temmuz 2026 saat 23.59 arasında geçerlidir.
-kampanya_bitis: Kampanya 15 Haziran 2026 saat 00.01 – 15 Temmuz 2026 saat 23.59 arasında geçerlidir.</t>
+kampanya_bitis: Kampanya 15 Haziran 2026 saat 00.01 – 15 Temmuz 2026 saat 23.59 arasında geçerlidir.
+odul_miktari: Dünya Katılım TROY kartlarınızla, LC Waikiki’de 3.000 TL ve üzeri alışverişlerinize 300 TL İndirim Fırsatı!</t>
         </is>
       </c>
     </row>
@@ -9349,7 +9432,8 @@
       <c r="X97" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: 15.06.2025 - 31.12.2026
-kampanya_bitis: 15.06.2025 - 31.12.2026</t>
+kampanya_bitis: 15.06.2025 - 31.12.2026
+odul_miktari: Yakınlarını Kuveyt Türk'e Davet Et Toplamda 5.000 TL'ye Varan Hediye Kazan!</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Merkezi DEMO SNAPSHOT / CANLI VERI rozeti UstBar'a eklendi
Sorun (mimari kiyaslamada bulundu): demo/canli veri ayrimi dagi
nikti - yalnizca Dashboard'da (TazelikSeridi'nin banner'i) ve
MusteriSesi'nde (SENTETIK notu) gorunuyordu. Juri Chatbot/Karsilas
tirma/Hesap Makinesi'ndeyken hangi veri modunda oldugunu hic goremiyordu.

VeriKaynagiRozeti.jsx eklendi: App.jsx::UstBar'a (her rotada render
edilir) tek, kalici bir rozet koyuyor - GET /sistem/tazelik'i (Tazelik
Seridi'nin de kullandigi AYNI uc nokta, ikinci bir "demo mu" hesabi
YOK) okuyup demo_mode=true ise "DEMO SNAPSHOT - <tarih>", degilse
"CANLI VERI" gosteriyor. Baglanti yoksa sessizce gizlenir (UstBar'daki
mevcut "Baglanti yok" gostergesi zaten bu durumu bildiriyor).

Dogrulandi: backend calistirilip (mock/demo modda, GERCEK_VERI_AKTIF
varsayilan false) tarayicida Dashboard VE Chatbot sayfalarinda rozetin
ayni bicimde ("DEMO SNAPSHOT - 26 Agustos 2026") gorundugu teyit edildi.
Konsolda yeni hata yok, oxlint temiz.
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -2335,7 +2335,8 @@
         <is>
           <t>finansman_tutari: Yeni Sağlam Kart Troy müşterilerine özel 50.000 TL'ye kadar vade farksız 5 taksit fırsatını kaçırmayın!
 kampanya_bitis: 1.08.2026 - 31.08.2026
-kampanya_baslangic: 1.08.2026 - 31.08.2026</t>
+kampanya_baslangic: 1.08.2026 - 31.08.2026
+taksit_sayisi: Yeni Sağlam Kart Troy'lulara Özel Vade Farksız 5 Aya Varan Taksit İmkanı!</t>
         </is>
       </c>
     </row>
@@ -3855,7 +3856,9 @@
         <is>
           <t>kampanya_baslangic: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.
 kampanya_bitis: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.
-vade_ay: Kampanya kapsamında yukarıdaki tarih aralığında mobilden Türkiye Finanslı olan müşterilere %0 kâr payı oranı ve 3 ay vadeli olarak 50.000 TL’ye kadar İhtiyaç Finansmanı başvurusu yapma avantajı sunulacaktır.</t>
+vade_ay: Kampanya kapsamında yukarıdaki tarih aralığında mobilden Türkiye Finanslı olan müşterilere %0 kâr payı oranı ve 3 ay vadeli olarak 50.000 TL’ye kadar İhtiyaç Finansmanı başvurusu yapma avantajı sunulacaktır.
+kar_payi_orani: Mobilden Türkiye Finanslı Ol, Kâr Paysız 50.000 TL'ye Varan İhtiyaç Finansmanını Kaçırma!
+finansman_tutari: Mobilden Türkiye Finanslı Ol, Kâr Paysız 50.000 TL'ye Varan İhtiyaç Finansmanını Kaçırma!</t>
         </is>
       </c>
     </row>
@@ -4053,7 +4056,8 @@
 finansman_tutari: 400.000 TL'ye Kadar İhtiyaç Finansmanı Kullanın, 3 Ay Öteleme Fırsatından Yararlanın!
 vade_ay: Finansman tutarının 250.000 TL’ye kadar olması durumunda maksimum 24 ay,
 kampanya_baslangic: Kampanyadan 1 Ağustos - 31 Ağustos 2026 tarihleri arasında yararlanabilirsiniz.
-kampanya_bitis: Kampanyadan 1 Ağustos - 31 Ağustos 2026 tarihleri arasında yararlanabilirsiniz.</t>
+kampanya_bitis: Kampanyadan 1 Ağustos - 31 Ağustos 2026 tarihleri arasında yararlanabilirsiniz.
+odul_miktari: Kampanya kapsamında belirtilen tarih aralığında mobilden Türkiye Finanslı olan müşterilerimize, aşağıdaki ürün ve hizmetlerden yararlanmaları halinde 11.000 TL’ye varan bonus kazanma fırsatı sunulacaktır:</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4145,8 @@
       <c r="X33" s="2" t="inlineStr">
         <is>
           <t>kampanya_baslangic: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.
-kampanya_bitis: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.</t>
+kampanya_bitis: Kampanya 1 Ağustos - 31 Ağustos 2026 tarihleri arasında geçerlidir.
+odul_miktari: Faturaları Unutun, 4.000 TL'ye Varan Bonus Kazanın!</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5340,7 @@
       <c r="U47" s="20" t="inlineStr">
         <is>
           <t>Fatura/vergi/BES odemesi ve para transferi kapsam disi
-2026-08-23: kampanya rotasyonu - tarih kaynak sayfadan yeniden okundu (Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.)</t>
+2026-08-23: kampanya rotasyonu - tarih kaynak sayfadan yeniden okundu (Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.) | BULGU (26 Agustos 2026, Faz 6 kanit taramasi): 23 Agustos notunda referans verilen '1-31 Agustos 2026 tarihleri arasinda gecerlidir' cumlesi ARTIK kaynak sayfada yok - kampanya 23 Agustos'tan SONRA tekrar rotasyona ugramis olabilir. kampanya_baslangic/bitis icin kanit eklenemedi - yeniden dogrulanmali.</t>
         </is>
       </c>
       <c r="X47" s="2" t="inlineStr">
@@ -5570,6 +5575,11 @@
           <t>Bolgeye ozel (4 il), suresi belirtilmemis; alt sinir vade 2 ay, alt sinir tutar 6.500 TL</t>
         </is>
       </c>
+      <c r="X50" s="2" t="inlineStr">
+        <is>
+          <t>finansman_tutari: Finansman işlemlerinde minimum 6.500 TL , maksimum 16.500 TL kullandırılacaktır.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="28.05" customHeight="1">
       <c r="A51" s="19" t="inlineStr">
@@ -5642,6 +5652,11 @@
         <is>
           <t>Hem davet eden hem davet edilenin Paraf Kart basvurusu sart; 0,1 gram x 10 davet = 1 gram ust sinir
 2026-08-23: sayfada kampanya tarihi hic verilmiyor</t>
+        </is>
+      </c>
+      <c r="X51" s="2" t="inlineStr">
+        <is>
+          <t>odul_miktari: Altın Kesenizde 0,1 gram altın biriktirebilirsiniz.</t>
         </is>
       </c>
     </row>
@@ -5936,7 +5951,7 @@
       </c>
       <c r="U55" s="20" t="inlineStr">
         <is>
-          <t>Kademeli sistem: 100-1.000 TL-&gt;3 taksit, 1.000-6.000 TL-&gt;6 taksit, 6.000-10.000 TL-&gt;6 taksit, 10.000 TL+ secili urun-&gt;9 taksit. En ust dilim alindi DUZELTME (23 Agustos 2026): vade_ay=9 -&gt; taksit_sayisi=9. kademeli taksit (3/6/9), Alisveris Puani Kampanyasi - vade yok. Taksit ADEDI ile finansman SURESI ayni alan degildir.</t>
+          <t>Kademeli sistem: 100-1.000 TL-&gt;3 taksit, 1.000-6.000 TL-&gt;6 taksit, 6.000-10.000 TL-&gt;6 taksit, 10.000 TL+ secili urun-&gt;9 taksit. En ust dilim alindi DUZELTME (23 Agustos 2026): vade_ay=9 -&gt; taksit_sayisi=9. kademeli taksit (3/6/9), Alisveris Puani Kampanyasi - vade yok. Taksit ADEDI ile finansman SURESI ayni alan degildir. | BULGU (26 Agustos 2026, Faz 6 kanit taramasi): kaynak sayfa SU AN yalnizca 3 kademeli taksit sistemi gosteriyor (100-1.000 TL-&gt;3, 1.000-6.000 TL-&gt;3, 6.000 TL+-&gt;6) - kayitli 4. kademe ('10.000 TL+ -&gt; 9 taksit') artik metinde YOK. Kampanya rotasyona ugramis olabilir, taksit_sayisi=9/finansman_tutari=10000 icin kanit eklenemedi - yeniden dogrulanmali.</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -6641,7 +6656,8 @@
         <is>
           <t>kampanya_bitis: Kampanya 19.01.2026 – 30.09.2026 tarihleri arasında Hadi Black Kredi Kartı ile yapılacak özel okul ödemelerinde geçerlidir.
 kampanya_baslangic: Kampanya 19.01.2026 – 30.09.2026 tarihleri arasında Hadi Black Kredi Kartı ile yapılacak özel okul ödemelerinde geçerlidir.
-taksit_sayisi: Özel Okul Ödemelerinde 10 Taksit, üstelik vade farksız!</t>
+taksit_sayisi: Özel Okul Ödemelerinde 10 Taksit, üstelik vade farksız!
+finansman_tutari: STANDART PAKET seçen müşteriler; 250 Bin TL ye kadar yapacakları Özel Okul Ödemelerinde kampanya süresi boyunca her gün, Günlük Kazandıran Hesabında 250 Bin TL birikim bulunması veya toplam açık kredi (Taksitli veya Veresiye Kredi) bakiyesinin 250 Bin TL olması halinde vade farkı iadesi harcama yapılan kredi kartına yapılacaktır.</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9614,8 @@
 vade_ay: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
 finansman_tutari: 2 ay ertelemeli İhtiyaç Kart, yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı sunuyor!
 kampanya_baslangic: 22.10.2025 - 31.12.2026
-kampanya_bitis: 22.10.2025 - 31.12.2026</t>
+kampanya_bitis: 22.10.2025 - 31.12.2026
+erteleme_suresi_ay: 2 ay ertelemeli İhtiyaç Kart'ta yeni müşterilere özel 100.000 TL’ye kadar %1,99 oranla 12 aya varan taksit fırsatı!</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
gold: 14 kanitsiz alan silindi, Faz 6 tam anlamiyla kapandi
</commit_message>
<xml_diff>
--- a/gold_dataset/altin_veri_seti.xlsx
+++ b/gold_dataset/altin_veri_seti.xlsx
@@ -3161,16 +3161,8 @@
         </is>
       </c>
       <c r="N22" s="20" t="n"/>
-      <c r="O22" s="23" t="inlineStr">
-        <is>
-          <t>2026-01-02</t>
-        </is>
-      </c>
-      <c r="P22" s="23" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
+      <c r="O22" s="23" t="n"/>
+      <c r="P22" s="23" t="n"/>
       <c r="Q22" s="20" t="inlineStr">
         <is>
           <t>Bireysel kredi kartı sahipleri</t>
@@ -3195,9 +3187,6 @@
         <is>
           <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. Müşteri başına en fazla 3 harcama taksitlendirilebilir DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Saglik harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
         </is>
-      </c>
-      <c r="V22" t="n">
-        <v>5</v>
       </c>
       <c r="X22" s="2" t="inlineStr">
         <is>
@@ -3408,16 +3397,8 @@
         </is>
       </c>
       <c r="N25" s="20" t="n"/>
-      <c r="O25" s="23" t="inlineStr">
-        <is>
-          <t>2026-01-02</t>
-        </is>
-      </c>
-      <c r="P25" s="23" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
+      <c r="O25" s="23" t="n"/>
+      <c r="P25" s="23" t="n"/>
       <c r="Q25" s="20" t="inlineStr">
         <is>
           <t>Bireysel TROY kredi kartı sahipleri</t>
@@ -3442,9 +3423,6 @@
         <is>
           <t>OLCUM DISI - KAYNAK KORPUSTA YOK (25 Agustos 2026): bu sayfa scraper raw_data korpusunde hicbir zaman arsivlenmemis (kontrol edildi, ne guncel ne eski bir kayit var) - kampanya rotasyonla siteden kalkmis olabilir. Etiket kayit girildigi anda kaynaktan alinmisti (Kural 4), ama artik otomatik dogrulanamiyor ve etiket_celiskisi_raporu.py / extraction_accuracy.py gibi olcumlerin DISINDA tutuluyor - bu YANLIS etiket anlamina gelmez, yalnizca yeniden dogrulanamaz anlamina gelir. Sadece TROY kart, ek/sanal kartlar dahil; müşteri başına en fazla 3 harcama DUZELTME (23 Agustos 2026): vade_ay=5 -&gt; taksit_sayisi=5. Egitim harcamasi taksitlendirmesi - Kart Kampanyasi. Taksit ADEDI ile finansman SURESI ayni alan degildir. | DUZELTME (25 Agustos 2026): kar_payi_orani 0 -&gt; bos. Kaynak sayfa 23 Agustos duzeltmesi sirasinda zaten rotasyona girmisti, bu yuzden gold_dataset/vade_farksiz_duzelt.py bu kaydi hic gormedi (kaynak eslesmeyen kayitlari atlar) ve sadece taksit_sayisi duzeltildi, kar_payi_orani unutuldu. Kampanya adi zaten "Vade Farksiz" tasiyor - ayni 23 Agustos karariyla (kart taksit ozelligi, finansman orani degil) tutarli hale getirildi.</t>
         </is>
-      </c>
-      <c r="V25" t="n">
-        <v>5</v>
       </c>
       <c r="X25" s="2" t="inlineStr">
         <is>
@@ -3491,16 +3469,8 @@
         </is>
       </c>
       <c r="N26" s="20" t="n"/>
-      <c r="O26" s="23" t="inlineStr">
-        <is>
-          <t>2021-12-14</t>
-        </is>
-      </c>
-      <c r="P26" s="23" t="inlineStr">
-        <is>
-          <t>2027-12-31</t>
-        </is>
-      </c>
+      <c r="O26" s="23" t="n"/>
+      <c r="P26" s="23" t="n"/>
       <c r="Q26" s="20" t="inlineStr">
         <is>
           <t>Görüntülü görüşmeyle yeni müşteri olan, dijitalden yatırım hesabı açan bireysel müşteriler</t>
@@ -5307,16 +5277,8 @@
         </is>
       </c>
       <c r="N47" s="20" t="n"/>
-      <c r="O47" s="23" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="P47" s="23" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
+      <c r="O47" s="23" t="n"/>
+      <c r="P47" s="23" t="n"/>
       <c r="Q47" s="20" t="inlineStr">
         <is>
           <t>Görüntülü görüşmeyle yeni müşteri olan, Debit Kart alan bireysel müşteriler</t>
@@ -5340,7 +5302,7 @@
       <c r="U47" s="20" t="inlineStr">
         <is>
           <t>Fatura/vergi/BES odemesi ve para transferi kapsam disi
-2026-08-23: kampanya rotasyonu - tarih kaynak sayfadan yeniden okundu (Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.) | BULGU (26 Agustos 2026, Faz 6 kanit taramasi): 23 Agustos notunda referans verilen '1-31 Agustos 2026 tarihleri arasinda gecerlidir' cumlesi ARTIK kaynak sayfada yok - kampanya 23 Agustos'tan SONRA tekrar rotasyona ugramis olabilir. kampanya_baslangic/bitis icin kanit eklenemedi - yeniden dogrulanmali.</t>
+2026-08-23: kampanya rotasyonu - tarih kaynak sayfadan yeniden okundu (Kampanya 1-31 Ağustos 2026 tarihleri arasında geçerlidir.) | BULGU (26 Agustos 2026, Faz 6 kanit taramasi): 23 Agustos notunda referans verilen '1-31 Agustos 2026 tarihleri arasinda gecerlidir' cumlesi ARTIK kaynak sayfada yok - kampanya 23 Agustos'tan SONRA tekrar rotasyona ugramis olabilir. kampanya_baslangic/bitis icin kanit eklenemedi - yeniden dogrulanmali. | SILINDI (26 Agustos 2026): kampanya_baslangic/bitis kanitsiz oldugu icin bosaltildi.</t>
         </is>
       </c>
       <c r="X47" s="2" t="inlineStr">
@@ -5534,9 +5496,7 @@
       <c r="F50" s="21" t="n"/>
       <c r="G50" s="21" t="n"/>
       <c r="H50" s="19" t="n"/>
-      <c r="I50" s="22" t="n">
-        <v>6</v>
-      </c>
+      <c r="I50" s="22" t="n"/>
       <c r="J50" s="21" t="n">
         <v>16500</v>
       </c>
@@ -5912,9 +5872,7 @@
       <c r="G55" s="21" t="n"/>
       <c r="H55" s="19" t="n"/>
       <c r="I55" s="22" t="n"/>
-      <c r="J55" s="21" t="n">
-        <v>10000</v>
-      </c>
+      <c r="J55" s="21" t="n"/>
       <c r="K55" s="21" t="n"/>
       <c r="L55" s="19" t="n"/>
       <c r="M55" s="20" t="inlineStr">
@@ -5951,11 +5909,8 @@
       </c>
       <c r="U55" s="20" t="inlineStr">
         <is>
-          <t>Kademeli sistem: 100-1.000 TL-&gt;3 taksit, 1.000-6.000 TL-&gt;6 taksit, 6.000-10.000 TL-&gt;6 taksit, 10.000 TL+ secili urun-&gt;9 taksit. En ust dilim alindi DUZELTME (23 Agustos 2026): vade_ay=9 -&gt; taksit_sayisi=9. kademeli taksit (3/6/9), Alisveris Puani Kampanyasi - vade yok. Taksit ADEDI ile finansman SURESI ayni alan degildir. | BULGU (26 Agustos 2026, Faz 6 kanit taramasi): kaynak sayfa SU AN yalnizca 3 kademeli taksit sistemi gosteriyor (100-1.000 TL-&gt;3, 1.000-6.000 TL-&gt;3, 6.000 TL+-&gt;6) - kayitli 4. kademe ('10.000 TL+ -&gt; 9 taksit') artik metinde YOK. Kampanya rotasyona ugramis olabilir, taksit_sayisi=9/finansman_tutari=10000 icin kanit eklenemedi - yeniden dogrulanmali.</t>
-        </is>
-      </c>
-      <c r="V55" t="n">
-        <v>9</v>
+          <t>Kademeli sistem: 100-1.000 TL-&gt;3 taksit, 1.000-6.000 TL-&gt;6 taksit, 6.000-10.000 TL-&gt;6 taksit, 10.000 TL+ secili urun-&gt;9 taksit. En ust dilim alindi DUZELTME (23 Agustos 2026): vade_ay=9 -&gt; taksit_sayisi=9. kademeli taksit (3/6/9), Alisveris Puani Kampanyasi - vade yok. Taksit ADEDI ile finansman SURESI ayni alan degildir. | BULGU (26 Agustos 2026, Faz 6 kanit taramasi): kaynak sayfa SU AN yalnizca 3 kademeli taksit sistemi gosteriyor (100-1.000 TL-&gt;3, 1.000-6.000 TL-&gt;3, 6.000 TL+-&gt;6) - kayitli 4. kademe ('10.000 TL+ -&gt; 9 taksit') artik metinde YOK. Kampanya rotasyona ugramis olabilir, taksit_sayisi=9/finansman_tutari=10000 icin kanit eklenemedi - yeniden dogrulanmali. | SILINDI (26 Agustos 2026): taksit_sayisi/finansman_tutari kanitsiz oldugu icin bosaltildi.</t>
+        </is>
       </c>
       <c r="X55" s="2" t="inlineStr">
         <is>
@@ -5989,15 +5944,9 @@
           <t>www.dunyakatilim.com.tr/kampanyalar/n11</t>
         </is>
       </c>
-      <c r="F56" s="21" t="n">
-        <v>0</v>
-      </c>
+      <c r="F56" s="21" t="n"/>
       <c r="G56" s="21" t="n"/>
-      <c r="H56" s="19" t="inlineStr">
-        <is>
-          <t>belirsiz</t>
-        </is>
-      </c>
+      <c r="H56" s="19" t="n"/>
       <c r="I56" s="22" t="n"/>
       <c r="J56" s="21" t="n">
         <v>2000</v>

</xml_diff>